<commit_message>
Daily scrape output - 2026-06-27
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F70"/>
+  <dimension ref="A1:F72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1148,10 +1148,10 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>10.74</v>
+        <v>10.75</v>
       </c>
       <c r="F28" t="n">
-        <v>2.74</v>
+        <v>2.86</v>
       </c>
     </row>
     <row r="29">
@@ -1226,10 +1226,10 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>9.210000000000001</v>
+        <v>8.960000000000001</v>
       </c>
       <c r="F31" t="n">
-        <v>-1.06</v>
+        <v>-1.04</v>
       </c>
     </row>
     <row r="32">
@@ -1252,7 +1252,7 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>8.69</v>
+        <v>8.449999999999999</v>
       </c>
       <c r="F32" t="n">
         <v>1.71</v>
@@ -1278,10 +1278,10 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>8.82</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="F33" t="n">
-        <v>1.15</v>
+        <v>1.66</v>
       </c>
     </row>
     <row r="34">
@@ -1356,7 +1356,7 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>10.09</v>
+        <v>10.07</v>
       </c>
       <c r="F36" t="n">
         <v>-4.25</v>
@@ -1408,10 +1408,10 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>9.640000000000001</v>
+        <v>9.65</v>
       </c>
       <c r="F38" t="n">
-        <v>0.49</v>
+        <v>0.51</v>
       </c>
     </row>
     <row r="39">
@@ -1512,10 +1512,10 @@
         </is>
       </c>
       <c r="E42" t="n">
-        <v>9.83</v>
+        <v>9.630000000000001</v>
       </c>
       <c r="F42" t="n">
-        <v>0.02</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="43">
@@ -1564,10 +1564,10 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>10.24</v>
+        <v>10.28</v>
       </c>
       <c r="F44" t="n">
-        <v>0.83</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="45">
@@ -1668,10 +1668,10 @@
         </is>
       </c>
       <c r="E48" t="n">
-        <v>11</v>
+        <v>11.16</v>
       </c>
       <c r="F48" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.55</v>
       </c>
     </row>
     <row r="49">
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E52" t="n">
-        <v>10.83</v>
+        <v>11.02</v>
       </c>
       <c r="F52" t="n">
-        <v>2.15</v>
+        <v>1.84</v>
       </c>
     </row>
     <row r="53">
@@ -1798,10 +1798,10 @@
         </is>
       </c>
       <c r="E53" t="n">
-        <v>10.63</v>
+        <v>10.62</v>
       </c>
       <c r="F53" t="n">
-        <v>-0.02</v>
+        <v>-0.09</v>
       </c>
     </row>
     <row r="54">
@@ -1850,10 +1850,10 @@
         </is>
       </c>
       <c r="E55" t="n">
-        <v>10.46</v>
+        <v>10.5</v>
       </c>
       <c r="F55" t="n">
-        <v>1.63</v>
+        <v>1.11</v>
       </c>
     </row>
     <row r="56">
@@ -1867,19 +1867,19 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Sundsvall</t>
+          <t>Nordic United</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Ostersunds FK</t>
+          <t>Oddevold</t>
         </is>
       </c>
       <c r="E56" t="n">
-        <v>9.83</v>
+        <v>9.56</v>
       </c>
       <c r="F56" t="n">
-        <v>-1.18</v>
+        <v>-0.35</v>
       </c>
     </row>
     <row r="57">
@@ -1893,45 +1893,45 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Varbergs BoIS</t>
+          <t>Sundsvall</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Osters</t>
+          <t>Ostersunds FK</t>
         </is>
       </c>
       <c r="E57" t="n">
-        <v>10.07</v>
+        <v>9.84</v>
       </c>
       <c r="F57" t="n">
-        <v>1.71</v>
+        <v>-1.16</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="n">
-        <v>46201</v>
+        <v>46200</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Sweden - Superettan</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Athletic Club</t>
+          <t>Varbergs BoIS</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Avai</t>
+          <t>Osters</t>
         </is>
       </c>
       <c r="E58" t="n">
-        <v>10.34</v>
+        <v>10.07</v>
       </c>
       <c r="F58" t="n">
-        <v>1.65</v>
+        <v>1.71</v>
       </c>
     </row>
     <row r="59">
@@ -1945,19 +1945,19 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Atletico Goianiense</t>
+          <t>Athletic Club</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Ponte Preta</t>
+          <t>Avai</t>
         </is>
       </c>
       <c r="E59" t="n">
-        <v>10.74</v>
+        <v>10.34</v>
       </c>
       <c r="F59" t="n">
-        <v>2.74</v>
+        <v>1.65</v>
       </c>
     </row>
     <row r="60">
@@ -1971,19 +1971,19 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Fortaleza</t>
+          <t>Atletico Goianiense</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Sport Recife</t>
+          <t>Ponte Preta</t>
         </is>
       </c>
       <c r="E60" t="n">
-        <v>10.34</v>
+        <v>10.74</v>
       </c>
       <c r="F60" t="n">
-        <v>1.9</v>
+        <v>2.74</v>
       </c>
     </row>
     <row r="61">
@@ -1997,19 +1997,19 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Juventude</t>
+          <t>Fortaleza</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Ceara</t>
+          <t>Sport Recife</t>
         </is>
       </c>
       <c r="E61" t="n">
-        <v>9.949999999999999</v>
+        <v>10.34</v>
       </c>
       <c r="F61" t="n">
-        <v>1.1</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="62">
@@ -2023,19 +2023,19 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Nautico</t>
+          <t>Juventude</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Goias</t>
+          <t>Ceara</t>
         </is>
       </c>
       <c r="E62" t="n">
-        <v>10.35</v>
+        <v>9.949999999999999</v>
       </c>
       <c r="F62" t="n">
-        <v>1.73</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="63">
@@ -2044,24 +2044,24 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>FIFA - World Cup</t>
+          <t>Brazil - Serie B</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Algeria</t>
+          <t>Nautico</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>Goias</t>
         </is>
       </c>
       <c r="E63" t="n">
-        <v>8.02</v>
+        <v>10.35</v>
       </c>
       <c r="F63" t="n">
-        <v>-0.16</v>
+        <v>1.73</v>
       </c>
     </row>
     <row r="64">
@@ -2075,19 +2075,19 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Algeria</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Austria</t>
         </is>
       </c>
       <c r="E64" t="n">
-        <v>8.74</v>
+        <v>7.82</v>
       </c>
       <c r="F64" t="n">
-        <v>-3.17</v>
+        <v>-0.16</v>
       </c>
     </row>
     <row r="65">
@@ -2101,19 +2101,19 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E65" t="n">
-        <v>9.460000000000001</v>
+        <v>8.4</v>
       </c>
       <c r="F65" t="n">
-        <v>-2.42</v>
+        <v>-2.99</v>
       </c>
     </row>
     <row r="66">
@@ -2122,24 +2122,24 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Finland - Ykkosliiga</t>
+          <t>FIFA - World Cup</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>KaPa</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>JaPS</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="E66" t="n">
-        <v>10.1</v>
+        <v>9.359999999999999</v>
       </c>
       <c r="F66" t="n">
-        <v>0.96</v>
+        <v>-2.5</v>
       </c>
     </row>
     <row r="67">
@@ -2148,24 +2148,24 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Finland - Ykkosliiga</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Landskrona</t>
+          <t>KaPa</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Varnamo</t>
+          <t>JaPS</t>
         </is>
       </c>
       <c r="E67" t="n">
-        <v>10.35</v>
+        <v>10.1</v>
       </c>
       <c r="F67" t="n">
-        <v>0.67</v>
+        <v>0.96</v>
       </c>
     </row>
     <row r="68">
@@ -2179,19 +2179,19 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Norrkoping</t>
+          <t>Landskrona</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Norrby</t>
+          <t>Varnamo</t>
         </is>
       </c>
       <c r="E68" t="n">
-        <v>10.11</v>
+        <v>10.35</v>
       </c>
       <c r="F68" t="n">
-        <v>2.54</v>
+        <v>0.67</v>
       </c>
     </row>
     <row r="69">
@@ -2205,45 +2205,97 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Sandvikens IF</t>
+          <t>Norrkoping</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Helsingborgs</t>
+          <t>Norrby</t>
         </is>
       </c>
       <c r="E69" t="n">
-        <v>10.5</v>
+        <v>10.11</v>
       </c>
       <c r="F69" t="n">
-        <v>0.8100000000000001</v>
+        <v>2.54</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="1" t="n">
+        <v>46201</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Sandvikens IF</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Helsingborgs</t>
+        </is>
+      </c>
+      <c r="E70" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="F70" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="1" t="n">
         <v>46202</v>
       </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>FIFA - World Cup</t>
-        </is>
-      </c>
-      <c r="C70" t="inlineStr">
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
         <is>
           <t>Brazil</t>
         </is>
       </c>
-      <c r="D70" t="inlineStr">
+      <c r="D71" t="inlineStr">
         <is>
           <t>Japan</t>
         </is>
       </c>
-      <c r="E70" t="n">
-        <v>9.18</v>
-      </c>
-      <c r="F70" t="n">
-        <v>1.6</v>
+      <c r="E71" t="n">
+        <v>9.26</v>
+      </c>
+      <c r="F71" t="n">
+        <v>1.55</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="1" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Botafogo SP</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>CRB</t>
+        </is>
+      </c>
+      <c r="E72" t="n">
+        <v>10.65</v>
+      </c>
+      <c r="F72" t="n">
+        <v>1.18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily scrape output - 2026-06-28
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F72"/>
+  <dimension ref="A1:F76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1954,10 +1954,10 @@
         </is>
       </c>
       <c r="E59" t="n">
-        <v>10.34</v>
+        <v>10.33</v>
       </c>
       <c r="F59" t="n">
-        <v>1.65</v>
+        <v>1.68</v>
       </c>
     </row>
     <row r="60">
@@ -1980,10 +1980,10 @@
         </is>
       </c>
       <c r="E60" t="n">
-        <v>10.74</v>
+        <v>10.75</v>
       </c>
       <c r="F60" t="n">
-        <v>2.74</v>
+        <v>2.72</v>
       </c>
     </row>
     <row r="61">
@@ -2058,10 +2058,10 @@
         </is>
       </c>
       <c r="E63" t="n">
-        <v>10.35</v>
+        <v>10.36</v>
       </c>
       <c r="F63" t="n">
-        <v>1.73</v>
+        <v>1.72</v>
       </c>
     </row>
     <row r="64">
@@ -2136,10 +2136,10 @@
         </is>
       </c>
       <c r="E66" t="n">
-        <v>9.359999999999999</v>
+        <v>9.65</v>
       </c>
       <c r="F66" t="n">
-        <v>-2.5</v>
+        <v>-2.69</v>
       </c>
     </row>
     <row r="67">
@@ -2214,10 +2214,10 @@
         </is>
       </c>
       <c r="E69" t="n">
-        <v>10.11</v>
+        <v>10.13</v>
       </c>
       <c r="F69" t="n">
-        <v>2.54</v>
+        <v>2.53</v>
       </c>
     </row>
     <row r="70">
@@ -2266,7 +2266,7 @@
         </is>
       </c>
       <c r="E71" t="n">
-        <v>9.26</v>
+        <v>9.27</v>
       </c>
       <c r="F71" t="n">
         <v>1.55</v>
@@ -2274,28 +2274,132 @@
     </row>
     <row r="72">
       <c r="A72" s="1" t="n">
+        <v>46202</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Paraguay</t>
+        </is>
+      </c>
+      <c r="E72" t="n">
+        <v>9.24</v>
+      </c>
+      <c r="F72" t="n">
+        <v>3.42</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="1" t="n">
         <v>46203</v>
       </c>
-      <c r="B72" t="inlineStr">
+      <c r="B73" t="inlineStr">
         <is>
           <t>Brazil - Serie B</t>
         </is>
       </c>
-      <c r="C72" t="inlineStr">
+      <c r="C73" t="inlineStr">
         <is>
           <t>Botafogo SP</t>
         </is>
       </c>
-      <c r="D72" t="inlineStr">
+      <c r="D73" t="inlineStr">
         <is>
           <t>CRB</t>
         </is>
       </c>
-      <c r="E72" t="n">
-        <v>10.65</v>
-      </c>
-      <c r="F72" t="n">
-        <v>1.18</v>
+      <c r="E73" t="n">
+        <v>10.33</v>
+      </c>
+      <c r="F73" t="n">
+        <v>1.19</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="1" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="E74" t="n">
+        <v>9.19</v>
+      </c>
+      <c r="F74" t="n">
+        <v>3.11</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="1" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Ivory Coast</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Norway</t>
+        </is>
+      </c>
+      <c r="E75" t="n">
+        <v>8.77</v>
+      </c>
+      <c r="F75" t="n">
+        <v>-1.2</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="1" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Morocco</t>
+        </is>
+      </c>
+      <c r="E76" t="n">
+        <v>9.18</v>
+      </c>
+      <c r="F76" t="n">
+        <v>0.83</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily scrape output - 2026-06-29
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F76"/>
+  <dimension ref="A1:F87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2266,10 +2266,10 @@
         </is>
       </c>
       <c r="E71" t="n">
-        <v>9.27</v>
+        <v>8.98</v>
       </c>
       <c r="F71" t="n">
-        <v>1.55</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="72">
@@ -2292,36 +2292,36 @@
         </is>
       </c>
       <c r="E72" t="n">
-        <v>9.24</v>
+        <v>9.26</v>
       </c>
       <c r="F72" t="n">
-        <v>3.42</v>
+        <v>3.77</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="1" t="n">
-        <v>46203</v>
+        <v>46202</v>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Iceland - 1. Deild</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Botafogo SP</t>
+          <t>Afturelding</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>CRB</t>
+          <t>Aegir</t>
         </is>
       </c>
       <c r="E73" t="n">
-        <v>10.33</v>
+        <v>12.09</v>
       </c>
       <c r="F73" t="n">
-        <v>1.19</v>
+        <v>4.49</v>
       </c>
     </row>
     <row r="74">
@@ -2330,24 +2330,24 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>FIFA - World Cup</t>
+          <t>Brazil - Serie B</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Botafogo SP</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>CRB</t>
         </is>
       </c>
       <c r="E74" t="n">
-        <v>9.19</v>
+        <v>10.3</v>
       </c>
       <c r="F74" t="n">
-        <v>3.11</v>
+        <v>1.45</v>
       </c>
     </row>
     <row r="75">
@@ -2361,19 +2361,19 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Ivory Coast</t>
+          <t>France</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Norway</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="E75" t="n">
-        <v>8.77</v>
+        <v>9.23</v>
       </c>
       <c r="F75" t="n">
-        <v>-1.2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="76">
@@ -2387,19 +2387,305 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
+          <t>Ivory Coast</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Norway</t>
+        </is>
+      </c>
+      <c r="E76" t="n">
+        <v>9.039999999999999</v>
+      </c>
+      <c r="F76" t="n">
+        <v>-1.36</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="1" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
           <t>Netherlands</t>
         </is>
       </c>
-      <c r="D76" t="inlineStr">
+      <c r="D77" t="inlineStr">
         <is>
           <t>Morocco</t>
         </is>
       </c>
-      <c r="E76" t="n">
+      <c r="E77" t="n">
+        <v>8.94</v>
+      </c>
+      <c r="F77" t="n">
+        <v>0.87</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Belgium</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Senegal</t>
+        </is>
+      </c>
+      <c r="E78" t="n">
+        <v>9.07</v>
+      </c>
+      <c r="F78" t="n">
+        <v>0.55</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>DR Congo</t>
+        </is>
+      </c>
+      <c r="E79" t="n">
+        <v>9.609999999999999</v>
+      </c>
+      <c r="F79" t="n">
+        <v>4.26</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="E80" t="n">
+        <v>8.15</v>
+      </c>
+      <c r="F80" t="n">
+        <v>0.65</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="1" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Croatia</t>
+        </is>
+      </c>
+      <c r="E81" t="n">
+        <v>8.529999999999999</v>
+      </c>
+      <c r="F81" t="n">
+        <v>1.48</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="1" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="E82" t="n">
         <v>9.18</v>
       </c>
-      <c r="F76" t="n">
-        <v>0.83</v>
+      <c r="F82" t="n">
+        <v>3.25</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="1" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Bosnia and Herzegovina</t>
+        </is>
+      </c>
+      <c r="E83" t="n">
+        <v>9.32</v>
+      </c>
+      <c r="F83" t="n">
+        <v>3.02</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="1" t="n">
+        <v>46206</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Cape Verde</t>
+        </is>
+      </c>
+      <c r="E84" t="n">
+        <v>8.890000000000001</v>
+      </c>
+      <c r="F84" t="n">
+        <v>4.3</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="1" t="n">
+        <v>46206</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Egypt</t>
+        </is>
+      </c>
+      <c r="E85" t="n">
+        <v>8.49</v>
+      </c>
+      <c r="F85" t="n">
+        <v>-0.42</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="1" t="n">
+        <v>46206</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Algeria</t>
+        </is>
+      </c>
+      <c r="E86" t="n">
+        <v>9.16</v>
+      </c>
+      <c r="F86" t="n">
+        <v>1.34</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="1" t="n">
+        <v>46207</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Ghana</t>
+        </is>
+      </c>
+      <c r="E87" t="n">
+        <v>8.630000000000001</v>
+      </c>
+      <c r="F87" t="n">
+        <v>2.44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily scrape output - 2026-06-30
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -2370,10 +2370,10 @@
         </is>
       </c>
       <c r="E75" t="n">
-        <v>9.23</v>
+        <v>9.550000000000001</v>
       </c>
       <c r="F75" t="n">
-        <v>3</v>
+        <v>3.26</v>
       </c>
     </row>
     <row r="76">
@@ -2396,10 +2396,10 @@
         </is>
       </c>
       <c r="E76" t="n">
-        <v>9.039999999999999</v>
+        <v>9.18</v>
       </c>
       <c r="F76" t="n">
-        <v>-1.36</v>
+        <v>-1.46</v>
       </c>
     </row>
     <row r="77">
@@ -2448,10 +2448,10 @@
         </is>
       </c>
       <c r="E78" t="n">
-        <v>9.07</v>
+        <v>8.720000000000001</v>
       </c>
       <c r="F78" t="n">
-        <v>0.55</v>
+        <v>0.58</v>
       </c>
     </row>
     <row r="79">
@@ -2474,10 +2474,10 @@
         </is>
       </c>
       <c r="E79" t="n">
-        <v>9.609999999999999</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="F79" t="n">
-        <v>4.26</v>
+        <v>4.51</v>
       </c>
     </row>
     <row r="80">
@@ -2500,10 +2500,10 @@
         </is>
       </c>
       <c r="E80" t="n">
-        <v>8.15</v>
+        <v>7.68</v>
       </c>
       <c r="F80" t="n">
-        <v>0.65</v>
+        <v>0.63</v>
       </c>
     </row>
     <row r="81">
@@ -2526,10 +2526,10 @@
         </is>
       </c>
       <c r="E81" t="n">
-        <v>8.529999999999999</v>
+        <v>8.56</v>
       </c>
       <c r="F81" t="n">
-        <v>1.48</v>
+        <v>1.53</v>
       </c>
     </row>
     <row r="82">
@@ -2578,10 +2578,10 @@
         </is>
       </c>
       <c r="E83" t="n">
-        <v>9.32</v>
+        <v>9.31</v>
       </c>
       <c r="F83" t="n">
-        <v>3.02</v>
+        <v>2.92</v>
       </c>
     </row>
     <row r="84">
@@ -2630,10 +2630,10 @@
         </is>
       </c>
       <c r="E85" t="n">
-        <v>8.49</v>
+        <v>8.58</v>
       </c>
       <c r="F85" t="n">
-        <v>-0.42</v>
+        <v>-0.44</v>
       </c>
     </row>
     <row r="86">
@@ -2659,7 +2659,7 @@
         <v>9.16</v>
       </c>
       <c r="F86" t="n">
-        <v>1.34</v>
+        <v>1.22</v>
       </c>
     </row>
     <row r="87">
@@ -2682,10 +2682,10 @@
         </is>
       </c>
       <c r="E87" t="n">
-        <v>8.630000000000001</v>
+        <v>8.69</v>
       </c>
       <c r="F87" t="n">
-        <v>2.44</v>
+        <v>2.46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily scrape output - 2026-07-01
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F87"/>
+  <dimension ref="A1:F88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2448,10 +2448,10 @@
         </is>
       </c>
       <c r="E78" t="n">
-        <v>8.720000000000001</v>
+        <v>9.32</v>
       </c>
       <c r="F78" t="n">
-        <v>0.58</v>
+        <v>0.47</v>
       </c>
     </row>
     <row r="79">
@@ -2474,10 +2474,10 @@
         </is>
       </c>
       <c r="E79" t="n">
-        <v>9.619999999999999</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="F79" t="n">
-        <v>4.51</v>
+        <v>4.6</v>
       </c>
     </row>
     <row r="80">
@@ -2529,7 +2529,7 @@
         <v>8.56</v>
       </c>
       <c r="F81" t="n">
-        <v>1.53</v>
+        <v>1.45</v>
       </c>
     </row>
     <row r="82">
@@ -2552,10 +2552,10 @@
         </is>
       </c>
       <c r="E82" t="n">
-        <v>9.18</v>
+        <v>9.210000000000001</v>
       </c>
       <c r="F82" t="n">
-        <v>3.25</v>
+        <v>3.42</v>
       </c>
     </row>
     <row r="83">
@@ -2578,10 +2578,10 @@
         </is>
       </c>
       <c r="E83" t="n">
-        <v>9.31</v>
+        <v>9.65</v>
       </c>
       <c r="F83" t="n">
-        <v>2.92</v>
+        <v>3.26</v>
       </c>
     </row>
     <row r="84">
@@ -2607,7 +2607,7 @@
         <v>8.890000000000001</v>
       </c>
       <c r="F84" t="n">
-        <v>4.3</v>
+        <v>4.31</v>
       </c>
     </row>
     <row r="85">
@@ -2659,7 +2659,7 @@
         <v>9.16</v>
       </c>
       <c r="F86" t="n">
-        <v>1.22</v>
+        <v>1.39</v>
       </c>
     </row>
     <row r="87">
@@ -2673,19 +2673,45 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Morocco</t>
+        </is>
+      </c>
+      <c r="E87" t="n">
+        <v>9.07</v>
+      </c>
+      <c r="F87" t="n">
+        <v>-1.59</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="1" t="n">
+        <v>46207</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
           <t>Colombia</t>
         </is>
       </c>
-      <c r="D87" t="inlineStr">
+      <c r="D88" t="inlineStr">
         <is>
           <t>Ghana</t>
         </is>
       </c>
-      <c r="E87" t="n">
+      <c r="E88" t="n">
         <v>8.69</v>
       </c>
-      <c r="F87" t="n">
-        <v>2.46</v>
+      <c r="F88" t="n">
+        <v>2.44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily scrape output - 2026-07-02
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F88"/>
+  <dimension ref="A1:F93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2512,24 +2512,24 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>FIFA - World Cup</t>
+          <t>Brazil - Serie B</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Cuiaba</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Croatia</t>
+          <t>America Mineiro</t>
         </is>
       </c>
       <c r="E81" t="n">
-        <v>8.56</v>
+        <v>9.82</v>
       </c>
       <c r="F81" t="n">
-        <v>1.45</v>
+        <v>1.35</v>
       </c>
     </row>
     <row r="82">
@@ -2543,19 +2543,19 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>Croatia</t>
         </is>
       </c>
       <c r="E82" t="n">
-        <v>9.210000000000001</v>
+        <v>8.94</v>
       </c>
       <c r="F82" t="n">
-        <v>3.42</v>
+        <v>1.83</v>
       </c>
     </row>
     <row r="83">
@@ -2569,24 +2569,24 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Bosnia and Herzegovina</t>
+          <t>Austria</t>
         </is>
       </c>
       <c r="E83" t="n">
-        <v>9.65</v>
+        <v>9</v>
       </c>
       <c r="F83" t="n">
-        <v>3.26</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="1" t="n">
-        <v>46206</v>
+        <v>46205</v>
       </c>
       <c r="B84" t="inlineStr">
         <is>
@@ -2595,45 +2595,45 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Cape Verde</t>
+          <t>Bosnia and Herzegovina</t>
         </is>
       </c>
       <c r="E84" t="n">
-        <v>8.890000000000001</v>
+        <v>9.65</v>
       </c>
       <c r="F84" t="n">
-        <v>4.31</v>
+        <v>3.26</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="1" t="n">
-        <v>46206</v>
+        <v>46205</v>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>FIFA - World Cup</t>
+          <t>Norway - 1st Division</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Lyn</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Egypt</t>
+          <t>Asane Fotball</t>
         </is>
       </c>
       <c r="E85" t="n">
-        <v>8.58</v>
+        <v>10.79</v>
       </c>
       <c r="F85" t="n">
-        <v>-0.44</v>
+        <v>2.43</v>
       </c>
     </row>
     <row r="86">
@@ -2642,29 +2642,29 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>FIFA - World Cup</t>
+          <t>Brazil - Serie B</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Switzerland</t>
+          <t>Fortaleza</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Algeria</t>
+          <t>Ponte Preta</t>
         </is>
       </c>
       <c r="E86" t="n">
-        <v>9.16</v>
+        <v>10.34</v>
       </c>
       <c r="F86" t="n">
-        <v>1.39</v>
+        <v>3.56</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="1" t="n">
-        <v>46207</v>
+        <v>46206</v>
       </c>
       <c r="B87" t="inlineStr">
         <is>
@@ -2673,45 +2673,175 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Morocco</t>
+          <t>Cape Verde</t>
         </is>
       </c>
       <c r="E87" t="n">
-        <v>9.07</v>
+        <v>8.92</v>
       </c>
       <c r="F87" t="n">
-        <v>-1.59</v>
+        <v>4.42</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="1" t="n">
+        <v>46206</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Egypt</t>
+        </is>
+      </c>
+      <c r="E88" t="n">
+        <v>8.58</v>
+      </c>
+      <c r="F88" t="n">
+        <v>-0.44</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="1" t="n">
+        <v>46206</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Algeria</t>
+        </is>
+      </c>
+      <c r="E89" t="n">
+        <v>9.050000000000001</v>
+      </c>
+      <c r="F89" t="n">
+        <v>0.99</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="1" t="n">
         <v>46207</v>
       </c>
-      <c r="B88" t="inlineStr">
-        <is>
-          <t>FIFA - World Cup</t>
-        </is>
-      </c>
-      <c r="C88" t="inlineStr">
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Morocco</t>
+        </is>
+      </c>
+      <c r="E90" t="n">
+        <v>9.07</v>
+      </c>
+      <c r="F90" t="n">
+        <v>-1.59</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="1" t="n">
+        <v>46207</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
         <is>
           <t>Colombia</t>
         </is>
       </c>
-      <c r="D88" t="inlineStr">
+      <c r="D91" t="inlineStr">
         <is>
           <t>Ghana</t>
         </is>
       </c>
-      <c r="E88" t="n">
+      <c r="E91" t="n">
         <v>8.69</v>
       </c>
-      <c r="F88" t="n">
-        <v>2.44</v>
+      <c r="F91" t="n">
+        <v>2.46</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="1" t="n">
+        <v>46207</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Paraguay</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="E92" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="F92" t="n">
+        <v>-4.66</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="1" t="n">
+        <v>46208</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Norway</t>
+        </is>
+      </c>
+      <c r="E93" t="n">
+        <v>8.74</v>
+      </c>
+      <c r="F93" t="n">
+        <v>1.15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily scrape output - 2026-07-03
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F93"/>
+  <dimension ref="A1:F121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2682,10 +2682,10 @@
         </is>
       </c>
       <c r="E87" t="n">
-        <v>8.92</v>
+        <v>8.76</v>
       </c>
       <c r="F87" t="n">
-        <v>4.42</v>
+        <v>4.37</v>
       </c>
     </row>
     <row r="88">
@@ -2708,10 +2708,10 @@
         </is>
       </c>
       <c r="E88" t="n">
-        <v>8.58</v>
+        <v>8.67</v>
       </c>
       <c r="F88" t="n">
-        <v>-0.44</v>
+        <v>-0.54</v>
       </c>
     </row>
     <row r="89">
@@ -2742,106 +2742,834 @@
     </row>
     <row r="90">
       <c r="A90" s="1" t="n">
-        <v>46207</v>
+        <v>46206</v>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>FIFA - World Cup</t>
+          <t>Finland - Ykkosliiga</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>JaPS</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Morocco</t>
+          <t>SJK Akatemia</t>
         </is>
       </c>
       <c r="E90" t="n">
-        <v>9.07</v>
+        <v>10.4</v>
       </c>
       <c r="F90" t="n">
-        <v>-1.59</v>
+        <v>0.87</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="1" t="n">
-        <v>46207</v>
+        <v>46206</v>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>FIFA - World Cup</t>
+          <t>Finland - Ykkosliiga</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>KTP</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Ghana</t>
+          <t>JIPPO</t>
         </is>
       </c>
       <c r="E91" t="n">
-        <v>8.69</v>
+        <v>9.68</v>
       </c>
       <c r="F91" t="n">
-        <v>2.46</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="1" t="n">
-        <v>46207</v>
+        <v>46206</v>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>FIFA - World Cup</t>
+          <t>Iceland - 1. Deild</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Paraguay</t>
+          <t>Aegir</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Fylkir</t>
         </is>
       </c>
       <c r="E92" t="n">
-        <v>9.6</v>
+        <v>11.65</v>
       </c>
       <c r="F92" t="n">
-        <v>-4.66</v>
+        <v>-3.54</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="1" t="n">
+        <v>46206</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Iceland - 1. Deild</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>IR Reykjavik</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Afturelding</t>
+        </is>
+      </c>
+      <c r="E93" t="n">
+        <v>11.76</v>
+      </c>
+      <c r="F93" t="n">
+        <v>-1.09</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="1" t="n">
+        <v>46206</v>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Iceland - 1. Deild</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>UMF Njardvik</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Throttur Reykjavik</t>
+        </is>
+      </c>
+      <c r="E94" t="n">
+        <v>11.45</v>
+      </c>
+      <c r="F94" t="n">
+        <v>0.19</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="1" t="n">
+        <v>46206</v>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Kongsvinger</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Sogndal</t>
+        </is>
+      </c>
+      <c r="E95" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="F95" t="n">
+        <v>2.45</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="1" t="n">
+        <v>46206</v>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Ranheim</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Stabaek</t>
+        </is>
+      </c>
+      <c r="E96" t="n">
+        <v>11.28</v>
+      </c>
+      <c r="F96" t="n">
+        <v>-0.82</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="1" t="n">
+        <v>46206</v>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Raufoss</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Strommen</t>
+        </is>
+      </c>
+      <c r="E97" t="n">
+        <v>10.57</v>
+      </c>
+      <c r="F97" t="n">
+        <v>0.64</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="1" t="n">
+        <v>46207</v>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Criciuma</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Sport Recife</t>
+        </is>
+      </c>
+      <c r="E98" t="n">
+        <v>10.72</v>
+      </c>
+      <c r="F98" t="n">
+        <v>2.2</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="1" t="n">
+        <v>46207</v>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Goias</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Ceara</t>
+        </is>
+      </c>
+      <c r="E99" t="n">
+        <v>10.11</v>
+      </c>
+      <c r="F99" t="n">
+        <v>0.93</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="1" t="n">
+        <v>46207</v>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Gremio Novorizontino</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Atletico Goianiense</t>
+        </is>
+      </c>
+      <c r="E100" t="n">
+        <v>10.26</v>
+      </c>
+      <c r="F100" t="n">
+        <v>1.35</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="1" t="n">
+        <v>46207</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Londrina</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>CRB</t>
+        </is>
+      </c>
+      <c r="E101" t="n">
+        <v>10.57</v>
+      </c>
+      <c r="F101" t="n">
+        <v>-0.06</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="1" t="n">
+        <v>46207</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Morocco</t>
+        </is>
+      </c>
+      <c r="E102" t="n">
+        <v>8.85</v>
+      </c>
+      <c r="F102" t="n">
+        <v>-1.05</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="1" t="n">
+        <v>46207</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Ghana</t>
+        </is>
+      </c>
+      <c r="E103" t="n">
+        <v>8.82</v>
+      </c>
+      <c r="F103" t="n">
+        <v>2.61</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="1" t="n">
+        <v>46207</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Paraguay</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="E104" t="n">
+        <v>9.65</v>
+      </c>
+      <c r="F104" t="n">
+        <v>-4.72</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="1" t="n">
+        <v>46207</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>FC Lahti</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Gnistan</t>
+        </is>
+      </c>
+      <c r="E105" t="n">
+        <v>10.16</v>
+      </c>
+      <c r="F105" t="n">
+        <v>1.39</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="1" t="n">
+        <v>46207</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Jaro</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Ilves</t>
+        </is>
+      </c>
+      <c r="E106" t="n">
+        <v>9.609999999999999</v>
+      </c>
+      <c r="F106" t="n">
+        <v>-0.64</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="1" t="n">
+        <v>46207</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>SJK</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>TPS</t>
+        </is>
+      </c>
+      <c r="E107" t="n">
+        <v>10.28</v>
+      </c>
+      <c r="F107" t="n">
+        <v>2.45</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="1" t="n">
+        <v>46207</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>VPS</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>IFK Mariehamn</t>
+        </is>
+      </c>
+      <c r="E108" t="n">
+        <v>10.45</v>
+      </c>
+      <c r="F108" t="n">
+        <v>2.94</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="1" t="n">
+        <v>46207</v>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Finland - Ykkosliiga</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>EIF</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>PK-35</t>
+        </is>
+      </c>
+      <c r="E109" t="n">
+        <v>10.36</v>
+      </c>
+      <c r="F109" t="n">
+        <v>-0.17</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="1" t="n">
+        <v>46207</v>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Iceland - 1. Deild</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Leiknir Reykjavik</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Volsungur</t>
+        </is>
+      </c>
+      <c r="E110" t="n">
+        <v>11.61</v>
+      </c>
+      <c r="F110" t="n">
+        <v>2.92</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="1" t="n">
+        <v>46207</v>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Bryne</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Sandnes Ulf</t>
+        </is>
+      </c>
+      <c r="E111" t="n">
+        <v>10.85</v>
+      </c>
+      <c r="F111" t="n">
+        <v>1.48</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="1" t="n">
+        <v>46207</v>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Egersunds</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Moss</t>
+        </is>
+      </c>
+      <c r="E112" t="n">
+        <v>11.06</v>
+      </c>
+      <c r="F112" t="n">
+        <v>0.87</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="1" t="n">
+        <v>46207</v>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Hodd</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Stromsgodset</t>
+        </is>
+      </c>
+      <c r="E113" t="n">
+        <v>11</v>
+      </c>
+      <c r="F113" t="n">
+        <v>-3</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="1" t="n">
         <v>46208</v>
       </c>
-      <c r="B93" t="inlineStr">
-        <is>
-          <t>FIFA - World Cup</t>
-        </is>
-      </c>
-      <c r="C93" t="inlineStr">
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Nautico</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Juventude</t>
+        </is>
+      </c>
+      <c r="E114" t="n">
+        <v>10.26</v>
+      </c>
+      <c r="F114" t="n">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="1" t="n">
+        <v>46208</v>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
         <is>
           <t>Brazil</t>
         </is>
       </c>
-      <c r="D93" t="inlineStr">
+      <c r="D115" t="inlineStr">
         <is>
           <t>Norway</t>
         </is>
       </c>
-      <c r="E93" t="n">
-        <v>8.74</v>
-      </c>
-      <c r="F93" t="n">
-        <v>1.15</v>
+      <c r="E115" t="n">
+        <v>8.789999999999999</v>
+      </c>
+      <c r="F115" t="n">
+        <v>1.12</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="1" t="n">
+        <v>46208</v>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Finland - Ykkosliiga</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Mikkelin Palloilijat</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>FC Haka</t>
+        </is>
+      </c>
+      <c r="E116" t="n">
+        <v>10.55</v>
+      </c>
+      <c r="F116" t="n">
+        <v>-2.54</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="1" t="n">
+        <v>46208</v>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Odd BK</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Haugesund</t>
+        </is>
+      </c>
+      <c r="E117" t="n">
+        <v>10.95</v>
+      </c>
+      <c r="F117" t="n">
+        <v>0.83</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="1" t="n">
+        <v>46209</v>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Botafogo SP</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Avai</t>
+        </is>
+      </c>
+      <c r="E118" t="n">
+        <v>10.72</v>
+      </c>
+      <c r="F118" t="n">
+        <v>2.66</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="1" t="n">
+        <v>46209</v>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Vila Nova</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Sao Bernardo</t>
+        </is>
+      </c>
+      <c r="E119" t="n">
+        <v>10.22</v>
+      </c>
+      <c r="F119" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="1" t="n">
+        <v>46209</v>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="E120" t="n">
+        <v>8.449999999999999</v>
+      </c>
+      <c r="F120" t="n">
+        <v>-0.65</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="1" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Belgium</t>
+        </is>
+      </c>
+      <c r="E121" t="n">
+        <v>9.640000000000001</v>
+      </c>
+      <c r="F121" t="n">
+        <v>0.06</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily scrape output - 2026-07-04
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F121"/>
+  <dimension ref="A1:F122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2968,10 +2968,10 @@
         </is>
       </c>
       <c r="E98" t="n">
-        <v>10.72</v>
+        <v>10.82</v>
       </c>
       <c r="F98" t="n">
-        <v>2.2</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="99">
@@ -3020,10 +3020,10 @@
         </is>
       </c>
       <c r="E100" t="n">
-        <v>10.26</v>
+        <v>10.16</v>
       </c>
       <c r="F100" t="n">
-        <v>1.35</v>
+        <v>1.71</v>
       </c>
     </row>
     <row r="101">
@@ -3046,7 +3046,7 @@
         </is>
       </c>
       <c r="E101" t="n">
-        <v>10.57</v>
+        <v>10.59</v>
       </c>
       <c r="F101" t="n">
         <v>-0.06</v>
@@ -3072,10 +3072,10 @@
         </is>
       </c>
       <c r="E102" t="n">
-        <v>8.85</v>
+        <v>9.050000000000001</v>
       </c>
       <c r="F102" t="n">
-        <v>-1.05</v>
+        <v>-1.04</v>
       </c>
     </row>
     <row r="103">
@@ -3124,10 +3124,10 @@
         </is>
       </c>
       <c r="E104" t="n">
-        <v>9.65</v>
+        <v>9.550000000000001</v>
       </c>
       <c r="F104" t="n">
-        <v>-4.72</v>
+        <v>-4.66</v>
       </c>
     </row>
     <row r="105">
@@ -3202,10 +3202,10 @@
         </is>
       </c>
       <c r="E107" t="n">
-        <v>10.28</v>
+        <v>10.22</v>
       </c>
       <c r="F107" t="n">
-        <v>2.45</v>
+        <v>2.43</v>
       </c>
     </row>
     <row r="108">
@@ -3231,7 +3231,7 @@
         <v>10.45</v>
       </c>
       <c r="F108" t="n">
-        <v>2.94</v>
+        <v>2.96</v>
       </c>
     </row>
     <row r="109">
@@ -3332,10 +3332,10 @@
         </is>
       </c>
       <c r="E112" t="n">
-        <v>11.06</v>
+        <v>11</v>
       </c>
       <c r="F112" t="n">
-        <v>0.87</v>
+        <v>0.88</v>
       </c>
     </row>
     <row r="113">
@@ -3358,10 +3358,10 @@
         </is>
       </c>
       <c r="E113" t="n">
-        <v>11</v>
+        <v>11.09</v>
       </c>
       <c r="F113" t="n">
-        <v>-3</v>
+        <v>-3.01</v>
       </c>
     </row>
     <row r="114">
@@ -3410,7 +3410,7 @@
         </is>
       </c>
       <c r="E115" t="n">
-        <v>8.789999999999999</v>
+        <v>8.82</v>
       </c>
       <c r="F115" t="n">
         <v>1.12</v>
@@ -3540,10 +3540,10 @@
         </is>
       </c>
       <c r="E120" t="n">
-        <v>8.449999999999999</v>
+        <v>8.25</v>
       </c>
       <c r="F120" t="n">
-        <v>-0.65</v>
+        <v>-0.97</v>
       </c>
     </row>
     <row r="121">
@@ -3552,23 +3552,49 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>FIFA - World Cup</t>
+          <t>Brazil - Serie B</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
+          <t>Athletic Club</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Operario Ferroviario</t>
+        </is>
+      </c>
+      <c r="E121" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="F121" t="n">
+        <v>0.89</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="1" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="D121" t="inlineStr">
+      <c r="D122" t="inlineStr">
         <is>
           <t>Belgium</t>
         </is>
       </c>
-      <c r="E121" t="n">
-        <v>9.640000000000001</v>
-      </c>
-      <c r="F121" t="n">
+      <c r="E122" t="n">
+        <v>9.65</v>
+      </c>
+      <c r="F122" t="n">
         <v>0.06</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily scrape output - 2026-07-05
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F122"/>
+  <dimension ref="A1:F124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3410,10 +3410,10 @@
         </is>
       </c>
       <c r="E115" t="n">
-        <v>8.82</v>
+        <v>9.23</v>
       </c>
       <c r="F115" t="n">
-        <v>1.12</v>
+        <v>1.17</v>
       </c>
     </row>
     <row r="116">
@@ -3436,10 +3436,10 @@
         </is>
       </c>
       <c r="E116" t="n">
-        <v>10.55</v>
+        <v>10.36</v>
       </c>
       <c r="F116" t="n">
-        <v>-2.54</v>
+        <v>-1.92</v>
       </c>
     </row>
     <row r="117">
@@ -3517,7 +3517,7 @@
         <v>10.22</v>
       </c>
       <c r="F119" t="n">
-        <v>2</v>
+        <v>2.05</v>
       </c>
     </row>
     <row r="120">
@@ -3540,10 +3540,10 @@
         </is>
       </c>
       <c r="E120" t="n">
-        <v>8.25</v>
+        <v>8.27</v>
       </c>
       <c r="F120" t="n">
-        <v>-0.97</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="121">
@@ -3583,19 +3583,71 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Egypt</t>
+        </is>
+      </c>
+      <c r="E122" t="n">
+        <v>8.43</v>
+      </c>
+      <c r="F122" t="n">
+        <v>2.55</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="1" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="E123" t="n">
+        <v>8.76</v>
+      </c>
+      <c r="F123" t="n">
+        <v>-0.62</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="1" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="D122" t="inlineStr">
+      <c r="D124" t="inlineStr">
         <is>
           <t>Belgium</t>
         </is>
       </c>
-      <c r="E122" t="n">
-        <v>9.65</v>
-      </c>
-      <c r="F122" t="n">
-        <v>0.06</v>
+      <c r="E124" t="n">
+        <v>9.69</v>
+      </c>
+      <c r="F124" t="n">
+        <v>0.17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily scrape output - 2026-07-06
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F124"/>
+  <dimension ref="A1:F126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3488,10 +3488,10 @@
         </is>
       </c>
       <c r="E118" t="n">
-        <v>10.72</v>
+        <v>10.7</v>
       </c>
       <c r="F118" t="n">
-        <v>2.66</v>
+        <v>2.48</v>
       </c>
     </row>
     <row r="119">
@@ -3517,7 +3517,7 @@
         <v>10.22</v>
       </c>
       <c r="F119" t="n">
-        <v>2.05</v>
+        <v>2</v>
       </c>
     </row>
     <row r="120">
@@ -3548,28 +3548,28 @@
     </row>
     <row r="121">
       <c r="A121" s="1" t="n">
-        <v>46210</v>
+        <v>46209</v>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>FIFA - World Cup</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Athletic Club</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Operario Ferroviario</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="E121" t="n">
-        <v>10.3</v>
+        <v>9.859999999999999</v>
       </c>
       <c r="F121" t="n">
-        <v>0.89</v>
+        <v>-1.54</v>
       </c>
     </row>
     <row r="122">
@@ -3578,24 +3578,24 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>FIFA - World Cup</t>
+          <t>Brazil - Serie B</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Athletic Club</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Egypt</t>
+          <t>Operario Ferroviario</t>
         </is>
       </c>
       <c r="E122" t="n">
-        <v>8.43</v>
+        <v>10.29</v>
       </c>
       <c r="F122" t="n">
-        <v>2.55</v>
+        <v>1.18</v>
       </c>
     </row>
     <row r="123">
@@ -3609,19 +3609,19 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Switzerland</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Egypt</t>
         </is>
       </c>
       <c r="E123" t="n">
-        <v>8.76</v>
+        <v>8.210000000000001</v>
       </c>
       <c r="F123" t="n">
-        <v>-0.62</v>
+        <v>2.34</v>
       </c>
     </row>
     <row r="124">
@@ -3635,19 +3635,71 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="E124" t="n">
+        <v>8.81</v>
+      </c>
+      <c r="F124" t="n">
+        <v>-0.62</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="1" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="D124" t="inlineStr">
+      <c r="D125" t="inlineStr">
         <is>
           <t>Belgium</t>
         </is>
       </c>
-      <c r="E124" t="n">
-        <v>9.69</v>
-      </c>
-      <c r="F124" t="n">
-        <v>0.17</v>
+      <c r="E125" t="n">
+        <v>10.05</v>
+      </c>
+      <c r="F125" t="n">
+        <v>0.13</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="1" t="n">
+        <v>46212</v>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Morocco</t>
+        </is>
+      </c>
+      <c r="E126" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="F126" t="n">
+        <v>2.52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily scrape output - 2026-07-07
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F126"/>
+  <dimension ref="A1:F127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3592,10 +3592,10 @@
         </is>
       </c>
       <c r="E122" t="n">
-        <v>10.29</v>
+        <v>10.49</v>
       </c>
       <c r="F122" t="n">
-        <v>1.18</v>
+        <v>0.9399999999999999</v>
       </c>
     </row>
     <row r="123">
@@ -3618,10 +3618,10 @@
         </is>
       </c>
       <c r="E123" t="n">
-        <v>8.210000000000001</v>
+        <v>8.81</v>
       </c>
       <c r="F123" t="n">
-        <v>2.34</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="124">
@@ -3644,10 +3644,10 @@
         </is>
       </c>
       <c r="E124" t="n">
-        <v>8.81</v>
+        <v>9.06</v>
       </c>
       <c r="F124" t="n">
-        <v>-0.62</v>
+        <v>-0.38</v>
       </c>
     </row>
     <row r="125">
@@ -3696,10 +3696,36 @@
         </is>
       </c>
       <c r="E126" t="n">
-        <v>9.1</v>
+        <v>9.48</v>
       </c>
       <c r="F126" t="n">
-        <v>2.52</v>
+        <v>2.55</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="1" t="n">
+        <v>46214</v>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Norway</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="E127" t="n">
+        <v>9.539999999999999</v>
+      </c>
+      <c r="F127" t="n">
+        <v>-1.13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily scrape output - 2026-07-08
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F127"/>
+  <dimension ref="A1:F129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3678,54 +3678,106 @@
     </row>
     <row r="126">
       <c r="A126" s="1" t="n">
-        <v>46212</v>
+        <v>46211</v>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>FIFA - World Cup</t>
+          <t>Brazil - Serie B</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Ponte Preta</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Morocco</t>
+          <t>Criciuma</t>
         </is>
       </c>
       <c r="E126" t="n">
-        <v>9.48</v>
+        <v>10.64</v>
       </c>
       <c r="F126" t="n">
-        <v>2.55</v>
+        <v>-1.18</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="1" t="n">
+        <v>46212</v>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Morocco</t>
+        </is>
+      </c>
+      <c r="E127" t="n">
+        <v>9.41</v>
+      </c>
+      <c r="F127" t="n">
+        <v>2.73</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="1" t="n">
+        <v>46213</v>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Belgium</t>
+        </is>
+      </c>
+      <c r="E128" t="n">
+        <v>9.31</v>
+      </c>
+      <c r="F128" t="n">
+        <v>2.2</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="1" t="n">
         <v>46214</v>
       </c>
-      <c r="B127" t="inlineStr">
-        <is>
-          <t>FIFA - World Cup</t>
-        </is>
-      </c>
-      <c r="C127" t="inlineStr">
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
         <is>
           <t>Norway</t>
         </is>
       </c>
-      <c r="D127" t="inlineStr">
+      <c r="D129" t="inlineStr">
         <is>
           <t>England</t>
         </is>
       </c>
-      <c r="E127" t="n">
-        <v>9.539999999999999</v>
-      </c>
-      <c r="F127" t="n">
-        <v>-1.13</v>
+      <c r="E129" t="n">
+        <v>9.51</v>
+      </c>
+      <c r="F129" t="n">
+        <v>-0.98</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily scrape output - 2026-07-09
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F129"/>
+  <dimension ref="A1:F130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3722,10 +3722,10 @@
         </is>
       </c>
       <c r="E127" t="n">
-        <v>9.41</v>
+        <v>9.48</v>
       </c>
       <c r="F127" t="n">
-        <v>2.73</v>
+        <v>2.98</v>
       </c>
     </row>
     <row r="128">
@@ -3748,10 +3748,10 @@
         </is>
       </c>
       <c r="E128" t="n">
-        <v>9.31</v>
+        <v>9.539999999999999</v>
       </c>
       <c r="F128" t="n">
-        <v>2.2</v>
+        <v>2.23</v>
       </c>
     </row>
     <row r="129">
@@ -3774,10 +3774,36 @@
         </is>
       </c>
       <c r="E129" t="n">
-        <v>9.51</v>
+        <v>9.550000000000001</v>
       </c>
       <c r="F129" t="n">
-        <v>-0.98</v>
+        <v>-0.96</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="1" t="n">
+        <v>46215</v>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="E130" t="n">
+        <v>8.51</v>
+      </c>
+      <c r="F130" t="n">
+        <v>1.59</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily scrape output - 2026-07-10
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F130"/>
+  <dimension ref="A1:F151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3734,76 +3734,622 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>FIFA - World Cup</t>
+          <t>Brazil - Serie B</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Juventude</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Belgium</t>
+          <t>Vila Nova</t>
         </is>
       </c>
       <c r="E128" t="n">
-        <v>9.539999999999999</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="F128" t="n">
-        <v>2.23</v>
+        <v>1.49</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="1" t="n">
-        <v>46214</v>
+        <v>46213</v>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>FIFA - World Cup</t>
+          <t>Brazil - Serie B</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Norway</t>
+          <t>Sport Recife</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>England</t>
+          <t>Botafogo SP</t>
         </is>
       </c>
       <c r="E129" t="n">
-        <v>9.550000000000001</v>
+        <v>9.83</v>
       </c>
       <c r="F129" t="n">
-        <v>-0.96</v>
+        <v>1.37</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="1" t="n">
+        <v>46213</v>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Belgium</t>
+        </is>
+      </c>
+      <c r="E130" t="n">
+        <v>10.02</v>
+      </c>
+      <c r="F130" t="n">
+        <v>2.91</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="1" t="n">
+        <v>46213</v>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>VPS</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>SJK</t>
+        </is>
+      </c>
+      <c r="E131" t="n">
+        <v>9.82</v>
+      </c>
+      <c r="F131" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="1" t="n">
+        <v>46213</v>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Finland - Ykkosliiga</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>KTP</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>JaPS</t>
+        </is>
+      </c>
+      <c r="E132" t="n">
+        <v>10.52</v>
+      </c>
+      <c r="F132" t="n">
+        <v>2.65</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="1" t="n">
+        <v>46213</v>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Finland - Ykkosliiga</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>PK-35</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>KaPa</t>
+        </is>
+      </c>
+      <c r="E133" t="n">
+        <v>10.07</v>
+      </c>
+      <c r="F133" t="n">
+        <v>1.88</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="1" t="n">
+        <v>46213</v>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Iceland - 1. Deild</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Aegir</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>HK Kopavogur</t>
+        </is>
+      </c>
+      <c r="E134" t="n">
+        <v>11.57</v>
+      </c>
+      <c r="F134" t="n">
+        <v>-3.01</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="1" t="n">
+        <v>46213</v>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Iceland - 1. Deild</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>IR Reykjavik</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Throttur Reykjavik</t>
+        </is>
+      </c>
+      <c r="E135" t="n">
+        <v>11.49</v>
+      </c>
+      <c r="F135" t="n">
+        <v>-0.7</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="1" t="n">
+        <v>46213</v>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Iceland - 1. Deild</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>UMF Njardvik</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>UMF Grindavik</t>
+        </is>
+      </c>
+      <c r="E136" t="n">
+        <v>11.55</v>
+      </c>
+      <c r="F136" t="n">
+        <v>3.38</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="1" t="n">
+        <v>46214</v>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Norway</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="E137" t="n">
+        <v>9.630000000000001</v>
+      </c>
+      <c r="F137" t="n">
+        <v>-0.97</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="1" t="n">
+        <v>46214</v>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>FC Lahti</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>HJK Helsinki</t>
+        </is>
+      </c>
+      <c r="E138" t="n">
+        <v>10.18</v>
+      </c>
+      <c r="F138" t="n">
+        <v>-0.34</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="1" t="n">
+        <v>46214</v>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Gnistan</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>IFK Mariehamn</t>
+        </is>
+      </c>
+      <c r="E139" t="n">
+        <v>10.57</v>
+      </c>
+      <c r="F139" t="n">
+        <v>2.44</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="1" t="n">
+        <v>46214</v>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>TPS</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>AC Oulu</t>
+        </is>
+      </c>
+      <c r="E140" t="n">
+        <v>9.82</v>
+      </c>
+      <c r="F140" t="n">
+        <v>-0.42</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="1" t="n">
+        <v>46214</v>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Finland - Ykkosliiga</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>FC Haka</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>EIF</t>
+        </is>
+      </c>
+      <c r="E141" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="F141" t="n">
+        <v>2.42</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="1" t="n">
+        <v>46214</v>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Finland - Ykkosliiga</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>HJK Klubi 04</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>JIPPO</t>
+        </is>
+      </c>
+      <c r="E142" t="n">
+        <v>9.84</v>
+      </c>
+      <c r="F142" t="n">
+        <v>-1.67</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="1" t="n">
+        <v>46214</v>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Finland - Ykkosliiga</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>SJK Akatemia</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Mikkelin Palloilijat</t>
+        </is>
+      </c>
+      <c r="E143" t="n">
+        <v>10.13</v>
+      </c>
+      <c r="F143" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="1" t="n">
         <v>46215</v>
       </c>
-      <c r="B130" t="inlineStr">
-        <is>
-          <t>FIFA - World Cup</t>
-        </is>
-      </c>
-      <c r="C130" t="inlineStr">
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Atletico Goianiense</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Fortaleza</t>
+        </is>
+      </c>
+      <c r="E144" t="n">
+        <v>10.11</v>
+      </c>
+      <c r="F144" t="n">
+        <v>0.91</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="1" t="n">
+        <v>46215</v>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Avai</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>Nautico</t>
+        </is>
+      </c>
+      <c r="E145" t="n">
+        <v>10.53</v>
+      </c>
+      <c r="F145" t="n">
+        <v>-0.6</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="1" t="n">
+        <v>46215</v>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>CRB</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>Goias</t>
+        </is>
+      </c>
+      <c r="E146" t="n">
+        <v>10.63</v>
+      </c>
+      <c r="F146" t="n">
+        <v>1.61</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="1" t="n">
+        <v>46215</v>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Operario Ferroviario</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Gremio Novorizontino</t>
+        </is>
+      </c>
+      <c r="E147" t="n">
+        <v>10.22</v>
+      </c>
+      <c r="F147" t="n">
+        <v>0.42</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="1" t="n">
+        <v>46215</v>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Sao Bernardo</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>Cuiaba</t>
+        </is>
+      </c>
+      <c r="E148" t="n">
+        <v>9.789999999999999</v>
+      </c>
+      <c r="F148" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="1" t="n">
+        <v>46215</v>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
         <is>
           <t>Argentina</t>
         </is>
       </c>
-      <c r="D130" t="inlineStr">
+      <c r="D149" t="inlineStr">
         <is>
           <t>Switzerland</t>
         </is>
       </c>
-      <c r="E130" t="n">
-        <v>8.51</v>
-      </c>
-      <c r="F130" t="n">
-        <v>1.59</v>
+      <c r="E149" t="n">
+        <v>8.449999999999999</v>
+      </c>
+      <c r="F149" t="n">
+        <v>1.58</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="1" t="n">
+        <v>46216</v>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>America Mineiro</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Londrina</t>
+        </is>
+      </c>
+      <c r="E150" t="n">
+        <v>10.67</v>
+      </c>
+      <c r="F150" t="n">
+        <v>1.83</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="1" t="n">
+        <v>46216</v>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Ceara</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Athletic Club</t>
+        </is>
+      </c>
+      <c r="E151" t="n">
+        <v>10.47</v>
+      </c>
+      <c r="F151" t="n">
+        <v>2.22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily scrape output - 2026-07-11
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F151"/>
+  <dimension ref="A1:F152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3982,10 +3982,10 @@
         </is>
       </c>
       <c r="E137" t="n">
-        <v>9.630000000000001</v>
+        <v>9.73</v>
       </c>
       <c r="F137" t="n">
-        <v>-0.97</v>
+        <v>-1.13</v>
       </c>
     </row>
     <row r="138">
@@ -4037,7 +4037,7 @@
         <v>10.57</v>
       </c>
       <c r="F139" t="n">
-        <v>2.44</v>
+        <v>2.48</v>
       </c>
     </row>
     <row r="140">
@@ -4146,28 +4146,28 @@
     </row>
     <row r="144">
       <c r="A144" s="1" t="n">
-        <v>46215</v>
+        <v>46214</v>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Iceland - 1. Deild</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Atletico Goianiense</t>
+          <t>Volsungur</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>Fortaleza</t>
+          <t>Afturelding</t>
         </is>
       </c>
       <c r="E144" t="n">
-        <v>10.11</v>
+        <v>11.87</v>
       </c>
       <c r="F144" t="n">
-        <v>0.91</v>
+        <v>-3.44</v>
       </c>
     </row>
     <row r="145">
@@ -4181,19 +4181,19 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>Avai</t>
+          <t>Atletico Goianiense</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>Nautico</t>
+          <t>Fortaleza</t>
         </is>
       </c>
       <c r="E145" t="n">
-        <v>10.53</v>
+        <v>10.11</v>
       </c>
       <c r="F145" t="n">
-        <v>-0.6</v>
+        <v>0.91</v>
       </c>
     </row>
     <row r="146">
@@ -4207,19 +4207,19 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>CRB</t>
+          <t>Avai</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>Goias</t>
+          <t>Nautico</t>
         </is>
       </c>
       <c r="E146" t="n">
-        <v>10.63</v>
+        <v>9.85</v>
       </c>
       <c r="F146" t="n">
-        <v>1.61</v>
+        <v>-0.59</v>
       </c>
     </row>
     <row r="147">
@@ -4233,19 +4233,19 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>Operario Ferroviario</t>
+          <t>CRB</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>Gremio Novorizontino</t>
+          <t>Goias</t>
         </is>
       </c>
       <c r="E147" t="n">
-        <v>10.22</v>
+        <v>10.63</v>
       </c>
       <c r="F147" t="n">
-        <v>0.42</v>
+        <v>1.61</v>
       </c>
     </row>
     <row r="148">
@@ -4259,19 +4259,19 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Sao Bernardo</t>
+          <t>Operario Ferroviario</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>Cuiaba</t>
+          <t>Gremio Novorizontino</t>
         </is>
       </c>
       <c r="E148" t="n">
-        <v>9.789999999999999</v>
+        <v>10.22</v>
       </c>
       <c r="F148" t="n">
-        <v>-0.07000000000000001</v>
+        <v>0.42</v>
       </c>
     </row>
     <row r="149">
@@ -4280,50 +4280,50 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>FIFA - World Cup</t>
+          <t>Brazil - Serie B</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Sao Bernardo</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>Switzerland</t>
+          <t>Cuiaba</t>
         </is>
       </c>
       <c r="E149" t="n">
-        <v>8.449999999999999</v>
+        <v>9.789999999999999</v>
       </c>
       <c r="F149" t="n">
-        <v>1.58</v>
+        <v>-0.07000000000000001</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="1" t="n">
-        <v>46216</v>
+        <v>46215</v>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>FIFA - World Cup</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>America Mineiro</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>Londrina</t>
+          <t>Switzerland</t>
         </is>
       </c>
       <c r="E150" t="n">
-        <v>10.67</v>
+        <v>8.32</v>
       </c>
       <c r="F150" t="n">
-        <v>1.83</v>
+        <v>1.55</v>
       </c>
     </row>
     <row r="151">
@@ -4337,19 +4337,45 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
+          <t>America Mineiro</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Londrina</t>
+        </is>
+      </c>
+      <c r="E151" t="n">
+        <v>9.710000000000001</v>
+      </c>
+      <c r="F151" t="n">
+        <v>1.89</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="1" t="n">
+        <v>46216</v>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
           <t>Ceara</t>
         </is>
       </c>
-      <c r="D151" t="inlineStr">
+      <c r="D152" t="inlineStr">
         <is>
           <t>Athletic Club</t>
         </is>
       </c>
-      <c r="E151" t="n">
-        <v>10.47</v>
-      </c>
-      <c r="F151" t="n">
-        <v>2.22</v>
+      <c r="E152" t="n">
+        <v>11.03</v>
+      </c>
+      <c r="F152" t="n">
+        <v>2.01</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily scrape output - 2026-07-12
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F152"/>
+  <dimension ref="A1:F154"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4190,10 +4190,10 @@
         </is>
       </c>
       <c r="E145" t="n">
-        <v>10.11</v>
+        <v>10.16</v>
       </c>
       <c r="F145" t="n">
-        <v>0.91</v>
+        <v>0.93</v>
       </c>
     </row>
     <row r="146">
@@ -4216,10 +4216,10 @@
         </is>
       </c>
       <c r="E146" t="n">
-        <v>9.85</v>
+        <v>9.859999999999999</v>
       </c>
       <c r="F146" t="n">
-        <v>-0.59</v>
+        <v>-0.61</v>
       </c>
     </row>
     <row r="147">
@@ -4268,10 +4268,10 @@
         </is>
       </c>
       <c r="E148" t="n">
-        <v>10.22</v>
+        <v>10.21</v>
       </c>
       <c r="F148" t="n">
-        <v>0.42</v>
+        <v>0.61</v>
       </c>
     </row>
     <row r="149">
@@ -4376,6 +4376,58 @@
       </c>
       <c r="F152" t="n">
         <v>2.01</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="1" t="n">
+        <v>46216</v>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Iceland - 1. Deild</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Vestri</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>Fylkir</t>
+        </is>
+      </c>
+      <c r="E153" t="n">
+        <v>11.21</v>
+      </c>
+      <c r="F153" t="n">
+        <v>-1.42</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="1" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="E154" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="F154" t="n">
+        <v>0.13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily scrape output - 2026-07-13
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F154"/>
+  <dimension ref="A1:F155"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4346,10 +4346,10 @@
         </is>
       </c>
       <c r="E151" t="n">
-        <v>9.710000000000001</v>
+        <v>9.74</v>
       </c>
       <c r="F151" t="n">
-        <v>1.89</v>
+        <v>1.88</v>
       </c>
     </row>
     <row r="152">
@@ -4398,10 +4398,10 @@
         </is>
       </c>
       <c r="E153" t="n">
-        <v>11.21</v>
+        <v>10.93</v>
       </c>
       <c r="F153" t="n">
-        <v>-1.42</v>
+        <v>-1.35</v>
       </c>
     </row>
     <row r="154">
@@ -4424,10 +4424,36 @@
         </is>
       </c>
       <c r="E154" t="n">
-        <v>9.6</v>
+        <v>9.640000000000001</v>
       </c>
       <c r="F154" t="n">
         <v>0.13</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="1" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E155" t="n">
+        <v>8.359999999999999</v>
+      </c>
+      <c r="F155" t="n">
+        <v>0.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily scrape output - 2026-07-14
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F155"/>
+  <dimension ref="A1:F156"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4424,36 +4424,62 @@
         </is>
       </c>
       <c r="E154" t="n">
-        <v>9.640000000000001</v>
+        <v>9.550000000000001</v>
       </c>
       <c r="F154" t="n">
-        <v>0.13</v>
+        <v>0.36</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="1" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Iceland - 1. Deild</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>HK Kopavogur</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>IR Reykjavik</t>
+        </is>
+      </c>
+      <c r="E155" t="n">
+        <v>11.73</v>
+      </c>
+      <c r="F155" t="n">
+        <v>1.36</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="1" t="n">
         <v>46218</v>
       </c>
-      <c r="B155" t="inlineStr">
-        <is>
-          <t>FIFA - World Cup</t>
-        </is>
-      </c>
-      <c r="C155" t="inlineStr">
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
         <is>
           <t>England</t>
         </is>
       </c>
-      <c r="D155" t="inlineStr">
+      <c r="D156" t="inlineStr">
         <is>
           <t>Argentina</t>
         </is>
       </c>
-      <c r="E155" t="n">
-        <v>8.359999999999999</v>
-      </c>
-      <c r="F155" t="n">
-        <v>0.6</v>
+      <c r="E156" t="n">
+        <v>8.32</v>
+      </c>
+      <c r="F156" t="n">
+        <v>0.49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily scrape output - 2026-07-15
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F156"/>
+  <dimension ref="A1:F157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4476,10 +4476,36 @@
         </is>
       </c>
       <c r="E156" t="n">
-        <v>8.32</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="F156" t="n">
-        <v>0.49</v>
+        <v>0.84</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="1" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Finland - Ykkosliiga</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>JIPPO</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Mikkelin Palloilijat</t>
+        </is>
+      </c>
+      <c r="E157" t="n">
+        <v>10.02</v>
+      </c>
+      <c r="F157" t="n">
+        <v>2.87</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily scrape output - 2026-07-16
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F157"/>
+  <dimension ref="A1:F159"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4508,6 +4508,58 @@
         <v>2.87</v>
       </c>
     </row>
+    <row r="158">
+      <c r="A158" s="1" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>CRB</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>Nautico</t>
+        </is>
+      </c>
+      <c r="E158" t="n">
+        <v>10.67</v>
+      </c>
+      <c r="F158" t="n">
+        <v>0.87</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="1" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Iceland - 1. Deild</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Afturelding</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>Leiknir Reykjavik</t>
+        </is>
+      </c>
+      <c r="E159" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="F159" t="n">
+        <v>2.86</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily scrape output - 2026-07-17
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F159"/>
+  <dimension ref="A1:F189"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4560,6 +4560,786 @@
         <v>2.86</v>
       </c>
     </row>
+    <row r="160">
+      <c r="A160" s="1" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>America Mineiro</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>Ceara</t>
+        </is>
+      </c>
+      <c r="E160" t="n">
+        <v>10.36</v>
+      </c>
+      <c r="F160" t="n">
+        <v>0.45</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="1" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Juventude</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>Cuiaba</t>
+        </is>
+      </c>
+      <c r="E161" t="n">
+        <v>9.720000000000001</v>
+      </c>
+      <c r="F161" t="n">
+        <v>1.68</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="1" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Sao Bernardo</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>Avai</t>
+        </is>
+      </c>
+      <c r="E162" t="n">
+        <v>10.36</v>
+      </c>
+      <c r="F162" t="n">
+        <v>1.82</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="1" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Finland - Ykkosliiga</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>HJK Klubi 04</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>FC Haka</t>
+        </is>
+      </c>
+      <c r="E163" t="n">
+        <v>10.07</v>
+      </c>
+      <c r="F163" t="n">
+        <v>-1.67</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="1" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Finland - Ykkosliiga</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>KaPa</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>SJK Akatemia</t>
+        </is>
+      </c>
+      <c r="E164" t="n">
+        <v>10.15</v>
+      </c>
+      <c r="F164" t="n">
+        <v>1.06</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="1" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Iceland - 1. Deild</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>Fylkir</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>UMF Njardvik</t>
+        </is>
+      </c>
+      <c r="E165" t="n">
+        <v>11.55</v>
+      </c>
+      <c r="F165" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="1" t="n">
+        <v>46221</v>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Atletico Goianiense</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>Athletic Club</t>
+        </is>
+      </c>
+      <c r="E166" t="n">
+        <v>10.65</v>
+      </c>
+      <c r="F166" t="n">
+        <v>1.64</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="1" t="n">
+        <v>46221</v>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>Criciuma</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>Vila Nova</t>
+        </is>
+      </c>
+      <c r="E167" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="F167" t="n">
+        <v>2.24</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="1" t="n">
+        <v>46221</v>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>Fortaleza</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>Gremio Novorizontino</t>
+        </is>
+      </c>
+      <c r="E168" t="n">
+        <v>10.26</v>
+      </c>
+      <c r="F168" t="n">
+        <v>1.71</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="1" t="n">
+        <v>46221</v>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>Londrina</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>Botafogo SP</t>
+        </is>
+      </c>
+      <c r="E169" t="n">
+        <v>10.55</v>
+      </c>
+      <c r="F169" t="n">
+        <v>0.16</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="1" t="n">
+        <v>46221</v>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>Ponte Preta</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>Goias</t>
+        </is>
+      </c>
+      <c r="E170" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="F170" t="n">
+        <v>-1.15</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="1" t="n">
+        <v>46221</v>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>Sport Recife</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>Operario Ferroviario</t>
+        </is>
+      </c>
+      <c r="E171" t="n">
+        <v>10.36</v>
+      </c>
+      <c r="F171" t="n">
+        <v>1.72</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="1" t="n">
+        <v>46221</v>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="E172" t="n">
+        <v>9.09</v>
+      </c>
+      <c r="F172" t="n">
+        <v>1.38</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="1" t="n">
+        <v>46221</v>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>AC Oulu</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>Gnistan</t>
+        </is>
+      </c>
+      <c r="E173" t="n">
+        <v>10.28</v>
+      </c>
+      <c r="F173" t="n">
+        <v>1.19</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="1" t="n">
+        <v>46221</v>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>HJK Helsinki</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>VPS</t>
+        </is>
+      </c>
+      <c r="E174" t="n">
+        <v>10.55</v>
+      </c>
+      <c r="F174" t="n">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="1" t="n">
+        <v>46221</v>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>SJK</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>KuPS</t>
+        </is>
+      </c>
+      <c r="E175" t="n">
+        <v>10.14</v>
+      </c>
+      <c r="F175" t="n">
+        <v>-0.88</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="1" t="n">
+        <v>46221</v>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>Finland - Ykkosliiga</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>EIF</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>JaPS</t>
+        </is>
+      </c>
+      <c r="E176" t="n">
+        <v>10.27</v>
+      </c>
+      <c r="F176" t="n">
+        <v>1.09</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="1" t="n">
+        <v>46221</v>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>Finland - Ykkosliiga</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>KTP</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>PK-35</t>
+        </is>
+      </c>
+      <c r="E177" t="n">
+        <v>10.51</v>
+      </c>
+      <c r="F177" t="n">
+        <v>1.42</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="1" t="n">
+        <v>46221</v>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>Iceland - 1. Deild</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>Throttur Reykjavik</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>Volsungur</t>
+        </is>
+      </c>
+      <c r="E178" t="n">
+        <v>11.98</v>
+      </c>
+      <c r="F178" t="n">
+        <v>4.63</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="1" t="n">
+        <v>46221</v>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Iceland - 1. Deild</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>UMF Grindavik</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>IR Reykjavik</t>
+        </is>
+      </c>
+      <c r="E179" t="n">
+        <v>11.49</v>
+      </c>
+      <c r="F179" t="n">
+        <v>-0.8100000000000001</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="1" t="n">
+        <v>46221</v>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Oddevold</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>Varbergs BoIS</t>
+        </is>
+      </c>
+      <c r="E180" t="n">
+        <v>9.880000000000001</v>
+      </c>
+      <c r="F180" t="n">
+        <v>0.65</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="1" t="n">
+        <v>46221</v>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Osters</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>Brage</t>
+        </is>
+      </c>
+      <c r="E181" t="n">
+        <v>10.83</v>
+      </c>
+      <c r="F181" t="n">
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="1" t="n">
+        <v>46221</v>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>Ostersunds FK</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>Landskrona</t>
+        </is>
+      </c>
+      <c r="E182" t="n">
+        <v>10.16</v>
+      </c>
+      <c r="F182" t="n">
+        <v>0.98</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="1" t="n">
+        <v>46222</v>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>FIFA - World Cup</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E183" t="n">
+        <v>8.210000000000001</v>
+      </c>
+      <c r="F183" t="n">
+        <v>1.12</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="1" t="n">
+        <v>46222</v>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>Jaro</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>Inter Turku</t>
+        </is>
+      </c>
+      <c r="E184" t="n">
+        <v>9.970000000000001</v>
+      </c>
+      <c r="F184" t="n">
+        <v>-2.19</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="1" t="n">
+        <v>46222</v>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>Norrkoping</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>Sandvikens IF</t>
+        </is>
+      </c>
+      <c r="E185" t="n">
+        <v>10.55</v>
+      </c>
+      <c r="F185" t="n">
+        <v>2.37</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="1" t="n">
+        <v>46222</v>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>Varnamo</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>Ljungskile</t>
+        </is>
+      </c>
+      <c r="E186" t="n">
+        <v>10.67</v>
+      </c>
+      <c r="F186" t="n">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="1" t="n">
+        <v>46223</v>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>IFK Mariehamn</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>FC Lahti</t>
+        </is>
+      </c>
+      <c r="E187" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="F187" t="n">
+        <v>-2.23</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="1" t="n">
+        <v>46223</v>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>TPS</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>Ilves</t>
+        </is>
+      </c>
+      <c r="E188" t="n">
+        <v>9.869999999999999</v>
+      </c>
+      <c r="F188" t="n">
+        <v>-0.46</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="1" t="n">
+        <v>46223</v>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>Norrby</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>Sundsvall</t>
+        </is>
+      </c>
+      <c r="E189" t="n">
+        <v>10.28</v>
+      </c>
+      <c r="F189" t="n">
+        <v>1.44</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily scrape output - 2026-07-18
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F189"/>
+  <dimension ref="A1:F192"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4736,10 +4736,10 @@
         </is>
       </c>
       <c r="E166" t="n">
-        <v>10.65</v>
+        <v>10.19</v>
       </c>
       <c r="F166" t="n">
-        <v>1.64</v>
+        <v>1.65</v>
       </c>
     </row>
     <row r="167">
@@ -4840,10 +4840,10 @@
         </is>
       </c>
       <c r="E170" t="n">
-        <v>10.1</v>
+        <v>9.98</v>
       </c>
       <c r="F170" t="n">
-        <v>-1.15</v>
+        <v>-1.13</v>
       </c>
     </row>
     <row r="171">
@@ -4892,10 +4892,10 @@
         </is>
       </c>
       <c r="E172" t="n">
-        <v>9.09</v>
+        <v>9.470000000000001</v>
       </c>
       <c r="F172" t="n">
-        <v>1.38</v>
+        <v>1.46</v>
       </c>
     </row>
     <row r="173">
@@ -4918,10 +4918,10 @@
         </is>
       </c>
       <c r="E173" t="n">
-        <v>10.28</v>
+        <v>10.32</v>
       </c>
       <c r="F173" t="n">
-        <v>1.19</v>
+        <v>1.37</v>
       </c>
     </row>
     <row r="174">
@@ -4970,10 +4970,10 @@
         </is>
       </c>
       <c r="E175" t="n">
-        <v>10.14</v>
+        <v>10.09</v>
       </c>
       <c r="F175" t="n">
-        <v>-0.88</v>
+        <v>-0.45</v>
       </c>
     </row>
     <row r="176">
@@ -4996,10 +4996,10 @@
         </is>
       </c>
       <c r="E176" t="n">
-        <v>10.27</v>
+        <v>10.26</v>
       </c>
       <c r="F176" t="n">
-        <v>1.09</v>
+        <v>1.16</v>
       </c>
     </row>
     <row r="177">
@@ -5074,10 +5074,10 @@
         </is>
       </c>
       <c r="E179" t="n">
-        <v>11.49</v>
+        <v>11.55</v>
       </c>
       <c r="F179" t="n">
-        <v>-0.8100000000000001</v>
+        <v>-0.82</v>
       </c>
     </row>
     <row r="180">
@@ -5126,7 +5126,7 @@
         </is>
       </c>
       <c r="E181" t="n">
-        <v>10.83</v>
+        <v>10.79</v>
       </c>
       <c r="F181" t="n">
         <v>0.95</v>
@@ -5178,10 +5178,10 @@
         </is>
       </c>
       <c r="E183" t="n">
-        <v>8.210000000000001</v>
+        <v>8.220000000000001</v>
       </c>
       <c r="F183" t="n">
-        <v>1.12</v>
+        <v>1.22</v>
       </c>
     </row>
     <row r="184">
@@ -5207,7 +5207,7 @@
         <v>9.970000000000001</v>
       </c>
       <c r="F184" t="n">
-        <v>-2.19</v>
+        <v>-2.21</v>
       </c>
     </row>
     <row r="185">
@@ -5233,7 +5233,7 @@
         <v>10.55</v>
       </c>
       <c r="F185" t="n">
-        <v>2.37</v>
+        <v>2.36</v>
       </c>
     </row>
     <row r="186">
@@ -5334,10 +5334,88 @@
         </is>
       </c>
       <c r="E189" t="n">
-        <v>10.28</v>
+        <v>10.26</v>
       </c>
       <c r="F189" t="n">
-        <v>1.44</v>
+        <v>1.41</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="1" t="n">
+        <v>46224</v>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>Avai</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>America Mineiro</t>
+        </is>
+      </c>
+      <c r="E190" t="n">
+        <v>10.13</v>
+      </c>
+      <c r="F190" t="n">
+        <v>0.33</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="1" t="n">
+        <v>46224</v>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>Finland - Ykkosliiga</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>KaPa</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>HJK Klubi 04</t>
+        </is>
+      </c>
+      <c r="E191" t="n">
+        <v>9.99</v>
+      </c>
+      <c r="F191" t="n">
+        <v>0.98</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="1" t="n">
+        <v>46224</v>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>Falkenbergs</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>Helsingborgs</t>
+        </is>
+      </c>
+      <c r="E192" t="n">
+        <v>10.32</v>
+      </c>
+      <c r="F192" t="n">
+        <v>0.38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily scrape output - 2026-07-19
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F192"/>
+  <dimension ref="A1:F196"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5178,10 +5178,10 @@
         </is>
       </c>
       <c r="E183" t="n">
-        <v>8.220000000000001</v>
+        <v>8.210000000000001</v>
       </c>
       <c r="F183" t="n">
-        <v>1.22</v>
+        <v>1.35</v>
       </c>
     </row>
     <row r="184">
@@ -5221,19 +5221,19 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>Norrkoping</t>
+          <t>Nordic United</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>Sandvikens IF</t>
+          <t>Orebro SK</t>
         </is>
       </c>
       <c r="E185" t="n">
-        <v>10.55</v>
+        <v>9.68</v>
       </c>
       <c r="F185" t="n">
-        <v>2.36</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="186">
@@ -5247,45 +5247,45 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>Varnamo</t>
+          <t>Norrkoping</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>Ljungskile</t>
+          <t>Sandvikens IF</t>
         </is>
       </c>
       <c r="E186" t="n">
-        <v>10.67</v>
+        <v>10.58</v>
       </c>
       <c r="F186" t="n">
-        <v>0.12</v>
+        <v>2.36</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="1" t="n">
-        <v>46223</v>
+        <v>46222</v>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>Finland - Veikkausliiga</t>
+          <t>Sweden - Superettan</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>IFK Mariehamn</t>
+          <t>Varnamo</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>FC Lahti</t>
+          <t>Ljungskile</t>
         </is>
       </c>
       <c r="E187" t="n">
-        <v>10.2</v>
+        <v>10.67</v>
       </c>
       <c r="F187" t="n">
-        <v>-2.23</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="188">
@@ -5299,19 +5299,19 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>TPS</t>
+          <t>IFK Mariehamn</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>Ilves</t>
+          <t>FC Lahti</t>
         </is>
       </c>
       <c r="E188" t="n">
-        <v>9.869999999999999</v>
+        <v>10.2</v>
       </c>
       <c r="F188" t="n">
-        <v>-0.46</v>
+        <v>-2.23</v>
       </c>
     </row>
     <row r="189">
@@ -5320,76 +5320,76 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Finland - Veikkausliiga</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>Norrby</t>
+          <t>TPS</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>Sundsvall</t>
+          <t>Ilves</t>
         </is>
       </c>
       <c r="E189" t="n">
-        <v>10.26</v>
+        <v>9.869999999999999</v>
       </c>
       <c r="F189" t="n">
-        <v>1.41</v>
+        <v>-0.46</v>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="1" t="n">
-        <v>46224</v>
+        <v>46223</v>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Iceland - 1. Deild</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>Avai</t>
+          <t>HK Kopavogur</t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>America Mineiro</t>
+          <t>Vestri</t>
         </is>
       </c>
       <c r="E190" t="n">
-        <v>10.13</v>
+        <v>11.59</v>
       </c>
       <c r="F190" t="n">
-        <v>0.33</v>
+        <v>2.09</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="1" t="n">
-        <v>46224</v>
+        <v>46223</v>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>Finland - Ykkosliiga</t>
+          <t>Sweden - Superettan</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>KaPa</t>
+          <t>Norrby</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>HJK Klubi 04</t>
+          <t>Sundsvall</t>
         </is>
       </c>
       <c r="E191" t="n">
-        <v>9.99</v>
+        <v>10.26</v>
       </c>
       <c r="F191" t="n">
-        <v>0.98</v>
+        <v>1.41</v>
       </c>
     </row>
     <row r="192">
@@ -5398,24 +5398,128 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>Avai</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>America Mineiro</t>
+        </is>
+      </c>
+      <c r="E192" t="n">
+        <v>10.13</v>
+      </c>
+      <c r="F192" t="n">
+        <v>0.33</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="1" t="n">
+        <v>46224</v>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>Gremio Novorizontino</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>Criciuma</t>
+        </is>
+      </c>
+      <c r="E193" t="n">
+        <v>10.13</v>
+      </c>
+      <c r="F193" t="n">
+        <v>0.87</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="1" t="n">
+        <v>46224</v>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>Finland - Ykkosliiga</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>KaPa</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>HJK Klubi 04</t>
+        </is>
+      </c>
+      <c r="E194" t="n">
+        <v>9.99</v>
+      </c>
+      <c r="F194" t="n">
+        <v>0.98</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="1" t="n">
+        <v>46224</v>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
           <t>Sweden - Superettan</t>
         </is>
       </c>
-      <c r="C192" t="inlineStr">
+      <c r="C195" t="inlineStr">
         <is>
           <t>Falkenbergs</t>
         </is>
       </c>
-      <c r="D192" t="inlineStr">
+      <c r="D195" t="inlineStr">
         <is>
           <t>Helsingborgs</t>
         </is>
       </c>
-      <c r="E192" t="n">
+      <c r="E195" t="n">
         <v>10.32</v>
       </c>
-      <c r="F192" t="n">
+      <c r="F195" t="n">
         <v>0.38</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="1" t="n">
+        <v>46225</v>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>Vila Nova</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>Fortaleza</t>
+        </is>
+      </c>
+      <c r="E196" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="F196" t="n">
+        <v>0.16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily scrape output - 2026-07-20
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -5308,10 +5308,10 @@
         </is>
       </c>
       <c r="E188" t="n">
-        <v>10.2</v>
+        <v>9.960000000000001</v>
       </c>
       <c r="F188" t="n">
-        <v>-2.23</v>
+        <v>-2.17</v>
       </c>
     </row>
     <row r="189">
@@ -5334,10 +5334,10 @@
         </is>
       </c>
       <c r="E189" t="n">
-        <v>9.869999999999999</v>
+        <v>9.77</v>
       </c>
       <c r="F189" t="n">
-        <v>-0.46</v>
+        <v>-0.45</v>
       </c>
     </row>
     <row r="190">
@@ -5389,7 +5389,7 @@
         <v>10.26</v>
       </c>
       <c r="F191" t="n">
-        <v>1.41</v>
+        <v>1.38</v>
       </c>
     </row>
     <row r="192">
@@ -5490,10 +5490,10 @@
         </is>
       </c>
       <c r="E195" t="n">
-        <v>10.32</v>
+        <v>10.35</v>
       </c>
       <c r="F195" t="n">
-        <v>0.38</v>
+        <v>0.37</v>
       </c>
     </row>
     <row r="196">

</xml_diff>

<commit_message>
Daily scrape output - 2026-07-21
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -5412,10 +5412,10 @@
         </is>
       </c>
       <c r="E192" t="n">
-        <v>10.13</v>
+        <v>10.07</v>
       </c>
       <c r="F192" t="n">
-        <v>0.33</v>
+        <v>0.58</v>
       </c>
     </row>
     <row r="193">
@@ -5490,10 +5490,10 @@
         </is>
       </c>
       <c r="E195" t="n">
-        <v>10.35</v>
+        <v>10.5</v>
       </c>
       <c r="F195" t="n">
-        <v>0.37</v>
+        <v>0.36</v>
       </c>
     </row>
     <row r="196">
@@ -5516,10 +5516,10 @@
         </is>
       </c>
       <c r="E196" t="n">
-        <v>10.2</v>
+        <v>10.15</v>
       </c>
       <c r="F196" t="n">
-        <v>0.16</v>
+        <v>0.18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily scrape output - 2026-07-22
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F196"/>
+  <dimension ref="A1:F200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5507,19 +5507,123 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
+          <t>Ceara</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>CRB</t>
+        </is>
+      </c>
+      <c r="E196" t="n">
+        <v>10.74</v>
+      </c>
+      <c r="F196" t="n">
+        <v>1.36</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="1" t="n">
+        <v>46225</v>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>Goias</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>Sport Recife</t>
+        </is>
+      </c>
+      <c r="E197" t="n">
+        <v>10.22</v>
+      </c>
+      <c r="F197" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="1" t="n">
+        <v>46225</v>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>Operario Ferroviario</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>Ponte Preta</t>
+        </is>
+      </c>
+      <c r="E198" t="n">
+        <v>10.42</v>
+      </c>
+      <c r="F198" t="n">
+        <v>3.03</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="1" t="n">
+        <v>46225</v>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
           <t>Vila Nova</t>
         </is>
       </c>
-      <c r="D196" t="inlineStr">
+      <c r="D199" t="inlineStr">
         <is>
           <t>Fortaleza</t>
         </is>
       </c>
-      <c r="E196" t="n">
+      <c r="E199" t="n">
         <v>10.15</v>
       </c>
-      <c r="F196" t="n">
+      <c r="F199" t="n">
         <v>0.18</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="1" t="n">
+        <v>46226</v>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>Nautico</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>Londrina</t>
+        </is>
+      </c>
+      <c r="E200" t="n">
+        <v>10.65</v>
+      </c>
+      <c r="F200" t="n">
+        <v>2.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily scrape output - 2026-07-23
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F200"/>
+  <dimension ref="A1:F204"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5611,19 +5611,123 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
+          <t>Athletic Club</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>Sao Bernardo</t>
+        </is>
+      </c>
+      <c r="E200" t="n">
+        <v>10.16</v>
+      </c>
+      <c r="F200" t="n">
+        <v>1.68</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="1" t="n">
+        <v>46226</v>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>Cuiaba</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>Atletico Goianiense</t>
+        </is>
+      </c>
+      <c r="E201" t="n">
+        <v>9.550000000000001</v>
+      </c>
+      <c r="F201" t="n">
+        <v>1.35</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="1" t="n">
+        <v>46226</v>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
           <t>Nautico</t>
         </is>
       </c>
-      <c r="D200" t="inlineStr">
+      <c r="D202" t="inlineStr">
         <is>
           <t>Londrina</t>
         </is>
       </c>
-      <c r="E200" t="n">
+      <c r="E202" t="n">
         <v>10.65</v>
       </c>
-      <c r="F200" t="n">
+      <c r="F202" t="n">
         <v>2.6</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="1" t="n">
+        <v>46226</v>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>Iceland - 1. Deild</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>Leiknir Reykjavik</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>Throttur Reykjavik</t>
+        </is>
+      </c>
+      <c r="E203" t="n">
+        <v>11.52</v>
+      </c>
+      <c r="F203" t="n">
+        <v>-1.45</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="1" t="n">
+        <v>46227</v>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>Botafogo SP</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>Juventude</t>
+        </is>
+      </c>
+      <c r="E204" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="F204" t="n">
+        <v>0.98</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily scrape output - 2026-07-24
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F204"/>
+  <dimension ref="A1:F239"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5730,6 +5730,916 @@
         <v>0.98</v>
       </c>
     </row>
+    <row r="205">
+      <c r="A205" s="1" t="n">
+        <v>46227</v>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>Jaro</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>SJK</t>
+        </is>
+      </c>
+      <c r="E205" t="n">
+        <v>10.33</v>
+      </c>
+      <c r="F205" t="n">
+        <v>-1.89</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="1" t="n">
+        <v>46227</v>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>Iceland - 1. Deild</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>UMF Njardvik</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>HK Kopavogur</t>
+        </is>
+      </c>
+      <c r="E206" t="n">
+        <v>11.36</v>
+      </c>
+      <c r="F206" t="n">
+        <v>0.66</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="1" t="n">
+        <v>46227</v>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>Iceland - 1. Deild</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>Volsungur</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>UMF Grindavik</t>
+        </is>
+      </c>
+      <c r="E207" t="n">
+        <v>11.73</v>
+      </c>
+      <c r="F207" t="n">
+        <v>-0.36</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="1" t="n">
+        <v>46228</v>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>IFK Mariehamn</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>AC Oulu</t>
+        </is>
+      </c>
+      <c r="E208" t="n">
+        <v>9.93</v>
+      </c>
+      <c r="F208" t="n">
+        <v>-1.86</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="1" t="n">
+        <v>46228</v>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>KuPS</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>VPS</t>
+        </is>
+      </c>
+      <c r="E209" t="n">
+        <v>10.23</v>
+      </c>
+      <c r="F209" t="n">
+        <v>2.09</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="1" t="n">
+        <v>46228</v>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>Finland - Ykkosliiga</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>FC Haka</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>KaPa</t>
+        </is>
+      </c>
+      <c r="E210" t="n">
+        <v>10.77</v>
+      </c>
+      <c r="F210" t="n">
+        <v>2.17</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="1" t="n">
+        <v>46228</v>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>Finland - Ykkosliiga</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>JaPS</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>HJK Klubi 04</t>
+        </is>
+      </c>
+      <c r="E211" t="n">
+        <v>10.49</v>
+      </c>
+      <c r="F211" t="n">
+        <v>0.85</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="1" t="n">
+        <v>46228</v>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>Finland - Ykkosliiga</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>Mikkelin Palloilijat</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>KTP</t>
+        </is>
+      </c>
+      <c r="E212" t="n">
+        <v>10.52</v>
+      </c>
+      <c r="F212" t="n">
+        <v>-2.67</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="1" t="n">
+        <v>46228</v>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>Finland - Ykkosliiga</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>PK-35</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>JIPPO</t>
+        </is>
+      </c>
+      <c r="E213" t="n">
+        <v>9.67</v>
+      </c>
+      <c r="F213" t="n">
+        <v>-0.16</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="1" t="n">
+        <v>46228</v>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>Finland - Ykkosliiga</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>SJK Akatemia</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>EIF</t>
+        </is>
+      </c>
+      <c r="E214" t="n">
+        <v>10.15</v>
+      </c>
+      <c r="F214" t="n">
+        <v>-0.58</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="1" t="n">
+        <v>46228</v>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>Iceland - 1. Deild</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>IR Reykjavik</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>Fylkir</t>
+        </is>
+      </c>
+      <c r="E215" t="n">
+        <v>11.86</v>
+      </c>
+      <c r="F215" t="n">
+        <v>-1.14</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="1" t="n">
+        <v>46228</v>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>Haugesund</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>Bryne</t>
+        </is>
+      </c>
+      <c r="E216" t="n">
+        <v>10.94</v>
+      </c>
+      <c r="F216" t="n">
+        <v>1.67</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="1" t="n">
+        <v>46228</v>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>Stromsgodset</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>Lyn</t>
+        </is>
+      </c>
+      <c r="E217" t="n">
+        <v>11.09</v>
+      </c>
+      <c r="F217" t="n">
+        <v>3.56</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="1" t="n">
+        <v>46228</v>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>Varnamo</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>Brage</t>
+        </is>
+      </c>
+      <c r="E218" t="n">
+        <v>10.51</v>
+      </c>
+      <c r="F218" t="n">
+        <v>0.89</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="1" t="n">
+        <v>46229</v>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>America Mineiro</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>Goias</t>
+        </is>
+      </c>
+      <c r="E219" t="n">
+        <v>10.21</v>
+      </c>
+      <c r="F219" t="n">
+        <v>0.82</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="1" t="n">
+        <v>46229</v>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>Criciuma</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>Nautico</t>
+        </is>
+      </c>
+      <c r="E220" t="n">
+        <v>10.47</v>
+      </c>
+      <c r="F220" t="n">
+        <v>1.43</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="1" t="n">
+        <v>46229</v>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>Londrina</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>Gremio Novorizontino</t>
+        </is>
+      </c>
+      <c r="E221" t="n">
+        <v>10.45</v>
+      </c>
+      <c r="F221" t="n">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="1" t="n">
+        <v>46229</v>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>Sao Bernardo</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>Ceara</t>
+        </is>
+      </c>
+      <c r="E222" t="n">
+        <v>10.53</v>
+      </c>
+      <c r="F222" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="1" t="n">
+        <v>46229</v>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>HJK Helsinki</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>TPS</t>
+        </is>
+      </c>
+      <c r="E223" t="n">
+        <v>10.75</v>
+      </c>
+      <c r="F223" t="n">
+        <v>2.99</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="1" t="n">
+        <v>46229</v>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>Ilves</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>FC Lahti</t>
+        </is>
+      </c>
+      <c r="E224" t="n">
+        <v>9.970000000000001</v>
+      </c>
+      <c r="F224" t="n">
+        <v>0.51</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="1" t="n">
+        <v>46229</v>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>Inter Turku</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>Gnistan</t>
+        </is>
+      </c>
+      <c r="E225" t="n">
+        <v>10.55</v>
+      </c>
+      <c r="F225" t="n">
+        <v>3.05</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="1" t="n">
+        <v>46229</v>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>Asane Fotball</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>Egersunds</t>
+        </is>
+      </c>
+      <c r="E226" t="n">
+        <v>10.53</v>
+      </c>
+      <c r="F226" t="n">
+        <v>-1.71</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="1" t="n">
+        <v>46229</v>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>Moss</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>Raufoss</t>
+        </is>
+      </c>
+      <c r="E227" t="n">
+        <v>10.85</v>
+      </c>
+      <c r="F227" t="n">
+        <v>1.73</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="1" t="n">
+        <v>46229</v>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>Sandnes Ulf</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>Kongsvinger</t>
+        </is>
+      </c>
+      <c r="E228" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="F228" t="n">
+        <v>-0.64</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="1" t="n">
+        <v>46229</v>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>Sogndal</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>Ranheim</t>
+        </is>
+      </c>
+      <c r="E229" t="n">
+        <v>11.27</v>
+      </c>
+      <c r="F229" t="n">
+        <v>0.32</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="1" t="n">
+        <v>46229</v>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>Strommen</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>Odd BK</t>
+        </is>
+      </c>
+      <c r="E230" t="n">
+        <v>10.59</v>
+      </c>
+      <c r="F230" t="n">
+        <v>-1.44</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="1" t="n">
+        <v>46229</v>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>Ljungskile</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>Sandvikens IF</t>
+        </is>
+      </c>
+      <c r="E231" t="n">
+        <v>10.67</v>
+      </c>
+      <c r="F231" t="n">
+        <v>1.57</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="1" t="n">
+        <v>46229</v>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>Norrby</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>Ostersunds FK</t>
+        </is>
+      </c>
+      <c r="E232" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="F232" t="n">
+        <v>-0.2</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="1" t="n">
+        <v>46229</v>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>Sundsvall</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>Falkenbergs</t>
+        </is>
+      </c>
+      <c r="E233" t="n">
+        <v>10.24</v>
+      </c>
+      <c r="F233" t="n">
+        <v>-0.93</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="1" t="n">
+        <v>46230</v>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>Atletico Goianiense</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>Operario Ferroviario</t>
+        </is>
+      </c>
+      <c r="E234" t="n">
+        <v>10.36</v>
+      </c>
+      <c r="F234" t="n">
+        <v>2.05</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="1" t="n">
+        <v>46230</v>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>CRB</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>Vila Nova</t>
+        </is>
+      </c>
+      <c r="E235" t="n">
+        <v>10.45</v>
+      </c>
+      <c r="F235" t="n">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="1" t="n">
+        <v>46230</v>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>Sport Recife</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>Cuiaba</t>
+        </is>
+      </c>
+      <c r="E236" t="n">
+        <v>9.85</v>
+      </c>
+      <c r="F236" t="n">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="1" t="n">
+        <v>46230</v>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>Stabaek</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>Hodd</t>
+        </is>
+      </c>
+      <c r="E237" t="n">
+        <v>11.11</v>
+      </c>
+      <c r="F237" t="n">
+        <v>3.68</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="1" t="n">
+        <v>46230</v>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>Orebro SK</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>Oddevold</t>
+        </is>
+      </c>
+      <c r="E238" t="n">
+        <v>10.07</v>
+      </c>
+      <c r="F238" t="n">
+        <v>-0.04</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="1" t="n">
+        <v>46230</v>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>Osters</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>Varbergs BoIS</t>
+        </is>
+      </c>
+      <c r="E239" t="n">
+        <v>10.61</v>
+      </c>
+      <c r="F239" t="n">
+        <v>0.06</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily scrape output - 2026-07-25
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F239"/>
+  <dimension ref="A1:F243"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5828,10 +5828,10 @@
         </is>
       </c>
       <c r="E208" t="n">
-        <v>9.93</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="F208" t="n">
-        <v>-1.86</v>
+        <v>-1.72</v>
       </c>
     </row>
     <row r="209">
@@ -5857,7 +5857,7 @@
         <v>10.23</v>
       </c>
       <c r="F209" t="n">
-        <v>2.09</v>
+        <v>1.97</v>
       </c>
     </row>
     <row r="210">
@@ -5906,10 +5906,10 @@
         </is>
       </c>
       <c r="E211" t="n">
-        <v>10.49</v>
+        <v>10.33</v>
       </c>
       <c r="F211" t="n">
-        <v>0.85</v>
+        <v>0.86</v>
       </c>
     </row>
     <row r="212">
@@ -5958,10 +5958,10 @@
         </is>
       </c>
       <c r="E213" t="n">
-        <v>9.67</v>
+        <v>9.76</v>
       </c>
       <c r="F213" t="n">
-        <v>-0.16</v>
+        <v>-0.05</v>
       </c>
     </row>
     <row r="214">
@@ -5984,10 +5984,10 @@
         </is>
       </c>
       <c r="E214" t="n">
-        <v>10.15</v>
+        <v>10.11</v>
       </c>
       <c r="F214" t="n">
-        <v>-0.58</v>
+        <v>-0.6899999999999999</v>
       </c>
     </row>
     <row r="215">
@@ -6166,10 +6166,10 @@
         </is>
       </c>
       <c r="E221" t="n">
-        <v>10.45</v>
+        <v>10.57</v>
       </c>
       <c r="F221" t="n">
-        <v>0.04</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="222">
@@ -6218,10 +6218,10 @@
         </is>
       </c>
       <c r="E223" t="n">
-        <v>10.75</v>
+        <v>10.78</v>
       </c>
       <c r="F223" t="n">
-        <v>2.99</v>
+        <v>2.89</v>
       </c>
     </row>
     <row r="224">
@@ -6270,10 +6270,10 @@
         </is>
       </c>
       <c r="E225" t="n">
-        <v>10.55</v>
+        <v>10.56</v>
       </c>
       <c r="F225" t="n">
-        <v>3.05</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="226">
@@ -6296,10 +6296,10 @@
         </is>
       </c>
       <c r="E226" t="n">
-        <v>10.53</v>
+        <v>10.5</v>
       </c>
       <c r="F226" t="n">
-        <v>-1.71</v>
+        <v>-1.48</v>
       </c>
     </row>
     <row r="227">
@@ -6478,10 +6478,10 @@
         </is>
       </c>
       <c r="E233" t="n">
-        <v>10.24</v>
+        <v>10.18</v>
       </c>
       <c r="F233" t="n">
-        <v>-0.93</v>
+        <v>-0.9</v>
       </c>
     </row>
     <row r="234">
@@ -6507,7 +6507,7 @@
         <v>10.36</v>
       </c>
       <c r="F234" t="n">
-        <v>2.05</v>
+        <v>1.57</v>
       </c>
     </row>
     <row r="235">
@@ -6608,7 +6608,7 @@
         </is>
       </c>
       <c r="E238" t="n">
-        <v>10.07</v>
+        <v>10</v>
       </c>
       <c r="F238" t="n">
         <v>-0.04</v>
@@ -6634,10 +6634,114 @@
         </is>
       </c>
       <c r="E239" t="n">
-        <v>10.61</v>
+        <v>10.63</v>
       </c>
       <c r="F239" t="n">
-        <v>0.06</v>
+        <v>-0.31</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="1" t="n">
+        <v>46231</v>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>Juventude</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>Avai</t>
+        </is>
+      </c>
+      <c r="E240" t="n">
+        <v>10.22</v>
+      </c>
+      <c r="F240" t="n">
+        <v>2.98</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" s="1" t="n">
+        <v>46231</v>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>Ponte Preta</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>Athletic Club</t>
+        </is>
+      </c>
+      <c r="E241" t="n">
+        <v>10.35</v>
+      </c>
+      <c r="F241" t="n">
+        <v>-0.38</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" s="1" t="n">
+        <v>46231</v>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>Landskrona</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>Norrkoping</t>
+        </is>
+      </c>
+      <c r="E242" t="n">
+        <v>10.35</v>
+      </c>
+      <c r="F242" t="n">
+        <v>-0.57</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="1" t="n">
+        <v>46232</v>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>Fortaleza</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>Botafogo SP</t>
+        </is>
+      </c>
+      <c r="E243" t="n">
+        <v>10.56</v>
+      </c>
+      <c r="F243" t="n">
+        <v>2.57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily scrape output - 2026-07-26
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -6114,10 +6114,10 @@
         </is>
       </c>
       <c r="E219" t="n">
-        <v>10.21</v>
+        <v>10.18</v>
       </c>
       <c r="F219" t="n">
-        <v>0.82</v>
+        <v>0.71</v>
       </c>
     </row>
     <row r="220">
@@ -6166,10 +6166,10 @@
         </is>
       </c>
       <c r="E221" t="n">
-        <v>10.57</v>
+        <v>10.61</v>
       </c>
       <c r="F221" t="n">
-        <v>0.02</v>
+        <v>0</v>
       </c>
     </row>
     <row r="222">
@@ -6218,7 +6218,7 @@
         </is>
       </c>
       <c r="E223" t="n">
-        <v>10.78</v>
+        <v>10.79</v>
       </c>
       <c r="F223" t="n">
         <v>2.89</v>
@@ -6244,10 +6244,10 @@
         </is>
       </c>
       <c r="E224" t="n">
-        <v>9.970000000000001</v>
+        <v>9.949999999999999</v>
       </c>
       <c r="F224" t="n">
-        <v>0.51</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="225">
@@ -6270,10 +6270,10 @@
         </is>
       </c>
       <c r="E225" t="n">
-        <v>10.56</v>
+        <v>10.47</v>
       </c>
       <c r="F225" t="n">
-        <v>3.1</v>
+        <v>3.07</v>
       </c>
     </row>
     <row r="226">
@@ -6478,10 +6478,10 @@
         </is>
       </c>
       <c r="E233" t="n">
-        <v>10.18</v>
+        <v>10</v>
       </c>
       <c r="F233" t="n">
-        <v>-0.9</v>
+        <v>-0.89</v>
       </c>
     </row>
     <row r="234">
@@ -6608,10 +6608,10 @@
         </is>
       </c>
       <c r="E238" t="n">
-        <v>10</v>
+        <v>10.01</v>
       </c>
       <c r="F238" t="n">
-        <v>-0.04</v>
+        <v>-0.14</v>
       </c>
     </row>
     <row r="239">
@@ -6686,10 +6686,10 @@
         </is>
       </c>
       <c r="E241" t="n">
-        <v>10.35</v>
+        <v>10.28</v>
       </c>
       <c r="F241" t="n">
-        <v>-0.38</v>
+        <v>0.37</v>
       </c>
     </row>
     <row r="242">
@@ -6712,10 +6712,10 @@
         </is>
       </c>
       <c r="E242" t="n">
-        <v>10.35</v>
+        <v>10.33</v>
       </c>
       <c r="F242" t="n">
-        <v>-0.57</v>
+        <v>-0.54</v>
       </c>
     </row>
     <row r="243">

</xml_diff>

<commit_message>
Daily scrape output - 2026-07-27
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -6530,7 +6530,7 @@
         </is>
       </c>
       <c r="E235" t="n">
-        <v>10.45</v>
+        <v>10.35</v>
       </c>
       <c r="F235" t="n">
         <v>1.6</v>
@@ -6686,10 +6686,10 @@
         </is>
       </c>
       <c r="E241" t="n">
-        <v>10.28</v>
+        <v>10.34</v>
       </c>
       <c r="F241" t="n">
-        <v>0.37</v>
+        <v>0.33</v>
       </c>
     </row>
     <row r="242">
@@ -6712,10 +6712,10 @@
         </is>
       </c>
       <c r="E242" t="n">
-        <v>10.33</v>
+        <v>10.29</v>
       </c>
       <c r="F242" t="n">
-        <v>-0.54</v>
+        <v>-0.13</v>
       </c>
     </row>
     <row r="243">

</xml_diff>

<commit_message>
Daily scrape output - 2026-07-28
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F243"/>
+  <dimension ref="A1:F245"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6660,10 +6660,10 @@
         </is>
       </c>
       <c r="E240" t="n">
-        <v>10.22</v>
+        <v>10.05</v>
       </c>
       <c r="F240" t="n">
-        <v>2.98</v>
+        <v>2.96</v>
       </c>
     </row>
     <row r="241">
@@ -6686,10 +6686,10 @@
         </is>
       </c>
       <c r="E241" t="n">
-        <v>10.34</v>
+        <v>10.48</v>
       </c>
       <c r="F241" t="n">
-        <v>0.33</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="242">
@@ -6698,50 +6698,102 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Iceland - 1. Deild</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>Landskrona</t>
+          <t>Aegir</t>
         </is>
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t>Norrkoping</t>
+          <t>UMF Njardvik</t>
         </is>
       </c>
       <c r="E242" t="n">
-        <v>10.29</v>
+        <v>11.57</v>
       </c>
       <c r="F242" t="n">
-        <v>-0.13</v>
+        <v>-3.03</v>
       </c>
     </row>
     <row r="243">
       <c r="A243" s="1" t="n">
+        <v>46231</v>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>Helsingborgs</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>Nordic United</t>
+        </is>
+      </c>
+      <c r="E243" t="n">
+        <v>9.77</v>
+      </c>
+      <c r="F243" t="n">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="1" t="n">
+        <v>46231</v>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>Landskrona</t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>Norrkoping</t>
+        </is>
+      </c>
+      <c r="E244" t="n">
+        <v>10.32</v>
+      </c>
+      <c r="F244" t="n">
+        <v>-0.18</v>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="1" t="n">
         <v>46232</v>
       </c>
-      <c r="B243" t="inlineStr">
+      <c r="B245" t="inlineStr">
         <is>
           <t>Brazil - Serie B</t>
         </is>
       </c>
-      <c r="C243" t="inlineStr">
+      <c r="C245" t="inlineStr">
         <is>
           <t>Fortaleza</t>
         </is>
       </c>
-      <c r="D243" t="inlineStr">
+      <c r="D245" t="inlineStr">
         <is>
           <t>Botafogo SP</t>
         </is>
       </c>
-      <c r="E243" t="n">
+      <c r="E245" t="n">
         <v>10.56</v>
       </c>
-      <c r="F243" t="n">
-        <v>2.57</v>
+      <c r="F245" t="n">
+        <v>2.08</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily scrape output - 2026-07-29
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F245"/>
+  <dimension ref="A1:F249"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6796,6 +6796,110 @@
         <v>2.08</v>
       </c>
     </row>
+    <row r="246">
+      <c r="A246" s="1" t="n">
+        <v>46232</v>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>Finland - Ykkosliiga</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>Mikkelin Palloilijat</t>
+        </is>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>KaPa</t>
+        </is>
+      </c>
+      <c r="E246" t="n">
+        <v>10.45</v>
+      </c>
+      <c r="F246" t="n">
+        <v>0.13</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="1" t="n">
+        <v>46232</v>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>Iceland - 1. Deild</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>Fylkir</t>
+        </is>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>Volsungur</t>
+        </is>
+      </c>
+      <c r="E247" t="n">
+        <v>11.82</v>
+      </c>
+      <c r="F247" t="n">
+        <v>4.16</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" s="1" t="n">
+        <v>46232</v>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>Iceland - 1. Deild</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>Throttur Reykjavik</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>Afturelding</t>
+        </is>
+      </c>
+      <c r="E248" t="n">
+        <v>11.58</v>
+      </c>
+      <c r="F248" t="n">
+        <v>0.88</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" s="1" t="n">
+        <v>46232</v>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>Iceland - 1. Deild</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>UMF Grindavik</t>
+        </is>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>Leiknir Reykjavik</t>
+        </is>
+      </c>
+      <c r="E249" t="n">
+        <v>11.47</v>
+      </c>
+      <c r="F249" t="n">
+        <v>-0.29</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily scrape output - 2026-07-30
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F249"/>
+  <dimension ref="A1:F250"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6900,6 +6900,32 @@
         <v>-0.29</v>
       </c>
     </row>
+    <row r="250">
+      <c r="A250" s="1" t="n">
+        <v>46233</v>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>Finland - Ykkosliiga</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>JIPPO</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>JaPS</t>
+        </is>
+      </c>
+      <c r="E250" t="n">
+        <v>10.26</v>
+      </c>
+      <c r="F250" t="n">
+        <v>2.72</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily scrape output - 2026-07-31
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F250"/>
+  <dimension ref="A1:F289"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6926,6 +6926,1020 @@
         <v>2.72</v>
       </c>
     </row>
+    <row r="251">
+      <c r="A251" s="1" t="n">
+        <v>46234</v>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>Finland - Ykkosliiga</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>EIF</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>HJK Klubi 04</t>
+        </is>
+      </c>
+      <c r="E251" t="n">
+        <v>9.800000000000001</v>
+      </c>
+      <c r="F251" t="n">
+        <v>1.42</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="1" t="n">
+        <v>46234</v>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>Finland - Ykkosliiga</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>KTP</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>SJK Akatemia</t>
+        </is>
+      </c>
+      <c r="E252" t="n">
+        <v>10.74</v>
+      </c>
+      <c r="F252" t="n">
+        <v>3.37</v>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="1" t="n">
+        <v>46234</v>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>Finland - Ykkosliiga</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>PK-35</t>
+        </is>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>FC Haka</t>
+        </is>
+      </c>
+      <c r="E253" t="n">
+        <v>10.46</v>
+      </c>
+      <c r="F253" t="n">
+        <v>-0.19</v>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="1" t="n">
+        <v>46234</v>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>LKS Lodz</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>Polonia Bytom</t>
+        </is>
+      </c>
+      <c r="E254" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="F254" t="n">
+        <v>1.48</v>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="1" t="n">
+        <v>46234</v>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>Lechia Gdansk</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>Warta Poznan</t>
+        </is>
+      </c>
+      <c r="E255" t="n">
+        <v>10.05</v>
+      </c>
+      <c r="F255" t="n">
+        <v>0.87</v>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="1" t="n">
+        <v>46234</v>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>Motor Lublin</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>Jagiellonia Bialystok</t>
+        </is>
+      </c>
+      <c r="E256" t="n">
+        <v>10.04</v>
+      </c>
+      <c r="F256" t="n">
+        <v>-0.05</v>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="1" t="n">
+        <v>46234</v>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>Wisla Plock</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>Widzew Lodz</t>
+        </is>
+      </c>
+      <c r="E257" t="n">
+        <v>9.789999999999999</v>
+      </c>
+      <c r="F257" t="n">
+        <v>-0.32</v>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="1" t="n">
+        <v>46234</v>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>Arges Pitesti</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>Csikszereda</t>
+        </is>
+      </c>
+      <c r="E258" t="n">
+        <v>9.52</v>
+      </c>
+      <c r="F258" t="n">
+        <v>2.62</v>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="1" t="n">
+        <v>46234</v>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>Otelul Galati</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>Dinamo Bucuresti</t>
+        </is>
+      </c>
+      <c r="E259" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="F259" t="n">
+        <v>-1.02</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="1" t="n">
+        <v>46234</v>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>Oddevold</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>Norrby</t>
+        </is>
+      </c>
+      <c r="E260" t="n">
+        <v>10.46</v>
+      </c>
+      <c r="F260" t="n">
+        <v>1.94</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>FC Lahti</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>Jaro</t>
+        </is>
+      </c>
+      <c r="E261" t="n">
+        <v>9.859999999999999</v>
+      </c>
+      <c r="F261" t="n">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>Gnistan</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>KuPS</t>
+        </is>
+      </c>
+      <c r="E262" t="n">
+        <v>10.51</v>
+      </c>
+      <c r="F262" t="n">
+        <v>-2.05</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>TPS</t>
+        </is>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>IFK Mariehamn</t>
+        </is>
+      </c>
+      <c r="E263" t="n">
+        <v>10.32</v>
+      </c>
+      <c r="F263" t="n">
+        <v>2.35</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>Bryne</t>
+        </is>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>Stromsgodset</t>
+        </is>
+      </c>
+      <c r="E264" t="n">
+        <v>10.98</v>
+      </c>
+      <c r="F264" t="n">
+        <v>-0.97</v>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>Brage</t>
+        </is>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>Landskrona</t>
+        </is>
+      </c>
+      <c r="E265" t="n">
+        <v>10.46</v>
+      </c>
+      <c r="F265" t="n">
+        <v>0.36</v>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>Norrkoping</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>Helsingborgs</t>
+        </is>
+      </c>
+      <c r="E266" t="n">
+        <v>10.59</v>
+      </c>
+      <c r="F266" t="n">
+        <v>1.99</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>Ostersunds FK</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>Osters</t>
+        </is>
+      </c>
+      <c r="E267" t="n">
+        <v>10.61</v>
+      </c>
+      <c r="F267" t="n">
+        <v>1.32</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>Sandvikens IF</t>
+        </is>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>Sundsvall</t>
+        </is>
+      </c>
+      <c r="E268" t="n">
+        <v>10.32</v>
+      </c>
+      <c r="F268" t="n">
+        <v>1.91</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>Varbergs BoIS</t>
+        </is>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>Falkenbergs</t>
+        </is>
+      </c>
+      <c r="E269" t="n">
+        <v>9.98</v>
+      </c>
+      <c r="F269" t="n">
+        <v>1.57</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="1" t="n">
+        <v>46236</v>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>AC Oulu</t>
+        </is>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>Ilves</t>
+        </is>
+      </c>
+      <c r="E270" t="n">
+        <v>10.09</v>
+      </c>
+      <c r="F270" t="n">
+        <v>0.45</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="1" t="n">
+        <v>46236</v>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>VPS</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>Inter Turku</t>
+        </is>
+      </c>
+      <c r="E271" t="n">
+        <v>9.74</v>
+      </c>
+      <c r="F271" t="n">
+        <v>-0.11</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="1" t="n">
+        <v>46236</v>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>Egersunds</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>Sandnes Ulf</t>
+        </is>
+      </c>
+      <c r="E272" t="n">
+        <v>10.72</v>
+      </c>
+      <c r="F272" t="n">
+        <v>1.85</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" s="1" t="n">
+        <v>46236</v>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>Hodd</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>Moss</t>
+        </is>
+      </c>
+      <c r="E273" t="n">
+        <v>11</v>
+      </c>
+      <c r="F273" t="n">
+        <v>-0.33</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" s="1" t="n">
+        <v>46236</v>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>Kongsvinger</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>Strommen</t>
+        </is>
+      </c>
+      <c r="E274" t="n">
+        <v>11.09</v>
+      </c>
+      <c r="F274" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" s="1" t="n">
+        <v>46236</v>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>Lyn</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>Sogndal</t>
+        </is>
+      </c>
+      <c r="E275" t="n">
+        <v>11.16</v>
+      </c>
+      <c r="F275" t="n">
+        <v>0.96</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="1" t="n">
+        <v>46236</v>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>Odd BK</t>
+        </is>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>Asane Fotball</t>
+        </is>
+      </c>
+      <c r="E276" t="n">
+        <v>11.16</v>
+      </c>
+      <c r="F276" t="n">
+        <v>4.13</v>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" s="1" t="n">
+        <v>46236</v>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>Raufoss</t>
+        </is>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>Stabaek</t>
+        </is>
+      </c>
+      <c r="E277" t="n">
+        <v>11.11</v>
+      </c>
+      <c r="F277" t="n">
+        <v>-2.61</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" s="1" t="n">
+        <v>46236</v>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>Pogon Grodzisk Mazowiecki</t>
+        </is>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>Puszcza Niepolomice</t>
+        </is>
+      </c>
+      <c r="E278" t="n">
+        <v>10.76</v>
+      </c>
+      <c r="F278" t="n">
+        <v>0.82</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" s="1" t="n">
+        <v>46236</v>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>Ruch Chorzow</t>
+        </is>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>Miedz Legnica</t>
+        </is>
+      </c>
+      <c r="E279" t="n">
+        <v>10.68</v>
+      </c>
+      <c r="F279" t="n">
+        <v>0.17</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" s="1" t="n">
+        <v>46236</v>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>GKS Katowice</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>Radomiak Radom</t>
+        </is>
+      </c>
+      <c r="E280" t="n">
+        <v>10.34</v>
+      </c>
+      <c r="F280" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" s="1" t="n">
+        <v>46236</v>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>Legia Warsaw</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>Zaglebie Lubin</t>
+        </is>
+      </c>
+      <c r="E281" t="n">
+        <v>10.26</v>
+      </c>
+      <c r="F281" t="n">
+        <v>2.74</v>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" s="1" t="n">
+        <v>46236</v>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>Rapid Bucuresti</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>CFR Cluj</t>
+        </is>
+      </c>
+      <c r="E282" t="n">
+        <v>9.32</v>
+      </c>
+      <c r="F282" t="n">
+        <v>0.49</v>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" s="1" t="n">
+        <v>46237</v>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>SJK</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>HJK Helsinki</t>
+        </is>
+      </c>
+      <c r="E283" t="n">
+        <v>10.69</v>
+      </c>
+      <c r="F283" t="n">
+        <v>0.39</v>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" s="1" t="n">
+        <v>46237</v>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>Ranheim</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>Haugesund</t>
+        </is>
+      </c>
+      <c r="E284" t="n">
+        <v>11.44</v>
+      </c>
+      <c r="F284" t="n">
+        <v>-0.66</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" s="1" t="n">
+        <v>46237</v>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>Chrobry Glogow</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>Odra Opole</t>
+        </is>
+      </c>
+      <c r="E285" t="n">
+        <v>10.55</v>
+      </c>
+      <c r="F285" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" s="1" t="n">
+        <v>46237</v>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>Cracovia Krakow</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>Pogon Szczecin</t>
+        </is>
+      </c>
+      <c r="E286" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="F286" t="n">
+        <v>1.21</v>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" s="1" t="n">
+        <v>46237</v>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>FCSB</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>Farul Constanta</t>
+        </is>
+      </c>
+      <c r="E287" t="n">
+        <v>10.09</v>
+      </c>
+      <c r="F287" t="n">
+        <v>2.12</v>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" s="1" t="n">
+        <v>46237</v>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>Universitatea Cluj</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>Botosani</t>
+        </is>
+      </c>
+      <c r="E288" t="n">
+        <v>9.779999999999999</v>
+      </c>
+      <c r="F288" t="n">
+        <v>1.58</v>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" s="1" t="n">
+        <v>46237</v>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>Orebro SK</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>Varnamo</t>
+        </is>
+      </c>
+      <c r="E289" t="n">
+        <v>10.24</v>
+      </c>
+      <c r="F289" t="n">
+        <v>0.45</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily scrape output - 2026-08-01
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F289"/>
+  <dimension ref="A1:F296"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7232,10 +7232,10 @@
         </is>
       </c>
       <c r="E262" t="n">
-        <v>10.51</v>
+        <v>10.37</v>
       </c>
       <c r="F262" t="n">
-        <v>-2.05</v>
+        <v>-1.58</v>
       </c>
     </row>
     <row r="263">
@@ -7284,10 +7284,10 @@
         </is>
       </c>
       <c r="E264" t="n">
-        <v>10.98</v>
+        <v>11.33</v>
       </c>
       <c r="F264" t="n">
-        <v>-0.97</v>
+        <v>-1.06</v>
       </c>
     </row>
     <row r="265">
@@ -7296,24 +7296,24 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>Brage</t>
+          <t>Arka Gdynia</t>
         </is>
       </c>
       <c r="D265" t="inlineStr">
         <is>
-          <t>Landskrona</t>
+          <t>Stal Rzeszow</t>
         </is>
       </c>
       <c r="E265" t="n">
-        <v>10.46</v>
+        <v>10.97</v>
       </c>
       <c r="F265" t="n">
-        <v>0.36</v>
+        <v>2.42</v>
       </c>
     </row>
     <row r="266">
@@ -7322,24 +7322,24 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>Norrkoping</t>
+          <t>Pogon Siedlce</t>
         </is>
       </c>
       <c r="D266" t="inlineStr">
         <is>
-          <t>Helsingborgs</t>
+          <t>Nieciecza</t>
         </is>
       </c>
       <c r="E266" t="n">
-        <v>10.59</v>
+        <v>10.64</v>
       </c>
       <c r="F266" t="n">
-        <v>1.99</v>
+        <v>-1.59</v>
       </c>
     </row>
     <row r="267">
@@ -7348,24 +7348,24 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>Ostersunds FK</t>
+          <t>Polonia Warsaw</t>
         </is>
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>Osters</t>
+          <t>Unia Skierniewice</t>
         </is>
       </c>
       <c r="E267" t="n">
-        <v>10.61</v>
+        <v>10.62</v>
       </c>
       <c r="F267" t="n">
-        <v>1.32</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="268">
@@ -7374,24 +7374,24 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>Sandvikens IF</t>
+          <t>Piast Gliwice</t>
         </is>
       </c>
       <c r="D268" t="inlineStr">
         <is>
-          <t>Sundsvall</t>
+          <t>Wisla Krakow</t>
         </is>
       </c>
       <c r="E268" t="n">
-        <v>10.32</v>
+        <v>10.56</v>
       </c>
       <c r="F268" t="n">
-        <v>1.91</v>
+        <v>0.83</v>
       </c>
     </row>
     <row r="269">
@@ -7400,206 +7400,206 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>Varbergs BoIS</t>
+          <t>Wieczysta Krakow</t>
         </is>
       </c>
       <c r="D269" t="inlineStr">
         <is>
-          <t>Falkenbergs</t>
+          <t>Lech Poznan</t>
         </is>
       </c>
       <c r="E269" t="n">
-        <v>9.98</v>
+        <v>10.51</v>
       </c>
       <c r="F269" t="n">
-        <v>1.57</v>
+        <v>-1.18</v>
       </c>
     </row>
     <row r="270">
       <c r="A270" s="1" t="n">
-        <v>46236</v>
+        <v>46235</v>
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>Finland - Veikkausliiga</t>
+          <t>Romania - Liga 1</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>AC Oulu</t>
+          <t>Universitatea Craiova</t>
         </is>
       </c>
       <c r="D270" t="inlineStr">
         <is>
-          <t>Ilves</t>
+          <t>Petrolul Ploiesti</t>
         </is>
       </c>
       <c r="E270" t="n">
-        <v>10.09</v>
+        <v>9.67</v>
       </c>
       <c r="F270" t="n">
-        <v>0.45</v>
+        <v>2.99</v>
       </c>
     </row>
     <row r="271">
       <c r="A271" s="1" t="n">
-        <v>46236</v>
+        <v>46235</v>
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>Finland - Veikkausliiga</t>
+          <t>Romania - Liga 1</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>VPS</t>
+          <t>Voluntari</t>
         </is>
       </c>
       <c r="D271" t="inlineStr">
         <is>
-          <t>Inter Turku</t>
+          <t>UTA Arad</t>
         </is>
       </c>
       <c r="E271" t="n">
-        <v>9.74</v>
+        <v>9.380000000000001</v>
       </c>
       <c r="F271" t="n">
-        <v>-0.11</v>
+        <v>-0.08</v>
       </c>
     </row>
     <row r="272">
       <c r="A272" s="1" t="n">
-        <v>46236</v>
+        <v>46235</v>
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>Norway - 1st Division</t>
+          <t>Sweden - Superettan</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>Egersunds</t>
+          <t>Brage</t>
         </is>
       </c>
       <c r="D272" t="inlineStr">
         <is>
-          <t>Sandnes Ulf</t>
+          <t>Landskrona</t>
         </is>
       </c>
       <c r="E272" t="n">
-        <v>10.72</v>
+        <v>10.46</v>
       </c>
       <c r="F272" t="n">
-        <v>1.85</v>
+        <v>0.36</v>
       </c>
     </row>
     <row r="273">
       <c r="A273" s="1" t="n">
-        <v>46236</v>
+        <v>46235</v>
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>Norway - 1st Division</t>
+          <t>Sweden - Superettan</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>Hodd</t>
+          <t>Norrkoping</t>
         </is>
       </c>
       <c r="D273" t="inlineStr">
         <is>
-          <t>Moss</t>
+          <t>Helsingborgs</t>
         </is>
       </c>
       <c r="E273" t="n">
-        <v>11</v>
+        <v>10.59</v>
       </c>
       <c r="F273" t="n">
-        <v>-0.33</v>
+        <v>1.99</v>
       </c>
     </row>
     <row r="274">
       <c r="A274" s="1" t="n">
-        <v>46236</v>
+        <v>46235</v>
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>Norway - 1st Division</t>
+          <t>Sweden - Superettan</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>Kongsvinger</t>
+          <t>Ostersunds FK</t>
         </is>
       </c>
       <c r="D274" t="inlineStr">
         <is>
-          <t>Strommen</t>
+          <t>Osters</t>
         </is>
       </c>
       <c r="E274" t="n">
-        <v>11.09</v>
+        <v>10.16</v>
       </c>
       <c r="F274" t="n">
-        <v>3</v>
+        <v>1.49</v>
       </c>
     </row>
     <row r="275">
       <c r="A275" s="1" t="n">
-        <v>46236</v>
+        <v>46235</v>
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>Norway - 1st Division</t>
+          <t>Sweden - Superettan</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>Lyn</t>
+          <t>Sandvikens IF</t>
         </is>
       </c>
       <c r="D275" t="inlineStr">
         <is>
-          <t>Sogndal</t>
+          <t>Sundsvall</t>
         </is>
       </c>
       <c r="E275" t="n">
-        <v>11.16</v>
+        <v>10.31</v>
       </c>
       <c r="F275" t="n">
-        <v>0.96</v>
+        <v>1.57</v>
       </c>
     </row>
     <row r="276">
       <c r="A276" s="1" t="n">
-        <v>46236</v>
+        <v>46235</v>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>Norway - 1st Division</t>
+          <t>Sweden - Superettan</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>Odd BK</t>
+          <t>Varbergs BoIS</t>
         </is>
       </c>
       <c r="D276" t="inlineStr">
         <is>
-          <t>Asane Fotball</t>
+          <t>Falkenbergs</t>
         </is>
       </c>
       <c r="E276" t="n">
-        <v>11.16</v>
+        <v>9.949999999999999</v>
       </c>
       <c r="F276" t="n">
-        <v>4.13</v>
+        <v>1.57</v>
       </c>
     </row>
     <row r="277">
@@ -7608,24 +7608,24 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>Norway - 1st Division</t>
+          <t>Finland - Veikkausliiga</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>Raufoss</t>
+          <t>AC Oulu</t>
         </is>
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>Stabaek</t>
+          <t>Ilves</t>
         </is>
       </c>
       <c r="E277" t="n">
-        <v>11.11</v>
+        <v>10.2</v>
       </c>
       <c r="F277" t="n">
-        <v>-2.61</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="278">
@@ -7634,24 +7634,24 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>Poland - 1st Liga</t>
+          <t>Finland - Veikkausliiga</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>Pogon Grodzisk Mazowiecki</t>
+          <t>VPS</t>
         </is>
       </c>
       <c r="D278" t="inlineStr">
         <is>
-          <t>Puszcza Niepolomice</t>
+          <t>Inter Turku</t>
         </is>
       </c>
       <c r="E278" t="n">
-        <v>10.76</v>
+        <v>9.77</v>
       </c>
       <c r="F278" t="n">
-        <v>0.82</v>
+        <v>-0.16</v>
       </c>
     </row>
     <row r="279">
@@ -7660,24 +7660,24 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>Poland - 1st Liga</t>
+          <t>Norway - 1st Division</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>Ruch Chorzow</t>
+          <t>Egersunds</t>
         </is>
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>Miedz Legnica</t>
+          <t>Sandnes Ulf</t>
         </is>
       </c>
       <c r="E279" t="n">
-        <v>10.68</v>
+        <v>10.72</v>
       </c>
       <c r="F279" t="n">
-        <v>0.17</v>
+        <v>1.85</v>
       </c>
     </row>
     <row r="280">
@@ -7686,24 +7686,24 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Norway - 1st Division</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>GKS Katowice</t>
+          <t>Hodd</t>
         </is>
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>Radomiak Radom</t>
+          <t>Moss</t>
         </is>
       </c>
       <c r="E280" t="n">
-        <v>10.34</v>
+        <v>10.83</v>
       </c>
       <c r="F280" t="n">
-        <v>1</v>
+        <v>-0.19</v>
       </c>
     </row>
     <row r="281">
@@ -7712,24 +7712,24 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Norway - 1st Division</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>Legia Warsaw</t>
+          <t>Kongsvinger</t>
         </is>
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>Zaglebie Lubin</t>
+          <t>Strommen</t>
         </is>
       </c>
       <c r="E281" t="n">
-        <v>10.26</v>
+        <v>11.12</v>
       </c>
       <c r="F281" t="n">
-        <v>2.74</v>
+        <v>3.57</v>
       </c>
     </row>
     <row r="282">
@@ -7738,55 +7738,55 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>Romania - Liga 1</t>
+          <t>Norway - 1st Division</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>Rapid Bucuresti</t>
+          <t>Lyn</t>
         </is>
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>CFR Cluj</t>
+          <t>Sogndal</t>
         </is>
       </c>
       <c r="E282" t="n">
-        <v>9.32</v>
+        <v>10.67</v>
       </c>
       <c r="F282" t="n">
-        <v>0.49</v>
+        <v>1</v>
       </c>
     </row>
     <row r="283">
       <c r="A283" s="1" t="n">
-        <v>46237</v>
+        <v>46236</v>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>Finland - Veikkausliiga</t>
+          <t>Norway - 1st Division</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>SJK</t>
+          <t>Odd BK</t>
         </is>
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>HJK Helsinki</t>
+          <t>Asane Fotball</t>
         </is>
       </c>
       <c r="E283" t="n">
-        <v>10.69</v>
+        <v>11.16</v>
       </c>
       <c r="F283" t="n">
-        <v>0.39</v>
+        <v>4.13</v>
       </c>
     </row>
     <row r="284">
       <c r="A284" s="1" t="n">
-        <v>46237</v>
+        <v>46236</v>
       </c>
       <c r="B284" t="inlineStr">
         <is>
@@ -7795,24 +7795,24 @@
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>Ranheim</t>
+          <t>Raufoss</t>
         </is>
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>Haugesund</t>
+          <t>Stabaek</t>
         </is>
       </c>
       <c r="E284" t="n">
-        <v>11.44</v>
+        <v>11.11</v>
       </c>
       <c r="F284" t="n">
-        <v>-0.66</v>
+        <v>-2.61</v>
       </c>
     </row>
     <row r="285">
       <c r="A285" s="1" t="n">
-        <v>46237</v>
+        <v>46236</v>
       </c>
       <c r="B285" t="inlineStr">
         <is>
@@ -7821,123 +7821,305 @@
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>Chrobry Glogow</t>
+          <t>Pogon Grodzisk Mazowiecki</t>
         </is>
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>Odra Opole</t>
+          <t>Puszcza Niepolomice</t>
         </is>
       </c>
       <c r="E285" t="n">
-        <v>10.55</v>
+        <v>10.47</v>
       </c>
       <c r="F285" t="n">
-        <v>0.4</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="286">
       <c r="A286" s="1" t="n">
-        <v>46237</v>
+        <v>46236</v>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>Cracovia Krakow</t>
+          <t>Ruch Chorzow</t>
         </is>
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>Pogon Szczecin</t>
+          <t>Miedz Legnica</t>
         </is>
       </c>
       <c r="E286" t="n">
-        <v>10.3</v>
+        <v>10.68</v>
       </c>
       <c r="F286" t="n">
-        <v>1.21</v>
+        <v>0.17</v>
       </c>
     </row>
     <row r="287">
       <c r="A287" s="1" t="n">
-        <v>46237</v>
+        <v>46236</v>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>Romania - Liga 1</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>FCSB</t>
+          <t>GKS Katowice</t>
         </is>
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>Farul Constanta</t>
+          <t>Radomiak Radom</t>
         </is>
       </c>
       <c r="E287" t="n">
-        <v>10.09</v>
+        <v>10.34</v>
       </c>
       <c r="F287" t="n">
-        <v>2.12</v>
+        <v>1</v>
       </c>
     </row>
     <row r="288">
       <c r="A288" s="1" t="n">
-        <v>46237</v>
+        <v>46236</v>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>Romania - Liga 1</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>Universitatea Cluj</t>
+          <t>Legia Warsaw</t>
         </is>
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>Botosani</t>
+          <t>Zaglebie Lubin</t>
         </is>
       </c>
       <c r="E288" t="n">
-        <v>9.779999999999999</v>
+        <v>10.26</v>
       </c>
       <c r="F288" t="n">
-        <v>1.58</v>
+        <v>2.74</v>
       </c>
     </row>
     <row r="289">
       <c r="A289" s="1" t="n">
+        <v>46236</v>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>Rapid Bucuresti</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>CFR Cluj</t>
+        </is>
+      </c>
+      <c r="E289" t="n">
+        <v>9.32</v>
+      </c>
+      <c r="F289" t="n">
+        <v>0.49</v>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" s="1" t="n">
         <v>46237</v>
       </c>
-      <c r="B289" t="inlineStr">
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>SJK</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>HJK Helsinki</t>
+        </is>
+      </c>
+      <c r="E290" t="n">
+        <v>10.69</v>
+      </c>
+      <c r="F290" t="n">
+        <v>0.39</v>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" s="1" t="n">
+        <v>46237</v>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>Ranheim</t>
+        </is>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>Haugesund</t>
+        </is>
+      </c>
+      <c r="E291" t="n">
+        <v>11.04</v>
+      </c>
+      <c r="F291" t="n">
+        <v>-0.6</v>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" s="1" t="n">
+        <v>46237</v>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>Chrobry Glogow</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>Odra Opole</t>
+        </is>
+      </c>
+      <c r="E292" t="n">
+        <v>10.55</v>
+      </c>
+      <c r="F292" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" s="1" t="n">
+        <v>46237</v>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>Cracovia Krakow</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>Pogon Szczecin</t>
+        </is>
+      </c>
+      <c r="E293" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="F293" t="n">
+        <v>1.21</v>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" s="1" t="n">
+        <v>46237</v>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>FCSB</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>Farul Constanta</t>
+        </is>
+      </c>
+      <c r="E294" t="n">
+        <v>10.09</v>
+      </c>
+      <c r="F294" t="n">
+        <v>2.12</v>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" s="1" t="n">
+        <v>46237</v>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>Universitatea Cluj</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>Botosani</t>
+        </is>
+      </c>
+      <c r="E295" t="n">
+        <v>9.779999999999999</v>
+      </c>
+      <c r="F295" t="n">
+        <v>1.58</v>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" s="1" t="n">
+        <v>46237</v>
+      </c>
+      <c r="B296" t="inlineStr">
         <is>
           <t>Sweden - Superettan</t>
         </is>
       </c>
-      <c r="C289" t="inlineStr">
+      <c r="C296" t="inlineStr">
         <is>
           <t>Orebro SK</t>
         </is>
       </c>
-      <c r="D289" t="inlineStr">
+      <c r="D296" t="inlineStr">
         <is>
           <t>Varnamo</t>
         </is>
       </c>
-      <c r="E289" t="n">
-        <v>10.24</v>
-      </c>
-      <c r="F289" t="n">
-        <v>0.45</v>
+      <c r="E296" t="n">
+        <v>10.17</v>
+      </c>
+      <c r="F296" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily scrape output - 2026-08-02
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F296"/>
+  <dimension ref="A1:F299"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7622,7 +7622,7 @@
         </is>
       </c>
       <c r="E277" t="n">
-        <v>10.2</v>
+        <v>10.21</v>
       </c>
       <c r="F277" t="n">
         <v>0.52</v>
@@ -7648,10 +7648,10 @@
         </is>
       </c>
       <c r="E278" t="n">
-        <v>9.77</v>
+        <v>9.82</v>
       </c>
       <c r="F278" t="n">
-        <v>-0.16</v>
+        <v>-0.15</v>
       </c>
     </row>
     <row r="279">
@@ -7703,7 +7703,7 @@
         <v>10.83</v>
       </c>
       <c r="F280" t="n">
-        <v>-0.19</v>
+        <v>-0.13</v>
       </c>
     </row>
     <row r="281">
@@ -7752,7 +7752,7 @@
         </is>
       </c>
       <c r="E282" t="n">
-        <v>10.67</v>
+        <v>10.72</v>
       </c>
       <c r="F282" t="n">
         <v>1</v>
@@ -7778,10 +7778,10 @@
         </is>
       </c>
       <c r="E283" t="n">
-        <v>11.16</v>
+        <v>11.09</v>
       </c>
       <c r="F283" t="n">
-        <v>4.13</v>
+        <v>3.51</v>
       </c>
     </row>
     <row r="284">
@@ -7804,10 +7804,10 @@
         </is>
       </c>
       <c r="E284" t="n">
-        <v>11.11</v>
+        <v>11.17</v>
       </c>
       <c r="F284" t="n">
-        <v>-2.61</v>
+        <v>-2.62</v>
       </c>
     </row>
     <row r="285">
@@ -7859,7 +7859,7 @@
         <v>10.68</v>
       </c>
       <c r="F286" t="n">
-        <v>0.17</v>
+        <v>0.32</v>
       </c>
     </row>
     <row r="287">
@@ -7908,10 +7908,10 @@
         </is>
       </c>
       <c r="E288" t="n">
-        <v>10.26</v>
+        <v>10.13</v>
       </c>
       <c r="F288" t="n">
-        <v>2.74</v>
+        <v>2.72</v>
       </c>
     </row>
     <row r="289">
@@ -7920,102 +7920,102 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>Romania - Liga 1</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>Rapid Bucuresti</t>
+          <t>Slask Wroclaw</t>
         </is>
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>CFR Cluj</t>
+          <t>Rakow Czestochowa</t>
         </is>
       </c>
       <c r="E289" t="n">
-        <v>9.32</v>
+        <v>9.99</v>
       </c>
       <c r="F289" t="n">
-        <v>0.49</v>
+        <v>-0.84</v>
       </c>
     </row>
     <row r="290">
       <c r="A290" s="1" t="n">
-        <v>46237</v>
+        <v>46236</v>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>Finland - Veikkausliiga</t>
+          <t>Romania - Liga 1</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>SJK</t>
+          <t>Corvinul Hunedoara</t>
         </is>
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>HJK Helsinki</t>
+          <t>Sepsi</t>
         </is>
       </c>
       <c r="E290" t="n">
-        <v>10.69</v>
+        <v>9.380000000000001</v>
       </c>
       <c r="F290" t="n">
-        <v>0.39</v>
+        <v>1.21</v>
       </c>
     </row>
     <row r="291">
       <c r="A291" s="1" t="n">
-        <v>46237</v>
+        <v>46236</v>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>Norway - 1st Division</t>
+          <t>Romania - Liga 1</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>Ranheim</t>
+          <t>Rapid Bucuresti</t>
         </is>
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>Haugesund</t>
+          <t>CFR Cluj</t>
         </is>
       </c>
       <c r="E291" t="n">
-        <v>11.04</v>
+        <v>9.31</v>
       </c>
       <c r="F291" t="n">
-        <v>-0.6</v>
+        <v>0.53</v>
       </c>
     </row>
     <row r="292">
       <c r="A292" s="1" t="n">
-        <v>46237</v>
+        <v>46236</v>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>Poland - 1st Liga</t>
+          <t>Sweden - Superettan</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>Chrobry Glogow</t>
+          <t>Nordic United</t>
         </is>
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>Odra Opole</t>
+          <t>Ljungskile</t>
         </is>
       </c>
       <c r="E292" t="n">
-        <v>10.55</v>
+        <v>10.33</v>
       </c>
       <c r="F292" t="n">
-        <v>0.4</v>
+        <v>0.82</v>
       </c>
     </row>
     <row r="293">
@@ -8024,24 +8024,24 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Finland - Veikkausliiga</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>Cracovia Krakow</t>
+          <t>SJK</t>
         </is>
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>Pogon Szczecin</t>
+          <t>HJK Helsinki</t>
         </is>
       </c>
       <c r="E293" t="n">
-        <v>10.3</v>
+        <v>10.47</v>
       </c>
       <c r="F293" t="n">
-        <v>1.21</v>
+        <v>-0.05</v>
       </c>
     </row>
     <row r="294">
@@ -8050,24 +8050,24 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>Romania - Liga 1</t>
+          <t>Norway - 1st Division</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>FCSB</t>
+          <t>Ranheim</t>
         </is>
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>Farul Constanta</t>
+          <t>Haugesund</t>
         </is>
       </c>
       <c r="E294" t="n">
-        <v>10.09</v>
+        <v>11.04</v>
       </c>
       <c r="F294" t="n">
-        <v>2.12</v>
+        <v>-0.6</v>
       </c>
     </row>
     <row r="295">
@@ -8076,24 +8076,24 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>Romania - Liga 1</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>Universitatea Cluj</t>
+          <t>Chrobry Glogow</t>
         </is>
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>Botosani</t>
+          <t>Odra Opole</t>
         </is>
       </c>
       <c r="E295" t="n">
-        <v>9.779999999999999</v>
+        <v>10.55</v>
       </c>
       <c r="F295" t="n">
-        <v>1.58</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="296">
@@ -8102,23 +8102,101 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>Cracovia Krakow</t>
+        </is>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>Pogon Szczecin</t>
+        </is>
+      </c>
+      <c r="E296" t="n">
+        <v>10.26</v>
+      </c>
+      <c r="F296" t="n">
+        <v>1.35</v>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" s="1" t="n">
+        <v>46237</v>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>FCSB</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>Farul Constanta</t>
+        </is>
+      </c>
+      <c r="E297" t="n">
+        <v>10.09</v>
+      </c>
+      <c r="F297" t="n">
+        <v>2.12</v>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" s="1" t="n">
+        <v>46237</v>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>Universitatea Cluj</t>
+        </is>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>Botosani</t>
+        </is>
+      </c>
+      <c r="E298" t="n">
+        <v>9.779999999999999</v>
+      </c>
+      <c r="F298" t="n">
+        <v>1.58</v>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" s="1" t="n">
+        <v>46237</v>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
           <t>Sweden - Superettan</t>
         </is>
       </c>
-      <c r="C296" t="inlineStr">
+      <c r="C299" t="inlineStr">
         <is>
           <t>Orebro SK</t>
         </is>
       </c>
-      <c r="D296" t="inlineStr">
+      <c r="D299" t="inlineStr">
         <is>
           <t>Varnamo</t>
         </is>
       </c>
-      <c r="E296" t="n">
+      <c r="E299" t="n">
         <v>10.17</v>
       </c>
-      <c r="F296" t="n">
+      <c r="F299" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily scrape output - 2026-08-03
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -8038,10 +8038,10 @@
         </is>
       </c>
       <c r="E293" t="n">
-        <v>10.47</v>
+        <v>10.49</v>
       </c>
       <c r="F293" t="n">
-        <v>-0.05</v>
+        <v>-0.14</v>
       </c>
     </row>
     <row r="294">
@@ -8090,10 +8090,10 @@
         </is>
       </c>
       <c r="E295" t="n">
-        <v>10.55</v>
+        <v>10.45</v>
       </c>
       <c r="F295" t="n">
-        <v>0.4</v>
+        <v>0.41</v>
       </c>
     </row>
     <row r="296">
@@ -8116,10 +8116,10 @@
         </is>
       </c>
       <c r="E296" t="n">
-        <v>10.26</v>
+        <v>10.29</v>
       </c>
       <c r="F296" t="n">
-        <v>1.35</v>
+        <v>1.22</v>
       </c>
     </row>
     <row r="297">
@@ -8142,10 +8142,10 @@
         </is>
       </c>
       <c r="E297" t="n">
-        <v>10.09</v>
+        <v>10.11</v>
       </c>
       <c r="F297" t="n">
-        <v>2.12</v>
+        <v>2.15</v>
       </c>
     </row>
     <row r="298">

</xml_diff>

<commit_message>
Daily scrape output - 2026-08-06
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F299"/>
+  <dimension ref="A1:F300"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8200,6 +8200,32 @@
         <v>1</v>
       </c>
     </row>
+    <row r="300">
+      <c r="A300" s="1" t="n">
+        <v>46240</v>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>Iceland - 1. Deild</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>IR Reykjavik</t>
+        </is>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>Aegir</t>
+        </is>
+      </c>
+      <c r="E300" t="n">
+        <v>11.76</v>
+      </c>
+      <c r="F300" t="n">
+        <v>3.65</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily scrape output - 2026-08-07
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F300"/>
+  <dimension ref="A1:F315"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8226,6 +8226,396 @@
         <v>3.65</v>
       </c>
     </row>
+    <row r="301">
+      <c r="A301" s="1" t="n">
+        <v>46241</v>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>Ceara</t>
+        </is>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>Ponte Preta</t>
+        </is>
+      </c>
+      <c r="E301" t="n">
+        <v>10.73</v>
+      </c>
+      <c r="F301" t="n">
+        <v>3.35</v>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" s="1" t="n">
+        <v>46241</v>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>Operario Ferroviario</t>
+        </is>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>Sao Bernardo</t>
+        </is>
+      </c>
+      <c r="E302" t="n">
+        <v>10.45</v>
+      </c>
+      <c r="F302" t="n">
+        <v>1.94</v>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" s="1" t="n">
+        <v>46241</v>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>SJK</t>
+        </is>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>Gnistan</t>
+        </is>
+      </c>
+      <c r="E303" t="n">
+        <v>10.57</v>
+      </c>
+      <c r="F303" t="n">
+        <v>1.21</v>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" s="1" t="n">
+        <v>46241</v>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>Iceland - 1. Deild</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>Afturelding</t>
+        </is>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>UMF Grindavik</t>
+        </is>
+      </c>
+      <c r="E304" t="n">
+        <v>12.01</v>
+      </c>
+      <c r="F304" t="n">
+        <v>3.88</v>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" s="1" t="n">
+        <v>46241</v>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>Iceland - 1. Deild</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>Leiknir Reykjavik</t>
+        </is>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>Fylkir</t>
+        </is>
+      </c>
+      <c r="E305" t="n">
+        <v>11.45</v>
+      </c>
+      <c r="F305" t="n">
+        <v>-1.41</v>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" s="1" t="n">
+        <v>46241</v>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>Polonia Bytom</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>Pogon Siedlce</t>
+        </is>
+      </c>
+      <c r="E306" t="n">
+        <v>10.86</v>
+      </c>
+      <c r="F306" t="n">
+        <v>2.65</v>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" s="1" t="n">
+        <v>46241</v>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>Polonia Warsaw</t>
+        </is>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>Ruch Chorzow</t>
+        </is>
+      </c>
+      <c r="E307" t="n">
+        <v>10.84</v>
+      </c>
+      <c r="F307" t="n">
+        <v>1.33</v>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" s="1" t="n">
+        <v>46241</v>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>Wisla Krakow</t>
+        </is>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>Wisla Plock</t>
+        </is>
+      </c>
+      <c r="E308" t="n">
+        <v>10.94</v>
+      </c>
+      <c r="F308" t="n">
+        <v>2.22</v>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" s="1" t="n">
+        <v>46241</v>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>UTA Arad</t>
+        </is>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>Rapid Bucuresti</t>
+        </is>
+      </c>
+      <c r="E309" t="n">
+        <v>9.84</v>
+      </c>
+      <c r="F309" t="n">
+        <v>0.16</v>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" s="1" t="n">
+        <v>46241</v>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>Ostersunds FK</t>
+        </is>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>Sundsvall</t>
+        </is>
+      </c>
+      <c r="E310" t="n">
+        <v>10.32</v>
+      </c>
+      <c r="F310" t="n">
+        <v>3.07</v>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" s="1" t="n">
+        <v>46242</v>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>Miedz Legnica</t>
+        </is>
+      </c>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>Pogon Grodzisk Mazowiecki</t>
+        </is>
+      </c>
+      <c r="E311" t="n">
+        <v>11.21</v>
+      </c>
+      <c r="F311" t="n">
+        <v>1.98</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" s="1" t="n">
+        <v>46243</v>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>Cuiaba</t>
+        </is>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>Fortaleza</t>
+        </is>
+      </c>
+      <c r="E312" t="n">
+        <v>10.09</v>
+      </c>
+      <c r="F312" t="n">
+        <v>0.83</v>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" s="1" t="n">
+        <v>46243</v>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>Stromsgodset</t>
+        </is>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>Egersunds</t>
+        </is>
+      </c>
+      <c r="E313" t="n">
+        <v>11.29</v>
+      </c>
+      <c r="F313" t="n">
+        <v>2.09</v>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" s="1" t="n">
+        <v>46243</v>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>Jagiellonia Bialystok</t>
+        </is>
+      </c>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>Widzew Lodz</t>
+        </is>
+      </c>
+      <c r="E314" t="n">
+        <v>9.69</v>
+      </c>
+      <c r="F314" t="n">
+        <v>1.34</v>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>Goias</t>
+        </is>
+      </c>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>Londrina</t>
+        </is>
+      </c>
+      <c r="E315" t="n">
+        <v>10.87</v>
+      </c>
+      <c r="F315" t="n">
+        <v>2.16</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily scrape output - 2026-08-08
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F315"/>
+  <dimension ref="A1:F354"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8492,29 +8492,29 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Poland - 1st Liga</t>
+          <t>Brazil - Serie B</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>Miedz Legnica</t>
+          <t>Botafogo SP</t>
         </is>
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>Pogon Grodzisk Mazowiecki</t>
+          <t>America Mineiro</t>
         </is>
       </c>
       <c r="E311" t="n">
-        <v>11.21</v>
+        <v>10.61</v>
       </c>
       <c r="F311" t="n">
-        <v>1.98</v>
+        <v>1.72</v>
       </c>
     </row>
     <row r="312">
       <c r="A312" s="1" t="n">
-        <v>46243</v>
+        <v>46242</v>
       </c>
       <c r="B312" t="inlineStr">
         <is>
@@ -8523,97 +8523,1111 @@
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>Cuiaba</t>
+          <t>Vila Nova</t>
         </is>
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>Fortaleza</t>
+          <t>Sport Recife</t>
         </is>
       </c>
       <c r="E312" t="n">
-        <v>10.09</v>
+        <v>10.28</v>
       </c>
       <c r="F312" t="n">
-        <v>0.83</v>
+        <v>1.06</v>
       </c>
     </row>
     <row r="313">
       <c r="A313" s="1" t="n">
-        <v>46243</v>
+        <v>46242</v>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Norway - 1st Division</t>
+          <t>Finland - Veikkausliiga</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>Stromsgodset</t>
+          <t>Jaro</t>
         </is>
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>Egersunds</t>
+          <t>VPS</t>
         </is>
       </c>
       <c r="E313" t="n">
-        <v>11.29</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="F313" t="n">
-        <v>2.09</v>
+        <v>-1.45</v>
       </c>
     </row>
     <row r="314">
       <c r="A314" s="1" t="n">
-        <v>46243</v>
+        <v>46242</v>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Finland - Ykkosliiga</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>Jagiellonia Bialystok</t>
+          <t>KaPa</t>
         </is>
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>Widzew Lodz</t>
+          <t>EIF</t>
         </is>
       </c>
       <c r="E314" t="n">
-        <v>9.69</v>
+        <v>10.36</v>
       </c>
       <c r="F314" t="n">
-        <v>1.34</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="315">
       <c r="A315" s="1" t="n">
+        <v>46242</v>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>Finland - Ykkosliiga</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>SJK Akatemia</t>
+        </is>
+      </c>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>PK-35</t>
+        </is>
+      </c>
+      <c r="E315" t="n">
+        <v>10.47</v>
+      </c>
+      <c r="F315" t="n">
+        <v>-1.49</v>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" s="1" t="n">
+        <v>46242</v>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>Iceland - 1. Deild</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>UMF Njardvik</t>
+        </is>
+      </c>
+      <c r="D316" t="inlineStr">
+        <is>
+          <t>Vestri</t>
+        </is>
+      </c>
+      <c r="E316" t="n">
+        <v>11.15</v>
+      </c>
+      <c r="F316" t="n">
+        <v>2.47</v>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" s="1" t="n">
+        <v>46242</v>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>Stabaek</t>
+        </is>
+      </c>
+      <c r="D317" t="inlineStr">
+        <is>
+          <t>Lyn</t>
+        </is>
+      </c>
+      <c r="E317" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="F317" t="n">
+        <v>2.71</v>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" s="1" t="n">
+        <v>46242</v>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>Miedz Legnica</t>
+        </is>
+      </c>
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>Pogon Grodzisk Mazowiecki</t>
+        </is>
+      </c>
+      <c r="E318" t="n">
+        <v>11.16</v>
+      </c>
+      <c r="F318" t="n">
+        <v>1.97</v>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" s="1" t="n">
+        <v>46242</v>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>Podbeskidzie Bielsko-Biala</t>
+        </is>
+      </c>
+      <c r="D319" t="inlineStr">
+        <is>
+          <t>Lechia Gdansk</t>
+        </is>
+      </c>
+      <c r="E319" t="n">
+        <v>9.83</v>
+      </c>
+      <c r="F319" t="n">
+        <v>2.18</v>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" s="1" t="n">
+        <v>46242</v>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>Puszcza Niepolomice</t>
+        </is>
+      </c>
+      <c r="D320" t="inlineStr">
+        <is>
+          <t>Odra Opole</t>
+        </is>
+      </c>
+      <c r="E320" t="n">
+        <v>10.04</v>
+      </c>
+      <c r="F320" t="n">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" s="1" t="n">
+        <v>46242</v>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>Stal Mielec</t>
+        </is>
+      </c>
+      <c r="D321" t="inlineStr">
+        <is>
+          <t>Stal Rzeszow</t>
+        </is>
+      </c>
+      <c r="E321" t="n">
+        <v>11.13</v>
+      </c>
+      <c r="F321" t="n">
+        <v>1.02</v>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" s="1" t="n">
+        <v>46242</v>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>Korona Kielce</t>
+        </is>
+      </c>
+      <c r="D322" t="inlineStr">
+        <is>
+          <t>Legia Warsaw</t>
+        </is>
+      </c>
+      <c r="E322" t="n">
+        <v>9.83</v>
+      </c>
+      <c r="F322" t="n">
+        <v>-0.32</v>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" s="1" t="n">
+        <v>46242</v>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>Pogon Szczecin</t>
+        </is>
+      </c>
+      <c r="D323" t="inlineStr">
+        <is>
+          <t>Motor Lublin</t>
+        </is>
+      </c>
+      <c r="E323" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="F323" t="n">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" s="1" t="n">
+        <v>46242</v>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>Radomiak Radom</t>
+        </is>
+      </c>
+      <c r="D324" t="inlineStr">
+        <is>
+          <t>Gornik Zabrze</t>
+        </is>
+      </c>
+      <c r="E324" t="n">
+        <v>10.59</v>
+      </c>
+      <c r="F324" t="n">
+        <v>-1.16</v>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" s="1" t="n">
+        <v>46242</v>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>Dinamo Bucuresti</t>
+        </is>
+      </c>
+      <c r="D325" t="inlineStr">
+        <is>
+          <t>Voluntari</t>
+        </is>
+      </c>
+      <c r="E325" t="n">
+        <v>9.34</v>
+      </c>
+      <c r="F325" t="n">
+        <v>2.95</v>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" s="1" t="n">
+        <v>46242</v>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>Farul Constanta</t>
+        </is>
+      </c>
+      <c r="D326" t="inlineStr">
+        <is>
+          <t>Csikszereda</t>
+        </is>
+      </c>
+      <c r="E326" t="n">
+        <v>9.65</v>
+      </c>
+      <c r="F326" t="n">
+        <v>3.17</v>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" s="1" t="n">
+        <v>46242</v>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>Falkenbergs</t>
+        </is>
+      </c>
+      <c r="D327" t="inlineStr">
+        <is>
+          <t>Nordic United</t>
+        </is>
+      </c>
+      <c r="E327" t="n">
+        <v>9.82</v>
+      </c>
+      <c r="F327" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" s="1" t="n">
+        <v>46242</v>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>Ljungskile</t>
+        </is>
+      </c>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>Oddevold</t>
+        </is>
+      </c>
+      <c r="E328" t="n">
+        <v>10.45</v>
+      </c>
+      <c r="F328" t="n">
+        <v>0.17</v>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" s="1" t="n">
+        <v>46242</v>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>Norrkoping</t>
+        </is>
+      </c>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>Brage</t>
+        </is>
+      </c>
+      <c r="E329" t="n">
+        <v>10.46</v>
+      </c>
+      <c r="F329" t="n">
+        <v>2.36</v>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" s="1" t="n">
+        <v>46242</v>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>Osters</t>
+        </is>
+      </c>
+      <c r="D330" t="inlineStr">
+        <is>
+          <t>Landskrona</t>
+        </is>
+      </c>
+      <c r="E330" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="F330" t="n">
+        <v>0.17</v>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" s="1" t="n">
+        <v>46243</v>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>Cuiaba</t>
+        </is>
+      </c>
+      <c r="D331" t="inlineStr">
+        <is>
+          <t>Fortaleza</t>
+        </is>
+      </c>
+      <c r="E331" t="n">
+        <v>10.11</v>
+      </c>
+      <c r="F331" t="n">
+        <v>0.67</v>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" s="1" t="n">
+        <v>46243</v>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>Gremio Novorizontino</t>
+        </is>
+      </c>
+      <c r="D332" t="inlineStr">
+        <is>
+          <t>Juventude</t>
+        </is>
+      </c>
+      <c r="E332" t="n">
+        <v>10.15</v>
+      </c>
+      <c r="F332" t="n">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" s="1" t="n">
+        <v>46243</v>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>Nautico</t>
+        </is>
+      </c>
+      <c r="D333" t="inlineStr">
+        <is>
+          <t>Atletico Goianiense</t>
+        </is>
+      </c>
+      <c r="E333" t="n">
+        <v>10.29</v>
+      </c>
+      <c r="F333" t="n">
+        <v>1.89</v>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" s="1" t="n">
+        <v>46243</v>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>AC Oulu</t>
+        </is>
+      </c>
+      <c r="D334" t="inlineStr">
+        <is>
+          <t>HJK Helsinki</t>
+        </is>
+      </c>
+      <c r="E334" t="n">
+        <v>10.45</v>
+      </c>
+      <c r="F334" t="n">
+        <v>-0.9399999999999999</v>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" s="1" t="n">
+        <v>46243</v>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>Ilves</t>
+        </is>
+      </c>
+      <c r="D335" t="inlineStr">
+        <is>
+          <t>IFK Mariehamn</t>
+        </is>
+      </c>
+      <c r="E335" t="n">
+        <v>11.16</v>
+      </c>
+      <c r="F335" t="n">
+        <v>3.48</v>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" s="1" t="n">
+        <v>46243</v>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>Inter Turku</t>
+        </is>
+      </c>
+      <c r="D336" t="inlineStr">
+        <is>
+          <t>FC Lahti</t>
+        </is>
+      </c>
+      <c r="E336" t="n">
+        <v>9.970000000000001</v>
+      </c>
+      <c r="F336" t="n">
+        <v>1.66</v>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" s="1" t="n">
+        <v>46243</v>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>KuPS</t>
+        </is>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>TPS</t>
+        </is>
+      </c>
+      <c r="E337" t="n">
+        <v>10.22</v>
+      </c>
+      <c r="F337" t="n">
+        <v>3.03</v>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" s="1" t="n">
+        <v>46243</v>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>Finland - Ykkosliiga</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>HJK Klubi 04</t>
+        </is>
+      </c>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t>KTP</t>
+        </is>
+      </c>
+      <c r="E338" t="n">
+        <v>10.55</v>
+      </c>
+      <c r="F338" t="n">
+        <v>-1.67</v>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" s="1" t="n">
+        <v>46243</v>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>Asane Fotball</t>
+        </is>
+      </c>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>Kongsvinger</t>
+        </is>
+      </c>
+      <c r="E339" t="n">
+        <v>11.24</v>
+      </c>
+      <c r="F339" t="n">
+        <v>-2.66</v>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" s="1" t="n">
+        <v>46243</v>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>Haugesund</t>
+        </is>
+      </c>
+      <c r="D340" t="inlineStr">
+        <is>
+          <t>Raufoss</t>
+        </is>
+      </c>
+      <c r="E340" t="n">
+        <v>11.38</v>
+      </c>
+      <c r="F340" t="n">
+        <v>3.75</v>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" s="1" t="n">
+        <v>46243</v>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>Sandnes Ulf</t>
+        </is>
+      </c>
+      <c r="D341" t="inlineStr">
+        <is>
+          <t>Hodd</t>
+        </is>
+      </c>
+      <c r="E341" t="n">
+        <v>10.61</v>
+      </c>
+      <c r="F341" t="n">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" s="1" t="n">
+        <v>46243</v>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>Sogndal</t>
+        </is>
+      </c>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t>Bryne</t>
+        </is>
+      </c>
+      <c r="E342" t="n">
+        <v>10.83</v>
+      </c>
+      <c r="F342" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" s="1" t="n">
+        <v>46243</v>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>Stromsgodset</t>
+        </is>
+      </c>
+      <c r="D343" t="inlineStr">
+        <is>
+          <t>Egersunds</t>
+        </is>
+      </c>
+      <c r="E343" t="n">
+        <v>11.29</v>
+      </c>
+      <c r="F343" t="n">
+        <v>2.09</v>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" s="1" t="n">
+        <v>46243</v>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>LKS Lodz</t>
+        </is>
+      </c>
+      <c r="D344" t="inlineStr">
+        <is>
+          <t>Chrobry Glogow</t>
+        </is>
+      </c>
+      <c r="E344" t="n">
+        <v>10.97</v>
+      </c>
+      <c r="F344" t="n">
+        <v>2.37</v>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" s="1" t="n">
+        <v>46243</v>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>Jagiellonia Bialystok</t>
+        </is>
+      </c>
+      <c r="D345" t="inlineStr">
+        <is>
+          <t>Widzew Lodz</t>
+        </is>
+      </c>
+      <c r="E345" t="n">
+        <v>9.69</v>
+      </c>
+      <c r="F345" t="n">
+        <v>1.34</v>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" s="1" t="n">
+        <v>46243</v>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>Lech Poznan</t>
+        </is>
+      </c>
+      <c r="D346" t="inlineStr">
+        <is>
+          <t>Piast Gliwice</t>
+        </is>
+      </c>
+      <c r="E346" t="n">
+        <v>10.67</v>
+      </c>
+      <c r="F346" t="n">
+        <v>2.47</v>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" s="1" t="n">
+        <v>46243</v>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>Petrolul Ploiesti</t>
+        </is>
+      </c>
+      <c r="D347" t="inlineStr">
+        <is>
+          <t>Otelul Galati</t>
+        </is>
+      </c>
+      <c r="E347" t="n">
+        <v>9.42</v>
+      </c>
+      <c r="F347" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" s="1" t="n">
+        <v>46243</v>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>Universitatea Craiova</t>
+        </is>
+      </c>
+      <c r="D348" t="inlineStr">
+        <is>
+          <t>Arges Pitesti</t>
+        </is>
+      </c>
+      <c r="E348" t="n">
+        <v>9.23</v>
+      </c>
+      <c r="F348" t="n">
+        <v>3.12</v>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" s="1" t="n">
+        <v>46243</v>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>Varbergs BoIS</t>
+        </is>
+      </c>
+      <c r="D349" t="inlineStr">
+        <is>
+          <t>Sandvikens IF</t>
+        </is>
+      </c>
+      <c r="E349" t="n">
+        <v>10.32</v>
+      </c>
+      <c r="F349" t="n">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" s="1" t="n">
         <v>46244</v>
       </c>
-      <c r="B315" t="inlineStr">
+      <c r="B350" t="inlineStr">
         <is>
           <t>Brazil - Serie B</t>
         </is>
       </c>
-      <c r="C315" t="inlineStr">
+      <c r="C350" t="inlineStr">
         <is>
           <t>Goias</t>
         </is>
       </c>
-      <c r="D315" t="inlineStr">
+      <c r="D350" t="inlineStr">
         <is>
           <t>Londrina</t>
         </is>
       </c>
-      <c r="E315" t="n">
+      <c r="E350" t="n">
         <v>10.87</v>
       </c>
-      <c r="F315" t="n">
+      <c r="F350" t="n">
         <v>2.16</v>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>CFR Cluj</t>
+        </is>
+      </c>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>Universitatea Cluj</t>
+        </is>
+      </c>
+      <c r="E351" t="n">
+        <v>9.68</v>
+      </c>
+      <c r="F351" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>Norrby</t>
+        </is>
+      </c>
+      <c r="D352" t="inlineStr">
+        <is>
+          <t>Orebro SK</t>
+        </is>
+      </c>
+      <c r="E352" t="n">
+        <v>10.46</v>
+      </c>
+      <c r="F352" t="n">
+        <v>0.62</v>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" s="1" t="n">
+        <v>46245</v>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>Avai</t>
+        </is>
+      </c>
+      <c r="D353" t="inlineStr">
+        <is>
+          <t>CRB</t>
+        </is>
+      </c>
+      <c r="E353" t="n">
+        <v>10.14</v>
+      </c>
+      <c r="F353" t="n">
+        <v>-0.02</v>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" s="1" t="n">
+        <v>46245</v>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>Helsingborgs</t>
+        </is>
+      </c>
+      <c r="D354" t="inlineStr">
+        <is>
+          <t>Varnamo</t>
+        </is>
+      </c>
+      <c r="E354" t="n">
+        <v>10.45</v>
+      </c>
+      <c r="F354" t="n">
+        <v>0.6899999999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily scrape output - 2026-08-09
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F354"/>
+  <dimension ref="A1:F359"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9017,19 +9017,19 @@
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>Cuiaba</t>
+          <t>Athletic Club</t>
         </is>
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>Fortaleza</t>
+          <t>Criciuma</t>
         </is>
       </c>
       <c r="E331" t="n">
-        <v>10.11</v>
+        <v>10.15</v>
       </c>
       <c r="F331" t="n">
-        <v>0.67</v>
+        <v>-0.14</v>
       </c>
     </row>
     <row r="332">
@@ -9043,19 +9043,19 @@
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>Gremio Novorizontino</t>
+          <t>Cuiaba</t>
         </is>
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>Juventude</t>
+          <t>Fortaleza</t>
         </is>
       </c>
       <c r="E332" t="n">
-        <v>10.15</v>
+        <v>10.11</v>
       </c>
       <c r="F332" t="n">
-        <v>1.2</v>
+        <v>0.67</v>
       </c>
     </row>
     <row r="333">
@@ -9069,19 +9069,19 @@
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>Nautico</t>
+          <t>Gremio Novorizontino</t>
         </is>
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>Atletico Goianiense</t>
+          <t>Juventude</t>
         </is>
       </c>
       <c r="E333" t="n">
-        <v>10.29</v>
+        <v>10.15</v>
       </c>
       <c r="F333" t="n">
-        <v>1.89</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="334">
@@ -9090,24 +9090,24 @@
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>Finland - Veikkausliiga</t>
+          <t>Brazil - Serie B</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>AC Oulu</t>
+          <t>Nautico</t>
         </is>
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>HJK Helsinki</t>
+          <t>Atletico Goianiense</t>
         </is>
       </c>
       <c r="E334" t="n">
-        <v>10.45</v>
+        <v>10.31</v>
       </c>
       <c r="F334" t="n">
-        <v>-0.9399999999999999</v>
+        <v>1.89</v>
       </c>
     </row>
     <row r="335">
@@ -9121,19 +9121,19 @@
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>Ilves</t>
+          <t>AC Oulu</t>
         </is>
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>IFK Mariehamn</t>
+          <t>HJK Helsinki</t>
         </is>
       </c>
       <c r="E335" t="n">
-        <v>11.16</v>
+        <v>10.43</v>
       </c>
       <c r="F335" t="n">
-        <v>3.48</v>
+        <v>-0.9399999999999999</v>
       </c>
     </row>
     <row r="336">
@@ -9147,19 +9147,19 @@
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>Inter Turku</t>
+          <t>Ilves</t>
         </is>
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>FC Lahti</t>
+          <t>IFK Mariehamn</t>
         </is>
       </c>
       <c r="E336" t="n">
-        <v>9.970000000000001</v>
+        <v>11.16</v>
       </c>
       <c r="F336" t="n">
-        <v>1.66</v>
+        <v>3.48</v>
       </c>
     </row>
     <row r="337">
@@ -9173,19 +9173,19 @@
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>KuPS</t>
+          <t>Inter Turku</t>
         </is>
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>TPS</t>
+          <t>FC Lahti</t>
         </is>
       </c>
       <c r="E337" t="n">
-        <v>10.22</v>
+        <v>9.82</v>
       </c>
       <c r="F337" t="n">
-        <v>3.03</v>
+        <v>1.66</v>
       </c>
     </row>
     <row r="338">
@@ -9194,24 +9194,24 @@
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>Finland - Ykkosliiga</t>
+          <t>Finland - Veikkausliiga</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>HJK Klubi 04</t>
+          <t>KuPS</t>
         </is>
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>KTP</t>
+          <t>TPS</t>
         </is>
       </c>
       <c r="E338" t="n">
-        <v>10.55</v>
+        <v>10.11</v>
       </c>
       <c r="F338" t="n">
-        <v>-1.67</v>
+        <v>2.99</v>
       </c>
     </row>
     <row r="339">
@@ -9220,24 +9220,24 @@
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>Norway - 1st Division</t>
+          <t>Finland - Ykkosliiga</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>Asane Fotball</t>
+          <t>HJK Klubi 04</t>
         </is>
       </c>
       <c r="D339" t="inlineStr">
         <is>
-          <t>Kongsvinger</t>
+          <t>KTP</t>
         </is>
       </c>
       <c r="E339" t="n">
-        <v>11.24</v>
+        <v>10.55</v>
       </c>
       <c r="F339" t="n">
-        <v>-2.66</v>
+        <v>-1.67</v>
       </c>
     </row>
     <row r="340">
@@ -9246,24 +9246,24 @@
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>Norway - 1st Division</t>
+          <t>Iceland - 1. Deild</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>Haugesund</t>
+          <t>Volsungur</t>
         </is>
       </c>
       <c r="D340" t="inlineStr">
         <is>
-          <t>Raufoss</t>
+          <t>HK Kopavogur</t>
         </is>
       </c>
       <c r="E340" t="n">
-        <v>11.38</v>
+        <v>11.58</v>
       </c>
       <c r="F340" t="n">
-        <v>3.75</v>
+        <v>-2.46</v>
       </c>
     </row>
     <row r="341">
@@ -9277,19 +9277,19 @@
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>Sandnes Ulf</t>
+          <t>Asane Fotball</t>
         </is>
       </c>
       <c r="D341" t="inlineStr">
         <is>
-          <t>Hodd</t>
+          <t>Kongsvinger</t>
         </is>
       </c>
       <c r="E341" t="n">
-        <v>10.61</v>
+        <v>11.16</v>
       </c>
       <c r="F341" t="n">
-        <v>1.4</v>
+        <v>-2.63</v>
       </c>
     </row>
     <row r="342">
@@ -9303,19 +9303,19 @@
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>Sogndal</t>
+          <t>Haugesund</t>
         </is>
       </c>
       <c r="D342" t="inlineStr">
         <is>
-          <t>Bryne</t>
+          <t>Raufoss</t>
         </is>
       </c>
       <c r="E342" t="n">
-        <v>10.83</v>
+        <v>11.38</v>
       </c>
       <c r="F342" t="n">
-        <v>0</v>
+        <v>3.75</v>
       </c>
     </row>
     <row r="343">
@@ -9329,19 +9329,19 @@
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>Stromsgodset</t>
+          <t>Sandnes Ulf</t>
         </is>
       </c>
       <c r="D343" t="inlineStr">
         <is>
-          <t>Egersunds</t>
+          <t>Hodd</t>
         </is>
       </c>
       <c r="E343" t="n">
-        <v>11.29</v>
+        <v>10.61</v>
       </c>
       <c r="F343" t="n">
-        <v>2.09</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="344">
@@ -9350,24 +9350,24 @@
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>Poland - 1st Liga</t>
+          <t>Norway - 1st Division</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>LKS Lodz</t>
+          <t>Sogndal</t>
         </is>
       </c>
       <c r="D344" t="inlineStr">
         <is>
-          <t>Chrobry Glogow</t>
+          <t>Bryne</t>
         </is>
       </c>
       <c r="E344" t="n">
-        <v>10.97</v>
+        <v>10.85</v>
       </c>
       <c r="F344" t="n">
-        <v>2.37</v>
+        <v>0</v>
       </c>
     </row>
     <row r="345">
@@ -9376,24 +9376,24 @@
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Norway - 1st Division</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>Jagiellonia Bialystok</t>
+          <t>Strommen</t>
         </is>
       </c>
       <c r="D345" t="inlineStr">
         <is>
-          <t>Widzew Lodz</t>
+          <t>Ranheim</t>
         </is>
       </c>
       <c r="E345" t="n">
-        <v>9.69</v>
+        <v>10.78</v>
       </c>
       <c r="F345" t="n">
-        <v>1.34</v>
+        <v>0</v>
       </c>
     </row>
     <row r="346">
@@ -9402,24 +9402,24 @@
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Norway - 1st Division</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>Lech Poznan</t>
+          <t>Stromsgodset</t>
         </is>
       </c>
       <c r="D346" t="inlineStr">
         <is>
-          <t>Piast Gliwice</t>
+          <t>Egersunds</t>
         </is>
       </c>
       <c r="E346" t="n">
-        <v>10.67</v>
+        <v>11.29</v>
       </c>
       <c r="F346" t="n">
-        <v>2.47</v>
+        <v>2.09</v>
       </c>
     </row>
     <row r="347">
@@ -9428,24 +9428,24 @@
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>Romania - Liga 1</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>Petrolul Ploiesti</t>
+          <t>LKS Lodz</t>
         </is>
       </c>
       <c r="D347" t="inlineStr">
         <is>
-          <t>Otelul Galati</t>
+          <t>Chrobry Glogow</t>
         </is>
       </c>
       <c r="E347" t="n">
-        <v>9.42</v>
+        <v>10.7</v>
       </c>
       <c r="F347" t="n">
-        <v>0.4</v>
+        <v>2.37</v>
       </c>
     </row>
     <row r="348">
@@ -9454,24 +9454,24 @@
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>Romania - Liga 1</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>Universitatea Craiova</t>
+          <t>Jagiellonia Bialystok</t>
         </is>
       </c>
       <c r="D348" t="inlineStr">
         <is>
-          <t>Arges Pitesti</t>
+          <t>Widzew Lodz</t>
         </is>
       </c>
       <c r="E348" t="n">
-        <v>9.23</v>
+        <v>9.69</v>
       </c>
       <c r="F348" t="n">
-        <v>3.12</v>
+        <v>1.34</v>
       </c>
     </row>
     <row r="349">
@@ -9480,55 +9480,55 @@
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>Varbergs BoIS</t>
+          <t>Lech Poznan</t>
         </is>
       </c>
       <c r="D349" t="inlineStr">
         <is>
-          <t>Sandvikens IF</t>
+          <t>Piast Gliwice</t>
         </is>
       </c>
       <c r="E349" t="n">
-        <v>10.32</v>
+        <v>10.67</v>
       </c>
       <c r="F349" t="n">
-        <v>1.2</v>
+        <v>2.47</v>
       </c>
     </row>
     <row r="350">
       <c r="A350" s="1" t="n">
-        <v>46244</v>
+        <v>46243</v>
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>Goias</t>
+          <t>Slask Wroclaw</t>
         </is>
       </c>
       <c r="D350" t="inlineStr">
         <is>
-          <t>Londrina</t>
+          <t>Cracovia Krakow</t>
         </is>
       </c>
       <c r="E350" t="n">
-        <v>10.87</v>
+        <v>10.63</v>
       </c>
       <c r="F350" t="n">
-        <v>2.16</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="351">
       <c r="A351" s="1" t="n">
-        <v>46244</v>
+        <v>46243</v>
       </c>
       <c r="B351" t="inlineStr">
         <is>
@@ -9537,96 +9537,226 @@
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>CFR Cluj</t>
+          <t>Petrolul Ploiesti</t>
         </is>
       </c>
       <c r="D351" t="inlineStr">
         <is>
-          <t>Universitatea Cluj</t>
+          <t>Otelul Galati</t>
         </is>
       </c>
       <c r="E351" t="n">
-        <v>9.68</v>
+        <v>9.41</v>
       </c>
       <c r="F351" t="n">
-        <v>2</v>
+        <v>0.51</v>
       </c>
     </row>
     <row r="352">
       <c r="A352" s="1" t="n">
-        <v>46244</v>
+        <v>46243</v>
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Romania - Liga 1</t>
         </is>
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>Norrby</t>
+          <t>Universitatea Craiova</t>
         </is>
       </c>
       <c r="D352" t="inlineStr">
         <is>
-          <t>Orebro SK</t>
+          <t>Arges Pitesti</t>
         </is>
       </c>
       <c r="E352" t="n">
-        <v>10.46</v>
+        <v>9.17</v>
       </c>
       <c r="F352" t="n">
-        <v>0.62</v>
+        <v>2.43</v>
       </c>
     </row>
     <row r="353">
       <c r="A353" s="1" t="n">
-        <v>46245</v>
+        <v>46243</v>
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Sweden - Superettan</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>Avai</t>
+          <t>Varbergs BoIS</t>
         </is>
       </c>
       <c r="D353" t="inlineStr">
         <is>
-          <t>CRB</t>
+          <t>Sandvikens IF</t>
         </is>
       </c>
       <c r="E353" t="n">
-        <v>10.14</v>
+        <v>10.35</v>
       </c>
       <c r="F353" t="n">
-        <v>-0.02</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="354">
       <c r="A354" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>Goias</t>
+        </is>
+      </c>
+      <c r="D354" t="inlineStr">
+        <is>
+          <t>Londrina</t>
+        </is>
+      </c>
+      <c r="E354" t="n">
+        <v>10.87</v>
+      </c>
+      <c r="F354" t="n">
+        <v>2.16</v>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>Moss</t>
+        </is>
+      </c>
+      <c r="D355" t="inlineStr">
+        <is>
+          <t>Odd BK</t>
+        </is>
+      </c>
+      <c r="E355" t="n">
+        <v>10.83</v>
+      </c>
+      <c r="F355" t="n">
+        <v>-0.92</v>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>CFR Cluj</t>
+        </is>
+      </c>
+      <c r="D356" t="inlineStr">
+        <is>
+          <t>Universitatea Cluj</t>
+        </is>
+      </c>
+      <c r="E356" t="n">
+        <v>9.68</v>
+      </c>
+      <c r="F356" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>Norrby</t>
+        </is>
+      </c>
+      <c r="D357" t="inlineStr">
+        <is>
+          <t>Orebro SK</t>
+        </is>
+      </c>
+      <c r="E357" t="n">
+        <v>10.46</v>
+      </c>
+      <c r="F357" t="n">
+        <v>0.62</v>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" s="1" t="n">
         <v>46245</v>
       </c>
-      <c r="B354" t="inlineStr">
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>Avai</t>
+        </is>
+      </c>
+      <c r="D358" t="inlineStr">
+        <is>
+          <t>CRB</t>
+        </is>
+      </c>
+      <c r="E358" t="n">
+        <v>10.14</v>
+      </c>
+      <c r="F358" t="n">
+        <v>-0.02</v>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" s="1" t="n">
+        <v>46245</v>
+      </c>
+      <c r="B359" t="inlineStr">
         <is>
           <t>Sweden - Superettan</t>
         </is>
       </c>
-      <c r="C354" t="inlineStr">
+      <c r="C359" t="inlineStr">
         <is>
           <t>Helsingborgs</t>
         </is>
       </c>
-      <c r="D354" t="inlineStr">
+      <c r="D359" t="inlineStr">
         <is>
           <t>Varnamo</t>
         </is>
       </c>
-      <c r="E354" t="n">
+      <c r="E359" t="n">
         <v>10.45</v>
       </c>
-      <c r="F354" t="n">
+      <c r="F359" t="n">
         <v>0.6899999999999999</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily scrape output - 2026-08-10
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F359"/>
+  <dimension ref="A1:F362"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9650,10 +9650,10 @@
         </is>
       </c>
       <c r="E355" t="n">
-        <v>10.83</v>
+        <v>10.8</v>
       </c>
       <c r="F355" t="n">
-        <v>-0.92</v>
+        <v>-0.93</v>
       </c>
     </row>
     <row r="356">
@@ -9662,24 +9662,24 @@
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>Romania - Liga 1</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="C356" t="inlineStr">
         <is>
-          <t>CFR Cluj</t>
+          <t>Unia Skierniewice</t>
         </is>
       </c>
       <c r="D356" t="inlineStr">
         <is>
-          <t>Universitatea Cluj</t>
+          <t>Arka Gdynia</t>
         </is>
       </c>
       <c r="E356" t="n">
-        <v>9.68</v>
+        <v>10.58</v>
       </c>
       <c r="F356" t="n">
-        <v>2</v>
+        <v>-0.5600000000000001</v>
       </c>
     </row>
     <row r="357">
@@ -9688,75 +9688,153 @@
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Romania - Liga 1</t>
         </is>
       </c>
       <c r="C357" t="inlineStr">
         <is>
-          <t>Norrby</t>
+          <t>Botosani</t>
         </is>
       </c>
       <c r="D357" t="inlineStr">
         <is>
-          <t>Orebro SK</t>
+          <t>Corvinul Hunedoara</t>
         </is>
       </c>
       <c r="E357" t="n">
-        <v>10.46</v>
+        <v>9.27</v>
       </c>
       <c r="F357" t="n">
-        <v>0.62</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="358">
       <c r="A358" s="1" t="n">
-        <v>46245</v>
+        <v>46244</v>
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Romania - Liga 1</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
         <is>
-          <t>Avai</t>
+          <t>CFR Cluj</t>
         </is>
       </c>
       <c r="D358" t="inlineStr">
         <is>
-          <t>CRB</t>
+          <t>Universitatea Cluj</t>
         </is>
       </c>
       <c r="E358" t="n">
-        <v>10.14</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="F358" t="n">
-        <v>-0.02</v>
+        <v>2</v>
       </c>
     </row>
     <row r="359">
       <c r="A359" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>Sepsi</t>
+        </is>
+      </c>
+      <c r="D359" t="inlineStr">
+        <is>
+          <t>FCSB</t>
+        </is>
+      </c>
+      <c r="E359" t="n">
+        <v>8.99</v>
+      </c>
+      <c r="F359" t="n">
+        <v>-1.4</v>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>Norrby</t>
+        </is>
+      </c>
+      <c r="D360" t="inlineStr">
+        <is>
+          <t>Orebro SK</t>
+        </is>
+      </c>
+      <c r="E360" t="n">
+        <v>10.61</v>
+      </c>
+      <c r="F360" t="n">
+        <v>0.51</v>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" s="1" t="n">
         <v>46245</v>
       </c>
-      <c r="B359" t="inlineStr">
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>Avai</t>
+        </is>
+      </c>
+      <c r="D361" t="inlineStr">
+        <is>
+          <t>CRB</t>
+        </is>
+      </c>
+      <c r="E361" t="n">
+        <v>9.970000000000001</v>
+      </c>
+      <c r="F361" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" s="1" t="n">
+        <v>46245</v>
+      </c>
+      <c r="B362" t="inlineStr">
         <is>
           <t>Sweden - Superettan</t>
         </is>
       </c>
-      <c r="C359" t="inlineStr">
+      <c r="C362" t="inlineStr">
         <is>
           <t>Helsingborgs</t>
         </is>
       </c>
-      <c r="D359" t="inlineStr">
+      <c r="D362" t="inlineStr">
         <is>
           <t>Varnamo</t>
         </is>
       </c>
-      <c r="E359" t="n">
+      <c r="E362" t="n">
         <v>10.45</v>
       </c>
-      <c r="F359" t="n">
+      <c r="F362" t="n">
         <v>0.6899999999999999</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily scrape output - 2026-08-11
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -9806,10 +9806,10 @@
         </is>
       </c>
       <c r="E361" t="n">
-        <v>9.970000000000001</v>
+        <v>9.890000000000001</v>
       </c>
       <c r="F361" t="n">
-        <v>0</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="362">
@@ -9832,10 +9832,10 @@
         </is>
       </c>
       <c r="E362" t="n">
-        <v>10.45</v>
+        <v>10.39</v>
       </c>
       <c r="F362" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily scrape output - 2026-08-13
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F362"/>
+  <dimension ref="A1:F367"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9838,6 +9838,136 @@
         <v>0.82</v>
       </c>
     </row>
+    <row r="363">
+      <c r="A363" s="1" t="n">
+        <v>46247</v>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>Iceland - 1. Deild</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>Aegir</t>
+        </is>
+      </c>
+      <c r="D363" t="inlineStr">
+        <is>
+          <t>Volsungur</t>
+        </is>
+      </c>
+      <c r="E363" t="n">
+        <v>11.28</v>
+      </c>
+      <c r="F363" t="n">
+        <v>-0.42</v>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" s="1" t="n">
+        <v>46247</v>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>Iceland - 1. Deild</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>Fylkir</t>
+        </is>
+      </c>
+      <c r="D364" t="inlineStr">
+        <is>
+          <t>Afturelding</t>
+        </is>
+      </c>
+      <c r="E364" t="n">
+        <v>11.18</v>
+      </c>
+      <c r="F364" t="n">
+        <v>1.37</v>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" s="1" t="n">
+        <v>46247</v>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>Iceland - 1. Deild</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>HK Kopavogur</t>
+        </is>
+      </c>
+      <c r="D365" t="inlineStr">
+        <is>
+          <t>Leiknir Reykjavik</t>
+        </is>
+      </c>
+      <c r="E365" t="n">
+        <v>11.86</v>
+      </c>
+      <c r="F365" t="n">
+        <v>1.85</v>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" s="1" t="n">
+        <v>46247</v>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>Iceland - 1. Deild</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>UMF Grindavik</t>
+        </is>
+      </c>
+      <c r="D366" t="inlineStr">
+        <is>
+          <t>Throttur Reykjavik</t>
+        </is>
+      </c>
+      <c r="E366" t="n">
+        <v>11.38</v>
+      </c>
+      <c r="F366" t="n">
+        <v>-2.71</v>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" s="1" t="n">
+        <v>46247</v>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>Iceland - 1. Deild</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>Vestri</t>
+        </is>
+      </c>
+      <c r="D367" t="inlineStr">
+        <is>
+          <t>IR Reykjavik</t>
+        </is>
+      </c>
+      <c r="E367" t="n">
+        <v>11.57</v>
+      </c>
+      <c r="F367" t="n">
+        <v>0.04</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily scrape output - 2026-08-14
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F367"/>
+  <dimension ref="A1:F407"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9968,6 +9968,1046 @@
         <v>0.04</v>
       </c>
     </row>
+    <row r="368">
+      <c r="A368" s="1" t="n">
+        <v>46248</v>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>Ponte Preta</t>
+        </is>
+      </c>
+      <c r="D368" t="inlineStr">
+        <is>
+          <t>Nautico</t>
+        </is>
+      </c>
+      <c r="E368" t="n">
+        <v>10.36</v>
+      </c>
+      <c r="F368" t="n">
+        <v>-1.09</v>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" s="1" t="n">
+        <v>46248</v>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>Sao Bernardo</t>
+        </is>
+      </c>
+      <c r="D369" t="inlineStr">
+        <is>
+          <t>Botafogo SP</t>
+        </is>
+      </c>
+      <c r="E369" t="n">
+        <v>10.69</v>
+      </c>
+      <c r="F369" t="n">
+        <v>0.67</v>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" s="1" t="n">
+        <v>46248</v>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>Sport Recife</t>
+        </is>
+      </c>
+      <c r="D370" t="inlineStr">
+        <is>
+          <t>Londrina</t>
+        </is>
+      </c>
+      <c r="E370" t="n">
+        <v>10.96</v>
+      </c>
+      <c r="F370" t="n">
+        <v>2.41</v>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" s="1" t="n">
+        <v>46248</v>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>VPS</t>
+        </is>
+      </c>
+      <c r="D371" t="inlineStr">
+        <is>
+          <t>TPS</t>
+        </is>
+      </c>
+      <c r="E371" t="n">
+        <v>9.779999999999999</v>
+      </c>
+      <c r="F371" t="n">
+        <v>2.05</v>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" s="1" t="n">
+        <v>46248</v>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>Finland - Ykkosliiga</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>JaPS</t>
+        </is>
+      </c>
+      <c r="D372" t="inlineStr">
+        <is>
+          <t>FC Haka</t>
+        </is>
+      </c>
+      <c r="E372" t="n">
+        <v>10.38</v>
+      </c>
+      <c r="F372" t="n">
+        <v>-1.61</v>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" s="1" t="n">
+        <v>46248</v>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>Pogon Grodzisk Mazowiecki</t>
+        </is>
+      </c>
+      <c r="D373" t="inlineStr">
+        <is>
+          <t>Stal Rzeszow</t>
+        </is>
+      </c>
+      <c r="E373" t="n">
+        <v>11.67</v>
+      </c>
+      <c r="F373" t="n">
+        <v>0.66</v>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" s="1" t="n">
+        <v>46248</v>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>Ruch Chorzow</t>
+        </is>
+      </c>
+      <c r="D374" t="inlineStr">
+        <is>
+          <t>Lechia Gdansk</t>
+        </is>
+      </c>
+      <c r="E374" t="n">
+        <v>10.61</v>
+      </c>
+      <c r="F374" t="n">
+        <v>1.02</v>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" s="1" t="n">
+        <v>46248</v>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>Legia Warsaw</t>
+        </is>
+      </c>
+      <c r="D375" t="inlineStr">
+        <is>
+          <t>Radomiak Radom</t>
+        </is>
+      </c>
+      <c r="E375" t="n">
+        <v>10.05</v>
+      </c>
+      <c r="F375" t="n">
+        <v>2.49</v>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" s="1" t="n">
+        <v>46248</v>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>Arges Pitesti</t>
+        </is>
+      </c>
+      <c r="D376" t="inlineStr">
+        <is>
+          <t>Farul Constanta</t>
+        </is>
+      </c>
+      <c r="E376" t="n">
+        <v>9.539999999999999</v>
+      </c>
+      <c r="F376" t="n">
+        <v>0.65</v>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" s="1" t="n">
+        <v>46248</v>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>Voluntari</t>
+        </is>
+      </c>
+      <c r="D377" t="inlineStr">
+        <is>
+          <t>Petrolul Ploiesti</t>
+        </is>
+      </c>
+      <c r="E377" t="n">
+        <v>9.07</v>
+      </c>
+      <c r="F377" t="n">
+        <v>0.51</v>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" s="1" t="n">
+        <v>46248</v>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>Real Sociedad II</t>
+        </is>
+      </c>
+      <c r="D378" t="inlineStr">
+        <is>
+          <t>Castellon</t>
+        </is>
+      </c>
+      <c r="E378" t="n">
+        <v>9.48</v>
+      </c>
+      <c r="F378" t="n">
+        <v>-1.49</v>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" s="1" t="n">
+        <v>46248</v>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>Brage</t>
+        </is>
+      </c>
+      <c r="D379" t="inlineStr">
+        <is>
+          <t>Orebro SK</t>
+        </is>
+      </c>
+      <c r="E379" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="F379" t="n">
+        <v>0.89</v>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" s="1" t="n">
+        <v>46248</v>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>Landskrona</t>
+        </is>
+      </c>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t>Oddevold</t>
+        </is>
+      </c>
+      <c r="E380" t="n">
+        <v>10.11</v>
+      </c>
+      <c r="F380" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" s="1" t="n">
+        <v>46249</v>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>Atletico Goianiense</t>
+        </is>
+      </c>
+      <c r="D381" t="inlineStr">
+        <is>
+          <t>Vila Nova</t>
+        </is>
+      </c>
+      <c r="E381" t="n">
+        <v>10.23</v>
+      </c>
+      <c r="F381" t="n">
+        <v>1.03</v>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" s="1" t="n">
+        <v>46249</v>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>Ceara</t>
+        </is>
+      </c>
+      <c r="D382" t="inlineStr">
+        <is>
+          <t>Cuiaba</t>
+        </is>
+      </c>
+      <c r="E382" t="n">
+        <v>10.27</v>
+      </c>
+      <c r="F382" t="n">
+        <v>1.34</v>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" s="1" t="n">
+        <v>46249</v>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>Criciuma</t>
+        </is>
+      </c>
+      <c r="D383" t="inlineStr">
+        <is>
+          <t>Goias</t>
+        </is>
+      </c>
+      <c r="E383" t="n">
+        <v>10.53</v>
+      </c>
+      <c r="F383" t="n">
+        <v>2.11</v>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" s="1" t="n">
+        <v>46249</v>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>Juventude</t>
+        </is>
+      </c>
+      <c r="D384" t="inlineStr">
+        <is>
+          <t>Fortaleza</t>
+        </is>
+      </c>
+      <c r="E384" t="n">
+        <v>10.24</v>
+      </c>
+      <c r="F384" t="n">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" s="1" t="n">
+        <v>46249</v>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>IFK Mariehamn</t>
+        </is>
+      </c>
+      <c r="D385" t="inlineStr">
+        <is>
+          <t>SJK</t>
+        </is>
+      </c>
+      <c r="E385" t="n">
+        <v>10.72</v>
+      </c>
+      <c r="F385" t="n">
+        <v>-2.05</v>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" s="1" t="n">
+        <v>46249</v>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>Finland - Ykkosliiga</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>JIPPO</t>
+        </is>
+      </c>
+      <c r="D386" t="inlineStr">
+        <is>
+          <t>SJK Akatemia</t>
+        </is>
+      </c>
+      <c r="E386" t="n">
+        <v>10.18</v>
+      </c>
+      <c r="F386" t="n">
+        <v>2.98</v>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" s="1" t="n">
+        <v>46249</v>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>Finland - Ykkosliiga</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>KTP</t>
+        </is>
+      </c>
+      <c r="D387" t="inlineStr">
+        <is>
+          <t>KaPa</t>
+        </is>
+      </c>
+      <c r="E387" t="n">
+        <v>10.82</v>
+      </c>
+      <c r="F387" t="n">
+        <v>2.99</v>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" s="1" t="n">
+        <v>46249</v>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>Bryne</t>
+        </is>
+      </c>
+      <c r="D388" t="inlineStr">
+        <is>
+          <t>Moss</t>
+        </is>
+      </c>
+      <c r="E388" t="n">
+        <v>11.16</v>
+      </c>
+      <c r="F388" t="n">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" s="1" t="n">
+        <v>46249</v>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>Lyn</t>
+        </is>
+      </c>
+      <c r="D389" t="inlineStr">
+        <is>
+          <t>Odd BK</t>
+        </is>
+      </c>
+      <c r="E389" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="F389" t="n">
+        <v>-0.68</v>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" s="1" t="n">
+        <v>46249</v>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>Pogon Siedlce</t>
+        </is>
+      </c>
+      <c r="D390" t="inlineStr">
+        <is>
+          <t>Polonia Warsaw</t>
+        </is>
+      </c>
+      <c r="E390" t="n">
+        <v>10.74</v>
+      </c>
+      <c r="F390" t="n">
+        <v>-2.23</v>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" s="1" t="n">
+        <v>46249</v>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>Widzew Lodz</t>
+        </is>
+      </c>
+      <c r="D391" t="inlineStr">
+        <is>
+          <t>Korona Kielce</t>
+        </is>
+      </c>
+      <c r="E391" t="n">
+        <v>9.58</v>
+      </c>
+      <c r="F391" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" s="1" t="n">
+        <v>46249</v>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>Rapid Bucuresti</t>
+        </is>
+      </c>
+      <c r="D392" t="inlineStr">
+        <is>
+          <t>Dinamo Bucuresti</t>
+        </is>
+      </c>
+      <c r="E392" t="n">
+        <v>9.720000000000001</v>
+      </c>
+      <c r="F392" t="n">
+        <v>0.32</v>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" s="1" t="n">
+        <v>46249</v>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>Falkenbergs</t>
+        </is>
+      </c>
+      <c r="D393" t="inlineStr">
+        <is>
+          <t>Norrby</t>
+        </is>
+      </c>
+      <c r="E393" t="n">
+        <v>10.16</v>
+      </c>
+      <c r="F393" t="n">
+        <v>1.33</v>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" s="1" t="n">
+        <v>46249</v>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>Sandvikens IF</t>
+        </is>
+      </c>
+      <c r="D394" t="inlineStr">
+        <is>
+          <t>Norrkoping</t>
+        </is>
+      </c>
+      <c r="E394" t="n">
+        <v>10.55</v>
+      </c>
+      <c r="F394" t="n">
+        <v>-1.06</v>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>America Mineiro</t>
+        </is>
+      </c>
+      <c r="D395" t="inlineStr">
+        <is>
+          <t>Athletic Club</t>
+        </is>
+      </c>
+      <c r="E395" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="F395" t="n">
+        <v>1.19</v>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>CRB</t>
+        </is>
+      </c>
+      <c r="D396" t="inlineStr">
+        <is>
+          <t>Gremio Novorizontino</t>
+        </is>
+      </c>
+      <c r="E396" t="n">
+        <v>10.51</v>
+      </c>
+      <c r="F396" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>Operario Ferroviario</t>
+        </is>
+      </c>
+      <c r="D397" t="inlineStr">
+        <is>
+          <t>Avai</t>
+        </is>
+      </c>
+      <c r="E397" t="n">
+        <v>10.29</v>
+      </c>
+      <c r="F397" t="n">
+        <v>2.02</v>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>AC Oulu</t>
+        </is>
+      </c>
+      <c r="D398" t="inlineStr">
+        <is>
+          <t>Inter Turku</t>
+        </is>
+      </c>
+      <c r="E398" t="n">
+        <v>10.05</v>
+      </c>
+      <c r="F398" t="n">
+        <v>-0.49</v>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>FC Lahti</t>
+        </is>
+      </c>
+      <c r="D399" t="inlineStr">
+        <is>
+          <t>KuPS</t>
+        </is>
+      </c>
+      <c r="E399" t="n">
+        <v>10.07</v>
+      </c>
+      <c r="F399" t="n">
+        <v>-0.91</v>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>Finland - Ykkosliiga</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>Mikkelin Palloilijat</t>
+        </is>
+      </c>
+      <c r="D400" t="inlineStr">
+        <is>
+          <t>EIF</t>
+        </is>
+      </c>
+      <c r="E400" t="n">
+        <v>10.34</v>
+      </c>
+      <c r="F400" t="n">
+        <v>-0.49</v>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>Egersunds</t>
+        </is>
+      </c>
+      <c r="D401" t="inlineStr">
+        <is>
+          <t>Stabaek</t>
+        </is>
+      </c>
+      <c r="E401" t="n">
+        <v>11.09</v>
+      </c>
+      <c r="F401" t="n">
+        <v>-0.49</v>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>Hodd</t>
+        </is>
+      </c>
+      <c r="D402" t="inlineStr">
+        <is>
+          <t>Strommen</t>
+        </is>
+      </c>
+      <c r="E402" t="n">
+        <v>10.51</v>
+      </c>
+      <c r="F402" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>Raufoss</t>
+        </is>
+      </c>
+      <c r="D403" t="inlineStr">
+        <is>
+          <t>Asane Fotball</t>
+        </is>
+      </c>
+      <c r="E403" t="n">
+        <v>11.29</v>
+      </c>
+      <c r="F403" t="n">
+        <v>1.33</v>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>Stal Mielec</t>
+        </is>
+      </c>
+      <c r="D404" t="inlineStr">
+        <is>
+          <t>Polonia Bytom</t>
+        </is>
+      </c>
+      <c r="E404" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="F404" t="n">
+        <v>0.39</v>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>Burgos</t>
+        </is>
+      </c>
+      <c r="D405" t="inlineStr">
+        <is>
+          <t>Cordoba</t>
+        </is>
+      </c>
+      <c r="E405" t="n">
+        <v>9.359999999999999</v>
+      </c>
+      <c r="F405" t="n">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" s="1" t="n">
+        <v>46251</v>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>Gnistan</t>
+        </is>
+      </c>
+      <c r="D406" t="inlineStr">
+        <is>
+          <t>Ilves</t>
+        </is>
+      </c>
+      <c r="E406" t="n">
+        <v>10.59</v>
+      </c>
+      <c r="F406" t="n">
+        <v>0.47</v>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" s="1" t="n">
+        <v>46251</v>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>FCSB</t>
+        </is>
+      </c>
+      <c r="D407" t="inlineStr">
+        <is>
+          <t>Botosani</t>
+        </is>
+      </c>
+      <c r="E407" t="n">
+        <v>9.789999999999999</v>
+      </c>
+      <c r="F407" t="n">
+        <v>2.48</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily scrape output - 2026-08-15
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F407"/>
+  <dimension ref="A1:F427"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10430,10 +10430,10 @@
         </is>
       </c>
       <c r="E385" t="n">
-        <v>10.72</v>
+        <v>10.85</v>
       </c>
       <c r="F385" t="n">
-        <v>-2.05</v>
+        <v>-1.98</v>
       </c>
     </row>
     <row r="386">
@@ -10494,24 +10494,24 @@
       </c>
       <c r="B388" t="inlineStr">
         <is>
-          <t>Norway - 1st Division</t>
+          <t>Finland - Ykkosliiga</t>
         </is>
       </c>
       <c r="C388" t="inlineStr">
         <is>
-          <t>Bryne</t>
+          <t>PK-35</t>
         </is>
       </c>
       <c r="D388" t="inlineStr">
         <is>
-          <t>Moss</t>
+          <t>HJK Klubi 04</t>
         </is>
       </c>
       <c r="E388" t="n">
-        <v>11.16</v>
+        <v>10.48</v>
       </c>
       <c r="F388" t="n">
-        <v>1.9</v>
+        <v>2.02</v>
       </c>
     </row>
     <row r="389">
@@ -10525,19 +10525,19 @@
       </c>
       <c r="C389" t="inlineStr">
         <is>
-          <t>Lyn</t>
+          <t>Bryne</t>
         </is>
       </c>
       <c r="D389" t="inlineStr">
         <is>
-          <t>Odd BK</t>
+          <t>Moss</t>
         </is>
       </c>
       <c r="E389" t="n">
-        <v>10.7</v>
+        <v>11.16</v>
       </c>
       <c r="F389" t="n">
-        <v>-0.68</v>
+        <v>1.86</v>
       </c>
     </row>
     <row r="390">
@@ -10546,24 +10546,24 @@
       </c>
       <c r="B390" t="inlineStr">
         <is>
-          <t>Poland - 1st Liga</t>
+          <t>Norway - 1st Division</t>
         </is>
       </c>
       <c r="C390" t="inlineStr">
         <is>
-          <t>Pogon Siedlce</t>
+          <t>Lyn</t>
         </is>
       </c>
       <c r="D390" t="inlineStr">
         <is>
-          <t>Polonia Warsaw</t>
+          <t>Odd BK</t>
         </is>
       </c>
       <c r="E390" t="n">
-        <v>10.74</v>
+        <v>10.98</v>
       </c>
       <c r="F390" t="n">
-        <v>-2.23</v>
+        <v>-0.83</v>
       </c>
     </row>
     <row r="391">
@@ -10572,24 +10572,24 @@
       </c>
       <c r="B391" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Norway - 1st Division</t>
         </is>
       </c>
       <c r="C391" t="inlineStr">
         <is>
-          <t>Widzew Lodz</t>
+          <t>Ranheim</t>
         </is>
       </c>
       <c r="D391" t="inlineStr">
         <is>
-          <t>Korona Kielce</t>
+          <t>Stromsgodset</t>
         </is>
       </c>
       <c r="E391" t="n">
-        <v>9.58</v>
+        <v>11.66</v>
       </c>
       <c r="F391" t="n">
-        <v>0.3</v>
+        <v>-1.91</v>
       </c>
     </row>
     <row r="392">
@@ -10598,24 +10598,24 @@
       </c>
       <c r="B392" t="inlineStr">
         <is>
-          <t>Romania - Liga 1</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="C392" t="inlineStr">
         <is>
-          <t>Rapid Bucuresti</t>
+          <t>Chrobry Glogow</t>
         </is>
       </c>
       <c r="D392" t="inlineStr">
         <is>
-          <t>Dinamo Bucuresti</t>
+          <t>Podbeskidzie Bielsko-Biala</t>
         </is>
       </c>
       <c r="E392" t="n">
-        <v>9.720000000000001</v>
+        <v>10.78</v>
       </c>
       <c r="F392" t="n">
-        <v>0.32</v>
+        <v>-0.43</v>
       </c>
     </row>
     <row r="393">
@@ -10624,24 +10624,24 @@
       </c>
       <c r="B393" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="C393" t="inlineStr">
         <is>
-          <t>Falkenbergs</t>
+          <t>Odra Opole</t>
         </is>
       </c>
       <c r="D393" t="inlineStr">
         <is>
-          <t>Norrby</t>
+          <t>Warta Poznan</t>
         </is>
       </c>
       <c r="E393" t="n">
-        <v>10.16</v>
+        <v>10.33</v>
       </c>
       <c r="F393" t="n">
-        <v>1.33</v>
+        <v>0.14</v>
       </c>
     </row>
     <row r="394">
@@ -10650,255 +10650,255 @@
       </c>
       <c r="B394" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="C394" t="inlineStr">
         <is>
-          <t>Sandvikens IF</t>
+          <t>Pogon Siedlce</t>
         </is>
       </c>
       <c r="D394" t="inlineStr">
         <is>
-          <t>Norrkoping</t>
+          <t>Polonia Warsaw</t>
         </is>
       </c>
       <c r="E394" t="n">
-        <v>10.55</v>
+        <v>10.84</v>
       </c>
       <c r="F394" t="n">
-        <v>-1.06</v>
+        <v>-2.33</v>
       </c>
     </row>
     <row r="395">
       <c r="A395" s="1" t="n">
-        <v>46250</v>
+        <v>46249</v>
       </c>
       <c r="B395" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C395" t="inlineStr">
         <is>
-          <t>America Mineiro</t>
+          <t>Widzew Lodz</t>
         </is>
       </c>
       <c r="D395" t="inlineStr">
         <is>
-          <t>Athletic Club</t>
+          <t>Korona Kielce</t>
         </is>
       </c>
       <c r="E395" t="n">
-        <v>10.3</v>
+        <v>9.369999999999999</v>
       </c>
       <c r="F395" t="n">
-        <v>1.19</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="396">
       <c r="A396" s="1" t="n">
-        <v>46250</v>
+        <v>46249</v>
       </c>
       <c r="B396" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C396" t="inlineStr">
         <is>
-          <t>CRB</t>
+          <t>Zaglebie Lubin</t>
         </is>
       </c>
       <c r="D396" t="inlineStr">
         <is>
-          <t>Gremio Novorizontino</t>
+          <t>Slask Wroclaw</t>
         </is>
       </c>
       <c r="E396" t="n">
-        <v>10.51</v>
+        <v>10.67</v>
       </c>
       <c r="F396" t="n">
-        <v>1</v>
+        <v>0.61</v>
       </c>
     </row>
     <row r="397">
       <c r="A397" s="1" t="n">
-        <v>46250</v>
+        <v>46249</v>
       </c>
       <c r="B397" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Romania - Liga 1</t>
         </is>
       </c>
       <c r="C397" t="inlineStr">
         <is>
-          <t>Operario Ferroviario</t>
+          <t>Csikszereda</t>
         </is>
       </c>
       <c r="D397" t="inlineStr">
         <is>
-          <t>Avai</t>
+          <t>Sepsi</t>
         </is>
       </c>
       <c r="E397" t="n">
-        <v>10.29</v>
+        <v>8.960000000000001</v>
       </c>
       <c r="F397" t="n">
-        <v>2.02</v>
+        <v>-0.17</v>
       </c>
     </row>
     <row r="398">
       <c r="A398" s="1" t="n">
-        <v>46250</v>
+        <v>46249</v>
       </c>
       <c r="B398" t="inlineStr">
         <is>
-          <t>Finland - Veikkausliiga</t>
+          <t>Romania - Liga 1</t>
         </is>
       </c>
       <c r="C398" t="inlineStr">
         <is>
-          <t>AC Oulu</t>
+          <t>Rapid Bucuresti</t>
         </is>
       </c>
       <c r="D398" t="inlineStr">
         <is>
-          <t>Inter Turku</t>
+          <t>Dinamo Bucuresti</t>
         </is>
       </c>
       <c r="E398" t="n">
-        <v>10.05</v>
+        <v>9.720000000000001</v>
       </c>
       <c r="F398" t="n">
-        <v>-0.49</v>
+        <v>0.32</v>
       </c>
     </row>
     <row r="399">
       <c r="A399" s="1" t="n">
-        <v>46250</v>
+        <v>46249</v>
       </c>
       <c r="B399" t="inlineStr">
         <is>
-          <t>Finland - Veikkausliiga</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="C399" t="inlineStr">
         <is>
-          <t>FC Lahti</t>
+          <t>Cadiz</t>
         </is>
       </c>
       <c r="D399" t="inlineStr">
         <is>
-          <t>KuPS</t>
+          <t>Celta Vigo II</t>
         </is>
       </c>
       <c r="E399" t="n">
-        <v>10.07</v>
+        <v>9.24</v>
       </c>
       <c r="F399" t="n">
-        <v>-0.91</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="400">
       <c r="A400" s="1" t="n">
-        <v>46250</v>
+        <v>46249</v>
       </c>
       <c r="B400" t="inlineStr">
         <is>
-          <t>Finland - Ykkosliiga</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="C400" t="inlineStr">
         <is>
-          <t>Mikkelin Palloilijat</t>
+          <t>FC Andorra</t>
         </is>
       </c>
       <c r="D400" t="inlineStr">
         <is>
-          <t>EIF</t>
+          <t>Ceuta</t>
         </is>
       </c>
       <c r="E400" t="n">
-        <v>10.34</v>
+        <v>9.460000000000001</v>
       </c>
       <c r="F400" t="n">
-        <v>-0.49</v>
+        <v>2.37</v>
       </c>
     </row>
     <row r="401">
       <c r="A401" s="1" t="n">
-        <v>46250</v>
+        <v>46249</v>
       </c>
       <c r="B401" t="inlineStr">
         <is>
-          <t>Norway - 1st Division</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="C401" t="inlineStr">
         <is>
-          <t>Egersunds</t>
+          <t>Mallorca</t>
         </is>
       </c>
       <c r="D401" t="inlineStr">
         <is>
-          <t>Stabaek</t>
+          <t>Real Valladolid</t>
         </is>
       </c>
       <c r="E401" t="n">
-        <v>11.09</v>
+        <v>9.35</v>
       </c>
       <c r="F401" t="n">
-        <v>-0.49</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="402">
       <c r="A402" s="1" t="n">
-        <v>46250</v>
+        <v>46249</v>
       </c>
       <c r="B402" t="inlineStr">
         <is>
-          <t>Norway - 1st Division</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="C402" t="inlineStr">
         <is>
-          <t>Hodd</t>
+          <t>Real Oviedo</t>
         </is>
       </c>
       <c r="D402" t="inlineStr">
         <is>
-          <t>Strommen</t>
+          <t>Granada</t>
         </is>
       </c>
       <c r="E402" t="n">
-        <v>10.51</v>
+        <v>9.609999999999999</v>
       </c>
       <c r="F402" t="n">
-        <v>0.5600000000000001</v>
+        <v>1.57</v>
       </c>
     </row>
     <row r="403">
       <c r="A403" s="1" t="n">
-        <v>46250</v>
+        <v>46249</v>
       </c>
       <c r="B403" t="inlineStr">
         <is>
-          <t>Norway - 1st Division</t>
+          <t>Sweden - Superettan</t>
         </is>
       </c>
       <c r="C403" t="inlineStr">
         <is>
-          <t>Raufoss</t>
+          <t>Falkenbergs</t>
         </is>
       </c>
       <c r="D403" t="inlineStr">
         <is>
-          <t>Asane Fotball</t>
+          <t>Norrby</t>
         </is>
       </c>
       <c r="E403" t="n">
-        <v>11.29</v>
+        <v>10.16</v>
       </c>
       <c r="F403" t="n">
         <v>1.33</v>
@@ -10906,106 +10906,626 @@
     </row>
     <row r="404">
       <c r="A404" s="1" t="n">
-        <v>46250</v>
+        <v>46249</v>
       </c>
       <c r="B404" t="inlineStr">
         <is>
-          <t>Poland - 1st Liga</t>
+          <t>Sweden - Superettan</t>
         </is>
       </c>
       <c r="C404" t="inlineStr">
         <is>
-          <t>Stal Mielec</t>
+          <t>Ljungskile</t>
         </is>
       </c>
       <c r="D404" t="inlineStr">
         <is>
-          <t>Polonia Bytom</t>
+          <t>Osters</t>
         </is>
       </c>
       <c r="E404" t="n">
-        <v>10.8</v>
+        <v>11.06</v>
       </c>
       <c r="F404" t="n">
-        <v>0.39</v>
+        <v>1.17</v>
       </c>
     </row>
     <row r="405">
       <c r="A405" s="1" t="n">
-        <v>46250</v>
+        <v>46249</v>
       </c>
       <c r="B405" t="inlineStr">
         <is>
-          <t>Spain - Segunda</t>
+          <t>Sweden - Superettan</t>
         </is>
       </c>
       <c r="C405" t="inlineStr">
         <is>
-          <t>Burgos</t>
+          <t>Nordic United</t>
         </is>
       </c>
       <c r="D405" t="inlineStr">
         <is>
-          <t>Cordoba</t>
+          <t>Varbergs BoIS</t>
         </is>
       </c>
       <c r="E405" t="n">
-        <v>9.359999999999999</v>
+        <v>9.949999999999999</v>
       </c>
       <c r="F405" t="n">
-        <v>0.05</v>
+        <v>0.19</v>
       </c>
     </row>
     <row r="406">
       <c r="A406" s="1" t="n">
-        <v>46251</v>
+        <v>46249</v>
       </c>
       <c r="B406" t="inlineStr">
         <is>
-          <t>Finland - Veikkausliiga</t>
+          <t>Sweden - Superettan</t>
         </is>
       </c>
       <c r="C406" t="inlineStr">
         <is>
-          <t>Gnistan</t>
+          <t>Sandvikens IF</t>
         </is>
       </c>
       <c r="D406" t="inlineStr">
         <is>
-          <t>Ilves</t>
+          <t>Norrkoping</t>
         </is>
       </c>
       <c r="E406" t="n">
-        <v>10.59</v>
+        <v>10.55</v>
       </c>
       <c r="F406" t="n">
-        <v>0.47</v>
+        <v>-1.06</v>
       </c>
     </row>
     <row r="407">
       <c r="A407" s="1" t="n">
+        <v>46249</v>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>Sundsvall</t>
+        </is>
+      </c>
+      <c r="D407" t="inlineStr">
+        <is>
+          <t>Helsingborgs</t>
+        </is>
+      </c>
+      <c r="E407" t="n">
+        <v>10.32</v>
+      </c>
+      <c r="F407" t="n">
+        <v>-1.14</v>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>America Mineiro</t>
+        </is>
+      </c>
+      <c r="D408" t="inlineStr">
+        <is>
+          <t>Athletic Club</t>
+        </is>
+      </c>
+      <c r="E408" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="F408" t="n">
+        <v>1.19</v>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>CRB</t>
+        </is>
+      </c>
+      <c r="D409" t="inlineStr">
+        <is>
+          <t>Gremio Novorizontino</t>
+        </is>
+      </c>
+      <c r="E409" t="n">
+        <v>10.51</v>
+      </c>
+      <c r="F409" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>Operario Ferroviario</t>
+        </is>
+      </c>
+      <c r="D410" t="inlineStr">
+        <is>
+          <t>Avai</t>
+        </is>
+      </c>
+      <c r="E410" t="n">
+        <v>10.29</v>
+      </c>
+      <c r="F410" t="n">
+        <v>2.02</v>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>AC Oulu</t>
+        </is>
+      </c>
+      <c r="D411" t="inlineStr">
+        <is>
+          <t>Inter Turku</t>
+        </is>
+      </c>
+      <c r="E411" t="n">
+        <v>10.11</v>
+      </c>
+      <c r="F411" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>FC Lahti</t>
+        </is>
+      </c>
+      <c r="D412" t="inlineStr">
+        <is>
+          <t>KuPS</t>
+        </is>
+      </c>
+      <c r="E412" t="n">
+        <v>10.07</v>
+      </c>
+      <c r="F412" t="n">
+        <v>-0.88</v>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>HJK Helsinki</t>
+        </is>
+      </c>
+      <c r="D413" t="inlineStr">
+        <is>
+          <t>Jaro</t>
+        </is>
+      </c>
+      <c r="E413" t="n">
+        <v>10.65</v>
+      </c>
+      <c r="F413" t="n">
+        <v>3.52</v>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>Finland - Ykkosliiga</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>Mikkelin Palloilijat</t>
+        </is>
+      </c>
+      <c r="D414" t="inlineStr">
+        <is>
+          <t>EIF</t>
+        </is>
+      </c>
+      <c r="E414" t="n">
+        <v>10.34</v>
+      </c>
+      <c r="F414" t="n">
+        <v>-0.49</v>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>Egersunds</t>
+        </is>
+      </c>
+      <c r="D415" t="inlineStr">
+        <is>
+          <t>Stabaek</t>
+        </is>
+      </c>
+      <c r="E415" t="n">
+        <v>11.09</v>
+      </c>
+      <c r="F415" t="n">
+        <v>-0.49</v>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>Hodd</t>
+        </is>
+      </c>
+      <c r="D416" t="inlineStr">
+        <is>
+          <t>Strommen</t>
+        </is>
+      </c>
+      <c r="E416" t="n">
+        <v>10.51</v>
+      </c>
+      <c r="F416" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>Raufoss</t>
+        </is>
+      </c>
+      <c r="D417" t="inlineStr">
+        <is>
+          <t>Asane Fotball</t>
+        </is>
+      </c>
+      <c r="E417" t="n">
+        <v>10.79</v>
+      </c>
+      <c r="F417" t="n">
+        <v>1.35</v>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>Sogndal</t>
+        </is>
+      </c>
+      <c r="D418" t="inlineStr">
+        <is>
+          <t>Sandnes Ulf</t>
+        </is>
+      </c>
+      <c r="E418" t="n">
+        <v>11.16</v>
+      </c>
+      <c r="F418" t="n">
+        <v>0.82</v>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>Stal Mielec</t>
+        </is>
+      </c>
+      <c r="D419" t="inlineStr">
+        <is>
+          <t>Polonia Bytom</t>
+        </is>
+      </c>
+      <c r="E419" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="F419" t="n">
+        <v>0.39</v>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>Cracovia Krakow</t>
+        </is>
+      </c>
+      <c r="D420" t="inlineStr">
+        <is>
+          <t>Rakow Czestochowa</t>
+        </is>
+      </c>
+      <c r="E420" t="n">
+        <v>9.65</v>
+      </c>
+      <c r="F420" t="n">
+        <v>0.85</v>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>Motor Lublin</t>
+        </is>
+      </c>
+      <c r="D421" t="inlineStr">
+        <is>
+          <t>GKS Katowice</t>
+        </is>
+      </c>
+      <c r="E421" t="n">
+        <v>10.47</v>
+      </c>
+      <c r="F421" t="n">
+        <v>-0.2</v>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>Otelul Galati</t>
+        </is>
+      </c>
+      <c r="D422" t="inlineStr">
+        <is>
+          <t>Universitatea Craiova</t>
+        </is>
+      </c>
+      <c r="E422" t="n">
+        <v>9.359999999999999</v>
+      </c>
+      <c r="F422" t="n">
+        <v>-1.19</v>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>Burgos</t>
+        </is>
+      </c>
+      <c r="D423" t="inlineStr">
+        <is>
+          <t>Cordoba</t>
+        </is>
+      </c>
+      <c r="E423" t="n">
+        <v>9.359999999999999</v>
+      </c>
+      <c r="F423" t="n">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>Las Palmas</t>
+        </is>
+      </c>
+      <c r="D424" t="inlineStr">
+        <is>
+          <t>Albacete</t>
+        </is>
+      </c>
+      <c r="E424" t="n">
+        <v>9.67</v>
+      </c>
+      <c r="F424" t="n">
+        <v>2.39</v>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" s="1" t="n">
         <v>46251</v>
       </c>
-      <c r="B407" t="inlineStr">
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>Gnistan</t>
+        </is>
+      </c>
+      <c r="D425" t="inlineStr">
+        <is>
+          <t>Ilves</t>
+        </is>
+      </c>
+      <c r="E425" t="n">
+        <v>10.59</v>
+      </c>
+      <c r="F425" t="n">
+        <v>0.47</v>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" s="1" t="n">
+        <v>46251</v>
+      </c>
+      <c r="B426" t="inlineStr">
         <is>
           <t>Romania - Liga 1</t>
         </is>
       </c>
-      <c r="C407" t="inlineStr">
+      <c r="C426" t="inlineStr">
         <is>
           <t>FCSB</t>
         </is>
       </c>
-      <c r="D407" t="inlineStr">
+      <c r="D426" t="inlineStr">
         <is>
           <t>Botosani</t>
         </is>
       </c>
-      <c r="E407" t="n">
+      <c r="E426" t="n">
         <v>9.789999999999999</v>
       </c>
-      <c r="F407" t="n">
+      <c r="F426" t="n">
         <v>2.48</v>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" s="1" t="n">
+        <v>46251</v>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>Universitatea Cluj</t>
+        </is>
+      </c>
+      <c r="D427" t="inlineStr">
+        <is>
+          <t>UTA Arad</t>
+        </is>
+      </c>
+      <c r="E427" t="n">
+        <v>9.470000000000001</v>
+      </c>
+      <c r="F427" t="n">
+        <v>0.93</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily scrape output - 2026-08-16
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F427"/>
+  <dimension ref="A1:F443"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11054,10 +11054,10 @@
         </is>
       </c>
       <c r="E409" t="n">
-        <v>10.51</v>
+        <v>10.34</v>
       </c>
       <c r="F409" t="n">
-        <v>1</v>
+        <v>1.02</v>
       </c>
     </row>
     <row r="410">
@@ -11106,7 +11106,7 @@
         </is>
       </c>
       <c r="E411" t="n">
-        <v>10.11</v>
+        <v>10.09</v>
       </c>
       <c r="F411" t="n">
         <v>-1</v>
@@ -11184,10 +11184,10 @@
         </is>
       </c>
       <c r="E414" t="n">
-        <v>10.34</v>
+        <v>10.45</v>
       </c>
       <c r="F414" t="n">
-        <v>-0.49</v>
+        <v>-0.98</v>
       </c>
     </row>
     <row r="415">
@@ -11210,10 +11210,10 @@
         </is>
       </c>
       <c r="E415" t="n">
-        <v>11.09</v>
+        <v>11.1</v>
       </c>
       <c r="F415" t="n">
-        <v>-0.49</v>
+        <v>-0.47</v>
       </c>
     </row>
     <row r="416">
@@ -11239,7 +11239,7 @@
         <v>10.51</v>
       </c>
       <c r="F416" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="417">
@@ -11253,19 +11253,19 @@
       </c>
       <c r="C417" t="inlineStr">
         <is>
-          <t>Raufoss</t>
+          <t>Kongsvinger</t>
         </is>
       </c>
       <c r="D417" t="inlineStr">
         <is>
-          <t>Asane Fotball</t>
+          <t>Haugesund</t>
         </is>
       </c>
       <c r="E417" t="n">
-        <v>10.79</v>
+        <v>11.3</v>
       </c>
       <c r="F417" t="n">
-        <v>1.35</v>
+        <v>0.92</v>
       </c>
     </row>
     <row r="418">
@@ -11279,19 +11279,19 @@
       </c>
       <c r="C418" t="inlineStr">
         <is>
-          <t>Sogndal</t>
+          <t>Raufoss</t>
         </is>
       </c>
       <c r="D418" t="inlineStr">
         <is>
-          <t>Sandnes Ulf</t>
+          <t>Asane Fotball</t>
         </is>
       </c>
       <c r="E418" t="n">
-        <v>11.16</v>
+        <v>10.79</v>
       </c>
       <c r="F418" t="n">
-        <v>0.82</v>
+        <v>1.35</v>
       </c>
     </row>
     <row r="419">
@@ -11300,24 +11300,24 @@
       </c>
       <c r="B419" t="inlineStr">
         <is>
-          <t>Poland - 1st Liga</t>
+          <t>Norway - 1st Division</t>
         </is>
       </c>
       <c r="C419" t="inlineStr">
         <is>
-          <t>Stal Mielec</t>
+          <t>Sogndal</t>
         </is>
       </c>
       <c r="D419" t="inlineStr">
         <is>
-          <t>Polonia Bytom</t>
+          <t>Sandnes Ulf</t>
         </is>
       </c>
       <c r="E419" t="n">
-        <v>10.8</v>
+        <v>11.16</v>
       </c>
       <c r="F419" t="n">
-        <v>0.39</v>
+        <v>0.82</v>
       </c>
     </row>
     <row r="420">
@@ -11326,24 +11326,24 @@
       </c>
       <c r="B420" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="C420" t="inlineStr">
         <is>
-          <t>Cracovia Krakow</t>
+          <t>LKS Lodz</t>
         </is>
       </c>
       <c r="D420" t="inlineStr">
         <is>
-          <t>Rakow Czestochowa</t>
+          <t>Nieciecza</t>
         </is>
       </c>
       <c r="E420" t="n">
-        <v>9.65</v>
+        <v>10.85</v>
       </c>
       <c r="F420" t="n">
-        <v>0.85</v>
+        <v>0.49</v>
       </c>
     </row>
     <row r="421">
@@ -11352,24 +11352,24 @@
       </c>
       <c r="B421" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="C421" t="inlineStr">
         <is>
-          <t>Motor Lublin</t>
+          <t>Stal Mielec</t>
         </is>
       </c>
       <c r="D421" t="inlineStr">
         <is>
-          <t>GKS Katowice</t>
+          <t>Polonia Bytom</t>
         </is>
       </c>
       <c r="E421" t="n">
-        <v>10.47</v>
+        <v>10.8</v>
       </c>
       <c r="F421" t="n">
-        <v>-0.2</v>
+        <v>0.41</v>
       </c>
     </row>
     <row r="422">
@@ -11378,24 +11378,24 @@
       </c>
       <c r="B422" t="inlineStr">
         <is>
-          <t>Romania - Liga 1</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="C422" t="inlineStr">
         <is>
-          <t>Otelul Galati</t>
+          <t>Unia Skierniewice</t>
         </is>
       </c>
       <c r="D422" t="inlineStr">
         <is>
-          <t>Universitatea Craiova</t>
+          <t>Miedz Legnica</t>
         </is>
       </c>
       <c r="E422" t="n">
-        <v>9.359999999999999</v>
+        <v>10.97</v>
       </c>
       <c r="F422" t="n">
-        <v>-1.19</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="423">
@@ -11404,24 +11404,24 @@
       </c>
       <c r="B423" t="inlineStr">
         <is>
-          <t>Spain - Segunda</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C423" t="inlineStr">
         <is>
-          <t>Burgos</t>
+          <t>Cracovia Krakow</t>
         </is>
       </c>
       <c r="D423" t="inlineStr">
         <is>
-          <t>Cordoba</t>
+          <t>Rakow Czestochowa</t>
         </is>
       </c>
       <c r="E423" t="n">
-        <v>9.359999999999999</v>
+        <v>9.67</v>
       </c>
       <c r="F423" t="n">
-        <v>0.05</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="424">
@@ -11430,55 +11430,55 @@
       </c>
       <c r="B424" t="inlineStr">
         <is>
-          <t>Spain - Segunda</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C424" t="inlineStr">
         <is>
-          <t>Las Palmas</t>
+          <t>Gornik Zabrze</t>
         </is>
       </c>
       <c r="D424" t="inlineStr">
         <is>
-          <t>Albacete</t>
+          <t>Wisla Krakow</t>
         </is>
       </c>
       <c r="E424" t="n">
-        <v>9.67</v>
+        <v>10.61</v>
       </c>
       <c r="F424" t="n">
-        <v>2.39</v>
+        <v>1.63</v>
       </c>
     </row>
     <row r="425">
       <c r="A425" s="1" t="n">
-        <v>46251</v>
+        <v>46250</v>
       </c>
       <c r="B425" t="inlineStr">
         <is>
-          <t>Finland - Veikkausliiga</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C425" t="inlineStr">
         <is>
-          <t>Gnistan</t>
+          <t>Motor Lublin</t>
         </is>
       </c>
       <c r="D425" t="inlineStr">
         <is>
-          <t>Ilves</t>
+          <t>GKS Katowice</t>
         </is>
       </c>
       <c r="E425" t="n">
-        <v>10.59</v>
+        <v>10.45</v>
       </c>
       <c r="F425" t="n">
-        <v>0.47</v>
+        <v>-0.31</v>
       </c>
     </row>
     <row r="426">
       <c r="A426" s="1" t="n">
-        <v>46251</v>
+        <v>46250</v>
       </c>
       <c r="B426" t="inlineStr">
         <is>
@@ -11487,45 +11487,461 @@
       </c>
       <c r="C426" t="inlineStr">
         <is>
-          <t>FCSB</t>
+          <t>Corvinul Hunedoara</t>
         </is>
       </c>
       <c r="D426" t="inlineStr">
         <is>
-          <t>Botosani</t>
+          <t>CFR Cluj</t>
         </is>
       </c>
       <c r="E426" t="n">
-        <v>9.789999999999999</v>
+        <v>9.01</v>
       </c>
       <c r="F426" t="n">
-        <v>2.48</v>
+        <v>-0.32</v>
       </c>
     </row>
     <row r="427">
       <c r="A427" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>Otelul Galati</t>
+        </is>
+      </c>
+      <c r="D427" t="inlineStr">
+        <is>
+          <t>Universitatea Craiova</t>
+        </is>
+      </c>
+      <c r="E427" t="n">
+        <v>9.359999999999999</v>
+      </c>
+      <c r="F427" t="n">
+        <v>-1.19</v>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>Burgos</t>
+        </is>
+      </c>
+      <c r="D428" t="inlineStr">
+        <is>
+          <t>Cordoba</t>
+        </is>
+      </c>
+      <c r="E428" t="n">
+        <v>9.359999999999999</v>
+      </c>
+      <c r="F428" t="n">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>Eibar</t>
+        </is>
+      </c>
+      <c r="D429" t="inlineStr">
+        <is>
+          <t>Tenerife</t>
+        </is>
+      </c>
+      <c r="E429" t="n">
+        <v>9.18</v>
+      </c>
+      <c r="F429" t="n">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>Girona</t>
+        </is>
+      </c>
+      <c r="D430" t="inlineStr">
+        <is>
+          <t>Leganes</t>
+        </is>
+      </c>
+      <c r="E430" t="n">
+        <v>9.619999999999999</v>
+      </c>
+      <c r="F430" t="n">
+        <v>2.24</v>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>Las Palmas</t>
+        </is>
+      </c>
+      <c r="D431" t="inlineStr">
+        <is>
+          <t>Albacete</t>
+        </is>
+      </c>
+      <c r="E431" t="n">
+        <v>9.67</v>
+      </c>
+      <c r="F431" t="n">
+        <v>2.39</v>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>Varnamo</t>
+        </is>
+      </c>
+      <c r="D432" t="inlineStr">
+        <is>
+          <t>Ostersunds FK</t>
+        </is>
+      </c>
+      <c r="E432" t="n">
+        <v>10</v>
+      </c>
+      <c r="F432" t="n">
+        <v>-0.09</v>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" s="1" t="n">
         <v>46251</v>
       </c>
-      <c r="B427" t="inlineStr">
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>Gnistan</t>
+        </is>
+      </c>
+      <c r="D433" t="inlineStr">
+        <is>
+          <t>Ilves</t>
+        </is>
+      </c>
+      <c r="E433" t="n">
+        <v>10.62</v>
+      </c>
+      <c r="F433" t="n">
+        <v>-0</v>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" s="1" t="n">
+        <v>46251</v>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>Iceland - 1. Deild</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>Afturelding</t>
+        </is>
+      </c>
+      <c r="D434" t="inlineStr">
+        <is>
+          <t>HK Kopavogur</t>
+        </is>
+      </c>
+      <c r="E434" t="n">
+        <v>11.67</v>
+      </c>
+      <c r="F434" t="n">
+        <v>1.62</v>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" s="1" t="n">
+        <v>46251</v>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>Iceland - 1. Deild</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>IR Reykjavik</t>
+        </is>
+      </c>
+      <c r="D435" t="inlineStr">
+        <is>
+          <t>UMF Njardvik</t>
+        </is>
+      </c>
+      <c r="E435" t="n">
+        <v>11.28</v>
+      </c>
+      <c r="F435" t="n">
+        <v>-0.13</v>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" s="1" t="n">
+        <v>46251</v>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>Iceland - 1. Deild</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>Leiknir Reykjavik</t>
+        </is>
+      </c>
+      <c r="D436" t="inlineStr">
+        <is>
+          <t>Aegir</t>
+        </is>
+      </c>
+      <c r="E436" t="n">
+        <v>11.65</v>
+      </c>
+      <c r="F436" t="n">
+        <v>3.18</v>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" s="1" t="n">
+        <v>46251</v>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>Iceland - 1. Deild</t>
+        </is>
+      </c>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>Throttur Reykjavik</t>
+        </is>
+      </c>
+      <c r="D437" t="inlineStr">
+        <is>
+          <t>Fylkir</t>
+        </is>
+      </c>
+      <c r="E437" t="n">
+        <v>10.99</v>
+      </c>
+      <c r="F437" t="n">
+        <v>1.07</v>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" s="1" t="n">
+        <v>46251</v>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>Iceland - 1. Deild</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>Volsungur</t>
+        </is>
+      </c>
+      <c r="D438" t="inlineStr">
+        <is>
+          <t>Vestri</t>
+        </is>
+      </c>
+      <c r="E438" t="n">
+        <v>11.11</v>
+      </c>
+      <c r="F438" t="n">
+        <v>-0.66</v>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" s="1" t="n">
+        <v>46251</v>
+      </c>
+      <c r="B439" t="inlineStr">
         <is>
           <t>Romania - Liga 1</t>
         </is>
       </c>
-      <c r="C427" t="inlineStr">
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>FCSB</t>
+        </is>
+      </c>
+      <c r="D439" t="inlineStr">
+        <is>
+          <t>Botosani</t>
+        </is>
+      </c>
+      <c r="E439" t="n">
+        <v>9.789999999999999</v>
+      </c>
+      <c r="F439" t="n">
+        <v>2.48</v>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" s="1" t="n">
+        <v>46251</v>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr">
         <is>
           <t>Universitatea Cluj</t>
         </is>
       </c>
-      <c r="D427" t="inlineStr">
+      <c r="D440" t="inlineStr">
         <is>
           <t>UTA Arad</t>
         </is>
       </c>
-      <c r="E427" t="n">
+      <c r="E440" t="n">
         <v>9.470000000000001</v>
       </c>
-      <c r="F427" t="n">
+      <c r="F440" t="n">
         <v>0.93</v>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" s="1" t="n">
+        <v>46252</v>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>Londrina</t>
+        </is>
+      </c>
+      <c r="D441" t="inlineStr">
+        <is>
+          <t>Atletico Goianiense</t>
+        </is>
+      </c>
+      <c r="E441" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="F441" t="n">
+        <v>0.52</v>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" s="1" t="n">
+        <v>46253</v>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>Goias</t>
+        </is>
+      </c>
+      <c r="D442" t="inlineStr">
+        <is>
+          <t>Juventude</t>
+        </is>
+      </c>
+      <c r="E442" t="n">
+        <v>10.11</v>
+      </c>
+      <c r="F442" t="n">
+        <v>1.47</v>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" s="1" t="n">
+        <v>46253</v>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>Nautico</t>
+        </is>
+      </c>
+      <c r="D443" t="inlineStr">
+        <is>
+          <t>Ceara</t>
+        </is>
+      </c>
+      <c r="E443" t="n">
+        <v>10.57</v>
+      </c>
+      <c r="F443" t="n">
+        <v>1.44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily scrape output - 2026-08-17
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F443"/>
+  <dimension ref="A1:F446"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11704,10 +11704,10 @@
         </is>
       </c>
       <c r="E434" t="n">
-        <v>11.67</v>
+        <v>11.69</v>
       </c>
       <c r="F434" t="n">
-        <v>1.62</v>
+        <v>1.36</v>
       </c>
     </row>
     <row r="435">
@@ -11730,10 +11730,10 @@
         </is>
       </c>
       <c r="E435" t="n">
-        <v>11.28</v>
+        <v>11.45</v>
       </c>
       <c r="F435" t="n">
-        <v>-0.13</v>
+        <v>-0.64</v>
       </c>
     </row>
     <row r="436">
@@ -11756,10 +11756,10 @@
         </is>
       </c>
       <c r="E436" t="n">
-        <v>11.65</v>
+        <v>11.36</v>
       </c>
       <c r="F436" t="n">
-        <v>3.18</v>
+        <v>1.11</v>
       </c>
     </row>
     <row r="437">
@@ -11782,7 +11782,7 @@
         </is>
       </c>
       <c r="E437" t="n">
-        <v>10.99</v>
+        <v>11.07</v>
       </c>
       <c r="F437" t="n">
         <v>1.07</v>
@@ -11820,24 +11820,24 @@
       </c>
       <c r="B439" t="inlineStr">
         <is>
-          <t>Romania - Liga 1</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="C439" t="inlineStr">
         <is>
-          <t>FCSB</t>
+          <t>Arka Gdynia</t>
         </is>
       </c>
       <c r="D439" t="inlineStr">
         <is>
-          <t>Botosani</t>
+          <t>Puszcza Niepolomice</t>
         </is>
       </c>
       <c r="E439" t="n">
-        <v>9.789999999999999</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="F439" t="n">
-        <v>2.48</v>
+        <v>1.69</v>
       </c>
     </row>
     <row r="440">
@@ -11851,96 +11851,174 @@
       </c>
       <c r="C440" t="inlineStr">
         <is>
-          <t>Universitatea Cluj</t>
+          <t>FCSB</t>
         </is>
       </c>
       <c r="D440" t="inlineStr">
         <is>
-          <t>UTA Arad</t>
+          <t>Botosani</t>
         </is>
       </c>
       <c r="E440" t="n">
-        <v>9.470000000000001</v>
+        <v>9.789999999999999</v>
       </c>
       <c r="F440" t="n">
-        <v>0.93</v>
+        <v>2.48</v>
       </c>
     </row>
     <row r="441">
       <c r="A441" s="1" t="n">
-        <v>46252</v>
+        <v>46251</v>
       </c>
       <c r="B441" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Romania - Liga 1</t>
         </is>
       </c>
       <c r="C441" t="inlineStr">
         <is>
-          <t>Londrina</t>
+          <t>Universitatea Cluj</t>
         </is>
       </c>
       <c r="D441" t="inlineStr">
         <is>
-          <t>Atletico Goianiense</t>
+          <t>UTA Arad</t>
         </is>
       </c>
       <c r="E441" t="n">
-        <v>10.7</v>
+        <v>9.470000000000001</v>
       </c>
       <c r="F441" t="n">
-        <v>0.52</v>
+        <v>0.93</v>
       </c>
     </row>
     <row r="442">
       <c r="A442" s="1" t="n">
-        <v>46253</v>
+        <v>46251</v>
       </c>
       <c r="B442" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="C442" t="inlineStr">
         <is>
-          <t>Goias</t>
+          <t>Almeria</t>
         </is>
       </c>
       <c r="D442" t="inlineStr">
         <is>
-          <t>Juventude</t>
+          <t>Eldense</t>
         </is>
       </c>
       <c r="E442" t="n">
-        <v>10.11</v>
+        <v>9.640000000000001</v>
       </c>
       <c r="F442" t="n">
-        <v>1.47</v>
+        <v>2.69</v>
       </c>
     </row>
     <row r="443">
       <c r="A443" s="1" t="n">
+        <v>46251</v>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>Sporting Gijon</t>
+        </is>
+      </c>
+      <c r="D443" t="inlineStr">
+        <is>
+          <t>Sabadell</t>
+        </is>
+      </c>
+      <c r="E443" t="n">
+        <v>9.18</v>
+      </c>
+      <c r="F443" t="n">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" s="1" t="n">
+        <v>46252</v>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>Londrina</t>
+        </is>
+      </c>
+      <c r="D444" t="inlineStr">
+        <is>
+          <t>Atletico Goianiense</t>
+        </is>
+      </c>
+      <c r="E444" t="n">
+        <v>10.45</v>
+      </c>
+      <c r="F444" t="n">
+        <v>0.55</v>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" s="1" t="n">
         <v>46253</v>
       </c>
-      <c r="B443" t="inlineStr">
+      <c r="B445" t="inlineStr">
         <is>
           <t>Brazil - Serie B</t>
         </is>
       </c>
-      <c r="C443" t="inlineStr">
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>Goias</t>
+        </is>
+      </c>
+      <c r="D445" t="inlineStr">
+        <is>
+          <t>Juventude</t>
+        </is>
+      </c>
+      <c r="E445" t="n">
+        <v>10.11</v>
+      </c>
+      <c r="F445" t="n">
+        <v>1.47</v>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" s="1" t="n">
+        <v>46253</v>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr">
         <is>
           <t>Nautico</t>
         </is>
       </c>
-      <c r="D443" t="inlineStr">
+      <c r="D446" t="inlineStr">
         <is>
           <t>Ceara</t>
         </is>
       </c>
-      <c r="E443" t="n">
+      <c r="E446" t="n">
         <v>10.57</v>
       </c>
-      <c r="F443" t="n">
+      <c r="F446" t="n">
         <v>1.44</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily scrape output - 2026-08-18
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -11681,7 +11681,7 @@
         <v>10.62</v>
       </c>
       <c r="F433" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="434">
@@ -11964,10 +11964,10 @@
         </is>
       </c>
       <c r="E444" t="n">
-        <v>10.45</v>
+        <v>10.67</v>
       </c>
       <c r="F444" t="n">
-        <v>0.55</v>
+        <v>0.49</v>
       </c>
     </row>
     <row r="445">
@@ -12016,7 +12016,7 @@
         </is>
       </c>
       <c r="E446" t="n">
-        <v>10.57</v>
+        <v>10.6</v>
       </c>
       <c r="F446" t="n">
         <v>1.44</v>

</xml_diff>

<commit_message>
Daily scrape output - 2026-08-20
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F446"/>
+  <dimension ref="A1:F449"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12022,6 +12022,84 @@
         <v>1.44</v>
       </c>
     </row>
+    <row r="447">
+      <c r="A447" s="1" t="n">
+        <v>46254</v>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>Athletic Club</t>
+        </is>
+      </c>
+      <c r="D447" t="inlineStr">
+        <is>
+          <t>CRB</t>
+        </is>
+      </c>
+      <c r="E447" t="n">
+        <v>9.720000000000001</v>
+      </c>
+      <c r="F447" t="n">
+        <v>0.59</v>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" s="1" t="n">
+        <v>46254</v>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t>Gremio Novorizontino</t>
+        </is>
+      </c>
+      <c r="D448" t="inlineStr">
+        <is>
+          <t>America Mineiro</t>
+        </is>
+      </c>
+      <c r="E448" t="n">
+        <v>10.52</v>
+      </c>
+      <c r="F448" t="n">
+        <v>2.47</v>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" s="1" t="n">
+        <v>46254</v>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>Finland - Ykkosliiga</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>KaPa</t>
+        </is>
+      </c>
+      <c r="D449" t="inlineStr">
+        <is>
+          <t>JIPPO</t>
+        </is>
+      </c>
+      <c r="E449" t="n">
+        <v>10.09</v>
+      </c>
+      <c r="F449" t="n">
+        <v>-1.67</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily scrape output - 2026-08-21
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F449"/>
+  <dimension ref="A1:F456"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12100,6 +12100,188 @@
         <v>-1.67</v>
       </c>
     </row>
+    <row r="450">
+      <c r="A450" s="1" t="n">
+        <v>46255</v>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t>SJK</t>
+        </is>
+      </c>
+      <c r="D450" t="inlineStr">
+        <is>
+          <t>FC Lahti</t>
+        </is>
+      </c>
+      <c r="E450" t="n">
+        <v>10.34</v>
+      </c>
+      <c r="F450" t="n">
+        <v>0.31</v>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" s="1" t="n">
+        <v>46255</v>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>Finland - Ykkosliiga</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>PK-35</t>
+        </is>
+      </c>
+      <c r="D451" t="inlineStr">
+        <is>
+          <t>JaPS</t>
+        </is>
+      </c>
+      <c r="E451" t="n">
+        <v>10.69</v>
+      </c>
+      <c r="F451" t="n">
+        <v>1.96</v>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" s="1" t="n">
+        <v>46255</v>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>Iceland - 1. Deild</t>
+        </is>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t>Aegir</t>
+        </is>
+      </c>
+      <c r="D452" t="inlineStr">
+        <is>
+          <t>Afturelding</t>
+        </is>
+      </c>
+      <c r="E452" t="n">
+        <v>11.67</v>
+      </c>
+      <c r="F452" t="n">
+        <v>-4.42</v>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" s="1" t="n">
+        <v>46255</v>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>Iceland - 1. Deild</t>
+        </is>
+      </c>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t>Grotta</t>
+        </is>
+      </c>
+      <c r="D453" t="inlineStr">
+        <is>
+          <t>IR Reykjavik</t>
+        </is>
+      </c>
+      <c r="E453" t="n">
+        <v>12.05</v>
+      </c>
+      <c r="F453" t="n">
+        <v>-0.1</v>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" s="1" t="n">
+        <v>46255</v>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C454" t="inlineStr">
+        <is>
+          <t>Lechia Gdansk</t>
+        </is>
+      </c>
+      <c r="D454" t="inlineStr">
+        <is>
+          <t>Pogon Siedlce</t>
+        </is>
+      </c>
+      <c r="E454" t="n">
+        <v>10.58</v>
+      </c>
+      <c r="F454" t="n">
+        <v>1.36</v>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" s="1" t="n">
+        <v>46255</v>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>Cracovia Krakow</t>
+        </is>
+      </c>
+      <c r="D455" t="inlineStr">
+        <is>
+          <t>Wieczysta Krakow</t>
+        </is>
+      </c>
+      <c r="E455" t="n">
+        <v>10.45</v>
+      </c>
+      <c r="F455" t="n">
+        <v>1.38</v>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" s="1" t="n">
+        <v>46255</v>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C456" t="inlineStr">
+        <is>
+          <t>Petrolul Ploiesti</t>
+        </is>
+      </c>
+      <c r="D456" t="inlineStr">
+        <is>
+          <t>Rapid Bucuresti</t>
+        </is>
+      </c>
+      <c r="E456" t="n">
+        <v>9.57</v>
+      </c>
+      <c r="F456" t="n">
+        <v>-0.59</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily scrape output - 2026-08-22
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F456"/>
+  <dimension ref="A1:F504"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12282,6 +12282,1254 @@
         <v>-0.59</v>
       </c>
     </row>
+    <row r="457">
+      <c r="A457" s="1" t="n">
+        <v>46256</v>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>Ceara</t>
+        </is>
+      </c>
+      <c r="D457" t="inlineStr">
+        <is>
+          <t>Londrina</t>
+        </is>
+      </c>
+      <c r="E457" t="n">
+        <v>10.75</v>
+      </c>
+      <c r="F457" t="n">
+        <v>2.05</v>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" s="1" t="n">
+        <v>46256</v>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C458" t="inlineStr">
+        <is>
+          <t>Cuiaba</t>
+        </is>
+      </c>
+      <c r="D458" t="inlineStr">
+        <is>
+          <t>Goias</t>
+        </is>
+      </c>
+      <c r="E458" t="n">
+        <v>10.16</v>
+      </c>
+      <c r="F458" t="n">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" s="1" t="n">
+        <v>46256</v>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C459" t="inlineStr">
+        <is>
+          <t>Ilves</t>
+        </is>
+      </c>
+      <c r="D459" t="inlineStr">
+        <is>
+          <t>VPS</t>
+        </is>
+      </c>
+      <c r="E459" t="n">
+        <v>10.24</v>
+      </c>
+      <c r="F459" t="n">
+        <v>-0.02</v>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" s="1" t="n">
+        <v>46256</v>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C460" t="inlineStr">
+        <is>
+          <t>Jaro</t>
+        </is>
+      </c>
+      <c r="D460" t="inlineStr">
+        <is>
+          <t>AC Oulu</t>
+        </is>
+      </c>
+      <c r="E460" t="n">
+        <v>9.970000000000001</v>
+      </c>
+      <c r="F460" t="n">
+        <v>-0.93</v>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" s="1" t="n">
+        <v>46256</v>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>Finland - Ykkosliiga</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>EIF</t>
+        </is>
+      </c>
+      <c r="D461" t="inlineStr">
+        <is>
+          <t>KTP</t>
+        </is>
+      </c>
+      <c r="E461" t="n">
+        <v>10.59</v>
+      </c>
+      <c r="F461" t="n">
+        <v>-1.13</v>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" s="1" t="n">
+        <v>46256</v>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>Iceland - 1. Deild</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>Fylkir</t>
+        </is>
+      </c>
+      <c r="D462" t="inlineStr">
+        <is>
+          <t>UMF Grindavik</t>
+        </is>
+      </c>
+      <c r="E462" t="n">
+        <v>11.65</v>
+      </c>
+      <c r="F462" t="n">
+        <v>3.52</v>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" s="1" t="n">
+        <v>46256</v>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>Iceland - 1. Deild</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>HK Kopavogur</t>
+        </is>
+      </c>
+      <c r="D463" t="inlineStr">
+        <is>
+          <t>Throttur Reykjavik</t>
+        </is>
+      </c>
+      <c r="E463" t="n">
+        <v>11.45</v>
+      </c>
+      <c r="F463" t="n">
+        <v>-0</v>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" s="1" t="n">
+        <v>46256</v>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>Iceland - 1. Deild</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>UMF Njardvik</t>
+        </is>
+      </c>
+      <c r="D464" t="inlineStr">
+        <is>
+          <t>Volsungur</t>
+        </is>
+      </c>
+      <c r="E464" t="n">
+        <v>11.53</v>
+      </c>
+      <c r="F464" t="n">
+        <v>3.69</v>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" s="1" t="n">
+        <v>46256</v>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>Iceland - 1. Deild</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>Vestri</t>
+        </is>
+      </c>
+      <c r="D465" t="inlineStr">
+        <is>
+          <t>Leiknir Reykjavik</t>
+        </is>
+      </c>
+      <c r="E465" t="n">
+        <v>11.15</v>
+      </c>
+      <c r="F465" t="n">
+        <v>1.19</v>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" s="1" t="n">
+        <v>46256</v>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C466" t="inlineStr">
+        <is>
+          <t>Sandnes Ulf</t>
+        </is>
+      </c>
+      <c r="D466" t="inlineStr">
+        <is>
+          <t>Bryne</t>
+        </is>
+      </c>
+      <c r="E466" t="n">
+        <v>10.74</v>
+      </c>
+      <c r="F466" t="n">
+        <v>-0.32</v>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" s="1" t="n">
+        <v>46256</v>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>Nieciecza</t>
+        </is>
+      </c>
+      <c r="D467" t="inlineStr">
+        <is>
+          <t>Polonia Warsaw</t>
+        </is>
+      </c>
+      <c r="E467" t="n">
+        <v>11</v>
+      </c>
+      <c r="F467" t="n">
+        <v>0.34</v>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" s="1" t="n">
+        <v>46256</v>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>Podbeskidzie Bielsko-Biala</t>
+        </is>
+      </c>
+      <c r="D468" t="inlineStr">
+        <is>
+          <t>Odra Opole</t>
+        </is>
+      </c>
+      <c r="E468" t="n">
+        <v>10.34</v>
+      </c>
+      <c r="F468" t="n">
+        <v>0.49</v>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" s="1" t="n">
+        <v>46256</v>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>Piast Gliwice</t>
+        </is>
+      </c>
+      <c r="D469" t="inlineStr">
+        <is>
+          <t>Legia Warsaw</t>
+        </is>
+      </c>
+      <c r="E469" t="n">
+        <v>10.07</v>
+      </c>
+      <c r="F469" t="n">
+        <v>-0.5600000000000001</v>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" s="1" t="n">
+        <v>46256</v>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t>Slask Wroclaw</t>
+        </is>
+      </c>
+      <c r="D470" t="inlineStr">
+        <is>
+          <t>Widzew Lodz</t>
+        </is>
+      </c>
+      <c r="E470" t="n">
+        <v>10.16</v>
+      </c>
+      <c r="F470" t="n">
+        <v>-0.04</v>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" s="1" t="n">
+        <v>46256</v>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>Dinamo Bucuresti</t>
+        </is>
+      </c>
+      <c r="D471" t="inlineStr">
+        <is>
+          <t>Universitatea Cluj</t>
+        </is>
+      </c>
+      <c r="E471" t="n">
+        <v>9.640000000000001</v>
+      </c>
+      <c r="F471" t="n">
+        <v>2.49</v>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" s="1" t="n">
+        <v>46256</v>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>UTA Arad</t>
+        </is>
+      </c>
+      <c r="D472" t="inlineStr">
+        <is>
+          <t>Corvinul Hunedoara</t>
+        </is>
+      </c>
+      <c r="E472" t="n">
+        <v>9.66</v>
+      </c>
+      <c r="F472" t="n">
+        <v>1.14</v>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" s="1" t="n">
+        <v>46256</v>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>Albacete</t>
+        </is>
+      </c>
+      <c r="D473" t="inlineStr">
+        <is>
+          <t>Real Sociedad II</t>
+        </is>
+      </c>
+      <c r="E473" t="n">
+        <v>9.640000000000001</v>
+      </c>
+      <c r="F473" t="n">
+        <v>1.89</v>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" s="1" t="n">
+        <v>46256</v>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t>Ceuta</t>
+        </is>
+      </c>
+      <c r="D474" t="inlineStr">
+        <is>
+          <t>Las Palmas</t>
+        </is>
+      </c>
+      <c r="E474" t="n">
+        <v>9.02</v>
+      </c>
+      <c r="F474" t="n">
+        <v>-0.41</v>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" s="1" t="n">
+        <v>46256</v>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>Eldense</t>
+        </is>
+      </c>
+      <c r="D475" t="inlineStr">
+        <is>
+          <t>Cadiz</t>
+        </is>
+      </c>
+      <c r="E475" t="n">
+        <v>9.279999999999999</v>
+      </c>
+      <c r="F475" t="n">
+        <v>0.91</v>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" s="1" t="n">
+        <v>46256</v>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C476" t="inlineStr">
+        <is>
+          <t>Real Oviedo</t>
+        </is>
+      </c>
+      <c r="D476" t="inlineStr">
+        <is>
+          <t>Leganes</t>
+        </is>
+      </c>
+      <c r="E476" t="n">
+        <v>9.390000000000001</v>
+      </c>
+      <c r="F476" t="n">
+        <v>1.62</v>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" s="1" t="n">
+        <v>46257</v>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>Criciuma</t>
+        </is>
+      </c>
+      <c r="D477" t="inlineStr">
+        <is>
+          <t>Fortaleza</t>
+        </is>
+      </c>
+      <c r="E477" t="n">
+        <v>10.65</v>
+      </c>
+      <c r="F477" t="n">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" s="1" t="n">
+        <v>46257</v>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr">
+        <is>
+          <t>Ponte Preta</t>
+        </is>
+      </c>
+      <c r="D478" t="inlineStr">
+        <is>
+          <t>Avai</t>
+        </is>
+      </c>
+      <c r="E478" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="F478" t="n">
+        <v>0.39</v>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" s="1" t="n">
+        <v>46257</v>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>Sao Bernardo</t>
+        </is>
+      </c>
+      <c r="D479" t="inlineStr">
+        <is>
+          <t>Nautico</t>
+        </is>
+      </c>
+      <c r="E479" t="n">
+        <v>10.56</v>
+      </c>
+      <c r="F479" t="n">
+        <v>0.89</v>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" s="1" t="n">
+        <v>46257</v>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t>HJK Helsinki</t>
+        </is>
+      </c>
+      <c r="D480" t="inlineStr">
+        <is>
+          <t>Gnistan</t>
+        </is>
+      </c>
+      <c r="E480" t="n">
+        <v>10.87</v>
+      </c>
+      <c r="F480" t="n">
+        <v>2.23</v>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" s="1" t="n">
+        <v>46257</v>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>KuPS</t>
+        </is>
+      </c>
+      <c r="D481" t="inlineStr">
+        <is>
+          <t>IFK Mariehamn</t>
+        </is>
+      </c>
+      <c r="E481" t="n">
+        <v>10.57</v>
+      </c>
+      <c r="F481" t="n">
+        <v>4.27</v>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" s="1" t="n">
+        <v>46257</v>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t>TPS</t>
+        </is>
+      </c>
+      <c r="D482" t="inlineStr">
+        <is>
+          <t>Inter Turku</t>
+        </is>
+      </c>
+      <c r="E482" t="n">
+        <v>9.970000000000001</v>
+      </c>
+      <c r="F482" t="n">
+        <v>-1.02</v>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" s="1" t="n">
+        <v>46257</v>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>LKS Lodz</t>
+        </is>
+      </c>
+      <c r="D483" t="inlineStr">
+        <is>
+          <t>Stal Mielec</t>
+        </is>
+      </c>
+      <c r="E483" t="n">
+        <v>10.98</v>
+      </c>
+      <c r="F483" t="n">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" s="1" t="n">
+        <v>46257</v>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>GKS Katowice</t>
+        </is>
+      </c>
+      <c r="D484" t="inlineStr">
+        <is>
+          <t>Wisla Plock</t>
+        </is>
+      </c>
+      <c r="E484" t="n">
+        <v>10.38</v>
+      </c>
+      <c r="F484" t="n">
+        <v>1.49</v>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" s="1" t="n">
+        <v>46257</v>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>Radomiak Radom</t>
+        </is>
+      </c>
+      <c r="D485" t="inlineStr">
+        <is>
+          <t>Zaglebie Lubin</t>
+        </is>
+      </c>
+      <c r="E485" t="n">
+        <v>10.32</v>
+      </c>
+      <c r="F485" t="n">
+        <v>1.34</v>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" s="1" t="n">
+        <v>46257</v>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t>CFR Cluj</t>
+        </is>
+      </c>
+      <c r="D486" t="inlineStr">
+        <is>
+          <t>FCSB</t>
+        </is>
+      </c>
+      <c r="E486" t="n">
+        <v>9.73</v>
+      </c>
+      <c r="F486" t="n">
+        <v>0.33</v>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" s="1" t="n">
+        <v>46257</v>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t>Castellon</t>
+        </is>
+      </c>
+      <c r="D487" t="inlineStr">
+        <is>
+          <t>Sabadell</t>
+        </is>
+      </c>
+      <c r="E487" t="n">
+        <v>9.33</v>
+      </c>
+      <c r="F487" t="n">
+        <v>2.44</v>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" s="1" t="n">
+        <v>46257</v>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C488" t="inlineStr">
+        <is>
+          <t>Eibar</t>
+        </is>
+      </c>
+      <c r="D488" t="inlineStr">
+        <is>
+          <t>Real Valladolid</t>
+        </is>
+      </c>
+      <c r="E488" t="n">
+        <v>9.16</v>
+      </c>
+      <c r="F488" t="n">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" s="1" t="n">
+        <v>46257</v>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C489" t="inlineStr">
+        <is>
+          <t>Tenerife</t>
+        </is>
+      </c>
+      <c r="D489" t="inlineStr">
+        <is>
+          <t>Almeria</t>
+        </is>
+      </c>
+      <c r="E489" t="n">
+        <v>9.460000000000001</v>
+      </c>
+      <c r="F489" t="n">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" s="1" t="n">
+        <v>46257</v>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C490" t="inlineStr">
+        <is>
+          <t>Brage</t>
+        </is>
+      </c>
+      <c r="D490" t="inlineStr">
+        <is>
+          <t>Nordic United</t>
+        </is>
+      </c>
+      <c r="E490" t="n">
+        <v>9.359999999999999</v>
+      </c>
+      <c r="F490" t="n">
+        <v>0.53</v>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" s="1" t="n">
+        <v>46257</v>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C491" t="inlineStr">
+        <is>
+          <t>Norrby</t>
+        </is>
+      </c>
+      <c r="D491" t="inlineStr">
+        <is>
+          <t>Sandvikens IF</t>
+        </is>
+      </c>
+      <c r="E491" t="n">
+        <v>9.51</v>
+      </c>
+      <c r="F491" t="n">
+        <v>0.55</v>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" s="1" t="n">
+        <v>46257</v>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>Oddevold</t>
+        </is>
+      </c>
+      <c r="D492" t="inlineStr">
+        <is>
+          <t>Helsingborgs</t>
+        </is>
+      </c>
+      <c r="E492" t="n">
+        <v>8.789999999999999</v>
+      </c>
+      <c r="F492" t="n">
+        <v>1.49</v>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" s="1" t="n">
+        <v>46258</v>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t>Athletic Club</t>
+        </is>
+      </c>
+      <c r="D493" t="inlineStr">
+        <is>
+          <t>Gremio Novorizontino</t>
+        </is>
+      </c>
+      <c r="E493" t="n">
+        <v>10.18</v>
+      </c>
+      <c r="F493" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" s="1" t="n">
+        <v>46258</v>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>Sport Recife</t>
+        </is>
+      </c>
+      <c r="D494" t="inlineStr">
+        <is>
+          <t>America Mineiro</t>
+        </is>
+      </c>
+      <c r="E494" t="n">
+        <v>10.48</v>
+      </c>
+      <c r="F494" t="n">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" s="1" t="n">
+        <v>46258</v>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>Stal Rzeszow</t>
+        </is>
+      </c>
+      <c r="D495" t="inlineStr">
+        <is>
+          <t>Ruch Chorzow</t>
+        </is>
+      </c>
+      <c r="E495" t="n">
+        <v>10.78</v>
+      </c>
+      <c r="F495" t="n">
+        <v>-0.34</v>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" s="1" t="n">
+        <v>46258</v>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>Botosani</t>
+        </is>
+      </c>
+      <c r="D496" t="inlineStr">
+        <is>
+          <t>Csikszereda</t>
+        </is>
+      </c>
+      <c r="E496" t="n">
+        <v>9.720000000000001</v>
+      </c>
+      <c r="F496" t="n">
+        <v>2.51</v>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" s="1" t="n">
+        <v>46258</v>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>Otelul Galati</t>
+        </is>
+      </c>
+      <c r="D497" t="inlineStr">
+        <is>
+          <t>Arges Pitesti</t>
+        </is>
+      </c>
+      <c r="E497" t="n">
+        <v>9.539999999999999</v>
+      </c>
+      <c r="F497" t="n">
+        <v>0.45</v>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" s="1" t="n">
+        <v>46258</v>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>Norrkoping</t>
+        </is>
+      </c>
+      <c r="D498" t="inlineStr">
+        <is>
+          <t>Falkenbergs</t>
+        </is>
+      </c>
+      <c r="E498" t="n">
+        <v>9.220000000000001</v>
+      </c>
+      <c r="F498" t="n">
+        <v>2.1</v>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" s="1" t="n">
+        <v>46258</v>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>Ostersunds FK</t>
+        </is>
+      </c>
+      <c r="D499" t="inlineStr">
+        <is>
+          <t>Ljungskile</t>
+        </is>
+      </c>
+      <c r="E499" t="n">
+        <v>10.55</v>
+      </c>
+      <c r="F499" t="n">
+        <v>1.36</v>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" s="1" t="n">
+        <v>46258</v>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>Varnamo</t>
+        </is>
+      </c>
+      <c r="D500" t="inlineStr">
+        <is>
+          <t>Landskrona</t>
+        </is>
+      </c>
+      <c r="E500" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="F500" t="n">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" s="1" t="n">
+        <v>46259</v>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>Atletico Goianiense</t>
+        </is>
+      </c>
+      <c r="D501" t="inlineStr">
+        <is>
+          <t>Botafogo SP</t>
+        </is>
+      </c>
+      <c r="E501" t="n">
+        <v>10.67</v>
+      </c>
+      <c r="F501" t="n">
+        <v>1.99</v>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" s="1" t="n">
+        <v>46259</v>
+      </c>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C502" t="inlineStr">
+        <is>
+          <t>Juventude</t>
+        </is>
+      </c>
+      <c r="D502" t="inlineStr">
+        <is>
+          <t>CRB</t>
+        </is>
+      </c>
+      <c r="E502" t="n">
+        <v>10.16</v>
+      </c>
+      <c r="F502" t="n">
+        <v>1.44</v>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" s="1" t="n">
+        <v>46259</v>
+      </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C503" t="inlineStr">
+        <is>
+          <t>Orebro SK</t>
+        </is>
+      </c>
+      <c r="D503" t="inlineStr">
+        <is>
+          <t>Varbergs BoIS</t>
+        </is>
+      </c>
+      <c r="E503" t="n">
+        <v>9.57</v>
+      </c>
+      <c r="F503" t="n">
+        <v>0.21</v>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" s="1" t="n">
+        <v>46259</v>
+      </c>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C504" t="inlineStr">
+        <is>
+          <t>Osters</t>
+        </is>
+      </c>
+      <c r="D504" t="inlineStr">
+        <is>
+          <t>Sundsvall</t>
+        </is>
+      </c>
+      <c r="E504" t="n">
+        <v>10.63</v>
+      </c>
+      <c r="F504" t="n">
+        <v>2.18</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily scrape output - 2026-08-23
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F504"/>
+  <dimension ref="A1:F510"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12461,7 +12461,7 @@
         <v>11.45</v>
       </c>
       <c r="F463" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="464">
@@ -12839,19 +12839,19 @@
       </c>
       <c r="C478" t="inlineStr">
         <is>
-          <t>Ponte Preta</t>
+          <t>Operario Ferroviario</t>
         </is>
       </c>
       <c r="D478" t="inlineStr">
         <is>
-          <t>Avai</t>
+          <t>Vila Nova</t>
         </is>
       </c>
       <c r="E478" t="n">
-        <v>9.1</v>
+        <v>10.29</v>
       </c>
       <c r="F478" t="n">
-        <v>0.39</v>
+        <v>0.93</v>
       </c>
     </row>
     <row r="479">
@@ -12865,19 +12865,19 @@
       </c>
       <c r="C479" t="inlineStr">
         <is>
-          <t>Sao Bernardo</t>
+          <t>Ponte Preta</t>
         </is>
       </c>
       <c r="D479" t="inlineStr">
         <is>
-          <t>Nautico</t>
+          <t>Avai</t>
         </is>
       </c>
       <c r="E479" t="n">
-        <v>10.56</v>
+        <v>9.07</v>
       </c>
       <c r="F479" t="n">
-        <v>0.89</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="480">
@@ -12886,24 +12886,24 @@
       </c>
       <c r="B480" t="inlineStr">
         <is>
-          <t>Finland - Veikkausliiga</t>
+          <t>Brazil - Serie B</t>
         </is>
       </c>
       <c r="C480" t="inlineStr">
         <is>
-          <t>HJK Helsinki</t>
+          <t>Sao Bernardo</t>
         </is>
       </c>
       <c r="D480" t="inlineStr">
         <is>
-          <t>Gnistan</t>
+          <t>Nautico</t>
         </is>
       </c>
       <c r="E480" t="n">
-        <v>10.87</v>
+        <v>10.56</v>
       </c>
       <c r="F480" t="n">
-        <v>2.23</v>
+        <v>0.89</v>
       </c>
     </row>
     <row r="481">
@@ -12917,19 +12917,19 @@
       </c>
       <c r="C481" t="inlineStr">
         <is>
-          <t>KuPS</t>
+          <t>HJK Helsinki</t>
         </is>
       </c>
       <c r="D481" t="inlineStr">
         <is>
-          <t>IFK Mariehamn</t>
+          <t>Gnistan</t>
         </is>
       </c>
       <c r="E481" t="n">
-        <v>10.57</v>
+        <v>10.82</v>
       </c>
       <c r="F481" t="n">
-        <v>4.27</v>
+        <v>2.34</v>
       </c>
     </row>
     <row r="482">
@@ -12943,19 +12943,19 @@
       </c>
       <c r="C482" t="inlineStr">
         <is>
-          <t>TPS</t>
+          <t>KuPS</t>
         </is>
       </c>
       <c r="D482" t="inlineStr">
         <is>
-          <t>Inter Turku</t>
+          <t>IFK Mariehamn</t>
         </is>
       </c>
       <c r="E482" t="n">
-        <v>9.970000000000001</v>
+        <v>10.57</v>
       </c>
       <c r="F482" t="n">
-        <v>-1.02</v>
+        <v>4.27</v>
       </c>
     </row>
     <row r="483">
@@ -12964,24 +12964,24 @@
       </c>
       <c r="B483" t="inlineStr">
         <is>
-          <t>Poland - 1st Liga</t>
+          <t>Finland - Veikkausliiga</t>
         </is>
       </c>
       <c r="C483" t="inlineStr">
         <is>
-          <t>LKS Lodz</t>
+          <t>TPS</t>
         </is>
       </c>
       <c r="D483" t="inlineStr">
         <is>
-          <t>Stal Mielec</t>
+          <t>Inter Turku</t>
         </is>
       </c>
       <c r="E483" t="n">
-        <v>10.98</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="F483" t="n">
-        <v>1.9</v>
+        <v>-1.02</v>
       </c>
     </row>
     <row r="484">
@@ -12990,24 +12990,24 @@
       </c>
       <c r="B484" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="C484" t="inlineStr">
         <is>
-          <t>GKS Katowice</t>
+          <t>LKS Lodz</t>
         </is>
       </c>
       <c r="D484" t="inlineStr">
         <is>
-          <t>Wisla Plock</t>
+          <t>Stal Mielec</t>
         </is>
       </c>
       <c r="E484" t="n">
-        <v>10.38</v>
+        <v>10.98</v>
       </c>
       <c r="F484" t="n">
-        <v>1.49</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="485">
@@ -13016,24 +13016,24 @@
       </c>
       <c r="B485" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="C485" t="inlineStr">
         <is>
-          <t>Radomiak Radom</t>
+          <t>Miedz Legnica</t>
         </is>
       </c>
       <c r="D485" t="inlineStr">
         <is>
-          <t>Zaglebie Lubin</t>
+          <t>Arka Gdynia</t>
         </is>
       </c>
       <c r="E485" t="n">
-        <v>10.32</v>
+        <v>10.68</v>
       </c>
       <c r="F485" t="n">
-        <v>1.34</v>
+        <v>0.66</v>
       </c>
     </row>
     <row r="486">
@@ -13042,24 +13042,24 @@
       </c>
       <c r="B486" t="inlineStr">
         <is>
-          <t>Romania - Liga 1</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="C486" t="inlineStr">
         <is>
-          <t>CFR Cluj</t>
+          <t>Puszcza Niepolomice</t>
         </is>
       </c>
       <c r="D486" t="inlineStr">
         <is>
-          <t>FCSB</t>
+          <t>Unia Skierniewice</t>
         </is>
       </c>
       <c r="E486" t="n">
-        <v>9.73</v>
+        <v>9.99</v>
       </c>
       <c r="F486" t="n">
-        <v>0.33</v>
+        <v>0.31</v>
       </c>
     </row>
     <row r="487">
@@ -13068,24 +13068,24 @@
       </c>
       <c r="B487" t="inlineStr">
         <is>
-          <t>Spain - Segunda</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C487" t="inlineStr">
         <is>
-          <t>Castellon</t>
+          <t>GKS Katowice</t>
         </is>
       </c>
       <c r="D487" t="inlineStr">
         <is>
-          <t>Sabadell</t>
+          <t>Wisla Plock</t>
         </is>
       </c>
       <c r="E487" t="n">
-        <v>9.33</v>
+        <v>10.38</v>
       </c>
       <c r="F487" t="n">
-        <v>2.44</v>
+        <v>1.49</v>
       </c>
     </row>
     <row r="488">
@@ -13094,24 +13094,24 @@
       </c>
       <c r="B488" t="inlineStr">
         <is>
-          <t>Spain - Segunda</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C488" t="inlineStr">
         <is>
-          <t>Eibar</t>
+          <t>Radomiak Radom</t>
         </is>
       </c>
       <c r="D488" t="inlineStr">
         <is>
-          <t>Real Valladolid</t>
+          <t>Zaglebie Lubin</t>
         </is>
       </c>
       <c r="E488" t="n">
-        <v>9.16</v>
+        <v>10.32</v>
       </c>
       <c r="F488" t="n">
-        <v>1.2</v>
+        <v>1.34</v>
       </c>
     </row>
     <row r="489">
@@ -13120,24 +13120,24 @@
       </c>
       <c r="B489" t="inlineStr">
         <is>
-          <t>Spain - Segunda</t>
+          <t>Romania - Liga 1</t>
         </is>
       </c>
       <c r="C489" t="inlineStr">
         <is>
-          <t>Tenerife</t>
+          <t>CFR Cluj</t>
         </is>
       </c>
       <c r="D489" t="inlineStr">
         <is>
-          <t>Almeria</t>
+          <t>FCSB</t>
         </is>
       </c>
       <c r="E489" t="n">
-        <v>9.460000000000001</v>
+        <v>9.84</v>
       </c>
       <c r="F489" t="n">
-        <v>0.02</v>
+        <v>0.33</v>
       </c>
     </row>
     <row r="490">
@@ -13146,24 +13146,24 @@
       </c>
       <c r="B490" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Romania - Liga 1</t>
         </is>
       </c>
       <c r="C490" t="inlineStr">
         <is>
-          <t>Brage</t>
+          <t>Sepsi</t>
         </is>
       </c>
       <c r="D490" t="inlineStr">
         <is>
-          <t>Nordic United</t>
+          <t>Farul Constanta</t>
         </is>
       </c>
       <c r="E490" t="n">
-        <v>9.359999999999999</v>
+        <v>9.32</v>
       </c>
       <c r="F490" t="n">
-        <v>0.53</v>
+        <v>0.32</v>
       </c>
     </row>
     <row r="491">
@@ -13172,24 +13172,24 @@
       </c>
       <c r="B491" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="C491" t="inlineStr">
         <is>
-          <t>Norrby</t>
+          <t>Castellon</t>
         </is>
       </c>
       <c r="D491" t="inlineStr">
         <is>
-          <t>Sandvikens IF</t>
+          <t>Sabadell</t>
         </is>
       </c>
       <c r="E491" t="n">
-        <v>9.51</v>
+        <v>9.33</v>
       </c>
       <c r="F491" t="n">
-        <v>0.55</v>
+        <v>2.44</v>
       </c>
     </row>
     <row r="492">
@@ -13198,154 +13198,154 @@
       </c>
       <c r="B492" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="C492" t="inlineStr">
         <is>
-          <t>Oddevold</t>
+          <t>Eibar</t>
         </is>
       </c>
       <c r="D492" t="inlineStr">
         <is>
-          <t>Helsingborgs</t>
+          <t>Real Valladolid</t>
         </is>
       </c>
       <c r="E492" t="n">
-        <v>8.789999999999999</v>
+        <v>8.890000000000001</v>
       </c>
       <c r="F492" t="n">
-        <v>1.49</v>
+        <v>1.21</v>
       </c>
     </row>
     <row r="493">
       <c r="A493" s="1" t="n">
-        <v>46258</v>
+        <v>46257</v>
       </c>
       <c r="B493" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="C493" t="inlineStr">
         <is>
-          <t>Athletic Club</t>
+          <t>Sporting Gijon</t>
         </is>
       </c>
       <c r="D493" t="inlineStr">
         <is>
-          <t>Gremio Novorizontino</t>
+          <t>Burgos</t>
         </is>
       </c>
       <c r="E493" t="n">
-        <v>10.18</v>
+        <v>9.31</v>
       </c>
       <c r="F493" t="n">
-        <v>0.2</v>
+        <v>0.96</v>
       </c>
     </row>
     <row r="494">
       <c r="A494" s="1" t="n">
-        <v>46258</v>
+        <v>46257</v>
       </c>
       <c r="B494" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="C494" t="inlineStr">
         <is>
-          <t>Sport Recife</t>
+          <t>Tenerife</t>
         </is>
       </c>
       <c r="D494" t="inlineStr">
         <is>
-          <t>America Mineiro</t>
+          <t>Almeria</t>
         </is>
       </c>
       <c r="E494" t="n">
-        <v>10.48</v>
+        <v>9.18</v>
       </c>
       <c r="F494" t="n">
-        <v>1.9</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="495">
       <c r="A495" s="1" t="n">
-        <v>46258</v>
+        <v>46257</v>
       </c>
       <c r="B495" t="inlineStr">
         <is>
-          <t>Poland - 1st Liga</t>
+          <t>Sweden - Superettan</t>
         </is>
       </c>
       <c r="C495" t="inlineStr">
         <is>
-          <t>Stal Rzeszow</t>
+          <t>Brage</t>
         </is>
       </c>
       <c r="D495" t="inlineStr">
         <is>
-          <t>Ruch Chorzow</t>
+          <t>Nordic United</t>
         </is>
       </c>
       <c r="E495" t="n">
-        <v>10.78</v>
+        <v>9.609999999999999</v>
       </c>
       <c r="F495" t="n">
-        <v>-0.34</v>
+        <v>0.51</v>
       </c>
     </row>
     <row r="496">
       <c r="A496" s="1" t="n">
-        <v>46258</v>
+        <v>46257</v>
       </c>
       <c r="B496" t="inlineStr">
         <is>
-          <t>Romania - Liga 1</t>
+          <t>Sweden - Superettan</t>
         </is>
       </c>
       <c r="C496" t="inlineStr">
         <is>
-          <t>Botosani</t>
+          <t>Norrby</t>
         </is>
       </c>
       <c r="D496" t="inlineStr">
         <is>
-          <t>Csikszereda</t>
+          <t>Sandvikens IF</t>
         </is>
       </c>
       <c r="E496" t="n">
         <v>9.720000000000001</v>
       </c>
       <c r="F496" t="n">
-        <v>2.51</v>
+        <v>0.42</v>
       </c>
     </row>
     <row r="497">
       <c r="A497" s="1" t="n">
-        <v>46258</v>
+        <v>46257</v>
       </c>
       <c r="B497" t="inlineStr">
         <is>
-          <t>Romania - Liga 1</t>
+          <t>Sweden - Superettan</t>
         </is>
       </c>
       <c r="C497" t="inlineStr">
         <is>
-          <t>Otelul Galati</t>
+          <t>Oddevold</t>
         </is>
       </c>
       <c r="D497" t="inlineStr">
         <is>
-          <t>Arges Pitesti</t>
+          <t>Helsingborgs</t>
         </is>
       </c>
       <c r="E497" t="n">
-        <v>9.539999999999999</v>
+        <v>8.789999999999999</v>
       </c>
       <c r="F497" t="n">
-        <v>0.45</v>
+        <v>1.49</v>
       </c>
     </row>
     <row r="498">
@@ -13354,24 +13354,24 @@
       </c>
       <c r="B498" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Brazil - Serie B</t>
         </is>
       </c>
       <c r="C498" t="inlineStr">
         <is>
-          <t>Norrkoping</t>
+          <t>Athletic Club</t>
         </is>
       </c>
       <c r="D498" t="inlineStr">
         <is>
-          <t>Falkenbergs</t>
+          <t>Gremio Novorizontino</t>
         </is>
       </c>
       <c r="E498" t="n">
-        <v>9.220000000000001</v>
+        <v>10.18</v>
       </c>
       <c r="F498" t="n">
-        <v>2.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="499">
@@ -13380,24 +13380,24 @@
       </c>
       <c r="B499" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Brazil - Serie B</t>
         </is>
       </c>
       <c r="C499" t="inlineStr">
         <is>
-          <t>Ostersunds FK</t>
+          <t>Sport Recife</t>
         </is>
       </c>
       <c r="D499" t="inlineStr">
         <is>
-          <t>Ljungskile</t>
+          <t>America Mineiro</t>
         </is>
       </c>
       <c r="E499" t="n">
-        <v>10.55</v>
+        <v>10.75</v>
       </c>
       <c r="F499" t="n">
-        <v>1.36</v>
+        <v>1.89</v>
       </c>
     </row>
     <row r="500">
@@ -13406,128 +13406,284 @@
       </c>
       <c r="B500" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="C500" t="inlineStr">
         <is>
-          <t>Varnamo</t>
+          <t>Stal Rzeszow</t>
         </is>
       </c>
       <c r="D500" t="inlineStr">
         <is>
-          <t>Landskrona</t>
+          <t>Ruch Chorzow</t>
         </is>
       </c>
       <c r="E500" t="n">
-        <v>9.6</v>
+        <v>10.84</v>
       </c>
       <c r="F500" t="n">
-        <v>0.18</v>
+        <v>-0.83</v>
       </c>
     </row>
     <row r="501">
       <c r="A501" s="1" t="n">
-        <v>46259</v>
+        <v>46258</v>
       </c>
       <c r="B501" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Romania - Liga 1</t>
         </is>
       </c>
       <c r="C501" t="inlineStr">
         <is>
-          <t>Atletico Goianiense</t>
+          <t>Botosani</t>
         </is>
       </c>
       <c r="D501" t="inlineStr">
         <is>
-          <t>Botafogo SP</t>
+          <t>Csikszereda</t>
         </is>
       </c>
       <c r="E501" t="n">
-        <v>10.67</v>
+        <v>9.720000000000001</v>
       </c>
       <c r="F501" t="n">
-        <v>1.99</v>
+        <v>2.51</v>
       </c>
     </row>
     <row r="502">
       <c r="A502" s="1" t="n">
-        <v>46259</v>
+        <v>46258</v>
       </c>
       <c r="B502" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Romania - Liga 1</t>
         </is>
       </c>
       <c r="C502" t="inlineStr">
         <is>
-          <t>Juventude</t>
+          <t>Otelul Galati</t>
         </is>
       </c>
       <c r="D502" t="inlineStr">
         <is>
-          <t>CRB</t>
+          <t>Arges Pitesti</t>
         </is>
       </c>
       <c r="E502" t="n">
-        <v>10.16</v>
+        <v>9.539999999999999</v>
       </c>
       <c r="F502" t="n">
-        <v>1.44</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="503">
       <c r="A503" s="1" t="n">
-        <v>46259</v>
+        <v>46258</v>
       </c>
       <c r="B503" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="C503" t="inlineStr">
         <is>
-          <t>Orebro SK</t>
+          <t>Celta Vigo II</t>
         </is>
       </c>
       <c r="D503" t="inlineStr">
         <is>
-          <t>Varbergs BoIS</t>
+          <t>FC Andorra</t>
         </is>
       </c>
       <c r="E503" t="n">
-        <v>9.57</v>
+        <v>8.359999999999999</v>
       </c>
       <c r="F503" t="n">
-        <v>0.21</v>
+        <v>-0.84</v>
       </c>
     </row>
     <row r="504">
       <c r="A504" s="1" t="n">
+        <v>46258</v>
+      </c>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C504" t="inlineStr">
+        <is>
+          <t>Norrkoping</t>
+        </is>
+      </c>
+      <c r="D504" t="inlineStr">
+        <is>
+          <t>Falkenbergs</t>
+        </is>
+      </c>
+      <c r="E504" t="n">
+        <v>9.220000000000001</v>
+      </c>
+      <c r="F504" t="n">
+        <v>2.1</v>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" s="1" t="n">
+        <v>46258</v>
+      </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C505" t="inlineStr">
+        <is>
+          <t>Ostersunds FK</t>
+        </is>
+      </c>
+      <c r="D505" t="inlineStr">
+        <is>
+          <t>Ljungskile</t>
+        </is>
+      </c>
+      <c r="E505" t="n">
+        <v>10.55</v>
+      </c>
+      <c r="F505" t="n">
+        <v>1.36</v>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" s="1" t="n">
+        <v>46258</v>
+      </c>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C506" t="inlineStr">
+        <is>
+          <t>Varnamo</t>
+        </is>
+      </c>
+      <c r="D506" t="inlineStr">
+        <is>
+          <t>Landskrona</t>
+        </is>
+      </c>
+      <c r="E506" t="n">
+        <v>9.57</v>
+      </c>
+      <c r="F506" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" s="1" t="n">
         <v>46259</v>
       </c>
-      <c r="B504" t="inlineStr">
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C507" t="inlineStr">
+        <is>
+          <t>Atletico Goianiense</t>
+        </is>
+      </c>
+      <c r="D507" t="inlineStr">
+        <is>
+          <t>Botafogo SP</t>
+        </is>
+      </c>
+      <c r="E507" t="n">
+        <v>10.67</v>
+      </c>
+      <c r="F507" t="n">
+        <v>1.99</v>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" s="1" t="n">
+        <v>46259</v>
+      </c>
+      <c r="B508" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C508" t="inlineStr">
+        <is>
+          <t>Juventude</t>
+        </is>
+      </c>
+      <c r="D508" t="inlineStr">
+        <is>
+          <t>CRB</t>
+        </is>
+      </c>
+      <c r="E508" t="n">
+        <v>10.16</v>
+      </c>
+      <c r="F508" t="n">
+        <v>1.44</v>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" s="1" t="n">
+        <v>46259</v>
+      </c>
+      <c r="B509" t="inlineStr">
         <is>
           <t>Sweden - Superettan</t>
         </is>
       </c>
-      <c r="C504" t="inlineStr">
+      <c r="C509" t="inlineStr">
+        <is>
+          <t>Orebro SK</t>
+        </is>
+      </c>
+      <c r="D509" t="inlineStr">
+        <is>
+          <t>Varbergs BoIS</t>
+        </is>
+      </c>
+      <c r="E509" t="n">
+        <v>9.57</v>
+      </c>
+      <c r="F509" t="n">
+        <v>0.21</v>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" s="1" t="n">
+        <v>46259</v>
+      </c>
+      <c r="B510" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C510" t="inlineStr">
         <is>
           <t>Osters</t>
         </is>
       </c>
-      <c r="D504" t="inlineStr">
+      <c r="D510" t="inlineStr">
         <is>
           <t>Sundsvall</t>
         </is>
       </c>
-      <c r="E504" t="n">
-        <v>10.63</v>
-      </c>
-      <c r="F504" t="n">
-        <v>2.18</v>
+      <c r="E510" t="n">
+        <v>10.33</v>
+      </c>
+      <c r="F510" t="n">
+        <v>2.07</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily scrape output - 2026-08-24
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F510"/>
+  <dimension ref="A1:F511"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13368,10 +13368,10 @@
         </is>
       </c>
       <c r="E498" t="n">
-        <v>10.18</v>
+        <v>10.22</v>
       </c>
       <c r="F498" t="n">
-        <v>0.2</v>
+        <v>-0.11</v>
       </c>
     </row>
     <row r="499">
@@ -13394,10 +13394,10 @@
         </is>
       </c>
       <c r="E499" t="n">
-        <v>10.75</v>
+        <v>10.7</v>
       </c>
       <c r="F499" t="n">
-        <v>1.89</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="500">
@@ -13420,7 +13420,7 @@
         </is>
       </c>
       <c r="E500" t="n">
-        <v>10.84</v>
+        <v>10.96</v>
       </c>
       <c r="F500" t="n">
         <v>-0.83</v>
@@ -13498,10 +13498,10 @@
         </is>
       </c>
       <c r="E503" t="n">
-        <v>8.359999999999999</v>
+        <v>8.23</v>
       </c>
       <c r="F503" t="n">
-        <v>-0.84</v>
+        <v>-1.01</v>
       </c>
     </row>
     <row r="504">
@@ -13510,24 +13510,24 @@
       </c>
       <c r="B504" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="C504" t="inlineStr">
         <is>
-          <t>Norrkoping</t>
+          <t>Granada</t>
         </is>
       </c>
       <c r="D504" t="inlineStr">
         <is>
-          <t>Falkenbergs</t>
+          <t>Mallorca</t>
         </is>
       </c>
       <c r="E504" t="n">
-        <v>9.220000000000001</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="F504" t="n">
-        <v>2.1</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="505">
@@ -13541,19 +13541,19 @@
       </c>
       <c r="C505" t="inlineStr">
         <is>
-          <t>Ostersunds FK</t>
+          <t>Norrkoping</t>
         </is>
       </c>
       <c r="D505" t="inlineStr">
         <is>
-          <t>Ljungskile</t>
+          <t>Falkenbergs</t>
         </is>
       </c>
       <c r="E505" t="n">
-        <v>10.55</v>
+        <v>9.220000000000001</v>
       </c>
       <c r="F505" t="n">
-        <v>1.36</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="506">
@@ -13567,45 +13567,45 @@
       </c>
       <c r="C506" t="inlineStr">
         <is>
-          <t>Varnamo</t>
+          <t>Ostersunds FK</t>
         </is>
       </c>
       <c r="D506" t="inlineStr">
         <is>
-          <t>Landskrona</t>
+          <t>Ljungskile</t>
         </is>
       </c>
       <c r="E506" t="n">
-        <v>9.57</v>
+        <v>10.55</v>
       </c>
       <c r="F506" t="n">
-        <v>0.4</v>
+        <v>1.36</v>
       </c>
     </row>
     <row r="507">
       <c r="A507" s="1" t="n">
-        <v>46259</v>
+        <v>46258</v>
       </c>
       <c r="B507" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Sweden - Superettan</t>
         </is>
       </c>
       <c r="C507" t="inlineStr">
         <is>
-          <t>Atletico Goianiense</t>
+          <t>Varnamo</t>
         </is>
       </c>
       <c r="D507" t="inlineStr">
         <is>
-          <t>Botafogo SP</t>
+          <t>Landskrona</t>
         </is>
       </c>
       <c r="E507" t="n">
-        <v>10.67</v>
+        <v>9.57</v>
       </c>
       <c r="F507" t="n">
-        <v>1.99</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="508">
@@ -13619,19 +13619,19 @@
       </c>
       <c r="C508" t="inlineStr">
         <is>
-          <t>Juventude</t>
+          <t>Atletico Goianiense</t>
         </is>
       </c>
       <c r="D508" t="inlineStr">
         <is>
-          <t>CRB</t>
+          <t>Botafogo SP</t>
         </is>
       </c>
       <c r="E508" t="n">
-        <v>10.16</v>
+        <v>10.67</v>
       </c>
       <c r="F508" t="n">
-        <v>1.44</v>
+        <v>1.99</v>
       </c>
     </row>
     <row r="509">
@@ -13640,24 +13640,24 @@
       </c>
       <c r="B509" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Brazil - Serie B</t>
         </is>
       </c>
       <c r="C509" t="inlineStr">
         <is>
-          <t>Orebro SK</t>
+          <t>Juventude</t>
         </is>
       </c>
       <c r="D509" t="inlineStr">
         <is>
-          <t>Varbergs BoIS</t>
+          <t>CRB</t>
         </is>
       </c>
       <c r="E509" t="n">
-        <v>9.57</v>
+        <v>10.15</v>
       </c>
       <c r="F509" t="n">
-        <v>0.21</v>
+        <v>1.44</v>
       </c>
     </row>
     <row r="510">
@@ -13671,18 +13671,44 @@
       </c>
       <c r="C510" t="inlineStr">
         <is>
+          <t>Orebro SK</t>
+        </is>
+      </c>
+      <c r="D510" t="inlineStr">
+        <is>
+          <t>Varbergs BoIS</t>
+        </is>
+      </c>
+      <c r="E510" t="n">
+        <v>9.57</v>
+      </c>
+      <c r="F510" t="n">
+        <v>0.21</v>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" s="1" t="n">
+        <v>46259</v>
+      </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C511" t="inlineStr">
+        <is>
           <t>Osters</t>
         </is>
       </c>
-      <c r="D510" t="inlineStr">
+      <c r="D511" t="inlineStr">
         <is>
           <t>Sundsvall</t>
         </is>
       </c>
-      <c r="E510" t="n">
+      <c r="E511" t="n">
         <v>10.33</v>
       </c>
-      <c r="F510" t="n">
+      <c r="F511" t="n">
         <v>2.07</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily scrape output - 2026-08-25
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -13628,10 +13628,10 @@
         </is>
       </c>
       <c r="E508" t="n">
-        <v>10.67</v>
+        <v>10.36</v>
       </c>
       <c r="F508" t="n">
-        <v>1.99</v>
+        <v>1.83</v>
       </c>
     </row>
     <row r="509">
@@ -13654,10 +13654,10 @@
         </is>
       </c>
       <c r="E509" t="n">
-        <v>10.15</v>
+        <v>9.73</v>
       </c>
       <c r="F509" t="n">
-        <v>1.44</v>
+        <v>1.46</v>
       </c>
     </row>
     <row r="510">
@@ -13706,7 +13706,7 @@
         </is>
       </c>
       <c r="E511" t="n">
-        <v>10.33</v>
+        <v>10.49</v>
       </c>
       <c r="F511" t="n">
         <v>2.07</v>

</xml_diff>

<commit_message>
Daily scrape output - 2026-08-26
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F511"/>
+  <dimension ref="A1:F518"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13712,6 +13712,188 @@
         <v>2.07</v>
       </c>
     </row>
+    <row r="512">
+      <c r="A512" s="1" t="n">
+        <v>46260</v>
+      </c>
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C512" t="inlineStr">
+        <is>
+          <t>Asane Fotball</t>
+        </is>
+      </c>
+      <c r="D512" t="inlineStr">
+        <is>
+          <t>Lyn</t>
+        </is>
+      </c>
+      <c r="E512" t="n">
+        <v>11.68</v>
+      </c>
+      <c r="F512" t="n">
+        <v>-1.57</v>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" s="1" t="n">
+        <v>46260</v>
+      </c>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C513" t="inlineStr">
+        <is>
+          <t>Haugesund</t>
+        </is>
+      </c>
+      <c r="D513" t="inlineStr">
+        <is>
+          <t>Egersunds</t>
+        </is>
+      </c>
+      <c r="E513" t="n">
+        <v>11.09</v>
+      </c>
+      <c r="F513" t="n">
+        <v>1.52</v>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" s="1" t="n">
+        <v>46260</v>
+      </c>
+      <c r="B514" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C514" t="inlineStr">
+        <is>
+          <t>Moss</t>
+        </is>
+      </c>
+      <c r="D514" t="inlineStr">
+        <is>
+          <t>Sogndal</t>
+        </is>
+      </c>
+      <c r="E514" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="F514" t="n">
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" s="1" t="n">
+        <v>46260</v>
+      </c>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C515" t="inlineStr">
+        <is>
+          <t>Odd BK</t>
+        </is>
+      </c>
+      <c r="D515" t="inlineStr">
+        <is>
+          <t>Kongsvinger</t>
+        </is>
+      </c>
+      <c r="E515" t="n">
+        <v>11.04</v>
+      </c>
+      <c r="F515" t="n">
+        <v>0.55</v>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" s="1" t="n">
+        <v>46260</v>
+      </c>
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C516" t="inlineStr">
+        <is>
+          <t>Stabaek</t>
+        </is>
+      </c>
+      <c r="D516" t="inlineStr">
+        <is>
+          <t>Ranheim</t>
+        </is>
+      </c>
+      <c r="E516" t="n">
+        <v>11.24</v>
+      </c>
+      <c r="F516" t="n">
+        <v>2.66</v>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" s="1" t="n">
+        <v>46260</v>
+      </c>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C517" t="inlineStr">
+        <is>
+          <t>Strommen</t>
+        </is>
+      </c>
+      <c r="D517" t="inlineStr">
+        <is>
+          <t>Raufoss</t>
+        </is>
+      </c>
+      <c r="E517" t="n">
+        <v>10.63</v>
+      </c>
+      <c r="F517" t="n">
+        <v>0.85</v>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" s="1" t="n">
+        <v>46260</v>
+      </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C518" t="inlineStr">
+        <is>
+          <t>Stromsgodset</t>
+        </is>
+      </c>
+      <c r="D518" t="inlineStr">
+        <is>
+          <t>Hodd</t>
+        </is>
+      </c>
+      <c r="E518" t="n">
+        <v>11.66</v>
+      </c>
+      <c r="F518" t="n">
+        <v>4.89</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily scrape output - 2026-08-27
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F518"/>
+  <dimension ref="A1:F522"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13894,6 +13894,110 @@
         <v>4.89</v>
       </c>
     </row>
+    <row r="519">
+      <c r="A519" s="1" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>Finland - Ykkosliiga</t>
+        </is>
+      </c>
+      <c r="C519" t="inlineStr">
+        <is>
+          <t>JaPS</t>
+        </is>
+      </c>
+      <c r="D519" t="inlineStr">
+        <is>
+          <t>KaPa</t>
+        </is>
+      </c>
+      <c r="E519" t="n">
+        <v>10.51</v>
+      </c>
+      <c r="F519" t="n">
+        <v>0.82</v>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" s="1" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B520" t="inlineStr">
+        <is>
+          <t>Finland - Ykkosliiga</t>
+        </is>
+      </c>
+      <c r="C520" t="inlineStr">
+        <is>
+          <t>KTP</t>
+        </is>
+      </c>
+      <c r="D520" t="inlineStr">
+        <is>
+          <t>FC Haka</t>
+        </is>
+      </c>
+      <c r="E520" t="n">
+        <v>10.62</v>
+      </c>
+      <c r="F520" t="n">
+        <v>-0.04</v>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" s="1" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B521" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C521" t="inlineStr">
+        <is>
+          <t>Wisla Plock</t>
+        </is>
+      </c>
+      <c r="D521" t="inlineStr">
+        <is>
+          <t>Korona Kielce</t>
+        </is>
+      </c>
+      <c r="E521" t="n">
+        <v>10.22</v>
+      </c>
+      <c r="F521" t="n">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" s="1" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B522" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C522" t="inlineStr">
+        <is>
+          <t>Tenerife</t>
+        </is>
+      </c>
+      <c r="D522" t="inlineStr">
+        <is>
+          <t>Sporting Gijon</t>
+        </is>
+      </c>
+      <c r="E522" t="n">
+        <v>9.550000000000001</v>
+      </c>
+      <c r="F522" t="n">
+        <v>1.13</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily scrape output - 2026-08-28
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F522"/>
+  <dimension ref="A1:F574"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13900,24 +13900,24 @@
       </c>
       <c r="B519" t="inlineStr">
         <is>
-          <t>Finland - Ykkosliiga</t>
+          <t>Brazil - Serie B</t>
         </is>
       </c>
       <c r="C519" t="inlineStr">
         <is>
-          <t>JaPS</t>
+          <t>Goias</t>
         </is>
       </c>
       <c r="D519" t="inlineStr">
         <is>
-          <t>KaPa</t>
+          <t>Sao Bernardo</t>
         </is>
       </c>
       <c r="E519" t="n">
-        <v>10.51</v>
+        <v>10.72</v>
       </c>
       <c r="F519" t="n">
-        <v>0.82</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="520">
@@ -13926,24 +13926,24 @@
       </c>
       <c r="B520" t="inlineStr">
         <is>
-          <t>Finland - Ykkosliiga</t>
+          <t>Brazil - Serie B</t>
         </is>
       </c>
       <c r="C520" t="inlineStr">
         <is>
-          <t>KTP</t>
+          <t>Gremio Novorizontino</t>
         </is>
       </c>
       <c r="D520" t="inlineStr">
         <is>
-          <t>FC Haka</t>
+          <t>Sport Recife</t>
         </is>
       </c>
       <c r="E520" t="n">
-        <v>10.62</v>
+        <v>11</v>
       </c>
       <c r="F520" t="n">
-        <v>-0.04</v>
+        <v>2.38</v>
       </c>
     </row>
     <row r="521">
@@ -13952,24 +13952,24 @@
       </c>
       <c r="B521" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Brazil - Serie B</t>
         </is>
       </c>
       <c r="C521" t="inlineStr">
         <is>
-          <t>Wisla Plock</t>
+          <t>Nautico</t>
         </is>
       </c>
       <c r="D521" t="inlineStr">
         <is>
-          <t>Korona Kielce</t>
+          <t>Athletic Club</t>
         </is>
       </c>
       <c r="E521" t="n">
-        <v>10.22</v>
+        <v>10.52</v>
       </c>
       <c r="F521" t="n">
-        <v>0.12</v>
+        <v>1.94</v>
       </c>
     </row>
     <row r="522">
@@ -13978,24 +13978,1376 @@
       </c>
       <c r="B522" t="inlineStr">
         <is>
+          <t>Finland - Ykkosliiga</t>
+        </is>
+      </c>
+      <c r="C522" t="inlineStr">
+        <is>
+          <t>JaPS</t>
+        </is>
+      </c>
+      <c r="D522" t="inlineStr">
+        <is>
+          <t>KaPa</t>
+        </is>
+      </c>
+      <c r="E522" t="n">
+        <v>10.51</v>
+      </c>
+      <c r="F522" t="n">
+        <v>0.82</v>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" s="1" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B523" t="inlineStr">
+        <is>
+          <t>Finland - Ykkosliiga</t>
+        </is>
+      </c>
+      <c r="C523" t="inlineStr">
+        <is>
+          <t>KTP</t>
+        </is>
+      </c>
+      <c r="D523" t="inlineStr">
+        <is>
+          <t>FC Haka</t>
+        </is>
+      </c>
+      <c r="E523" t="n">
+        <v>10.62</v>
+      </c>
+      <c r="F523" t="n">
+        <v>-0.04</v>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" s="1" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B524" t="inlineStr">
+        <is>
+          <t>Iceland - 1. Deild</t>
+        </is>
+      </c>
+      <c r="C524" t="inlineStr">
+        <is>
+          <t>Throttur Reykjavik</t>
+        </is>
+      </c>
+      <c r="D524" t="inlineStr">
+        <is>
+          <t>Aegir</t>
+        </is>
+      </c>
+      <c r="E524" t="n">
+        <v>11.87</v>
+      </c>
+      <c r="F524" t="n">
+        <v>6.07</v>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" s="1" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B525" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C525" t="inlineStr">
+        <is>
+          <t>Odra Opole</t>
+        </is>
+      </c>
+      <c r="D525" t="inlineStr">
+        <is>
+          <t>LKS Lodz</t>
+        </is>
+      </c>
+      <c r="E525" t="n">
+        <v>10.57</v>
+      </c>
+      <c r="F525" t="n">
+        <v>-0.47</v>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" s="1" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B526" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C526" t="inlineStr">
+        <is>
+          <t>Legia Warsaw</t>
+        </is>
+      </c>
+      <c r="D526" t="inlineStr">
+        <is>
+          <t>Slask Wroclaw</t>
+        </is>
+      </c>
+      <c r="E526" t="n">
+        <v>10.07</v>
+      </c>
+      <c r="F526" t="n">
+        <v>2.71</v>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" s="1" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B527" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C527" t="inlineStr">
+        <is>
+          <t>Wisla Plock</t>
+        </is>
+      </c>
+      <c r="D527" t="inlineStr">
+        <is>
+          <t>Korona Kielce</t>
+        </is>
+      </c>
+      <c r="E527" t="n">
+        <v>10.22</v>
+      </c>
+      <c r="F527" t="n">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" s="1" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B528" t="inlineStr">
+        <is>
           <t>Spain - Segunda</t>
         </is>
       </c>
-      <c r="C522" t="inlineStr">
+      <c r="C528" t="inlineStr">
         <is>
           <t>Tenerife</t>
         </is>
       </c>
-      <c r="D522" t="inlineStr">
+      <c r="D528" t="inlineStr">
         <is>
           <t>Sporting Gijon</t>
         </is>
       </c>
-      <c r="E522" t="n">
-        <v>9.550000000000001</v>
-      </c>
-      <c r="F522" t="n">
+      <c r="E528" t="n">
+        <v>9.56</v>
+      </c>
+      <c r="F528" t="n">
         <v>1.13</v>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" s="1" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B529" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C529" t="inlineStr">
+        <is>
+          <t>Botafogo SP</t>
+        </is>
+      </c>
+      <c r="D529" t="inlineStr">
+        <is>
+          <t>Cuiaba</t>
+        </is>
+      </c>
+      <c r="E529" t="n">
+        <v>10.64</v>
+      </c>
+      <c r="F529" t="n">
+        <v>0.85</v>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" s="1" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B530" t="inlineStr">
+        <is>
+          <t>Finland - Ykkosliiga</t>
+        </is>
+      </c>
+      <c r="C530" t="inlineStr">
+        <is>
+          <t>EIF</t>
+        </is>
+      </c>
+      <c r="D530" t="inlineStr">
+        <is>
+          <t>JIPPO</t>
+        </is>
+      </c>
+      <c r="E530" t="n">
+        <v>10.07</v>
+      </c>
+      <c r="F530" t="n">
+        <v>-1.13</v>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" s="1" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B531" t="inlineStr">
+        <is>
+          <t>Finland - Ykkosliiga</t>
+        </is>
+      </c>
+      <c r="C531" t="inlineStr">
+        <is>
+          <t>Mikkelin Palloilijat</t>
+        </is>
+      </c>
+      <c r="D531" t="inlineStr">
+        <is>
+          <t>PK-35</t>
+        </is>
+      </c>
+      <c r="E531" t="n">
+        <v>10.21</v>
+      </c>
+      <c r="F531" t="n">
+        <v>-1.41</v>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" s="1" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B532" t="inlineStr">
+        <is>
+          <t>Iceland - 1. Deild</t>
+        </is>
+      </c>
+      <c r="C532" t="inlineStr">
+        <is>
+          <t>Leiknir Reykjavik</t>
+        </is>
+      </c>
+      <c r="D532" t="inlineStr">
+        <is>
+          <t>UMF Njardvik</t>
+        </is>
+      </c>
+      <c r="E532" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="F532" t="n">
+        <v>-1.19</v>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" s="1" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B533" t="inlineStr">
+        <is>
+          <t>Iceland - 1. Deild</t>
+        </is>
+      </c>
+      <c r="C533" t="inlineStr">
+        <is>
+          <t>UMF Grindavik</t>
+        </is>
+      </c>
+      <c r="D533" t="inlineStr">
+        <is>
+          <t>HK Kopavogur</t>
+        </is>
+      </c>
+      <c r="E533" t="n">
+        <v>11.53</v>
+      </c>
+      <c r="F533" t="n">
+        <v>-1.48</v>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" s="1" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B534" t="inlineStr">
+        <is>
+          <t>Iceland - 1. Deild</t>
+        </is>
+      </c>
+      <c r="C534" t="inlineStr">
+        <is>
+          <t>Volsungur</t>
+        </is>
+      </c>
+      <c r="D534" t="inlineStr">
+        <is>
+          <t>IR Reykjavik</t>
+        </is>
+      </c>
+      <c r="E534" t="n">
+        <v>11.65</v>
+      </c>
+      <c r="F534" t="n">
+        <v>-1.48</v>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" s="1" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B535" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C535" t="inlineStr">
+        <is>
+          <t>Bryne</t>
+        </is>
+      </c>
+      <c r="D535" t="inlineStr">
+        <is>
+          <t>Haugesund</t>
+        </is>
+      </c>
+      <c r="E535" t="n">
+        <v>10.63</v>
+      </c>
+      <c r="F535" t="n">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" s="1" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B536" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C536" t="inlineStr">
+        <is>
+          <t>Pogon Siedlce</t>
+        </is>
+      </c>
+      <c r="D536" t="inlineStr">
+        <is>
+          <t>Stal Mielec</t>
+        </is>
+      </c>
+      <c r="E536" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="F536" t="n">
+        <v>-0.86</v>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" s="1" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B537" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C537" t="inlineStr">
+        <is>
+          <t>Motor Lublin</t>
+        </is>
+      </c>
+      <c r="D537" t="inlineStr">
+        <is>
+          <t>Piast Gliwice</t>
+        </is>
+      </c>
+      <c r="E537" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="F537" t="n">
+        <v>0.48</v>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" s="1" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B538" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C538" t="inlineStr">
+        <is>
+          <t>Radomiak Radom</t>
+        </is>
+      </c>
+      <c r="D538" t="inlineStr">
+        <is>
+          <t>Cracovia Krakow</t>
+        </is>
+      </c>
+      <c r="E538" t="n">
+        <v>9.74</v>
+      </c>
+      <c r="F538" t="n">
+        <v>-0.59</v>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" s="1" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B539" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C539" t="inlineStr">
+        <is>
+          <t>Zaglebie Lubin</t>
+        </is>
+      </c>
+      <c r="D539" t="inlineStr">
+        <is>
+          <t>Pogon Szczecin</t>
+        </is>
+      </c>
+      <c r="E539" t="n">
+        <v>10.38</v>
+      </c>
+      <c r="F539" t="n">
+        <v>-0.35</v>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" s="1" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B540" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C540" t="inlineStr">
+        <is>
+          <t>Csikszereda</t>
+        </is>
+      </c>
+      <c r="D540" t="inlineStr">
+        <is>
+          <t>CFR Cluj</t>
+        </is>
+      </c>
+      <c r="E540" t="n">
+        <v>9.66</v>
+      </c>
+      <c r="F540" t="n">
+        <v>-1.54</v>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" s="1" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B541" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C541" t="inlineStr">
+        <is>
+          <t>Falkenbergs</t>
+        </is>
+      </c>
+      <c r="D541" t="inlineStr">
+        <is>
+          <t>Brage</t>
+        </is>
+      </c>
+      <c r="E541" t="n">
+        <v>10.07</v>
+      </c>
+      <c r="F541" t="n">
+        <v>0.52</v>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" s="1" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B542" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C542" t="inlineStr">
+        <is>
+          <t>Landskrona</t>
+        </is>
+      </c>
+      <c r="D542" t="inlineStr">
+        <is>
+          <t>Ostersunds FK</t>
+        </is>
+      </c>
+      <c r="E542" t="n">
+        <v>10.01</v>
+      </c>
+      <c r="F542" t="n">
+        <v>0.42</v>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" s="1" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B543" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C543" t="inlineStr">
+        <is>
+          <t>Ljungskile</t>
+        </is>
+      </c>
+      <c r="D543" t="inlineStr">
+        <is>
+          <t>Varnamo</t>
+        </is>
+      </c>
+      <c r="E543" t="n">
+        <v>10.61</v>
+      </c>
+      <c r="F543" t="n">
+        <v>1.11</v>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" s="1" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B544" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C544" t="inlineStr">
+        <is>
+          <t>Nordic United</t>
+        </is>
+      </c>
+      <c r="D544" t="inlineStr">
+        <is>
+          <t>Norrkoping</t>
+        </is>
+      </c>
+      <c r="E544" t="n">
+        <v>10.05</v>
+      </c>
+      <c r="F544" t="n">
+        <v>-0.49</v>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" s="1" t="n">
+        <v>46264</v>
+      </c>
+      <c r="B545" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C545" t="inlineStr">
+        <is>
+          <t>America Mineiro</t>
+        </is>
+      </c>
+      <c r="D545" t="inlineStr">
+        <is>
+          <t>Ponte Preta</t>
+        </is>
+      </c>
+      <c r="E545" t="n">
+        <v>10.45</v>
+      </c>
+      <c r="F545" t="n">
+        <v>2.45</v>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" s="1" t="n">
+        <v>46264</v>
+      </c>
+      <c r="B546" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C546" t="inlineStr">
+        <is>
+          <t>Avai</t>
+        </is>
+      </c>
+      <c r="D546" t="inlineStr">
+        <is>
+          <t>Atletico Goianiense</t>
+        </is>
+      </c>
+      <c r="E546" t="n">
+        <v>10.16</v>
+      </c>
+      <c r="F546" t="n">
+        <v>0.31</v>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" s="1" t="n">
+        <v>46264</v>
+      </c>
+      <c r="B547" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C547" t="inlineStr">
+        <is>
+          <t>CRB</t>
+        </is>
+      </c>
+      <c r="D547" t="inlineStr">
+        <is>
+          <t>Criciuma</t>
+        </is>
+      </c>
+      <c r="E547" t="n">
+        <v>10.51</v>
+      </c>
+      <c r="F547" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" s="1" t="n">
+        <v>46264</v>
+      </c>
+      <c r="B548" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C548" t="inlineStr">
+        <is>
+          <t>Vila Nova</t>
+        </is>
+      </c>
+      <c r="D548" t="inlineStr">
+        <is>
+          <t>Ceara</t>
+        </is>
+      </c>
+      <c r="E548" t="n">
+        <v>10.49</v>
+      </c>
+      <c r="F548" t="n">
+        <v>1.45</v>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" s="1" t="n">
+        <v>46264</v>
+      </c>
+      <c r="B549" t="inlineStr">
+        <is>
+          <t>Finland - Ykkosliiga</t>
+        </is>
+      </c>
+      <c r="C549" t="inlineStr">
+        <is>
+          <t>SJK Akatemia</t>
+        </is>
+      </c>
+      <c r="D549" t="inlineStr">
+        <is>
+          <t>HJK Klubi 04</t>
+        </is>
+      </c>
+      <c r="E549" t="n">
+        <v>10.22</v>
+      </c>
+      <c r="F549" t="n">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" s="1" t="n">
+        <v>46264</v>
+      </c>
+      <c r="B550" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C550" t="inlineStr">
+        <is>
+          <t>Egersunds</t>
+        </is>
+      </c>
+      <c r="D550" t="inlineStr">
+        <is>
+          <t>Asane Fotball</t>
+        </is>
+      </c>
+      <c r="E550" t="n">
+        <v>11.06</v>
+      </c>
+      <c r="F550" t="n">
+        <v>2.95</v>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" s="1" t="n">
+        <v>46264</v>
+      </c>
+      <c r="B551" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C551" t="inlineStr">
+        <is>
+          <t>Hodd</t>
+        </is>
+      </c>
+      <c r="D551" t="inlineStr">
+        <is>
+          <t>Stabaek</t>
+        </is>
+      </c>
+      <c r="E551" t="n">
+        <v>11.34</v>
+      </c>
+      <c r="F551" t="n">
+        <v>-3.03</v>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" s="1" t="n">
+        <v>46264</v>
+      </c>
+      <c r="B552" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C552" t="inlineStr">
+        <is>
+          <t>Kongsvinger</t>
+        </is>
+      </c>
+      <c r="D552" t="inlineStr">
+        <is>
+          <t>Lyn</t>
+        </is>
+      </c>
+      <c r="E552" t="n">
+        <v>11.06</v>
+      </c>
+      <c r="F552" t="n">
+        <v>1.71</v>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" s="1" t="n">
+        <v>46264</v>
+      </c>
+      <c r="B553" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C553" t="inlineStr">
+        <is>
+          <t>Moss</t>
+        </is>
+      </c>
+      <c r="D553" t="inlineStr">
+        <is>
+          <t>Strommen</t>
+        </is>
+      </c>
+      <c r="E553" t="n">
+        <v>10.55</v>
+      </c>
+      <c r="F553" t="n">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" s="1" t="n">
+        <v>46264</v>
+      </c>
+      <c r="B554" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C554" t="inlineStr">
+        <is>
+          <t>Ranheim</t>
+        </is>
+      </c>
+      <c r="D554" t="inlineStr">
+        <is>
+          <t>Odd BK</t>
+        </is>
+      </c>
+      <c r="E554" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="F554" t="n">
+        <v>-0.36</v>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" s="1" t="n">
+        <v>46264</v>
+      </c>
+      <c r="B555" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C555" t="inlineStr">
+        <is>
+          <t>Raufoss</t>
+        </is>
+      </c>
+      <c r="D555" t="inlineStr">
+        <is>
+          <t>Sandnes Ulf</t>
+        </is>
+      </c>
+      <c r="E555" t="n">
+        <v>10.98</v>
+      </c>
+      <c r="F555" t="n">
+        <v>-0.2</v>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" s="1" t="n">
+        <v>46264</v>
+      </c>
+      <c r="B556" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C556" t="inlineStr">
+        <is>
+          <t>Sogndal</t>
+        </is>
+      </c>
+      <c r="D556" t="inlineStr">
+        <is>
+          <t>Stromsgodset</t>
+        </is>
+      </c>
+      <c r="E556" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="F556" t="n">
+        <v>-2.6</v>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" s="1" t="n">
+        <v>46264</v>
+      </c>
+      <c r="B557" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C557" t="inlineStr">
+        <is>
+          <t>Chrobry Glogow</t>
+        </is>
+      </c>
+      <c r="D557" t="inlineStr">
+        <is>
+          <t>Ruch Chorzow</t>
+        </is>
+      </c>
+      <c r="E557" t="n">
+        <v>10.82</v>
+      </c>
+      <c r="F557" t="n">
+        <v>-0.54</v>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" s="1" t="n">
+        <v>46264</v>
+      </c>
+      <c r="B558" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C558" t="inlineStr">
+        <is>
+          <t>Gornik Zabrze</t>
+        </is>
+      </c>
+      <c r="D558" t="inlineStr">
+        <is>
+          <t>GKS Katowice</t>
+        </is>
+      </c>
+      <c r="E558" t="n">
+        <v>10.36</v>
+      </c>
+      <c r="F558" t="n">
+        <v>2.4</v>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" s="1" t="n">
+        <v>46264</v>
+      </c>
+      <c r="B559" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C559" t="inlineStr">
+        <is>
+          <t>Rakow Czestochowa</t>
+        </is>
+      </c>
+      <c r="D559" t="inlineStr">
+        <is>
+          <t>Jagiellonia Bialystok</t>
+        </is>
+      </c>
+      <c r="E559" t="n">
+        <v>9.67</v>
+      </c>
+      <c r="F559" t="n">
+        <v>0.53</v>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" s="1" t="n">
+        <v>46264</v>
+      </c>
+      <c r="B560" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C560" t="inlineStr">
+        <is>
+          <t>Widzew Lodz</t>
+        </is>
+      </c>
+      <c r="D560" t="inlineStr">
+        <is>
+          <t>Lech Poznan</t>
+        </is>
+      </c>
+      <c r="E560" t="n">
+        <v>10.14</v>
+      </c>
+      <c r="F560" t="n">
+        <v>-0.65</v>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" s="1" t="n">
+        <v>46264</v>
+      </c>
+      <c r="B561" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C561" t="inlineStr">
+        <is>
+          <t>FCSB</t>
+        </is>
+      </c>
+      <c r="D561" t="inlineStr">
+        <is>
+          <t>UTA Arad</t>
+        </is>
+      </c>
+      <c r="E561" t="n">
+        <v>10.01</v>
+      </c>
+      <c r="F561" t="n">
+        <v>2.61</v>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" s="1" t="n">
+        <v>46264</v>
+      </c>
+      <c r="B562" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C562" t="inlineStr">
+        <is>
+          <t>Farul Constanta</t>
+        </is>
+      </c>
+      <c r="D562" t="inlineStr">
+        <is>
+          <t>Botosani</t>
+        </is>
+      </c>
+      <c r="E562" t="n">
+        <v>9.25</v>
+      </c>
+      <c r="F562" t="n">
+        <v>1.36</v>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" s="1" t="n">
+        <v>46264</v>
+      </c>
+      <c r="B563" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C563" t="inlineStr">
+        <is>
+          <t>Cordoba</t>
+        </is>
+      </c>
+      <c r="D563" t="inlineStr">
+        <is>
+          <t>Granada</t>
+        </is>
+      </c>
+      <c r="E563" t="n">
+        <v>9.859999999999999</v>
+      </c>
+      <c r="F563" t="n">
+        <v>1.98</v>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" s="1" t="n">
+        <v>46264</v>
+      </c>
+      <c r="B564" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C564" t="inlineStr">
+        <is>
+          <t>FC Andorra</t>
+        </is>
+      </c>
+      <c r="D564" t="inlineStr">
+        <is>
+          <t>Eibar</t>
+        </is>
+      </c>
+      <c r="E564" t="n">
+        <v>9.15</v>
+      </c>
+      <c r="F564" t="n">
+        <v>1.44</v>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" s="1" t="n">
+        <v>46264</v>
+      </c>
+      <c r="B565" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C565" t="inlineStr">
+        <is>
+          <t>Sandvikens IF</t>
+        </is>
+      </c>
+      <c r="D565" t="inlineStr">
+        <is>
+          <t>Osters</t>
+        </is>
+      </c>
+      <c r="E565" t="n">
+        <v>10.79</v>
+      </c>
+      <c r="F565" t="n">
+        <v>0.64</v>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" s="1" t="n">
+        <v>46264</v>
+      </c>
+      <c r="B566" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C566" t="inlineStr">
+        <is>
+          <t>Varbergs BoIS</t>
+        </is>
+      </c>
+      <c r="D566" t="inlineStr">
+        <is>
+          <t>Oddevold</t>
+        </is>
+      </c>
+      <c r="E566" t="n">
+        <v>9.789999999999999</v>
+      </c>
+      <c r="F566" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" s="1" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B567" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C567" t="inlineStr">
+        <is>
+          <t>Fortaleza</t>
+        </is>
+      </c>
+      <c r="D567" t="inlineStr">
+        <is>
+          <t>Operario Ferroviario</t>
+        </is>
+      </c>
+      <c r="E567" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="F567" t="n">
+        <v>2.05</v>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" s="1" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B568" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C568" t="inlineStr">
+        <is>
+          <t>Gnistan</t>
+        </is>
+      </c>
+      <c r="D568" t="inlineStr">
+        <is>
+          <t>TPS</t>
+        </is>
+      </c>
+      <c r="E568" t="n">
+        <v>10.34</v>
+      </c>
+      <c r="F568" t="n">
+        <v>0.68</v>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" s="1" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B569" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C569" t="inlineStr">
+        <is>
+          <t>IFK Mariehamn</t>
+        </is>
+      </c>
+      <c r="D569" t="inlineStr">
+        <is>
+          <t>Jaro</t>
+        </is>
+      </c>
+      <c r="E569" t="n">
+        <v>10.24</v>
+      </c>
+      <c r="F569" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" s="1" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B570" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C570" t="inlineStr">
+        <is>
+          <t>Ilves</t>
+        </is>
+      </c>
+      <c r="D570" t="inlineStr">
+        <is>
+          <t>HJK Helsinki</t>
+        </is>
+      </c>
+      <c r="E570" t="n">
+        <v>10.87</v>
+      </c>
+      <c r="F570" t="n">
+        <v>-1.6</v>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" s="1" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B571" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C571" t="inlineStr">
+        <is>
+          <t>Inter Turku</t>
+        </is>
+      </c>
+      <c r="D571" t="inlineStr">
+        <is>
+          <t>KuPS</t>
+        </is>
+      </c>
+      <c r="E571" t="n">
+        <v>9.710000000000001</v>
+      </c>
+      <c r="F571" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" s="1" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B572" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C572" t="inlineStr">
+        <is>
+          <t>VPS</t>
+        </is>
+      </c>
+      <c r="D572" t="inlineStr">
+        <is>
+          <t>FC Lahti</t>
+        </is>
+      </c>
+      <c r="E572" t="n">
+        <v>9.73</v>
+      </c>
+      <c r="F572" t="n">
+        <v>1.06</v>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" s="1" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B573" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C573" t="inlineStr">
+        <is>
+          <t>Rapid Bucuresti</t>
+        </is>
+      </c>
+      <c r="D573" t="inlineStr">
+        <is>
+          <t>Universitatea Craiova</t>
+        </is>
+      </c>
+      <c r="E573" t="n">
+        <v>9.789999999999999</v>
+      </c>
+      <c r="F573" t="n">
+        <v>-0.67</v>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" s="1" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B574" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C574" t="inlineStr">
+        <is>
+          <t>Sundsvall</t>
+        </is>
+      </c>
+      <c r="D574" t="inlineStr">
+        <is>
+          <t>Norrby</t>
+        </is>
+      </c>
+      <c r="E574" t="n">
+        <v>10.13</v>
+      </c>
+      <c r="F574" t="n">
+        <v>-0.18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily scrape output - 2026-08-29
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F574"/>
+  <dimension ref="A1:F586"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14226,10 +14226,10 @@
         </is>
       </c>
       <c r="E531" t="n">
-        <v>10.21</v>
+        <v>10.2</v>
       </c>
       <c r="F531" t="n">
-        <v>-1.41</v>
+        <v>-1.36</v>
       </c>
     </row>
     <row r="532">
@@ -14243,19 +14243,19 @@
       </c>
       <c r="C532" t="inlineStr">
         <is>
-          <t>Leiknir Reykjavik</t>
+          <t>Afturelding</t>
         </is>
       </c>
       <c r="D532" t="inlineStr">
         <is>
-          <t>UMF Njardvik</t>
+          <t>Vestri</t>
         </is>
       </c>
       <c r="E532" t="n">
-        <v>11.3</v>
+        <v>11.32</v>
       </c>
       <c r="F532" t="n">
-        <v>-1.19</v>
+        <v>3.22</v>
       </c>
     </row>
     <row r="533">
@@ -14269,19 +14269,19 @@
       </c>
       <c r="C533" t="inlineStr">
         <is>
-          <t>UMF Grindavik</t>
+          <t>Leiknir Reykjavik</t>
         </is>
       </c>
       <c r="D533" t="inlineStr">
         <is>
-          <t>HK Kopavogur</t>
+          <t>UMF Njardvik</t>
         </is>
       </c>
       <c r="E533" t="n">
-        <v>11.53</v>
+        <v>11.3</v>
       </c>
       <c r="F533" t="n">
-        <v>-1.48</v>
+        <v>-1.19</v>
       </c>
     </row>
     <row r="534">
@@ -14295,16 +14295,16 @@
       </c>
       <c r="C534" t="inlineStr">
         <is>
-          <t>Volsungur</t>
+          <t>UMF Grindavik</t>
         </is>
       </c>
       <c r="D534" t="inlineStr">
         <is>
-          <t>IR Reykjavik</t>
+          <t>HK Kopavogur</t>
         </is>
       </c>
       <c r="E534" t="n">
-        <v>11.65</v>
+        <v>11.53</v>
       </c>
       <c r="F534" t="n">
         <v>-1.48</v>
@@ -14316,24 +14316,24 @@
       </c>
       <c r="B535" t="inlineStr">
         <is>
-          <t>Norway - 1st Division</t>
+          <t>Iceland - 1. Deild</t>
         </is>
       </c>
       <c r="C535" t="inlineStr">
         <is>
-          <t>Bryne</t>
+          <t>Volsungur</t>
         </is>
       </c>
       <c r="D535" t="inlineStr">
         <is>
-          <t>Haugesund</t>
+          <t>IR Reykjavik</t>
         </is>
       </c>
       <c r="E535" t="n">
-        <v>10.63</v>
+        <v>11.65</v>
       </c>
       <c r="F535" t="n">
-        <v>0.05</v>
+        <v>-1.48</v>
       </c>
     </row>
     <row r="536">
@@ -14342,24 +14342,24 @@
       </c>
       <c r="B536" t="inlineStr">
         <is>
-          <t>Poland - 1st Liga</t>
+          <t>Norway - 1st Division</t>
         </is>
       </c>
       <c r="C536" t="inlineStr">
         <is>
-          <t>Pogon Siedlce</t>
+          <t>Bryne</t>
         </is>
       </c>
       <c r="D536" t="inlineStr">
         <is>
-          <t>Stal Mielec</t>
+          <t>Haugesund</t>
         </is>
       </c>
       <c r="E536" t="n">
-        <v>10.8</v>
+        <v>10.63</v>
       </c>
       <c r="F536" t="n">
-        <v>-0.86</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="537">
@@ -14368,24 +14368,24 @@
       </c>
       <c r="B537" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="C537" t="inlineStr">
         <is>
-          <t>Motor Lublin</t>
+          <t>Pogon Siedlce</t>
         </is>
       </c>
       <c r="D537" t="inlineStr">
         <is>
-          <t>Piast Gliwice</t>
+          <t>Stal Mielec</t>
         </is>
       </c>
       <c r="E537" t="n">
-        <v>10.2</v>
+        <v>10.71</v>
       </c>
       <c r="F537" t="n">
-        <v>0.48</v>
+        <v>-0.83</v>
       </c>
     </row>
     <row r="538">
@@ -14394,24 +14394,24 @@
       </c>
       <c r="B538" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="C538" t="inlineStr">
         <is>
-          <t>Radomiak Radom</t>
+          <t>Polonia Warsaw</t>
         </is>
       </c>
       <c r="D538" t="inlineStr">
         <is>
-          <t>Cracovia Krakow</t>
+          <t>Lechia Gdansk</t>
         </is>
       </c>
       <c r="E538" t="n">
-        <v>9.74</v>
+        <v>10.83</v>
       </c>
       <c r="F538" t="n">
-        <v>-0.59</v>
+        <v>0.98</v>
       </c>
     </row>
     <row r="539">
@@ -14420,24 +14420,24 @@
       </c>
       <c r="B539" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="C539" t="inlineStr">
         <is>
-          <t>Zaglebie Lubin</t>
+          <t>Puszcza Niepolomice</t>
         </is>
       </c>
       <c r="D539" t="inlineStr">
         <is>
-          <t>Pogon Szczecin</t>
+          <t>Podbeskidzie Bielsko-Biala</t>
         </is>
       </c>
       <c r="E539" t="n">
-        <v>10.38</v>
+        <v>10.05</v>
       </c>
       <c r="F539" t="n">
-        <v>-0.35</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="540">
@@ -14446,24 +14446,24 @@
       </c>
       <c r="B540" t="inlineStr">
         <is>
-          <t>Romania - Liga 1</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C540" t="inlineStr">
         <is>
-          <t>Csikszereda</t>
+          <t>Motor Lublin</t>
         </is>
       </c>
       <c r="D540" t="inlineStr">
         <is>
-          <t>CFR Cluj</t>
+          <t>Piast Gliwice</t>
         </is>
       </c>
       <c r="E540" t="n">
-        <v>9.66</v>
+        <v>10.01</v>
       </c>
       <c r="F540" t="n">
-        <v>-1.54</v>
+        <v>0.49</v>
       </c>
     </row>
     <row r="541">
@@ -14472,24 +14472,24 @@
       </c>
       <c r="B541" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C541" t="inlineStr">
         <is>
-          <t>Falkenbergs</t>
+          <t>Radomiak Radom</t>
         </is>
       </c>
       <c r="D541" t="inlineStr">
         <is>
-          <t>Brage</t>
+          <t>Cracovia Krakow</t>
         </is>
       </c>
       <c r="E541" t="n">
-        <v>10.07</v>
+        <v>9.74</v>
       </c>
       <c r="F541" t="n">
-        <v>0.52</v>
+        <v>-0.59</v>
       </c>
     </row>
     <row r="542">
@@ -14498,24 +14498,24 @@
       </c>
       <c r="B542" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C542" t="inlineStr">
         <is>
-          <t>Landskrona</t>
+          <t>Wisla Krakow</t>
         </is>
       </c>
       <c r="D542" t="inlineStr">
         <is>
-          <t>Ostersunds FK</t>
+          <t>Wieczysta Krakow</t>
         </is>
       </c>
       <c r="E542" t="n">
-        <v>10.01</v>
+        <v>11.31</v>
       </c>
       <c r="F542" t="n">
-        <v>0.42</v>
+        <v>1.52</v>
       </c>
     </row>
     <row r="543">
@@ -14524,24 +14524,24 @@
       </c>
       <c r="B543" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C543" t="inlineStr">
         <is>
-          <t>Ljungskile</t>
+          <t>Zaglebie Lubin</t>
         </is>
       </c>
       <c r="D543" t="inlineStr">
         <is>
-          <t>Varnamo</t>
+          <t>Pogon Szczecin</t>
         </is>
       </c>
       <c r="E543" t="n">
-        <v>10.61</v>
+        <v>10.21</v>
       </c>
       <c r="F543" t="n">
-        <v>1.11</v>
+        <v>-0.18</v>
       </c>
     </row>
     <row r="544">
@@ -14550,99 +14550,99 @@
       </c>
       <c r="B544" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Romania - Liga 1</t>
         </is>
       </c>
       <c r="C544" t="inlineStr">
         <is>
-          <t>Nordic United</t>
+          <t>Arges Pitesti</t>
         </is>
       </c>
       <c r="D544" t="inlineStr">
         <is>
-          <t>Norrkoping</t>
+          <t>Sepsi</t>
         </is>
       </c>
       <c r="E544" t="n">
-        <v>10.05</v>
+        <v>8.67</v>
       </c>
       <c r="F544" t="n">
-        <v>-0.49</v>
+        <v>1.08</v>
       </c>
     </row>
     <row r="545">
       <c r="A545" s="1" t="n">
-        <v>46264</v>
+        <v>46263</v>
       </c>
       <c r="B545" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Romania - Liga 1</t>
         </is>
       </c>
       <c r="C545" t="inlineStr">
         <is>
-          <t>America Mineiro</t>
+          <t>Corvinul Hunedoara</t>
         </is>
       </c>
       <c r="D545" t="inlineStr">
         <is>
-          <t>Ponte Preta</t>
+          <t>Dinamo Bucuresti</t>
         </is>
       </c>
       <c r="E545" t="n">
-        <v>10.45</v>
+        <v>8.779999999999999</v>
       </c>
       <c r="F545" t="n">
-        <v>2.45</v>
+        <v>-0.59</v>
       </c>
     </row>
     <row r="546">
       <c r="A546" s="1" t="n">
-        <v>46264</v>
+        <v>46263</v>
       </c>
       <c r="B546" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Romania - Liga 1</t>
         </is>
       </c>
       <c r="C546" t="inlineStr">
         <is>
-          <t>Avai</t>
+          <t>Csikszereda</t>
         </is>
       </c>
       <c r="D546" t="inlineStr">
         <is>
-          <t>Atletico Goianiense</t>
+          <t>CFR Cluj</t>
         </is>
       </c>
       <c r="E546" t="n">
-        <v>10.16</v>
+        <v>9.449999999999999</v>
       </c>
       <c r="F546" t="n">
-        <v>0.31</v>
+        <v>-1.18</v>
       </c>
     </row>
     <row r="547">
       <c r="A547" s="1" t="n">
-        <v>46264</v>
+        <v>46263</v>
       </c>
       <c r="B547" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="C547" t="inlineStr">
         <is>
-          <t>CRB</t>
+          <t>Albacete</t>
         </is>
       </c>
       <c r="D547" t="inlineStr">
         <is>
-          <t>Criciuma</t>
+          <t>Real Oviedo</t>
         </is>
       </c>
       <c r="E547" t="n">
-        <v>10.51</v>
+        <v>9.460000000000001</v>
       </c>
       <c r="F547" t="n">
         <v>0.4</v>
@@ -14650,158 +14650,158 @@
     </row>
     <row r="548">
       <c r="A548" s="1" t="n">
-        <v>46264</v>
+        <v>46263</v>
       </c>
       <c r="B548" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="C548" t="inlineStr">
         <is>
-          <t>Vila Nova</t>
+          <t>Leganes</t>
         </is>
       </c>
       <c r="D548" t="inlineStr">
         <is>
-          <t>Ceara</t>
+          <t>Eldense</t>
         </is>
       </c>
       <c r="E548" t="n">
-        <v>10.49</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="F548" t="n">
-        <v>1.45</v>
+        <v>0.96</v>
       </c>
     </row>
     <row r="549">
       <c r="A549" s="1" t="n">
-        <v>46264</v>
+        <v>46263</v>
       </c>
       <c r="B549" t="inlineStr">
         <is>
-          <t>Finland - Ykkosliiga</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="C549" t="inlineStr">
         <is>
-          <t>SJK Akatemia</t>
+          <t>Sabadell</t>
         </is>
       </c>
       <c r="D549" t="inlineStr">
         <is>
-          <t>HJK Klubi 04</t>
+          <t>Almeria</t>
         </is>
       </c>
       <c r="E549" t="n">
-        <v>10.22</v>
+        <v>9.5</v>
       </c>
       <c r="F549" t="n">
-        <v>0.02</v>
+        <v>0.67</v>
       </c>
     </row>
     <row r="550">
       <c r="A550" s="1" t="n">
-        <v>46264</v>
+        <v>46263</v>
       </c>
       <c r="B550" t="inlineStr">
         <is>
-          <t>Norway - 1st Division</t>
+          <t>Sweden - Superettan</t>
         </is>
       </c>
       <c r="C550" t="inlineStr">
         <is>
-          <t>Egersunds</t>
+          <t>Falkenbergs</t>
         </is>
       </c>
       <c r="D550" t="inlineStr">
         <is>
-          <t>Asane Fotball</t>
+          <t>Brage</t>
         </is>
       </c>
       <c r="E550" t="n">
-        <v>11.06</v>
+        <v>10.06</v>
       </c>
       <c r="F550" t="n">
-        <v>2.95</v>
+        <v>0.53</v>
       </c>
     </row>
     <row r="551">
       <c r="A551" s="1" t="n">
-        <v>46264</v>
+        <v>46263</v>
       </c>
       <c r="B551" t="inlineStr">
         <is>
-          <t>Norway - 1st Division</t>
+          <t>Sweden - Superettan</t>
         </is>
       </c>
       <c r="C551" t="inlineStr">
         <is>
-          <t>Hodd</t>
+          <t>Landskrona</t>
         </is>
       </c>
       <c r="D551" t="inlineStr">
         <is>
-          <t>Stabaek</t>
+          <t>Ostersunds FK</t>
         </is>
       </c>
       <c r="E551" t="n">
-        <v>11.34</v>
+        <v>10.01</v>
       </c>
       <c r="F551" t="n">
-        <v>-3.03</v>
+        <v>0.42</v>
       </c>
     </row>
     <row r="552">
       <c r="A552" s="1" t="n">
-        <v>46264</v>
+        <v>46263</v>
       </c>
       <c r="B552" t="inlineStr">
         <is>
-          <t>Norway - 1st Division</t>
+          <t>Sweden - Superettan</t>
         </is>
       </c>
       <c r="C552" t="inlineStr">
         <is>
-          <t>Kongsvinger</t>
+          <t>Ljungskile</t>
         </is>
       </c>
       <c r="D552" t="inlineStr">
         <is>
-          <t>Lyn</t>
+          <t>Varnamo</t>
         </is>
       </c>
       <c r="E552" t="n">
-        <v>11.06</v>
+        <v>10.61</v>
       </c>
       <c r="F552" t="n">
-        <v>1.71</v>
+        <v>1.11</v>
       </c>
     </row>
     <row r="553">
       <c r="A553" s="1" t="n">
-        <v>46264</v>
+        <v>46263</v>
       </c>
       <c r="B553" t="inlineStr">
         <is>
-          <t>Norway - 1st Division</t>
+          <t>Sweden - Superettan</t>
         </is>
       </c>
       <c r="C553" t="inlineStr">
         <is>
-          <t>Moss</t>
+          <t>Nordic United</t>
         </is>
       </c>
       <c r="D553" t="inlineStr">
         <is>
-          <t>Strommen</t>
+          <t>Norrkoping</t>
         </is>
       </c>
       <c r="E553" t="n">
-        <v>10.55</v>
+        <v>10.05</v>
       </c>
       <c r="F553" t="n">
-        <v>1.2</v>
+        <v>-0.49</v>
       </c>
     </row>
     <row r="554">
@@ -14810,24 +14810,24 @@
       </c>
       <c r="B554" t="inlineStr">
         <is>
-          <t>Norway - 1st Division</t>
+          <t>Brazil - Serie B</t>
         </is>
       </c>
       <c r="C554" t="inlineStr">
         <is>
-          <t>Ranheim</t>
+          <t>America Mineiro</t>
         </is>
       </c>
       <c r="D554" t="inlineStr">
         <is>
-          <t>Odd BK</t>
+          <t>Ponte Preta</t>
         </is>
       </c>
       <c r="E554" t="n">
-        <v>11.2</v>
+        <v>10.45</v>
       </c>
       <c r="F554" t="n">
-        <v>-0.36</v>
+        <v>2.45</v>
       </c>
     </row>
     <row r="555">
@@ -14836,24 +14836,24 @@
       </c>
       <c r="B555" t="inlineStr">
         <is>
-          <t>Norway - 1st Division</t>
+          <t>Brazil - Serie B</t>
         </is>
       </c>
       <c r="C555" t="inlineStr">
         <is>
-          <t>Raufoss</t>
+          <t>Avai</t>
         </is>
       </c>
       <c r="D555" t="inlineStr">
         <is>
-          <t>Sandnes Ulf</t>
+          <t>Atletico Goianiense</t>
         </is>
       </c>
       <c r="E555" t="n">
-        <v>10.98</v>
+        <v>10.16</v>
       </c>
       <c r="F555" t="n">
-        <v>-0.2</v>
+        <v>0.31</v>
       </c>
     </row>
     <row r="556">
@@ -14862,24 +14862,24 @@
       </c>
       <c r="B556" t="inlineStr">
         <is>
-          <t>Norway - 1st Division</t>
+          <t>Brazil - Serie B</t>
         </is>
       </c>
       <c r="C556" t="inlineStr">
         <is>
-          <t>Sogndal</t>
+          <t>CRB</t>
         </is>
       </c>
       <c r="D556" t="inlineStr">
         <is>
-          <t>Stromsgodset</t>
+          <t>Criciuma</t>
         </is>
       </c>
       <c r="E556" t="n">
-        <v>11.5</v>
+        <v>10.51</v>
       </c>
       <c r="F556" t="n">
-        <v>-2.6</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="557">
@@ -14888,24 +14888,24 @@
       </c>
       <c r="B557" t="inlineStr">
         <is>
-          <t>Poland - 1st Liga</t>
+          <t>Brazil - Serie B</t>
         </is>
       </c>
       <c r="C557" t="inlineStr">
         <is>
-          <t>Chrobry Glogow</t>
+          <t>Vila Nova</t>
         </is>
       </c>
       <c r="D557" t="inlineStr">
         <is>
-          <t>Ruch Chorzow</t>
+          <t>Ceara</t>
         </is>
       </c>
       <c r="E557" t="n">
-        <v>10.82</v>
+        <v>10.49</v>
       </c>
       <c r="F557" t="n">
-        <v>-0.54</v>
+        <v>1.45</v>
       </c>
     </row>
     <row r="558">
@@ -14914,24 +14914,24 @@
       </c>
       <c r="B558" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Finland - Ykkosliiga</t>
         </is>
       </c>
       <c r="C558" t="inlineStr">
         <is>
-          <t>Gornik Zabrze</t>
+          <t>SJK Akatemia</t>
         </is>
       </c>
       <c r="D558" t="inlineStr">
         <is>
-          <t>GKS Katowice</t>
+          <t>HJK Klubi 04</t>
         </is>
       </c>
       <c r="E558" t="n">
-        <v>10.36</v>
+        <v>10.22</v>
       </c>
       <c r="F558" t="n">
-        <v>2.4</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="559">
@@ -14940,24 +14940,24 @@
       </c>
       <c r="B559" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Norway - 1st Division</t>
         </is>
       </c>
       <c r="C559" t="inlineStr">
         <is>
-          <t>Rakow Czestochowa</t>
+          <t>Egersunds</t>
         </is>
       </c>
       <c r="D559" t="inlineStr">
         <is>
-          <t>Jagiellonia Bialystok</t>
+          <t>Asane Fotball</t>
         </is>
       </c>
       <c r="E559" t="n">
-        <v>9.67</v>
+        <v>10.83</v>
       </c>
       <c r="F559" t="n">
-        <v>0.53</v>
+        <v>2.96</v>
       </c>
     </row>
     <row r="560">
@@ -14966,24 +14966,24 @@
       </c>
       <c r="B560" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Norway - 1st Division</t>
         </is>
       </c>
       <c r="C560" t="inlineStr">
         <is>
-          <t>Widzew Lodz</t>
+          <t>Hodd</t>
         </is>
       </c>
       <c r="D560" t="inlineStr">
         <is>
-          <t>Lech Poznan</t>
+          <t>Stabaek</t>
         </is>
       </c>
       <c r="E560" t="n">
-        <v>10.14</v>
+        <v>11.34</v>
       </c>
       <c r="F560" t="n">
-        <v>-0.65</v>
+        <v>-3.03</v>
       </c>
     </row>
     <row r="561">
@@ -14992,24 +14992,24 @@
       </c>
       <c r="B561" t="inlineStr">
         <is>
-          <t>Romania - Liga 1</t>
+          <t>Norway - 1st Division</t>
         </is>
       </c>
       <c r="C561" t="inlineStr">
         <is>
-          <t>FCSB</t>
+          <t>Kongsvinger</t>
         </is>
       </c>
       <c r="D561" t="inlineStr">
         <is>
-          <t>UTA Arad</t>
+          <t>Lyn</t>
         </is>
       </c>
       <c r="E561" t="n">
-        <v>10.01</v>
+        <v>11.06</v>
       </c>
       <c r="F561" t="n">
-        <v>2.61</v>
+        <v>1.88</v>
       </c>
     </row>
     <row r="562">
@@ -15018,24 +15018,24 @@
       </c>
       <c r="B562" t="inlineStr">
         <is>
-          <t>Romania - Liga 1</t>
+          <t>Norway - 1st Division</t>
         </is>
       </c>
       <c r="C562" t="inlineStr">
         <is>
-          <t>Farul Constanta</t>
+          <t>Moss</t>
         </is>
       </c>
       <c r="D562" t="inlineStr">
         <is>
-          <t>Botosani</t>
+          <t>Strommen</t>
         </is>
       </c>
       <c r="E562" t="n">
-        <v>9.25</v>
+        <v>10.55</v>
       </c>
       <c r="F562" t="n">
-        <v>1.36</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="563">
@@ -15044,24 +15044,24 @@
       </c>
       <c r="B563" t="inlineStr">
         <is>
-          <t>Spain - Segunda</t>
+          <t>Norway - 1st Division</t>
         </is>
       </c>
       <c r="C563" t="inlineStr">
         <is>
-          <t>Cordoba</t>
+          <t>Ranheim</t>
         </is>
       </c>
       <c r="D563" t="inlineStr">
         <is>
-          <t>Granada</t>
+          <t>Odd BK</t>
         </is>
       </c>
       <c r="E563" t="n">
-        <v>9.859999999999999</v>
+        <v>11.2</v>
       </c>
       <c r="F563" t="n">
-        <v>1.98</v>
+        <v>-0.36</v>
       </c>
     </row>
     <row r="564">
@@ -15070,24 +15070,24 @@
       </c>
       <c r="B564" t="inlineStr">
         <is>
-          <t>Spain - Segunda</t>
+          <t>Norway - 1st Division</t>
         </is>
       </c>
       <c r="C564" t="inlineStr">
         <is>
-          <t>FC Andorra</t>
+          <t>Raufoss</t>
         </is>
       </c>
       <c r="D564" t="inlineStr">
         <is>
-          <t>Eibar</t>
+          <t>Sandnes Ulf</t>
         </is>
       </c>
       <c r="E564" t="n">
-        <v>9.15</v>
+        <v>10.98</v>
       </c>
       <c r="F564" t="n">
-        <v>1.44</v>
+        <v>-0.2</v>
       </c>
     </row>
     <row r="565">
@@ -15096,24 +15096,24 @@
       </c>
       <c r="B565" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Norway - 1st Division</t>
         </is>
       </c>
       <c r="C565" t="inlineStr">
         <is>
-          <t>Sandvikens IF</t>
+          <t>Sogndal</t>
         </is>
       </c>
       <c r="D565" t="inlineStr">
         <is>
-          <t>Osters</t>
+          <t>Stromsgodset</t>
         </is>
       </c>
       <c r="E565" t="n">
-        <v>10.79</v>
+        <v>11.5</v>
       </c>
       <c r="F565" t="n">
-        <v>0.64</v>
+        <v>-2.59</v>
       </c>
     </row>
     <row r="566">
@@ -15122,232 +15122,544 @@
       </c>
       <c r="B566" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="C566" t="inlineStr">
         <is>
-          <t>Varbergs BoIS</t>
+          <t>Chrobry Glogow</t>
         </is>
       </c>
       <c r="D566" t="inlineStr">
         <is>
-          <t>Oddevold</t>
+          <t>Ruch Chorzow</t>
         </is>
       </c>
       <c r="E566" t="n">
-        <v>9.789999999999999</v>
+        <v>10.82</v>
       </c>
       <c r="F566" t="n">
-        <v>0.5600000000000001</v>
+        <v>-0.54</v>
       </c>
     </row>
     <row r="567">
       <c r="A567" s="1" t="n">
-        <v>46265</v>
+        <v>46264</v>
       </c>
       <c r="B567" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C567" t="inlineStr">
         <is>
-          <t>Fortaleza</t>
+          <t>Gornik Zabrze</t>
         </is>
       </c>
       <c r="D567" t="inlineStr">
         <is>
-          <t>Operario Ferroviario</t>
+          <t>GKS Katowice</t>
         </is>
       </c>
       <c r="E567" t="n">
-        <v>10.5</v>
+        <v>10.36</v>
       </c>
       <c r="F567" t="n">
-        <v>2.05</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="568">
       <c r="A568" s="1" t="n">
-        <v>46265</v>
+        <v>46264</v>
       </c>
       <c r="B568" t="inlineStr">
         <is>
-          <t>Finland - Veikkausliiga</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C568" t="inlineStr">
         <is>
-          <t>Gnistan</t>
+          <t>Rakow Czestochowa</t>
         </is>
       </c>
       <c r="D568" t="inlineStr">
         <is>
-          <t>TPS</t>
+          <t>Jagiellonia Bialystok</t>
         </is>
       </c>
       <c r="E568" t="n">
-        <v>10.34</v>
+        <v>9.67</v>
       </c>
       <c r="F568" t="n">
-        <v>0.68</v>
+        <v>0.53</v>
       </c>
     </row>
     <row r="569">
       <c r="A569" s="1" t="n">
-        <v>46265</v>
+        <v>46264</v>
       </c>
       <c r="B569" t="inlineStr">
         <is>
-          <t>Finland - Veikkausliiga</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C569" t="inlineStr">
         <is>
-          <t>IFK Mariehamn</t>
+          <t>Widzew Lodz</t>
         </is>
       </c>
       <c r="D569" t="inlineStr">
         <is>
-          <t>Jaro</t>
+          <t>Lech Poznan</t>
         </is>
       </c>
       <c r="E569" t="n">
-        <v>10.24</v>
+        <v>10.14</v>
       </c>
       <c r="F569" t="n">
-        <v>0</v>
+        <v>-0.65</v>
       </c>
     </row>
     <row r="570">
       <c r="A570" s="1" t="n">
-        <v>46265</v>
+        <v>46264</v>
       </c>
       <c r="B570" t="inlineStr">
         <is>
-          <t>Finland - Veikkausliiga</t>
+          <t>Romania - Liga 1</t>
         </is>
       </c>
       <c r="C570" t="inlineStr">
         <is>
-          <t>Ilves</t>
+          <t>FCSB</t>
         </is>
       </c>
       <c r="D570" t="inlineStr">
         <is>
-          <t>HJK Helsinki</t>
+          <t>UTA Arad</t>
         </is>
       </c>
       <c r="E570" t="n">
-        <v>10.87</v>
+        <v>10.01</v>
       </c>
       <c r="F570" t="n">
-        <v>-1.6</v>
+        <v>2.61</v>
       </c>
     </row>
     <row r="571">
       <c r="A571" s="1" t="n">
-        <v>46265</v>
+        <v>46264</v>
       </c>
       <c r="B571" t="inlineStr">
         <is>
-          <t>Finland - Veikkausliiga</t>
+          <t>Romania - Liga 1</t>
         </is>
       </c>
       <c r="C571" t="inlineStr">
         <is>
-          <t>Inter Turku</t>
+          <t>Farul Constanta</t>
         </is>
       </c>
       <c r="D571" t="inlineStr">
         <is>
-          <t>KuPS</t>
+          <t>Botosani</t>
         </is>
       </c>
       <c r="E571" t="n">
-        <v>9.710000000000001</v>
+        <v>9.25</v>
       </c>
       <c r="F571" t="n">
-        <v>0.9399999999999999</v>
+        <v>1.36</v>
       </c>
     </row>
     <row r="572">
       <c r="A572" s="1" t="n">
-        <v>46265</v>
+        <v>46264</v>
       </c>
       <c r="B572" t="inlineStr">
         <is>
-          <t>Finland - Veikkausliiga</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="C572" t="inlineStr">
         <is>
-          <t>VPS</t>
+          <t>Cordoba</t>
         </is>
       </c>
       <c r="D572" t="inlineStr">
         <is>
-          <t>FC Lahti</t>
+          <t>Granada</t>
         </is>
       </c>
       <c r="E572" t="n">
-        <v>9.73</v>
+        <v>9.859999999999999</v>
       </c>
       <c r="F572" t="n">
-        <v>1.06</v>
+        <v>1.98</v>
       </c>
     </row>
     <row r="573">
       <c r="A573" s="1" t="n">
-        <v>46265</v>
+        <v>46264</v>
       </c>
       <c r="B573" t="inlineStr">
         <is>
-          <t>Romania - Liga 1</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="C573" t="inlineStr">
         <is>
-          <t>Rapid Bucuresti</t>
+          <t>FC Andorra</t>
         </is>
       </c>
       <c r="D573" t="inlineStr">
         <is>
-          <t>Universitatea Craiova</t>
+          <t>Eibar</t>
         </is>
       </c>
       <c r="E573" t="n">
-        <v>9.789999999999999</v>
+        <v>9.15</v>
       </c>
       <c r="F573" t="n">
-        <v>-0.67</v>
+        <v>1.44</v>
       </c>
     </row>
     <row r="574">
       <c r="A574" s="1" t="n">
+        <v>46264</v>
+      </c>
+      <c r="B574" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C574" t="inlineStr">
+        <is>
+          <t>Sandvikens IF</t>
+        </is>
+      </c>
+      <c r="D574" t="inlineStr">
+        <is>
+          <t>Osters</t>
+        </is>
+      </c>
+      <c r="E574" t="n">
+        <v>10.79</v>
+      </c>
+      <c r="F574" t="n">
+        <v>0.64</v>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" s="1" t="n">
+        <v>46264</v>
+      </c>
+      <c r="B575" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C575" t="inlineStr">
+        <is>
+          <t>Varbergs BoIS</t>
+        </is>
+      </c>
+      <c r="D575" t="inlineStr">
+        <is>
+          <t>Oddevold</t>
+        </is>
+      </c>
+      <c r="E575" t="n">
+        <v>9.789999999999999</v>
+      </c>
+      <c r="F575" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" s="1" t="n">
         <v>46265</v>
       </c>
-      <c r="B574" t="inlineStr">
+      <c r="B576" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C576" t="inlineStr">
+        <is>
+          <t>Fortaleza</t>
+        </is>
+      </c>
+      <c r="D576" t="inlineStr">
+        <is>
+          <t>Operario Ferroviario</t>
+        </is>
+      </c>
+      <c r="E576" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="F576" t="n">
+        <v>2.05</v>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" s="1" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B577" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C577" t="inlineStr">
+        <is>
+          <t>AC Oulu</t>
+        </is>
+      </c>
+      <c r="D577" t="inlineStr">
+        <is>
+          <t>SJK</t>
+        </is>
+      </c>
+      <c r="E577" t="n">
+        <v>10.49</v>
+      </c>
+      <c r="F577" t="n">
+        <v>-0.06</v>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" s="1" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B578" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C578" t="inlineStr">
+        <is>
+          <t>Gnistan</t>
+        </is>
+      </c>
+      <c r="D578" t="inlineStr">
+        <is>
+          <t>TPS</t>
+        </is>
+      </c>
+      <c r="E578" t="n">
+        <v>10.22</v>
+      </c>
+      <c r="F578" t="n">
+        <v>0.68</v>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" s="1" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B579" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C579" t="inlineStr">
+        <is>
+          <t>IFK Mariehamn</t>
+        </is>
+      </c>
+      <c r="D579" t="inlineStr">
+        <is>
+          <t>Jaro</t>
+        </is>
+      </c>
+      <c r="E579" t="n">
+        <v>10.24</v>
+      </c>
+      <c r="F579" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" s="1" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B580" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C580" t="inlineStr">
+        <is>
+          <t>Ilves</t>
+        </is>
+      </c>
+      <c r="D580" t="inlineStr">
+        <is>
+          <t>HJK Helsinki</t>
+        </is>
+      </c>
+      <c r="E580" t="n">
+        <v>10.87</v>
+      </c>
+      <c r="F580" t="n">
+        <v>-1.6</v>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" s="1" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B581" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C581" t="inlineStr">
+        <is>
+          <t>Inter Turku</t>
+        </is>
+      </c>
+      <c r="D581" t="inlineStr">
+        <is>
+          <t>KuPS</t>
+        </is>
+      </c>
+      <c r="E581" t="n">
+        <v>9.710000000000001</v>
+      </c>
+      <c r="F581" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" s="1" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B582" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C582" t="inlineStr">
+        <is>
+          <t>VPS</t>
+        </is>
+      </c>
+      <c r="D582" t="inlineStr">
+        <is>
+          <t>FC Lahti</t>
+        </is>
+      </c>
+      <c r="E582" t="n">
+        <v>9.73</v>
+      </c>
+      <c r="F582" t="n">
+        <v>1.06</v>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" s="1" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B583" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C583" t="inlineStr">
+        <is>
+          <t>Rapid Bucuresti</t>
+        </is>
+      </c>
+      <c r="D583" t="inlineStr">
+        <is>
+          <t>Universitatea Craiova</t>
+        </is>
+      </c>
+      <c r="E583" t="n">
+        <v>9.789999999999999</v>
+      </c>
+      <c r="F583" t="n">
+        <v>-0.67</v>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" s="1" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B584" t="inlineStr">
         <is>
           <t>Sweden - Superettan</t>
         </is>
       </c>
-      <c r="C574" t="inlineStr">
+      <c r="C584" t="inlineStr">
         <is>
           <t>Sundsvall</t>
         </is>
       </c>
-      <c r="D574" t="inlineStr">
+      <c r="D584" t="inlineStr">
         <is>
           <t>Norrby</t>
         </is>
       </c>
-      <c r="E574" t="n">
-        <v>10.13</v>
-      </c>
-      <c r="F574" t="n">
-        <v>-0.18</v>
+      <c r="E584" t="n">
+        <v>9.82</v>
+      </c>
+      <c r="F584" t="n">
+        <v>-0.11</v>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" s="1" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B585" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C585" t="inlineStr">
+        <is>
+          <t>Londrina</t>
+        </is>
+      </c>
+      <c r="D585" t="inlineStr">
+        <is>
+          <t>Juventude</t>
+        </is>
+      </c>
+      <c r="E585" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="F585" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" s="1" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B586" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C586" t="inlineStr">
+        <is>
+          <t>Helsingborgs</t>
+        </is>
+      </c>
+      <c r="D586" t="inlineStr">
+        <is>
+          <t>Orebro SK</t>
+        </is>
+      </c>
+      <c r="E586" t="n">
+        <v>10.26</v>
+      </c>
+      <c r="F586" t="n">
+        <v>0.45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily scrape output - 2026-08-30
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F586"/>
+  <dimension ref="A1:F590"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14824,10 +14824,10 @@
         </is>
       </c>
       <c r="E554" t="n">
-        <v>10.45</v>
+        <v>10.63</v>
       </c>
       <c r="F554" t="n">
-        <v>2.45</v>
+        <v>3.51</v>
       </c>
     </row>
     <row r="555">
@@ -14928,10 +14928,10 @@
         </is>
       </c>
       <c r="E558" t="n">
-        <v>10.22</v>
+        <v>10.29</v>
       </c>
       <c r="F558" t="n">
-        <v>0.02</v>
+        <v>0</v>
       </c>
     </row>
     <row r="559">
@@ -14945,19 +14945,19 @@
       </c>
       <c r="C559" t="inlineStr">
         <is>
-          <t>Egersunds</t>
+          <t>Bryne</t>
         </is>
       </c>
       <c r="D559" t="inlineStr">
         <is>
-          <t>Asane Fotball</t>
+          <t>Haugesund</t>
         </is>
       </c>
       <c r="E559" t="n">
-        <v>10.83</v>
+        <v>10.79</v>
       </c>
       <c r="F559" t="n">
-        <v>2.96</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="560">
@@ -14971,19 +14971,19 @@
       </c>
       <c r="C560" t="inlineStr">
         <is>
-          <t>Hodd</t>
+          <t>Egersunds</t>
         </is>
       </c>
       <c r="D560" t="inlineStr">
         <is>
-          <t>Stabaek</t>
+          <t>Asane Fotball</t>
         </is>
       </c>
       <c r="E560" t="n">
-        <v>11.34</v>
+        <v>10.32</v>
       </c>
       <c r="F560" t="n">
-        <v>-3.03</v>
+        <v>3.44</v>
       </c>
     </row>
     <row r="561">
@@ -14997,19 +14997,19 @@
       </c>
       <c r="C561" t="inlineStr">
         <is>
-          <t>Kongsvinger</t>
+          <t>Hodd</t>
         </is>
       </c>
       <c r="D561" t="inlineStr">
         <is>
-          <t>Lyn</t>
+          <t>Stabaek</t>
         </is>
       </c>
       <c r="E561" t="n">
-        <v>11.06</v>
+        <v>11.34</v>
       </c>
       <c r="F561" t="n">
-        <v>1.88</v>
+        <v>-3.03</v>
       </c>
     </row>
     <row r="562">
@@ -15023,19 +15023,19 @@
       </c>
       <c r="C562" t="inlineStr">
         <is>
-          <t>Moss</t>
+          <t>Kongsvinger</t>
         </is>
       </c>
       <c r="D562" t="inlineStr">
         <is>
-          <t>Strommen</t>
+          <t>Lyn</t>
         </is>
       </c>
       <c r="E562" t="n">
-        <v>10.55</v>
+        <v>11.17</v>
       </c>
       <c r="F562" t="n">
-        <v>1.2</v>
+        <v>1.88</v>
       </c>
     </row>
     <row r="563">
@@ -15049,19 +15049,19 @@
       </c>
       <c r="C563" t="inlineStr">
         <is>
-          <t>Ranheim</t>
+          <t>Moss</t>
         </is>
       </c>
       <c r="D563" t="inlineStr">
         <is>
-          <t>Odd BK</t>
+          <t>Strommen</t>
         </is>
       </c>
       <c r="E563" t="n">
-        <v>11.2</v>
+        <v>10.55</v>
       </c>
       <c r="F563" t="n">
-        <v>-0.36</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="564">
@@ -15075,19 +15075,19 @@
       </c>
       <c r="C564" t="inlineStr">
         <is>
-          <t>Raufoss</t>
+          <t>Ranheim</t>
         </is>
       </c>
       <c r="D564" t="inlineStr">
         <is>
-          <t>Sandnes Ulf</t>
+          <t>Odd BK</t>
         </is>
       </c>
       <c r="E564" t="n">
-        <v>10.98</v>
+        <v>11.2</v>
       </c>
       <c r="F564" t="n">
-        <v>-0.2</v>
+        <v>-0.36</v>
       </c>
     </row>
     <row r="565">
@@ -15101,19 +15101,19 @@
       </c>
       <c r="C565" t="inlineStr">
         <is>
-          <t>Sogndal</t>
+          <t>Raufoss</t>
         </is>
       </c>
       <c r="D565" t="inlineStr">
         <is>
-          <t>Stromsgodset</t>
+          <t>Sandnes Ulf</t>
         </is>
       </c>
       <c r="E565" t="n">
-        <v>11.5</v>
+        <v>11</v>
       </c>
       <c r="F565" t="n">
-        <v>-2.59</v>
+        <v>-0.42</v>
       </c>
     </row>
     <row r="566">
@@ -15122,24 +15122,24 @@
       </c>
       <c r="B566" t="inlineStr">
         <is>
-          <t>Poland - 1st Liga</t>
+          <t>Norway - 1st Division</t>
         </is>
       </c>
       <c r="C566" t="inlineStr">
         <is>
-          <t>Chrobry Glogow</t>
+          <t>Sogndal</t>
         </is>
       </c>
       <c r="D566" t="inlineStr">
         <is>
-          <t>Ruch Chorzow</t>
+          <t>Stromsgodset</t>
         </is>
       </c>
       <c r="E566" t="n">
-        <v>10.82</v>
+        <v>11.94</v>
       </c>
       <c r="F566" t="n">
-        <v>-0.54</v>
+        <v>-2.69</v>
       </c>
     </row>
     <row r="567">
@@ -15148,24 +15148,24 @@
       </c>
       <c r="B567" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="C567" t="inlineStr">
         <is>
-          <t>Gornik Zabrze</t>
+          <t>Arka Gdynia</t>
         </is>
       </c>
       <c r="D567" t="inlineStr">
         <is>
-          <t>GKS Katowice</t>
+          <t>Polonia Bytom</t>
         </is>
       </c>
       <c r="E567" t="n">
-        <v>10.36</v>
+        <v>10.13</v>
       </c>
       <c r="F567" t="n">
-        <v>2.4</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="568">
@@ -15174,24 +15174,24 @@
       </c>
       <c r="B568" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="C568" t="inlineStr">
         <is>
-          <t>Rakow Czestochowa</t>
+          <t>Chrobry Glogow</t>
         </is>
       </c>
       <c r="D568" t="inlineStr">
         <is>
-          <t>Jagiellonia Bialystok</t>
+          <t>Ruch Chorzow</t>
         </is>
       </c>
       <c r="E568" t="n">
-        <v>9.67</v>
+        <v>10.61</v>
       </c>
       <c r="F568" t="n">
-        <v>0.53</v>
+        <v>-0.51</v>
       </c>
     </row>
     <row r="569">
@@ -15205,19 +15205,19 @@
       </c>
       <c r="C569" t="inlineStr">
         <is>
-          <t>Widzew Lodz</t>
+          <t>Gornik Zabrze</t>
         </is>
       </c>
       <c r="D569" t="inlineStr">
         <is>
-          <t>Lech Poznan</t>
+          <t>GKS Katowice</t>
         </is>
       </c>
       <c r="E569" t="n">
-        <v>10.14</v>
+        <v>10.36</v>
       </c>
       <c r="F569" t="n">
-        <v>-0.65</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="570">
@@ -15226,24 +15226,24 @@
       </c>
       <c r="B570" t="inlineStr">
         <is>
-          <t>Romania - Liga 1</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C570" t="inlineStr">
         <is>
-          <t>FCSB</t>
+          <t>Rakow Czestochowa</t>
         </is>
       </c>
       <c r="D570" t="inlineStr">
         <is>
-          <t>UTA Arad</t>
+          <t>Jagiellonia Bialystok</t>
         </is>
       </c>
       <c r="E570" t="n">
-        <v>10.01</v>
+        <v>9.640000000000001</v>
       </c>
       <c r="F570" t="n">
-        <v>2.61</v>
+        <v>0.54</v>
       </c>
     </row>
     <row r="571">
@@ -15252,24 +15252,24 @@
       </c>
       <c r="B571" t="inlineStr">
         <is>
-          <t>Romania - Liga 1</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C571" t="inlineStr">
         <is>
-          <t>Farul Constanta</t>
+          <t>Widzew Lodz</t>
         </is>
       </c>
       <c r="D571" t="inlineStr">
         <is>
-          <t>Botosani</t>
+          <t>Lech Poznan</t>
         </is>
       </c>
       <c r="E571" t="n">
-        <v>9.25</v>
+        <v>10.12</v>
       </c>
       <c r="F571" t="n">
-        <v>1.36</v>
+        <v>-0.64</v>
       </c>
     </row>
     <row r="572">
@@ -15278,24 +15278,24 @@
       </c>
       <c r="B572" t="inlineStr">
         <is>
-          <t>Spain - Segunda</t>
+          <t>Romania - Liga 1</t>
         </is>
       </c>
       <c r="C572" t="inlineStr">
         <is>
-          <t>Cordoba</t>
+          <t>FCSB</t>
         </is>
       </c>
       <c r="D572" t="inlineStr">
         <is>
-          <t>Granada</t>
+          <t>UTA Arad</t>
         </is>
       </c>
       <c r="E572" t="n">
-        <v>9.859999999999999</v>
+        <v>9.98</v>
       </c>
       <c r="F572" t="n">
-        <v>1.98</v>
+        <v>2.62</v>
       </c>
     </row>
     <row r="573">
@@ -15304,24 +15304,24 @@
       </c>
       <c r="B573" t="inlineStr">
         <is>
-          <t>Spain - Segunda</t>
+          <t>Romania - Liga 1</t>
         </is>
       </c>
       <c r="C573" t="inlineStr">
         <is>
-          <t>FC Andorra</t>
+          <t>Farul Constanta</t>
         </is>
       </c>
       <c r="D573" t="inlineStr">
         <is>
-          <t>Eibar</t>
+          <t>Botosani</t>
         </is>
       </c>
       <c r="E573" t="n">
-        <v>9.15</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="F573" t="n">
-        <v>1.44</v>
+        <v>1.42</v>
       </c>
     </row>
     <row r="574">
@@ -15330,24 +15330,24 @@
       </c>
       <c r="B574" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="C574" t="inlineStr">
         <is>
-          <t>Sandvikens IF</t>
+          <t>Cadiz</t>
         </is>
       </c>
       <c r="D574" t="inlineStr">
         <is>
-          <t>Osters</t>
+          <t>Real Valladolid</t>
         </is>
       </c>
       <c r="E574" t="n">
-        <v>10.79</v>
+        <v>9.359999999999999</v>
       </c>
       <c r="F574" t="n">
-        <v>0.64</v>
+        <v>-0.02</v>
       </c>
     </row>
     <row r="575">
@@ -15356,128 +15356,128 @@
       </c>
       <c r="B575" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="C575" t="inlineStr">
         <is>
-          <t>Varbergs BoIS</t>
+          <t>Cordoba</t>
         </is>
       </c>
       <c r="D575" t="inlineStr">
         <is>
-          <t>Oddevold</t>
+          <t>Granada</t>
         </is>
       </c>
       <c r="E575" t="n">
-        <v>9.789999999999999</v>
+        <v>9.859999999999999</v>
       </c>
       <c r="F575" t="n">
-        <v>0.5600000000000001</v>
+        <v>2.22</v>
       </c>
     </row>
     <row r="576">
       <c r="A576" s="1" t="n">
-        <v>46265</v>
+        <v>46264</v>
       </c>
       <c r="B576" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="C576" t="inlineStr">
         <is>
-          <t>Fortaleza</t>
+          <t>FC Andorra</t>
         </is>
       </c>
       <c r="D576" t="inlineStr">
         <is>
-          <t>Operario Ferroviario</t>
+          <t>Eibar</t>
         </is>
       </c>
       <c r="E576" t="n">
-        <v>10.5</v>
+        <v>9.15</v>
       </c>
       <c r="F576" t="n">
-        <v>2.05</v>
+        <v>1.49</v>
       </c>
     </row>
     <row r="577">
       <c r="A577" s="1" t="n">
-        <v>46265</v>
+        <v>46264</v>
       </c>
       <c r="B577" t="inlineStr">
         <is>
-          <t>Finland - Veikkausliiga</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="C577" t="inlineStr">
         <is>
-          <t>AC Oulu</t>
+          <t>Mallorca</t>
         </is>
       </c>
       <c r="D577" t="inlineStr">
         <is>
-          <t>SJK</t>
+          <t>Ceuta</t>
         </is>
       </c>
       <c r="E577" t="n">
-        <v>10.49</v>
+        <v>9.52</v>
       </c>
       <c r="F577" t="n">
-        <v>-0.06</v>
+        <v>1.17</v>
       </c>
     </row>
     <row r="578">
       <c r="A578" s="1" t="n">
-        <v>46265</v>
+        <v>46264</v>
       </c>
       <c r="B578" t="inlineStr">
         <is>
-          <t>Finland - Veikkausliiga</t>
+          <t>Sweden - Superettan</t>
         </is>
       </c>
       <c r="C578" t="inlineStr">
         <is>
-          <t>Gnistan</t>
+          <t>Sandvikens IF</t>
         </is>
       </c>
       <c r="D578" t="inlineStr">
         <is>
-          <t>TPS</t>
+          <t>Osters</t>
         </is>
       </c>
       <c r="E578" t="n">
-        <v>10.22</v>
+        <v>10.77</v>
       </c>
       <c r="F578" t="n">
-        <v>0.68</v>
+        <v>0.65</v>
       </c>
     </row>
     <row r="579">
       <c r="A579" s="1" t="n">
-        <v>46265</v>
+        <v>46264</v>
       </c>
       <c r="B579" t="inlineStr">
         <is>
-          <t>Finland - Veikkausliiga</t>
+          <t>Sweden - Superettan</t>
         </is>
       </c>
       <c r="C579" t="inlineStr">
         <is>
-          <t>IFK Mariehamn</t>
+          <t>Varbergs BoIS</t>
         </is>
       </c>
       <c r="D579" t="inlineStr">
         <is>
-          <t>Jaro</t>
+          <t>Oddevold</t>
         </is>
       </c>
       <c r="E579" t="n">
-        <v>10.24</v>
+        <v>9.789999999999999</v>
       </c>
       <c r="F579" t="n">
-        <v>0</v>
+        <v>0.5600000000000001</v>
       </c>
     </row>
     <row r="580">
@@ -15486,24 +15486,24 @@
       </c>
       <c r="B580" t="inlineStr">
         <is>
-          <t>Finland - Veikkausliiga</t>
+          <t>Brazil - Serie B</t>
         </is>
       </c>
       <c r="C580" t="inlineStr">
         <is>
-          <t>Ilves</t>
+          <t>Fortaleza</t>
         </is>
       </c>
       <c r="D580" t="inlineStr">
         <is>
-          <t>HJK Helsinki</t>
+          <t>Operario Ferroviario</t>
         </is>
       </c>
       <c r="E580" t="n">
-        <v>10.87</v>
+        <v>10.5</v>
       </c>
       <c r="F580" t="n">
-        <v>-1.6</v>
+        <v>2.05</v>
       </c>
     </row>
     <row r="581">
@@ -15517,19 +15517,19 @@
       </c>
       <c r="C581" t="inlineStr">
         <is>
-          <t>Inter Turku</t>
+          <t>AC Oulu</t>
         </is>
       </c>
       <c r="D581" t="inlineStr">
         <is>
-          <t>KuPS</t>
+          <t>SJK</t>
         </is>
       </c>
       <c r="E581" t="n">
-        <v>9.710000000000001</v>
+        <v>10.49</v>
       </c>
       <c r="F581" t="n">
-        <v>0.9399999999999999</v>
+        <v>-0.06</v>
       </c>
     </row>
     <row r="582">
@@ -15543,19 +15543,19 @@
       </c>
       <c r="C582" t="inlineStr">
         <is>
-          <t>VPS</t>
+          <t>Gnistan</t>
         </is>
       </c>
       <c r="D582" t="inlineStr">
         <is>
-          <t>FC Lahti</t>
+          <t>TPS</t>
         </is>
       </c>
       <c r="E582" t="n">
-        <v>9.73</v>
+        <v>10.23</v>
       </c>
       <c r="F582" t="n">
-        <v>1.06</v>
+        <v>0.66</v>
       </c>
     </row>
     <row r="583">
@@ -15564,24 +15564,24 @@
       </c>
       <c r="B583" t="inlineStr">
         <is>
-          <t>Romania - Liga 1</t>
+          <t>Finland - Veikkausliiga</t>
         </is>
       </c>
       <c r="C583" t="inlineStr">
         <is>
-          <t>Rapid Bucuresti</t>
+          <t>IFK Mariehamn</t>
         </is>
       </c>
       <c r="D583" t="inlineStr">
         <is>
-          <t>Universitatea Craiova</t>
+          <t>Jaro</t>
         </is>
       </c>
       <c r="E583" t="n">
-        <v>9.789999999999999</v>
+        <v>10.24</v>
       </c>
       <c r="F583" t="n">
-        <v>-0.67</v>
+        <v>0</v>
       </c>
     </row>
     <row r="584">
@@ -15590,75 +15590,179 @@
       </c>
       <c r="B584" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Finland - Veikkausliiga</t>
         </is>
       </c>
       <c r="C584" t="inlineStr">
         <is>
-          <t>Sundsvall</t>
+          <t>Ilves</t>
         </is>
       </c>
       <c r="D584" t="inlineStr">
         <is>
-          <t>Norrby</t>
+          <t>HJK Helsinki</t>
         </is>
       </c>
       <c r="E584" t="n">
-        <v>9.82</v>
+        <v>10.81</v>
       </c>
       <c r="F584" t="n">
-        <v>-0.11</v>
+        <v>-1.58</v>
       </c>
     </row>
     <row r="585">
       <c r="A585" s="1" t="n">
-        <v>46266</v>
+        <v>46265</v>
       </c>
       <c r="B585" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Finland - Veikkausliiga</t>
         </is>
       </c>
       <c r="C585" t="inlineStr">
         <is>
-          <t>Londrina</t>
+          <t>Inter Turku</t>
         </is>
       </c>
       <c r="D585" t="inlineStr">
         <is>
-          <t>Juventude</t>
+          <t>KuPS</t>
         </is>
       </c>
       <c r="E585" t="n">
-        <v>10.5</v>
+        <v>9.710000000000001</v>
       </c>
       <c r="F585" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.9399999999999999</v>
       </c>
     </row>
     <row r="586">
       <c r="A586" s="1" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B586" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C586" t="inlineStr">
+        <is>
+          <t>VPS</t>
+        </is>
+      </c>
+      <c r="D586" t="inlineStr">
+        <is>
+          <t>FC Lahti</t>
+        </is>
+      </c>
+      <c r="E586" t="n">
+        <v>9.73</v>
+      </c>
+      <c r="F586" t="n">
+        <v>1.06</v>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" s="1" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B587" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C587" t="inlineStr">
+        <is>
+          <t>Rapid Bucuresti</t>
+        </is>
+      </c>
+      <c r="D587" t="inlineStr">
+        <is>
+          <t>Universitatea Craiova</t>
+        </is>
+      </c>
+      <c r="E587" t="n">
+        <v>9.82</v>
+      </c>
+      <c r="F587" t="n">
+        <v>-0.67</v>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" s="1" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B588" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C588" t="inlineStr">
+        <is>
+          <t>Sundsvall</t>
+        </is>
+      </c>
+      <c r="D588" t="inlineStr">
+        <is>
+          <t>Norrby</t>
+        </is>
+      </c>
+      <c r="E588" t="n">
+        <v>9.789999999999999</v>
+      </c>
+      <c r="F588" t="n">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" s="1" t="n">
         <v>46266</v>
       </c>
-      <c r="B586" t="inlineStr">
+      <c r="B589" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C589" t="inlineStr">
+        <is>
+          <t>Londrina</t>
+        </is>
+      </c>
+      <c r="D589" t="inlineStr">
+        <is>
+          <t>Juventude</t>
+        </is>
+      </c>
+      <c r="E589" t="n">
+        <v>10.6</v>
+      </c>
+      <c r="F589" t="n">
+        <v>0.52</v>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" s="1" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B590" t="inlineStr">
         <is>
           <t>Sweden - Superettan</t>
         </is>
       </c>
-      <c r="C586" t="inlineStr">
+      <c r="C590" t="inlineStr">
         <is>
           <t>Helsingborgs</t>
         </is>
       </c>
-      <c r="D586" t="inlineStr">
+      <c r="D590" t="inlineStr">
         <is>
           <t>Orebro SK</t>
         </is>
       </c>
-      <c r="E586" t="n">
+      <c r="E590" t="n">
         <v>10.26</v>
       </c>
-      <c r="F586" t="n">
+      <c r="F590" t="n">
         <v>0.45</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily scrape output - 2026-08-31
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F590"/>
+  <dimension ref="A1:F592"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15526,10 +15526,10 @@
         </is>
       </c>
       <c r="E581" t="n">
-        <v>10.49</v>
+        <v>10.26</v>
       </c>
       <c r="F581" t="n">
-        <v>-0.06</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="582">
@@ -15552,10 +15552,10 @@
         </is>
       </c>
       <c r="E582" t="n">
-        <v>10.23</v>
+        <v>10.14</v>
       </c>
       <c r="F582" t="n">
-        <v>0.66</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="583">
@@ -15578,10 +15578,10 @@
         </is>
       </c>
       <c r="E583" t="n">
-        <v>10.24</v>
+        <v>10.2</v>
       </c>
       <c r="F583" t="n">
-        <v>0</v>
+        <v>0.38</v>
       </c>
     </row>
     <row r="584">
@@ -15604,7 +15604,7 @@
         </is>
       </c>
       <c r="E584" t="n">
-        <v>10.81</v>
+        <v>10.74</v>
       </c>
       <c r="F584" t="n">
         <v>-1.58</v>
@@ -15630,10 +15630,10 @@
         </is>
       </c>
       <c r="E585" t="n">
-        <v>9.710000000000001</v>
+        <v>9.69</v>
       </c>
       <c r="F585" t="n">
-        <v>0.9399999999999999</v>
+        <v>1.38</v>
       </c>
     </row>
     <row r="586">
@@ -15685,7 +15685,7 @@
         <v>9.82</v>
       </c>
       <c r="F587" t="n">
-        <v>-0.67</v>
+        <v>-0.49</v>
       </c>
     </row>
     <row r="588">
@@ -15694,75 +15694,127 @@
       </c>
       <c r="B588" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="C588" t="inlineStr">
         <is>
-          <t>Sundsvall</t>
+          <t>Burgos</t>
         </is>
       </c>
       <c r="D588" t="inlineStr">
         <is>
-          <t>Norrby</t>
+          <t>Real Sociedad II</t>
         </is>
       </c>
       <c r="E588" t="n">
-        <v>9.789999999999999</v>
+        <v>9.25</v>
       </c>
       <c r="F588" t="n">
-        <v>0.11</v>
+        <v>1.84</v>
       </c>
     </row>
     <row r="589">
       <c r="A589" s="1" t="n">
-        <v>46266</v>
+        <v>46265</v>
       </c>
       <c r="B589" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="C589" t="inlineStr">
         <is>
-          <t>Londrina</t>
+          <t>Celta Vigo II</t>
         </is>
       </c>
       <c r="D589" t="inlineStr">
         <is>
-          <t>Juventude</t>
+          <t>Castellon</t>
         </is>
       </c>
       <c r="E589" t="n">
-        <v>10.6</v>
+        <v>9.18</v>
       </c>
       <c r="F589" t="n">
-        <v>0.52</v>
+        <v>-1.43</v>
       </c>
     </row>
     <row r="590">
       <c r="A590" s="1" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B590" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C590" t="inlineStr">
+        <is>
+          <t>Sundsvall</t>
+        </is>
+      </c>
+      <c r="D590" t="inlineStr">
+        <is>
+          <t>Norrby</t>
+        </is>
+      </c>
+      <c r="E590" t="n">
+        <v>9.789999999999999</v>
+      </c>
+      <c r="F590" t="n">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" s="1" t="n">
         <v>46266</v>
       </c>
-      <c r="B590" t="inlineStr">
+      <c r="B591" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C591" t="inlineStr">
+        <is>
+          <t>Londrina</t>
+        </is>
+      </c>
+      <c r="D591" t="inlineStr">
+        <is>
+          <t>Juventude</t>
+        </is>
+      </c>
+      <c r="E591" t="n">
+        <v>10.6</v>
+      </c>
+      <c r="F591" t="n">
+        <v>0.52</v>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" s="1" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B592" t="inlineStr">
         <is>
           <t>Sweden - Superettan</t>
         </is>
       </c>
-      <c r="C590" t="inlineStr">
+      <c r="C592" t="inlineStr">
         <is>
           <t>Helsingborgs</t>
         </is>
       </c>
-      <c r="D590" t="inlineStr">
+      <c r="D592" t="inlineStr">
         <is>
           <t>Orebro SK</t>
         </is>
       </c>
-      <c r="E590" t="n">
+      <c r="E592" t="n">
         <v>10.26</v>
       </c>
-      <c r="F590" t="n">
+      <c r="F592" t="n">
         <v>0.45</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily scrape output - 2026-09-01
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -15786,10 +15786,10 @@
         </is>
       </c>
       <c r="E591" t="n">
-        <v>10.6</v>
+        <v>10.56</v>
       </c>
       <c r="F591" t="n">
-        <v>0.52</v>
+        <v>0.47</v>
       </c>
     </row>
     <row r="592">
@@ -15812,7 +15812,7 @@
         </is>
       </c>
       <c r="E592" t="n">
-        <v>10.26</v>
+        <v>10.28</v>
       </c>
       <c r="F592" t="n">
         <v>0.45</v>

</xml_diff>

<commit_message>
Daily scrape output - 2026-09-03
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F592"/>
+  <dimension ref="A1:F603"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15818,6 +15818,292 @@
         <v>0.45</v>
       </c>
     </row>
+    <row r="593">
+      <c r="A593" s="1" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B593" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C593" t="inlineStr">
+        <is>
+          <t>Nautico</t>
+        </is>
+      </c>
+      <c r="D593" t="inlineStr">
+        <is>
+          <t>Botafogo SP</t>
+        </is>
+      </c>
+      <c r="E593" t="n">
+        <v>10.96</v>
+      </c>
+      <c r="F593" t="n">
+        <v>2.05</v>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" s="1" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B594" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C594" t="inlineStr">
+        <is>
+          <t>Lech Poznan</t>
+        </is>
+      </c>
+      <c r="D594" t="inlineStr">
+        <is>
+          <t>Jagiellonia Bialystok</t>
+        </is>
+      </c>
+      <c r="E594" t="n">
+        <v>10.51</v>
+      </c>
+      <c r="F594" t="n">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" s="1" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B595" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C595" t="inlineStr">
+        <is>
+          <t>Rakow Czestochowa</t>
+        </is>
+      </c>
+      <c r="D595" t="inlineStr">
+        <is>
+          <t>Gornik Zabrze</t>
+        </is>
+      </c>
+      <c r="E595" t="n">
+        <v>9.869999999999999</v>
+      </c>
+      <c r="F595" t="n">
+        <v>0.45</v>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" s="1" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B596" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C596" t="inlineStr">
+        <is>
+          <t>Las Palmas</t>
+        </is>
+      </c>
+      <c r="D596" t="inlineStr">
+        <is>
+          <t>Leganes</t>
+        </is>
+      </c>
+      <c r="E596" t="n">
+        <v>9</v>
+      </c>
+      <c r="F596" t="n">
+        <v>1.56</v>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" s="1" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B597" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C597" t="inlineStr">
+        <is>
+          <t>Ceuta</t>
+        </is>
+      </c>
+      <c r="D597" t="inlineStr">
+        <is>
+          <t>Celta Vigo II</t>
+        </is>
+      </c>
+      <c r="E597" t="n">
+        <v>8.470000000000001</v>
+      </c>
+      <c r="F597" t="n">
+        <v>1.37</v>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" s="1" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B598" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C598" t="inlineStr">
+        <is>
+          <t>Eldense</t>
+        </is>
+      </c>
+      <c r="D598" t="inlineStr">
+        <is>
+          <t>Mallorca</t>
+        </is>
+      </c>
+      <c r="E598" t="n">
+        <v>9.58</v>
+      </c>
+      <c r="F598" t="n">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" s="1" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B599" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C599" t="inlineStr">
+        <is>
+          <t>Real Sociedad II</t>
+        </is>
+      </c>
+      <c r="D599" t="inlineStr">
+        <is>
+          <t>Tenerife</t>
+        </is>
+      </c>
+      <c r="E599" t="n">
+        <v>9.640000000000001</v>
+      </c>
+      <c r="F599" t="n">
+        <v>0.16</v>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" s="1" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B600" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C600" t="inlineStr">
+        <is>
+          <t>Real Valladolid</t>
+        </is>
+      </c>
+      <c r="D600" t="inlineStr">
+        <is>
+          <t>FC Andorra</t>
+        </is>
+      </c>
+      <c r="E600" t="n">
+        <v>9</v>
+      </c>
+      <c r="F600" t="n">
+        <v>0.58</v>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" s="1" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B601" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C601" t="inlineStr">
+        <is>
+          <t>Sporting Gijon</t>
+        </is>
+      </c>
+      <c r="D601" t="inlineStr">
+        <is>
+          <t>Girona</t>
+        </is>
+      </c>
+      <c r="E601" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="F601" t="n">
+        <v>-0.41</v>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" s="1" t="n">
+        <v>46271</v>
+      </c>
+      <c r="B602" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C602" t="inlineStr">
+        <is>
+          <t>Almeria</t>
+        </is>
+      </c>
+      <c r="D602" t="inlineStr">
+        <is>
+          <t>Cadiz</t>
+        </is>
+      </c>
+      <c r="E602" t="n">
+        <v>9.550000000000001</v>
+      </c>
+      <c r="F602" t="n">
+        <v>2.2</v>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" s="1" t="n">
+        <v>46271</v>
+      </c>
+      <c r="B603" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C603" t="inlineStr">
+        <is>
+          <t>Real Oviedo</t>
+        </is>
+      </c>
+      <c r="D603" t="inlineStr">
+        <is>
+          <t>Burgos</t>
+        </is>
+      </c>
+      <c r="E603" t="n">
+        <v>9.09</v>
+      </c>
+      <c r="F603" t="n">
+        <v>1.6</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily scrape output - 2026-09-04
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F603"/>
+  <dimension ref="A1:F656"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15902,206 +15902,1584 @@
       </c>
       <c r="B596" t="inlineStr">
         <is>
-          <t>Spain - Segunda</t>
+          <t>Brazil - Serie B</t>
         </is>
       </c>
       <c r="C596" t="inlineStr">
         <is>
-          <t>Las Palmas</t>
+          <t>Athletic Club</t>
         </is>
       </c>
       <c r="D596" t="inlineStr">
         <is>
-          <t>Leganes</t>
+          <t>Vila Nova</t>
         </is>
       </c>
       <c r="E596" t="n">
-        <v>9</v>
+        <v>10.22</v>
       </c>
       <c r="F596" t="n">
-        <v>1.56</v>
+        <v>0.33</v>
       </c>
     </row>
     <row r="597">
       <c r="A597" s="1" t="n">
-        <v>46270</v>
+        <v>46269</v>
       </c>
       <c r="B597" t="inlineStr">
         <is>
-          <t>Spain - Segunda</t>
+          <t>Brazil - Serie B</t>
         </is>
       </c>
       <c r="C597" t="inlineStr">
         <is>
-          <t>Ceuta</t>
+          <t>Criciuma</t>
         </is>
       </c>
       <c r="D597" t="inlineStr">
         <is>
-          <t>Celta Vigo II</t>
+          <t>Cuiaba</t>
         </is>
       </c>
       <c r="E597" t="n">
-        <v>8.470000000000001</v>
+        <v>10.26</v>
       </c>
       <c r="F597" t="n">
-        <v>1.37</v>
+        <v>2.07</v>
       </c>
     </row>
     <row r="598">
       <c r="A598" s="1" t="n">
-        <v>46270</v>
+        <v>46269</v>
       </c>
       <c r="B598" t="inlineStr">
         <is>
-          <t>Spain - Segunda</t>
+          <t>Finland - Ykkosliiga</t>
         </is>
       </c>
       <c r="C598" t="inlineStr">
         <is>
-          <t>Eldense</t>
+          <t>JIPPO</t>
         </is>
       </c>
       <c r="D598" t="inlineStr">
         <is>
-          <t>Mallorca</t>
+          <t>KTP</t>
         </is>
       </c>
       <c r="E598" t="n">
-        <v>9.58</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="F598" t="n">
-        <v>0.15</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="599">
       <c r="A599" s="1" t="n">
-        <v>46270</v>
+        <v>46269</v>
       </c>
       <c r="B599" t="inlineStr">
         <is>
-          <t>Spain - Segunda</t>
+          <t>Finland - Ykkosliiga</t>
         </is>
       </c>
       <c r="C599" t="inlineStr">
         <is>
-          <t>Real Sociedad II</t>
+          <t>PK-35</t>
         </is>
       </c>
       <c r="D599" t="inlineStr">
         <is>
-          <t>Tenerife</t>
+          <t>EIF</t>
         </is>
       </c>
       <c r="E599" t="n">
-        <v>9.640000000000001</v>
+        <v>10.71</v>
       </c>
       <c r="F599" t="n">
-        <v>0.16</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="600">
       <c r="A600" s="1" t="n">
-        <v>46270</v>
+        <v>46269</v>
       </c>
       <c r="B600" t="inlineStr">
         <is>
-          <t>Spain - Segunda</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="C600" t="inlineStr">
         <is>
-          <t>Real Valladolid</t>
+          <t>Nieciecza</t>
         </is>
       </c>
       <c r="D600" t="inlineStr">
         <is>
-          <t>FC Andorra</t>
+          <t>Lechia Gdansk</t>
         </is>
       </c>
       <c r="E600" t="n">
-        <v>9</v>
+        <v>10.18</v>
       </c>
       <c r="F600" t="n">
-        <v>0.58</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="601">
       <c r="A601" s="1" t="n">
-        <v>46270</v>
+        <v>46269</v>
       </c>
       <c r="B601" t="inlineStr">
         <is>
-          <t>Spain - Segunda</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="C601" t="inlineStr">
         <is>
-          <t>Sporting Gijon</t>
+          <t>Pogon Grodzisk Mazowiecki</t>
         </is>
       </c>
       <c r="D601" t="inlineStr">
         <is>
-          <t>Girona</t>
+          <t>Warta Poznan</t>
         </is>
       </c>
       <c r="E601" t="n">
-        <v>9.199999999999999</v>
+        <v>10.58</v>
       </c>
       <c r="F601" t="n">
-        <v>-0.41</v>
+        <v>0.07000000000000001</v>
       </c>
     </row>
     <row r="602">
       <c r="A602" s="1" t="n">
-        <v>46271</v>
+        <v>46269</v>
       </c>
       <c r="B602" t="inlineStr">
         <is>
-          <t>Spain - Segunda</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C602" t="inlineStr">
         <is>
-          <t>Almeria</t>
+          <t>Piast Gliwice</t>
         </is>
       </c>
       <c r="D602" t="inlineStr">
         <is>
-          <t>Cadiz</t>
+          <t>GKS Katowice</t>
         </is>
       </c>
       <c r="E602" t="n">
-        <v>9.550000000000001</v>
+        <v>9.869999999999999</v>
       </c>
       <c r="F602" t="n">
-        <v>2.2</v>
+        <v>0.93</v>
       </c>
     </row>
     <row r="603">
       <c r="A603" s="1" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B603" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C603" t="inlineStr">
+        <is>
+          <t>CFR Cluj</t>
+        </is>
+      </c>
+      <c r="D603" t="inlineStr">
+        <is>
+          <t>Farul Constanta</t>
+        </is>
+      </c>
+      <c r="E603" t="n">
+        <v>9.470000000000001</v>
+      </c>
+      <c r="F603" t="n">
+        <v>1.57</v>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" s="1" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B604" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C604" t="inlineStr">
+        <is>
+          <t>Las Palmas</t>
+        </is>
+      </c>
+      <c r="D604" t="inlineStr">
+        <is>
+          <t>Leganes</t>
+        </is>
+      </c>
+      <c r="E604" t="n">
+        <v>9</v>
+      </c>
+      <c r="F604" t="n">
+        <v>1.91</v>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" s="1" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B605" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C605" t="inlineStr">
+        <is>
+          <t>Norrkoping</t>
+        </is>
+      </c>
+      <c r="D605" t="inlineStr">
+        <is>
+          <t>Ljungskile</t>
+        </is>
+      </c>
+      <c r="E605" t="n">
+        <v>10.01</v>
+      </c>
+      <c r="F605" t="n">
+        <v>2.23</v>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" s="1" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B606" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C606" t="inlineStr">
+        <is>
+          <t>Osters</t>
+        </is>
+      </c>
+      <c r="D606" t="inlineStr">
+        <is>
+          <t>Nordic United</t>
+        </is>
+      </c>
+      <c r="E606" t="n">
+        <v>10.04</v>
+      </c>
+      <c r="F606" t="n">
+        <v>-0.32</v>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" s="1" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B607" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C607" t="inlineStr">
+        <is>
+          <t>CRB</t>
+        </is>
+      </c>
+      <c r="D607" t="inlineStr">
+        <is>
+          <t>America Mineiro</t>
+        </is>
+      </c>
+      <c r="E607" t="n">
+        <v>10.67</v>
+      </c>
+      <c r="F607" t="n">
+        <v>1.96</v>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" s="1" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B608" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C608" t="inlineStr">
+        <is>
+          <t>Ceara</t>
+        </is>
+      </c>
+      <c r="D608" t="inlineStr">
+        <is>
+          <t>Sport Recife</t>
+        </is>
+      </c>
+      <c r="E608" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="F608" t="n">
+        <v>1.84</v>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" s="1" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B609" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C609" t="inlineStr">
+        <is>
+          <t>Goias</t>
+        </is>
+      </c>
+      <c r="D609" t="inlineStr">
+        <is>
+          <t>Fortaleza</t>
+        </is>
+      </c>
+      <c r="E609" t="n">
+        <v>10.49</v>
+      </c>
+      <c r="F609" t="n">
+        <v>0.54</v>
+      </c>
+    </row>
+    <row r="610">
+      <c r="A610" s="1" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B610" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C610" t="inlineStr">
+        <is>
+          <t>Gremio Novorizontino</t>
+        </is>
+      </c>
+      <c r="D610" t="inlineStr">
+        <is>
+          <t>Avai</t>
+        </is>
+      </c>
+      <c r="E610" t="n">
+        <v>10.99</v>
+      </c>
+      <c r="F610" t="n">
+        <v>2.97</v>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" s="1" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B611" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C611" t="inlineStr">
+        <is>
+          <t>Juventude</t>
+        </is>
+      </c>
+      <c r="D611" t="inlineStr">
+        <is>
+          <t>Atletico Goianiense</t>
+        </is>
+      </c>
+      <c r="E611" t="n">
+        <v>9.99</v>
+      </c>
+      <c r="F611" t="n">
+        <v>1.06</v>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" s="1" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B612" t="inlineStr">
+        <is>
+          <t>Iceland - 1. Deild</t>
+        </is>
+      </c>
+      <c r="C612" t="inlineStr">
+        <is>
+          <t>Aegir</t>
+        </is>
+      </c>
+      <c r="D612" t="inlineStr">
+        <is>
+          <t>UMF Grindavik</t>
+        </is>
+      </c>
+      <c r="E612" t="n">
+        <v>11.41</v>
+      </c>
+      <c r="F612" t="n">
+        <v>-1.83</v>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" s="1" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B613" t="inlineStr">
+        <is>
+          <t>Iceland - 1. Deild</t>
+        </is>
+      </c>
+      <c r="C613" t="inlineStr">
+        <is>
+          <t>HK Kopavogur</t>
+        </is>
+      </c>
+      <c r="D613" t="inlineStr">
+        <is>
+          <t>Fylkir</t>
+        </is>
+      </c>
+      <c r="E613" t="n">
+        <v>11.66</v>
+      </c>
+      <c r="F613" t="n">
+        <v>-0.37</v>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" s="1" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B614" t="inlineStr">
+        <is>
+          <t>Iceland - 1. Deild</t>
+        </is>
+      </c>
+      <c r="C614" t="inlineStr">
+        <is>
+          <t>IR Reykjavik</t>
+        </is>
+      </c>
+      <c r="D614" t="inlineStr">
+        <is>
+          <t>Leiknir Reykjavik</t>
+        </is>
+      </c>
+      <c r="E614" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="F614" t="n">
+        <v>1.07</v>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" s="1" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B615" t="inlineStr">
+        <is>
+          <t>Iceland - 1. Deild</t>
+        </is>
+      </c>
+      <c r="C615" t="inlineStr">
+        <is>
+          <t>UMF Njardvik</t>
+        </is>
+      </c>
+      <c r="D615" t="inlineStr">
+        <is>
+          <t>Afturelding</t>
+        </is>
+      </c>
+      <c r="E615" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="F615" t="n">
+        <v>0.06</v>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" s="1" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B616" t="inlineStr">
+        <is>
+          <t>Iceland - 1. Deild</t>
+        </is>
+      </c>
+      <c r="C616" t="inlineStr">
+        <is>
+          <t>Vestri</t>
+        </is>
+      </c>
+      <c r="D616" t="inlineStr">
+        <is>
+          <t>Throttur Reykjavik</t>
+        </is>
+      </c>
+      <c r="E616" t="n">
+        <v>11.01</v>
+      </c>
+      <c r="F616" t="n">
+        <v>-1.68</v>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" s="1" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B617" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C617" t="inlineStr">
+        <is>
+          <t>Asane Fotball</t>
+        </is>
+      </c>
+      <c r="D617" t="inlineStr">
+        <is>
+          <t>Hodd</t>
+        </is>
+      </c>
+      <c r="E617" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="F617" t="n">
+        <v>0.09</v>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" s="1" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B618" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C618" t="inlineStr">
+        <is>
+          <t>Haugesund</t>
+        </is>
+      </c>
+      <c r="D618" t="inlineStr">
+        <is>
+          <t>Sogndal</t>
+        </is>
+      </c>
+      <c r="E618" t="n">
+        <v>11.16</v>
+      </c>
+      <c r="F618" t="n">
+        <v>2.49</v>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" s="1" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B619" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C619" t="inlineStr">
+        <is>
+          <t>Kongsvinger</t>
+        </is>
+      </c>
+      <c r="D619" t="inlineStr">
+        <is>
+          <t>Raufoss</t>
+        </is>
+      </c>
+      <c r="E619" t="n">
+        <v>11.77</v>
+      </c>
+      <c r="F619" t="n">
+        <v>3.57</v>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" s="1" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B620" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C620" t="inlineStr">
+        <is>
+          <t>Odd BK</t>
+        </is>
+      </c>
+      <c r="D620" t="inlineStr">
+        <is>
+          <t>Stromsgodset</t>
+        </is>
+      </c>
+      <c r="E620" t="n">
+        <v>11.12</v>
+      </c>
+      <c r="F620" t="n">
+        <v>-0.97</v>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" s="1" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B621" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C621" t="inlineStr">
+        <is>
+          <t>Sandnes Ulf</t>
+        </is>
+      </c>
+      <c r="D621" t="inlineStr">
+        <is>
+          <t>Ranheim</t>
+        </is>
+      </c>
+      <c r="E621" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="F621" t="n">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" s="1" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B622" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C622" t="inlineStr">
+        <is>
+          <t>Stabaek</t>
+        </is>
+      </c>
+      <c r="D622" t="inlineStr">
+        <is>
+          <t>Moss</t>
+        </is>
+      </c>
+      <c r="E622" t="n">
+        <v>11.73</v>
+      </c>
+      <c r="F622" t="n">
+        <v>3.4</v>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" s="1" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B623" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C623" t="inlineStr">
+        <is>
+          <t>Strommen</t>
+        </is>
+      </c>
+      <c r="D623" t="inlineStr">
+        <is>
+          <t>Bryne</t>
+        </is>
+      </c>
+      <c r="E623" t="n">
+        <v>10.51</v>
+      </c>
+      <c r="F623" t="n">
+        <v>-0.64</v>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" s="1" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B624" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C624" t="inlineStr">
+        <is>
+          <t>Miedz Legnica</t>
+        </is>
+      </c>
+      <c r="D624" t="inlineStr">
+        <is>
+          <t>Chrobry Glogow</t>
+        </is>
+      </c>
+      <c r="E624" t="n">
+        <v>10.67</v>
+      </c>
+      <c r="F624" t="n">
+        <v>1.86</v>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" s="1" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B625" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C625" t="inlineStr">
+        <is>
+          <t>Stal Mielec</t>
+        </is>
+      </c>
+      <c r="D625" t="inlineStr">
+        <is>
+          <t>Odra Opole</t>
+        </is>
+      </c>
+      <c r="E625" t="n">
+        <v>10.55</v>
+      </c>
+      <c r="F625" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" s="1" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B626" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C626" t="inlineStr">
+        <is>
+          <t>Stal Rzeszow</t>
+        </is>
+      </c>
+      <c r="D626" t="inlineStr">
+        <is>
+          <t>Polonia Warsaw</t>
+        </is>
+      </c>
+      <c r="E626" t="n">
+        <v>11.29</v>
+      </c>
+      <c r="F626" t="n">
+        <v>-0.84</v>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" s="1" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B627" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C627" t="inlineStr">
+        <is>
+          <t>Motor Lublin</t>
+        </is>
+      </c>
+      <c r="D627" t="inlineStr">
+        <is>
+          <t>Legia Warsaw</t>
+        </is>
+      </c>
+      <c r="E627" t="n">
+        <v>9.76</v>
+      </c>
+      <c r="F627" t="n">
+        <v>-1.07</v>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" s="1" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B628" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C628" t="inlineStr">
+        <is>
+          <t>Widzew Lodz</t>
+        </is>
+      </c>
+      <c r="D628" t="inlineStr">
+        <is>
+          <t>Radomiak Radom</t>
+        </is>
+      </c>
+      <c r="E628" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="F628" t="n">
+        <v>2.53</v>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" s="1" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B629" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C629" t="inlineStr">
+        <is>
+          <t>Dinamo Bucuresti</t>
+        </is>
+      </c>
+      <c r="D629" t="inlineStr">
+        <is>
+          <t>FCSB</t>
+        </is>
+      </c>
+      <c r="E629" t="n">
+        <v>9.640000000000001</v>
+      </c>
+      <c r="F629" t="n">
+        <v>0.65</v>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" s="1" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B630" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C630" t="inlineStr">
+        <is>
+          <t>UTA Arad</t>
+        </is>
+      </c>
+      <c r="D630" t="inlineStr">
+        <is>
+          <t>Csikszereda</t>
+        </is>
+      </c>
+      <c r="E630" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="F630" t="n">
+        <v>3.07</v>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" s="1" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B631" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C631" t="inlineStr">
+        <is>
+          <t>Ceuta</t>
+        </is>
+      </c>
+      <c r="D631" t="inlineStr">
+        <is>
+          <t>Celta Vigo II</t>
+        </is>
+      </c>
+      <c r="E631" t="n">
+        <v>8.470000000000001</v>
+      </c>
+      <c r="F631" t="n">
+        <v>1.37</v>
+      </c>
+    </row>
+    <row r="632">
+      <c r="A632" s="1" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B632" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C632" t="inlineStr">
+        <is>
+          <t>Eldense</t>
+        </is>
+      </c>
+      <c r="D632" t="inlineStr">
+        <is>
+          <t>Mallorca</t>
+        </is>
+      </c>
+      <c r="E632" t="n">
+        <v>9.57</v>
+      </c>
+      <c r="F632" t="n">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="633">
+      <c r="A633" s="1" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B633" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C633" t="inlineStr">
+        <is>
+          <t>Real Sociedad II</t>
+        </is>
+      </c>
+      <c r="D633" t="inlineStr">
+        <is>
+          <t>Tenerife</t>
+        </is>
+      </c>
+      <c r="E633" t="n">
+        <v>9.640000000000001</v>
+      </c>
+      <c r="F633" t="n">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" s="1" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B634" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C634" t="inlineStr">
+        <is>
+          <t>Real Valladolid</t>
+        </is>
+      </c>
+      <c r="D634" t="inlineStr">
+        <is>
+          <t>FC Andorra</t>
+        </is>
+      </c>
+      <c r="E634" t="n">
+        <v>9</v>
+      </c>
+      <c r="F634" t="n">
+        <v>0.58</v>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" s="1" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B635" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C635" t="inlineStr">
+        <is>
+          <t>Sporting Gijon</t>
+        </is>
+      </c>
+      <c r="D635" t="inlineStr">
+        <is>
+          <t>Girona</t>
+        </is>
+      </c>
+      <c r="E635" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="F635" t="n">
+        <v>-0.41</v>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" s="1" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B636" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C636" t="inlineStr">
+        <is>
+          <t>Brage</t>
+        </is>
+      </c>
+      <c r="D636" t="inlineStr">
+        <is>
+          <t>Sundsvall</t>
+        </is>
+      </c>
+      <c r="E636" t="n">
+        <v>10.46</v>
+      </c>
+      <c r="F636" t="n">
+        <v>1.65</v>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" s="1" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B637" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C637" t="inlineStr">
+        <is>
+          <t>Helsingborgs</t>
+        </is>
+      </c>
+      <c r="D637" t="inlineStr">
+        <is>
+          <t>Sandvikens IF</t>
+        </is>
+      </c>
+      <c r="E637" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="F637" t="n">
+        <v>1.06</v>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" s="1" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B638" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C638" t="inlineStr">
+        <is>
+          <t>Norrby</t>
+        </is>
+      </c>
+      <c r="D638" t="inlineStr">
+        <is>
+          <t>Landskrona</t>
+        </is>
+      </c>
+      <c r="E638" t="n">
+        <v>10.17</v>
+      </c>
+      <c r="F638" t="n">
+        <v>-1.06</v>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" s="1" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B639" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C639" t="inlineStr">
+        <is>
+          <t>Oddevold</t>
+        </is>
+      </c>
+      <c r="D639" t="inlineStr">
+        <is>
+          <t>Falkenbergs</t>
+        </is>
+      </c>
+      <c r="E639" t="n">
+        <v>9.16</v>
+      </c>
+      <c r="F639" t="n">
+        <v>1.51</v>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" s="1" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B640" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C640" t="inlineStr">
+        <is>
+          <t>Varnamo</t>
+        </is>
+      </c>
+      <c r="D640" t="inlineStr">
+        <is>
+          <t>Varbergs BoIS</t>
+        </is>
+      </c>
+      <c r="E640" t="n">
+        <v>9.73</v>
+      </c>
+      <c r="F640" t="n">
+        <v>-0.47</v>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" s="1" t="n">
         <v>46271</v>
       </c>
-      <c r="B603" t="inlineStr">
+      <c r="B641" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C641" t="inlineStr">
+        <is>
+          <t>Londrina</t>
+        </is>
+      </c>
+      <c r="D641" t="inlineStr">
+        <is>
+          <t>Operario Ferroviario</t>
+        </is>
+      </c>
+      <c r="E641" t="n">
+        <v>10.45</v>
+      </c>
+      <c r="F641" t="n">
+        <v>1.02</v>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" s="1" t="n">
+        <v>46271</v>
+      </c>
+      <c r="B642" t="inlineStr">
+        <is>
+          <t>Finland - Ykkosliiga</t>
+        </is>
+      </c>
+      <c r="C642" t="inlineStr">
+        <is>
+          <t>FC Haka</t>
+        </is>
+      </c>
+      <c r="D642" t="inlineStr">
+        <is>
+          <t>Mikkelin Palloilijat</t>
+        </is>
+      </c>
+      <c r="E642" t="n">
+        <v>10.84</v>
+      </c>
+      <c r="F642" t="n">
+        <v>3.67</v>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" s="1" t="n">
+        <v>46271</v>
+      </c>
+      <c r="B643" t="inlineStr">
+        <is>
+          <t>Finland - Ykkosliiga</t>
+        </is>
+      </c>
+      <c r="C643" t="inlineStr">
+        <is>
+          <t>SJK Akatemia</t>
+        </is>
+      </c>
+      <c r="D643" t="inlineStr">
+        <is>
+          <t>JaPS</t>
+        </is>
+      </c>
+      <c r="E643" t="n">
+        <v>10.61</v>
+      </c>
+      <c r="F643" t="n">
+        <v>-0.5600000000000001</v>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" s="1" t="n">
+        <v>46271</v>
+      </c>
+      <c r="B644" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C644" t="inlineStr">
+        <is>
+          <t>Lyn</t>
+        </is>
+      </c>
+      <c r="D644" t="inlineStr">
+        <is>
+          <t>Egersunds</t>
+        </is>
+      </c>
+      <c r="E644" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="F644" t="n">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" s="1" t="n">
+        <v>46271</v>
+      </c>
+      <c r="B645" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C645" t="inlineStr">
+        <is>
+          <t>Pogon Siedlce</t>
+        </is>
+      </c>
+      <c r="D645" t="inlineStr">
+        <is>
+          <t>Puszcza Niepolomice</t>
+        </is>
+      </c>
+      <c r="E645" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="F645" t="n">
+        <v>-0.17</v>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" s="1" t="n">
+        <v>46271</v>
+      </c>
+      <c r="B646" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C646" t="inlineStr">
+        <is>
+          <t>Cracovia Krakow</t>
+        </is>
+      </c>
+      <c r="D646" t="inlineStr">
+        <is>
+          <t>Gornik Zabrze</t>
+        </is>
+      </c>
+      <c r="E646" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="F646" t="n">
+        <v>0.38</v>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" s="1" t="n">
+        <v>46271</v>
+      </c>
+      <c r="B647" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C647" t="inlineStr">
+        <is>
+          <t>Lech Poznan</t>
+        </is>
+      </c>
+      <c r="D647" t="inlineStr">
+        <is>
+          <t>Rakow Czestochowa</t>
+        </is>
+      </c>
+      <c r="E647" t="n">
+        <v>10.26</v>
+      </c>
+      <c r="F647" t="n">
+        <v>2.85</v>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" s="1" t="n">
+        <v>46271</v>
+      </c>
+      <c r="B648" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C648" t="inlineStr">
+        <is>
+          <t>Otelul Galati</t>
+        </is>
+      </c>
+      <c r="D648" t="inlineStr">
+        <is>
+          <t>Rapid Bucuresti</t>
+        </is>
+      </c>
+      <c r="E648" t="n">
+        <v>9.41</v>
+      </c>
+      <c r="F648" t="n">
+        <v>0.32</v>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" s="1" t="n">
+        <v>46271</v>
+      </c>
+      <c r="B649" t="inlineStr">
         <is>
           <t>Spain - Segunda</t>
         </is>
       </c>
-      <c r="C603" t="inlineStr">
+      <c r="C649" t="inlineStr">
+        <is>
+          <t>Almeria</t>
+        </is>
+      </c>
+      <c r="D649" t="inlineStr">
+        <is>
+          <t>Cadiz</t>
+        </is>
+      </c>
+      <c r="E649" t="n">
+        <v>9.550000000000001</v>
+      </c>
+      <c r="F649" t="n">
+        <v>2.2</v>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" s="1" t="n">
+        <v>46271</v>
+      </c>
+      <c r="B650" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C650" t="inlineStr">
+        <is>
+          <t>Castellon</t>
+        </is>
+      </c>
+      <c r="D650" t="inlineStr">
+        <is>
+          <t>Albacete</t>
+        </is>
+      </c>
+      <c r="E650" t="n">
+        <v>10.32</v>
+      </c>
+      <c r="F650" t="n">
+        <v>2.53</v>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" s="1" t="n">
+        <v>46271</v>
+      </c>
+      <c r="B651" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C651" t="inlineStr">
+        <is>
+          <t>Eibar</t>
+        </is>
+      </c>
+      <c r="D651" t="inlineStr">
+        <is>
+          <t>Granada</t>
+        </is>
+      </c>
+      <c r="E651" t="n">
+        <v>9</v>
+      </c>
+      <c r="F651" t="n">
+        <v>1.86</v>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" s="1" t="n">
+        <v>46271</v>
+      </c>
+      <c r="B652" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C652" t="inlineStr">
         <is>
           <t>Real Oviedo</t>
         </is>
       </c>
-      <c r="D603" t="inlineStr">
+      <c r="D652" t="inlineStr">
         <is>
           <t>Burgos</t>
         </is>
       </c>
-      <c r="E603" t="n">
+      <c r="E652" t="n">
         <v>9.09</v>
       </c>
-      <c r="F603" t="n">
+      <c r="F652" t="n">
         <v>1.6</v>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" s="1" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B653" t="inlineStr">
+        <is>
+          <t>Finland - Ykkosliiga</t>
+        </is>
+      </c>
+      <c r="C653" t="inlineStr">
+        <is>
+          <t>HJK Klubi 04</t>
+        </is>
+      </c>
+      <c r="D653" t="inlineStr">
+        <is>
+          <t>KaPa</t>
+        </is>
+      </c>
+      <c r="E653" t="n">
+        <v>10.53</v>
+      </c>
+      <c r="F653" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" s="1" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B654" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C654" t="inlineStr">
+        <is>
+          <t>Pogon Szczecin</t>
+        </is>
+      </c>
+      <c r="D654" t="inlineStr">
+        <is>
+          <t>Wisla Plock</t>
+        </is>
+      </c>
+      <c r="E654" t="n">
+        <v>10.43</v>
+      </c>
+      <c r="F654" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" s="1" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B655" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C655" t="inlineStr">
+        <is>
+          <t>Universitatea Craiova</t>
+        </is>
+      </c>
+      <c r="D655" t="inlineStr">
+        <is>
+          <t>Universitatea Cluj</t>
+        </is>
+      </c>
+      <c r="E655" t="n">
+        <v>9.34</v>
+      </c>
+      <c r="F655" t="n">
+        <v>2.67</v>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" s="1" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B656" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C656" t="inlineStr">
+        <is>
+          <t>Orebro SK</t>
+        </is>
+      </c>
+      <c r="D656" t="inlineStr">
+        <is>
+          <t>Ostersunds FK</t>
+        </is>
+      </c>
+      <c r="E656" t="n">
+        <v>10.13</v>
+      </c>
+      <c r="F656" t="n">
+        <v>-0.02</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily scrape output - 2026-09-05
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F656"/>
+  <dimension ref="A1:F665"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16231,7 +16231,7 @@
         <v>10.1</v>
       </c>
       <c r="F608" t="n">
-        <v>1.84</v>
+        <v>1.61</v>
       </c>
     </row>
     <row r="609">
@@ -16254,10 +16254,10 @@
         </is>
       </c>
       <c r="E609" t="n">
-        <v>10.49</v>
+        <v>10.34</v>
       </c>
       <c r="F609" t="n">
-        <v>0.54</v>
+        <v>0.55</v>
       </c>
     </row>
     <row r="610">
@@ -16306,10 +16306,10 @@
         </is>
       </c>
       <c r="E611" t="n">
-        <v>9.99</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="F611" t="n">
-        <v>1.06</v>
+        <v>1.18</v>
       </c>
     </row>
     <row r="612">
@@ -16332,10 +16332,10 @@
         </is>
       </c>
       <c r="E612" t="n">
-        <v>11.41</v>
+        <v>11.45</v>
       </c>
       <c r="F612" t="n">
-        <v>-1.83</v>
+        <v>-2.03</v>
       </c>
     </row>
     <row r="613">
@@ -16349,19 +16349,19 @@
       </c>
       <c r="C613" t="inlineStr">
         <is>
-          <t>HK Kopavogur</t>
+          <t>Grotta</t>
         </is>
       </c>
       <c r="D613" t="inlineStr">
         <is>
-          <t>Fylkir</t>
+          <t>Volsungur</t>
         </is>
       </c>
       <c r="E613" t="n">
-        <v>11.66</v>
+        <v>11.8</v>
       </c>
       <c r="F613" t="n">
-        <v>-0.37</v>
+        <v>1.21</v>
       </c>
     </row>
     <row r="614">
@@ -16375,19 +16375,19 @@
       </c>
       <c r="C614" t="inlineStr">
         <is>
-          <t>IR Reykjavik</t>
+          <t>HK Kopavogur</t>
         </is>
       </c>
       <c r="D614" t="inlineStr">
         <is>
-          <t>Leiknir Reykjavik</t>
+          <t>Fylkir</t>
         </is>
       </c>
       <c r="E614" t="n">
-        <v>11.7</v>
+        <v>11.66</v>
       </c>
       <c r="F614" t="n">
-        <v>1.07</v>
+        <v>-0.37</v>
       </c>
     </row>
     <row r="615">
@@ -16401,19 +16401,19 @@
       </c>
       <c r="C615" t="inlineStr">
         <is>
-          <t>UMF Njardvik</t>
+          <t>IR Reykjavik</t>
         </is>
       </c>
       <c r="D615" t="inlineStr">
         <is>
-          <t>Afturelding</t>
+          <t>Leiknir Reykjavik</t>
         </is>
       </c>
       <c r="E615" t="n">
-        <v>11.2</v>
+        <v>11.85</v>
       </c>
       <c r="F615" t="n">
-        <v>0.06</v>
+        <v>1.07</v>
       </c>
     </row>
     <row r="616">
@@ -16427,19 +16427,19 @@
       </c>
       <c r="C616" t="inlineStr">
         <is>
-          <t>Vestri</t>
+          <t>UMF Njardvik</t>
         </is>
       </c>
       <c r="D616" t="inlineStr">
         <is>
-          <t>Throttur Reykjavik</t>
+          <t>Afturelding</t>
         </is>
       </c>
       <c r="E616" t="n">
-        <v>11.01</v>
+        <v>11.79</v>
       </c>
       <c r="F616" t="n">
-        <v>-1.68</v>
+        <v>-0.03</v>
       </c>
     </row>
     <row r="617">
@@ -16448,24 +16448,24 @@
       </c>
       <c r="B617" t="inlineStr">
         <is>
-          <t>Norway - 1st Division</t>
+          <t>Iceland - 1. Deild</t>
         </is>
       </c>
       <c r="C617" t="inlineStr">
         <is>
-          <t>Asane Fotball</t>
+          <t>Vestri</t>
         </is>
       </c>
       <c r="D617" t="inlineStr">
         <is>
-          <t>Hodd</t>
+          <t>Throttur Reykjavik</t>
         </is>
       </c>
       <c r="E617" t="n">
-        <v>10.8</v>
+        <v>10.97</v>
       </c>
       <c r="F617" t="n">
-        <v>0.09</v>
+        <v>-1.67</v>
       </c>
     </row>
     <row r="618">
@@ -16479,19 +16479,19 @@
       </c>
       <c r="C618" t="inlineStr">
         <is>
-          <t>Haugesund</t>
+          <t>Asane Fotball</t>
         </is>
       </c>
       <c r="D618" t="inlineStr">
         <is>
-          <t>Sogndal</t>
+          <t>Hodd</t>
         </is>
       </c>
       <c r="E618" t="n">
-        <v>11.16</v>
+        <v>10.73</v>
       </c>
       <c r="F618" t="n">
-        <v>2.49</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="619">
@@ -16505,19 +16505,19 @@
       </c>
       <c r="C619" t="inlineStr">
         <is>
-          <t>Kongsvinger</t>
+          <t>Haugesund</t>
         </is>
       </c>
       <c r="D619" t="inlineStr">
         <is>
-          <t>Raufoss</t>
+          <t>Sogndal</t>
         </is>
       </c>
       <c r="E619" t="n">
-        <v>11.77</v>
+        <v>11.34</v>
       </c>
       <c r="F619" t="n">
-        <v>3.57</v>
+        <v>2.51</v>
       </c>
     </row>
     <row r="620">
@@ -16531,19 +16531,19 @@
       </c>
       <c r="C620" t="inlineStr">
         <is>
-          <t>Odd BK</t>
+          <t>Kongsvinger</t>
         </is>
       </c>
       <c r="D620" t="inlineStr">
         <is>
-          <t>Stromsgodset</t>
+          <t>Raufoss</t>
         </is>
       </c>
       <c r="E620" t="n">
-        <v>11.12</v>
+        <v>11.89</v>
       </c>
       <c r="F620" t="n">
-        <v>-0.97</v>
+        <v>3.73</v>
       </c>
     </row>
     <row r="621">
@@ -16557,19 +16557,19 @@
       </c>
       <c r="C621" t="inlineStr">
         <is>
-          <t>Sandnes Ulf</t>
+          <t>Odd BK</t>
         </is>
       </c>
       <c r="D621" t="inlineStr">
         <is>
-          <t>Ranheim</t>
+          <t>Stromsgodset</t>
         </is>
       </c>
       <c r="E621" t="n">
-        <v>11.2</v>
+        <v>11.16</v>
       </c>
       <c r="F621" t="n">
-        <v>0.15</v>
+        <v>-0.97</v>
       </c>
     </row>
     <row r="622">
@@ -16583,19 +16583,19 @@
       </c>
       <c r="C622" t="inlineStr">
         <is>
-          <t>Stabaek</t>
+          <t>Sandnes Ulf</t>
         </is>
       </c>
       <c r="D622" t="inlineStr">
         <is>
-          <t>Moss</t>
+          <t>Ranheim</t>
         </is>
       </c>
       <c r="E622" t="n">
-        <v>11.73</v>
+        <v>11.02</v>
       </c>
       <c r="F622" t="n">
-        <v>3.4</v>
+        <v>0.19</v>
       </c>
     </row>
     <row r="623">
@@ -16609,19 +16609,19 @@
       </c>
       <c r="C623" t="inlineStr">
         <is>
-          <t>Strommen</t>
+          <t>Stabaek</t>
         </is>
       </c>
       <c r="D623" t="inlineStr">
         <is>
-          <t>Bryne</t>
+          <t>Moss</t>
         </is>
       </c>
       <c r="E623" t="n">
-        <v>10.51</v>
+        <v>11.86</v>
       </c>
       <c r="F623" t="n">
-        <v>-0.64</v>
+        <v>3.51</v>
       </c>
     </row>
     <row r="624">
@@ -16630,24 +16630,24 @@
       </c>
       <c r="B624" t="inlineStr">
         <is>
-          <t>Poland - 1st Liga</t>
+          <t>Norway - 1st Division</t>
         </is>
       </c>
       <c r="C624" t="inlineStr">
         <is>
-          <t>Miedz Legnica</t>
+          <t>Strommen</t>
         </is>
       </c>
       <c r="D624" t="inlineStr">
         <is>
-          <t>Chrobry Glogow</t>
+          <t>Bryne</t>
         </is>
       </c>
       <c r="E624" t="n">
-        <v>10.67</v>
+        <v>10.32</v>
       </c>
       <c r="F624" t="n">
-        <v>1.86</v>
+        <v>-0.62</v>
       </c>
     </row>
     <row r="625">
@@ -16661,19 +16661,19 @@
       </c>
       <c r="C625" t="inlineStr">
         <is>
-          <t>Stal Mielec</t>
+          <t>Miedz Legnica</t>
         </is>
       </c>
       <c r="D625" t="inlineStr">
         <is>
-          <t>Odra Opole</t>
+          <t>Chrobry Glogow</t>
         </is>
       </c>
       <c r="E625" t="n">
-        <v>10.55</v>
+        <v>10.83</v>
       </c>
       <c r="F625" t="n">
-        <v>0.2</v>
+        <v>1.86</v>
       </c>
     </row>
     <row r="626">
@@ -16687,19 +16687,19 @@
       </c>
       <c r="C626" t="inlineStr">
         <is>
-          <t>Stal Rzeszow</t>
+          <t>Stal Mielec</t>
         </is>
       </c>
       <c r="D626" t="inlineStr">
         <is>
-          <t>Polonia Warsaw</t>
+          <t>Odra Opole</t>
         </is>
       </c>
       <c r="E626" t="n">
-        <v>11.29</v>
+        <v>11.01</v>
       </c>
       <c r="F626" t="n">
-        <v>-0.84</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="627">
@@ -16708,24 +16708,24 @@
       </c>
       <c r="B627" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="C627" t="inlineStr">
         <is>
-          <t>Motor Lublin</t>
+          <t>Stal Rzeszow</t>
         </is>
       </c>
       <c r="D627" t="inlineStr">
         <is>
-          <t>Legia Warsaw</t>
+          <t>Polonia Warsaw</t>
         </is>
       </c>
       <c r="E627" t="n">
-        <v>9.76</v>
+        <v>11.71</v>
       </c>
       <c r="F627" t="n">
-        <v>-1.07</v>
+        <v>-0.9</v>
       </c>
     </row>
     <row r="628">
@@ -16739,19 +16739,19 @@
       </c>
       <c r="C628" t="inlineStr">
         <is>
-          <t>Widzew Lodz</t>
+          <t>Korona Kielce</t>
         </is>
       </c>
       <c r="D628" t="inlineStr">
         <is>
-          <t>Radomiak Radom</t>
+          <t>Wisla Krakow</t>
         </is>
       </c>
       <c r="E628" t="n">
-        <v>10.2</v>
+        <v>9.949999999999999</v>
       </c>
       <c r="F628" t="n">
-        <v>2.53</v>
+        <v>0.33</v>
       </c>
     </row>
     <row r="629">
@@ -16760,24 +16760,24 @@
       </c>
       <c r="B629" t="inlineStr">
         <is>
-          <t>Romania - Liga 1</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C629" t="inlineStr">
         <is>
-          <t>Dinamo Bucuresti</t>
+          <t>Motor Lublin</t>
         </is>
       </c>
       <c r="D629" t="inlineStr">
         <is>
-          <t>FCSB</t>
+          <t>Legia Warsaw</t>
         </is>
       </c>
       <c r="E629" t="n">
-        <v>9.640000000000001</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="F629" t="n">
-        <v>0.65</v>
+        <v>-1.06</v>
       </c>
     </row>
     <row r="630">
@@ -16786,24 +16786,24 @@
       </c>
       <c r="B630" t="inlineStr">
         <is>
-          <t>Romania - Liga 1</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C630" t="inlineStr">
         <is>
-          <t>UTA Arad</t>
+          <t>Widzew Lodz</t>
         </is>
       </c>
       <c r="D630" t="inlineStr">
         <is>
-          <t>Csikszereda</t>
+          <t>Radomiak Radom</t>
         </is>
       </c>
       <c r="E630" t="n">
-        <v>9.6</v>
+        <v>10.21</v>
       </c>
       <c r="F630" t="n">
-        <v>3.07</v>
+        <v>2.49</v>
       </c>
     </row>
     <row r="631">
@@ -16812,24 +16812,24 @@
       </c>
       <c r="B631" t="inlineStr">
         <is>
-          <t>Spain - Segunda</t>
+          <t>Romania - Liga 1</t>
         </is>
       </c>
       <c r="C631" t="inlineStr">
         <is>
-          <t>Ceuta</t>
+          <t>Botosani</t>
         </is>
       </c>
       <c r="D631" t="inlineStr">
         <is>
-          <t>Celta Vigo II</t>
+          <t>Sepsi</t>
         </is>
       </c>
       <c r="E631" t="n">
-        <v>8.470000000000001</v>
+        <v>9.76</v>
       </c>
       <c r="F631" t="n">
-        <v>1.37</v>
+        <v>1.14</v>
       </c>
     </row>
     <row r="632">
@@ -16838,24 +16838,24 @@
       </c>
       <c r="B632" t="inlineStr">
         <is>
-          <t>Spain - Segunda</t>
+          <t>Romania - Liga 1</t>
         </is>
       </c>
       <c r="C632" t="inlineStr">
         <is>
-          <t>Eldense</t>
+          <t>Dinamo Bucuresti</t>
         </is>
       </c>
       <c r="D632" t="inlineStr">
         <is>
-          <t>Mallorca</t>
+          <t>FCSB</t>
         </is>
       </c>
       <c r="E632" t="n">
-        <v>9.57</v>
+        <v>9.67</v>
       </c>
       <c r="F632" t="n">
-        <v>0.11</v>
+        <v>1.35</v>
       </c>
     </row>
     <row r="633">
@@ -16864,24 +16864,24 @@
       </c>
       <c r="B633" t="inlineStr">
         <is>
-          <t>Spain - Segunda</t>
+          <t>Romania - Liga 1</t>
         </is>
       </c>
       <c r="C633" t="inlineStr">
         <is>
-          <t>Real Sociedad II</t>
+          <t>UTA Arad</t>
         </is>
       </c>
       <c r="D633" t="inlineStr">
         <is>
-          <t>Tenerife</t>
+          <t>Csikszereda</t>
         </is>
       </c>
       <c r="E633" t="n">
-        <v>9.640000000000001</v>
+        <v>9.609999999999999</v>
       </c>
       <c r="F633" t="n">
-        <v>0.15</v>
+        <v>3.23</v>
       </c>
     </row>
     <row r="634">
@@ -16895,19 +16895,19 @@
       </c>
       <c r="C634" t="inlineStr">
         <is>
-          <t>Real Valladolid</t>
+          <t>Ceuta</t>
         </is>
       </c>
       <c r="D634" t="inlineStr">
         <is>
-          <t>FC Andorra</t>
+          <t>Celta Vigo II</t>
         </is>
       </c>
       <c r="E634" t="n">
-        <v>9</v>
+        <v>8.470000000000001</v>
       </c>
       <c r="F634" t="n">
-        <v>0.58</v>
+        <v>1.37</v>
       </c>
     </row>
     <row r="635">
@@ -16921,19 +16921,19 @@
       </c>
       <c r="C635" t="inlineStr">
         <is>
-          <t>Sporting Gijon</t>
+          <t>Eldense</t>
         </is>
       </c>
       <c r="D635" t="inlineStr">
         <is>
-          <t>Girona</t>
+          <t>Mallorca</t>
         </is>
       </c>
       <c r="E635" t="n">
-        <v>9.199999999999999</v>
+        <v>9.65</v>
       </c>
       <c r="F635" t="n">
-        <v>-0.41</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="636">
@@ -16942,24 +16942,24 @@
       </c>
       <c r="B636" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="C636" t="inlineStr">
         <is>
-          <t>Brage</t>
+          <t>Real Sociedad II</t>
         </is>
       </c>
       <c r="D636" t="inlineStr">
         <is>
-          <t>Sundsvall</t>
+          <t>Tenerife</t>
         </is>
       </c>
       <c r="E636" t="n">
-        <v>10.46</v>
+        <v>9.529999999999999</v>
       </c>
       <c r="F636" t="n">
-        <v>1.65</v>
+        <v>0.17</v>
       </c>
     </row>
     <row r="637">
@@ -16968,24 +16968,24 @@
       </c>
       <c r="B637" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="C637" t="inlineStr">
         <is>
-          <t>Helsingborgs</t>
+          <t>Real Valladolid</t>
         </is>
       </c>
       <c r="D637" t="inlineStr">
         <is>
-          <t>Sandvikens IF</t>
+          <t>FC Andorra</t>
         </is>
       </c>
       <c r="E637" t="n">
-        <v>10.2</v>
+        <v>9</v>
       </c>
       <c r="F637" t="n">
-        <v>1.06</v>
+        <v>0.58</v>
       </c>
     </row>
     <row r="638">
@@ -16994,24 +16994,24 @@
       </c>
       <c r="B638" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="C638" t="inlineStr">
         <is>
-          <t>Norrby</t>
+          <t>Sporting Gijon</t>
         </is>
       </c>
       <c r="D638" t="inlineStr">
         <is>
-          <t>Landskrona</t>
+          <t>Girona</t>
         </is>
       </c>
       <c r="E638" t="n">
-        <v>10.17</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="F638" t="n">
-        <v>-1.06</v>
+        <v>-0.41</v>
       </c>
     </row>
     <row r="639">
@@ -17025,19 +17025,19 @@
       </c>
       <c r="C639" t="inlineStr">
         <is>
-          <t>Oddevold</t>
+          <t>Brage</t>
         </is>
       </c>
       <c r="D639" t="inlineStr">
         <is>
-          <t>Falkenbergs</t>
+          <t>Sundsvall</t>
         </is>
       </c>
       <c r="E639" t="n">
-        <v>9.16</v>
+        <v>10.57</v>
       </c>
       <c r="F639" t="n">
-        <v>1.51</v>
+        <v>1.83</v>
       </c>
     </row>
     <row r="640">
@@ -17051,97 +17051,97 @@
       </c>
       <c r="C640" t="inlineStr">
         <is>
-          <t>Varnamo</t>
+          <t>Helsingborgs</t>
         </is>
       </c>
       <c r="D640" t="inlineStr">
         <is>
-          <t>Varbergs BoIS</t>
+          <t>Sandvikens IF</t>
         </is>
       </c>
       <c r="E640" t="n">
-        <v>9.73</v>
+        <v>10.21</v>
       </c>
       <c r="F640" t="n">
-        <v>-0.47</v>
+        <v>1.06</v>
       </c>
     </row>
     <row r="641">
       <c r="A641" s="1" t="n">
-        <v>46271</v>
+        <v>46270</v>
       </c>
       <c r="B641" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Sweden - Superettan</t>
         </is>
       </c>
       <c r="C641" t="inlineStr">
         <is>
-          <t>Londrina</t>
+          <t>Norrby</t>
         </is>
       </c>
       <c r="D641" t="inlineStr">
         <is>
-          <t>Operario Ferroviario</t>
+          <t>Landskrona</t>
         </is>
       </c>
       <c r="E641" t="n">
-        <v>10.45</v>
+        <v>9.960000000000001</v>
       </c>
       <c r="F641" t="n">
-        <v>1.02</v>
+        <v>-0.9</v>
       </c>
     </row>
     <row r="642">
       <c r="A642" s="1" t="n">
-        <v>46271</v>
+        <v>46270</v>
       </c>
       <c r="B642" t="inlineStr">
         <is>
-          <t>Finland - Ykkosliiga</t>
+          <t>Sweden - Superettan</t>
         </is>
       </c>
       <c r="C642" t="inlineStr">
         <is>
-          <t>FC Haka</t>
+          <t>Oddevold</t>
         </is>
       </c>
       <c r="D642" t="inlineStr">
         <is>
-          <t>Mikkelin Palloilijat</t>
+          <t>Falkenbergs</t>
         </is>
       </c>
       <c r="E642" t="n">
-        <v>10.84</v>
+        <v>9.16</v>
       </c>
       <c r="F642" t="n">
-        <v>3.67</v>
+        <v>1.51</v>
       </c>
     </row>
     <row r="643">
       <c r="A643" s="1" t="n">
-        <v>46271</v>
+        <v>46270</v>
       </c>
       <c r="B643" t="inlineStr">
         <is>
-          <t>Finland - Ykkosliiga</t>
+          <t>Sweden - Superettan</t>
         </is>
       </c>
       <c r="C643" t="inlineStr">
         <is>
-          <t>SJK Akatemia</t>
+          <t>Varnamo</t>
         </is>
       </c>
       <c r="D643" t="inlineStr">
         <is>
-          <t>JaPS</t>
+          <t>Varbergs BoIS</t>
         </is>
       </c>
       <c r="E643" t="n">
-        <v>10.61</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="F643" t="n">
-        <v>-0.5600000000000001</v>
+        <v>-0.13</v>
       </c>
     </row>
     <row r="644">
@@ -17150,24 +17150,24 @@
       </c>
       <c r="B644" t="inlineStr">
         <is>
-          <t>Norway - 1st Division</t>
+          <t>Brazil - Serie B</t>
         </is>
       </c>
       <c r="C644" t="inlineStr">
         <is>
-          <t>Lyn</t>
+          <t>Londrina</t>
         </is>
       </c>
       <c r="D644" t="inlineStr">
         <is>
-          <t>Egersunds</t>
+          <t>Operario Ferroviario</t>
         </is>
       </c>
       <c r="E644" t="n">
-        <v>10.8</v>
+        <v>10.45</v>
       </c>
       <c r="F644" t="n">
-        <v>0.12</v>
+        <v>1.02</v>
       </c>
     </row>
     <row r="645">
@@ -17176,24 +17176,24 @@
       </c>
       <c r="B645" t="inlineStr">
         <is>
-          <t>Poland - 1st Liga</t>
+          <t>Brazil - Serie B</t>
         </is>
       </c>
       <c r="C645" t="inlineStr">
         <is>
-          <t>Pogon Siedlce</t>
+          <t>Ponte Preta</t>
         </is>
       </c>
       <c r="D645" t="inlineStr">
         <is>
-          <t>Puszcza Niepolomice</t>
+          <t>Sao Bernardo</t>
         </is>
       </c>
       <c r="E645" t="n">
-        <v>10.3</v>
+        <v>10.76</v>
       </c>
       <c r="F645" t="n">
-        <v>-0.17</v>
+        <v>-2.66</v>
       </c>
     </row>
     <row r="646">
@@ -17202,24 +17202,24 @@
       </c>
       <c r="B646" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Finland - Ykkosliiga</t>
         </is>
       </c>
       <c r="C646" t="inlineStr">
         <is>
-          <t>Cracovia Krakow</t>
+          <t>FC Haka</t>
         </is>
       </c>
       <c r="D646" t="inlineStr">
         <is>
-          <t>Gornik Zabrze</t>
+          <t>Mikkelin Palloilijat</t>
         </is>
       </c>
       <c r="E646" t="n">
-        <v>10.8</v>
+        <v>10.84</v>
       </c>
       <c r="F646" t="n">
-        <v>0.38</v>
+        <v>3.67</v>
       </c>
     </row>
     <row r="647">
@@ -17228,24 +17228,24 @@
       </c>
       <c r="B647" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Finland - Ykkosliiga</t>
         </is>
       </c>
       <c r="C647" t="inlineStr">
         <is>
-          <t>Lech Poznan</t>
+          <t>SJK Akatemia</t>
         </is>
       </c>
       <c r="D647" t="inlineStr">
         <is>
-          <t>Rakow Czestochowa</t>
+          <t>JaPS</t>
         </is>
       </c>
       <c r="E647" t="n">
-        <v>10.26</v>
+        <v>10.61</v>
       </c>
       <c r="F647" t="n">
-        <v>2.85</v>
+        <v>-0.5600000000000001</v>
       </c>
     </row>
     <row r="648">
@@ -17254,24 +17254,24 @@
       </c>
       <c r="B648" t="inlineStr">
         <is>
-          <t>Romania - Liga 1</t>
+          <t>Norway - 1st Division</t>
         </is>
       </c>
       <c r="C648" t="inlineStr">
         <is>
-          <t>Otelul Galati</t>
+          <t>Lyn</t>
         </is>
       </c>
       <c r="D648" t="inlineStr">
         <is>
-          <t>Rapid Bucuresti</t>
+          <t>Egersunds</t>
         </is>
       </c>
       <c r="E648" t="n">
-        <v>9.41</v>
+        <v>10.8</v>
       </c>
       <c r="F648" t="n">
-        <v>0.32</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="649">
@@ -17280,24 +17280,24 @@
       </c>
       <c r="B649" t="inlineStr">
         <is>
-          <t>Spain - Segunda</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="C649" t="inlineStr">
         <is>
-          <t>Almeria</t>
+          <t>Pogon Siedlce</t>
         </is>
       </c>
       <c r="D649" t="inlineStr">
         <is>
-          <t>Cadiz</t>
+          <t>Puszcza Niepolomice</t>
         </is>
       </c>
       <c r="E649" t="n">
-        <v>9.550000000000001</v>
+        <v>10.3</v>
       </c>
       <c r="F649" t="n">
-        <v>2.2</v>
+        <v>-0.17</v>
       </c>
     </row>
     <row r="650">
@@ -17306,24 +17306,24 @@
       </c>
       <c r="B650" t="inlineStr">
         <is>
-          <t>Spain - Segunda</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C650" t="inlineStr">
         <is>
-          <t>Castellon</t>
+          <t>Cracovia Krakow</t>
         </is>
       </c>
       <c r="D650" t="inlineStr">
         <is>
-          <t>Albacete</t>
+          <t>Gornik Zabrze</t>
         </is>
       </c>
       <c r="E650" t="n">
-        <v>10.32</v>
+        <v>10.8</v>
       </c>
       <c r="F650" t="n">
-        <v>2.53</v>
+        <v>0.38</v>
       </c>
     </row>
     <row r="651">
@@ -17332,24 +17332,24 @@
       </c>
       <c r="B651" t="inlineStr">
         <is>
-          <t>Spain - Segunda</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C651" t="inlineStr">
         <is>
-          <t>Eibar</t>
+          <t>Lech Poznan</t>
         </is>
       </c>
       <c r="D651" t="inlineStr">
         <is>
-          <t>Granada</t>
+          <t>Rakow Czestochowa</t>
         </is>
       </c>
       <c r="E651" t="n">
-        <v>9</v>
+        <v>10.26</v>
       </c>
       <c r="F651" t="n">
-        <v>1.86</v>
+        <v>2.85</v>
       </c>
     </row>
     <row r="652">
@@ -17358,128 +17358,362 @@
       </c>
       <c r="B652" t="inlineStr">
         <is>
-          <t>Spain - Segunda</t>
+          <t>Romania - Liga 1</t>
         </is>
       </c>
       <c r="C652" t="inlineStr">
         <is>
-          <t>Real Oviedo</t>
+          <t>Otelul Galati</t>
         </is>
       </c>
       <c r="D652" t="inlineStr">
         <is>
-          <t>Burgos</t>
+          <t>Rapid Bucuresti</t>
         </is>
       </c>
       <c r="E652" t="n">
-        <v>9.09</v>
+        <v>9.470000000000001</v>
       </c>
       <c r="F652" t="n">
-        <v>1.6</v>
+        <v>-0.18</v>
       </c>
     </row>
     <row r="653">
       <c r="A653" s="1" t="n">
-        <v>46272</v>
+        <v>46271</v>
       </c>
       <c r="B653" t="inlineStr">
         <is>
-          <t>Finland - Ykkosliiga</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="C653" t="inlineStr">
         <is>
-          <t>HJK Klubi 04</t>
+          <t>Almeria</t>
         </is>
       </c>
       <c r="D653" t="inlineStr">
         <is>
-          <t>KaPa</t>
+          <t>Cadiz</t>
         </is>
       </c>
       <c r="E653" t="n">
-        <v>10.53</v>
+        <v>9.56</v>
       </c>
       <c r="F653" t="n">
-        <v>0.9399999999999999</v>
+        <v>2.22</v>
       </c>
     </row>
     <row r="654">
       <c r="A654" s="1" t="n">
-        <v>46272</v>
+        <v>46271</v>
       </c>
       <c r="B654" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="C654" t="inlineStr">
         <is>
-          <t>Pogon Szczecin</t>
+          <t>Castellon</t>
         </is>
       </c>
       <c r="D654" t="inlineStr">
         <is>
-          <t>Wisla Plock</t>
+          <t>Albacete</t>
         </is>
       </c>
       <c r="E654" t="n">
-        <v>10.43</v>
+        <v>10.32</v>
       </c>
       <c r="F654" t="n">
-        <v>0.9399999999999999</v>
+        <v>2.53</v>
       </c>
     </row>
     <row r="655">
       <c r="A655" s="1" t="n">
-        <v>46272</v>
+        <v>46271</v>
       </c>
       <c r="B655" t="inlineStr">
         <is>
-          <t>Romania - Liga 1</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="C655" t="inlineStr">
         <is>
-          <t>Universitatea Craiova</t>
+          <t>Eibar</t>
         </is>
       </c>
       <c r="D655" t="inlineStr">
         <is>
-          <t>Universitatea Cluj</t>
+          <t>Granada</t>
         </is>
       </c>
       <c r="E655" t="n">
-        <v>9.34</v>
+        <v>9</v>
       </c>
       <c r="F655" t="n">
-        <v>2.67</v>
+        <v>1.86</v>
       </c>
     </row>
     <row r="656">
       <c r="A656" s="1" t="n">
+        <v>46271</v>
+      </c>
+      <c r="B656" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C656" t="inlineStr">
+        <is>
+          <t>Real Oviedo</t>
+        </is>
+      </c>
+      <c r="D656" t="inlineStr">
+        <is>
+          <t>Burgos</t>
+        </is>
+      </c>
+      <c r="E656" t="n">
+        <v>9.09</v>
+      </c>
+      <c r="F656" t="n">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" s="1" t="n">
         <v>46272</v>
       </c>
-      <c r="B656" t="inlineStr">
+      <c r="B657" t="inlineStr">
+        <is>
+          <t>Finland - Ykkosliiga</t>
+        </is>
+      </c>
+      <c r="C657" t="inlineStr">
+        <is>
+          <t>HJK Klubi 04</t>
+        </is>
+      </c>
+      <c r="D657" t="inlineStr">
+        <is>
+          <t>KaPa</t>
+        </is>
+      </c>
+      <c r="E657" t="n">
+        <v>10.53</v>
+      </c>
+      <c r="F657" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" s="1" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B658" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C658" t="inlineStr">
+        <is>
+          <t>Pogon Szczecin</t>
+        </is>
+      </c>
+      <c r="D658" t="inlineStr">
+        <is>
+          <t>Wisla Plock</t>
+        </is>
+      </c>
+      <c r="E658" t="n">
+        <v>10.45</v>
+      </c>
+      <c r="F658" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" s="1" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B659" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C659" t="inlineStr">
+        <is>
+          <t>Universitatea Craiova</t>
+        </is>
+      </c>
+      <c r="D659" t="inlineStr">
+        <is>
+          <t>Universitatea Cluj</t>
+        </is>
+      </c>
+      <c r="E659" t="n">
+        <v>9.34</v>
+      </c>
+      <c r="F659" t="n">
+        <v>2.67</v>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" s="1" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B660" t="inlineStr">
         <is>
           <t>Sweden - Superettan</t>
         </is>
       </c>
-      <c r="C656" t="inlineStr">
+      <c r="C660" t="inlineStr">
         <is>
           <t>Orebro SK</t>
         </is>
       </c>
-      <c r="D656" t="inlineStr">
+      <c r="D660" t="inlineStr">
         <is>
           <t>Ostersunds FK</t>
         </is>
       </c>
-      <c r="E656" t="n">
+      <c r="E660" t="n">
         <v>10.13</v>
       </c>
-      <c r="F656" t="n">
+      <c r="F660" t="n">
         <v>-0.02</v>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" s="1" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B661" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C661" t="inlineStr">
+        <is>
+          <t>Cuiaba</t>
+        </is>
+      </c>
+      <c r="D661" t="inlineStr">
+        <is>
+          <t>Athletic Club</t>
+        </is>
+      </c>
+      <c r="E661" t="n">
+        <v>10.14</v>
+      </c>
+      <c r="F661" t="n">
+        <v>2.16</v>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" s="1" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B662" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C662" t="inlineStr">
+        <is>
+          <t>FC Lahti</t>
+        </is>
+      </c>
+      <c r="D662" t="inlineStr">
+        <is>
+          <t>IFK Mariehamn</t>
+        </is>
+      </c>
+      <c r="E662" t="n">
+        <v>10.53</v>
+      </c>
+      <c r="F662" t="n">
+        <v>2.96</v>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" s="1" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B663" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C663" t="inlineStr">
+        <is>
+          <t>Gnistan</t>
+        </is>
+      </c>
+      <c r="D663" t="inlineStr">
+        <is>
+          <t>KuPS</t>
+        </is>
+      </c>
+      <c r="E663" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="F663" t="n">
+        <v>-0.57</v>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" s="1" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B664" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C664" t="inlineStr">
+        <is>
+          <t>Ilves</t>
+        </is>
+      </c>
+      <c r="D664" t="inlineStr">
+        <is>
+          <t>Jaro</t>
+        </is>
+      </c>
+      <c r="E664" t="n">
+        <v>10.22</v>
+      </c>
+      <c r="F664" t="n">
+        <v>2.2</v>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" s="1" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B665" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C665" t="inlineStr">
+        <is>
+          <t>VPS</t>
+        </is>
+      </c>
+      <c r="D665" t="inlineStr">
+        <is>
+          <t>AC Oulu</t>
+        </is>
+      </c>
+      <c r="E665" t="n">
+        <v>9.74</v>
+      </c>
+      <c r="F665" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily scrape output - 2026-09-06
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F665"/>
+  <dimension ref="A1:F672"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17242,10 +17242,10 @@
         </is>
       </c>
       <c r="E647" t="n">
-        <v>10.61</v>
+        <v>10.94</v>
       </c>
       <c r="F647" t="n">
-        <v>-0.5600000000000001</v>
+        <v>-0.61</v>
       </c>
     </row>
     <row r="648">
@@ -17268,10 +17268,10 @@
         </is>
       </c>
       <c r="E648" t="n">
-        <v>10.8</v>
+        <v>10.79</v>
       </c>
       <c r="F648" t="n">
-        <v>0.12</v>
+        <v>0.42</v>
       </c>
     </row>
     <row r="649">
@@ -17285,19 +17285,19 @@
       </c>
       <c r="C649" t="inlineStr">
         <is>
-          <t>Pogon Siedlce</t>
+          <t>Arka Gdynia</t>
         </is>
       </c>
       <c r="D649" t="inlineStr">
         <is>
-          <t>Puszcza Niepolomice</t>
+          <t>LKS Lodz</t>
         </is>
       </c>
       <c r="E649" t="n">
-        <v>10.3</v>
+        <v>10.21</v>
       </c>
       <c r="F649" t="n">
-        <v>-0.17</v>
+        <v>0.62</v>
       </c>
     </row>
     <row r="650">
@@ -17306,24 +17306,24 @@
       </c>
       <c r="B650" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="C650" t="inlineStr">
         <is>
-          <t>Cracovia Krakow</t>
+          <t>Pogon Siedlce</t>
         </is>
       </c>
       <c r="D650" t="inlineStr">
         <is>
-          <t>Gornik Zabrze</t>
+          <t>Puszcza Niepolomice</t>
         </is>
       </c>
       <c r="E650" t="n">
-        <v>10.8</v>
+        <v>10.3</v>
       </c>
       <c r="F650" t="n">
-        <v>0.38</v>
+        <v>-0.17</v>
       </c>
     </row>
     <row r="651">
@@ -17332,24 +17332,24 @@
       </c>
       <c r="B651" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="C651" t="inlineStr">
         <is>
-          <t>Lech Poznan</t>
+          <t>Polonia Bytom</t>
         </is>
       </c>
       <c r="D651" t="inlineStr">
         <is>
-          <t>Rakow Czestochowa</t>
+          <t>Podbeskidzie Bielsko-Biala</t>
         </is>
       </c>
       <c r="E651" t="n">
-        <v>10.26</v>
+        <v>10.07</v>
       </c>
       <c r="F651" t="n">
-        <v>2.85</v>
+        <v>0.58</v>
       </c>
     </row>
     <row r="652">
@@ -17358,24 +17358,24 @@
       </c>
       <c r="B652" t="inlineStr">
         <is>
-          <t>Romania - Liga 1</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C652" t="inlineStr">
         <is>
-          <t>Otelul Galati</t>
+          <t>Cracovia Krakow</t>
         </is>
       </c>
       <c r="D652" t="inlineStr">
         <is>
-          <t>Rapid Bucuresti</t>
+          <t>Gornik Zabrze</t>
         </is>
       </c>
       <c r="E652" t="n">
-        <v>9.470000000000001</v>
+        <v>11.05</v>
       </c>
       <c r="F652" t="n">
-        <v>-0.18</v>
+        <v>0.36</v>
       </c>
     </row>
     <row r="653">
@@ -17384,24 +17384,24 @@
       </c>
       <c r="B653" t="inlineStr">
         <is>
-          <t>Spain - Segunda</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C653" t="inlineStr">
         <is>
-          <t>Almeria</t>
+          <t>Jagiellonia Bialystok</t>
         </is>
       </c>
       <c r="D653" t="inlineStr">
         <is>
-          <t>Cadiz</t>
+          <t>Slask Wroclaw</t>
         </is>
       </c>
       <c r="E653" t="n">
-        <v>9.56</v>
+        <v>9.58</v>
       </c>
       <c r="F653" t="n">
-        <v>2.22</v>
+        <v>2.36</v>
       </c>
     </row>
     <row r="654">
@@ -17410,24 +17410,24 @@
       </c>
       <c r="B654" t="inlineStr">
         <is>
-          <t>Spain - Segunda</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C654" t="inlineStr">
         <is>
-          <t>Castellon</t>
+          <t>Lech Poznan</t>
         </is>
       </c>
       <c r="D654" t="inlineStr">
         <is>
-          <t>Albacete</t>
+          <t>Rakow Czestochowa</t>
         </is>
       </c>
       <c r="E654" t="n">
-        <v>10.32</v>
+        <v>10.26</v>
       </c>
       <c r="F654" t="n">
-        <v>2.53</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="655">
@@ -17436,24 +17436,24 @@
       </c>
       <c r="B655" t="inlineStr">
         <is>
-          <t>Spain - Segunda</t>
+          <t>Romania - Liga 1</t>
         </is>
       </c>
       <c r="C655" t="inlineStr">
         <is>
-          <t>Eibar</t>
+          <t>Otelul Galati</t>
         </is>
       </c>
       <c r="D655" t="inlineStr">
         <is>
-          <t>Granada</t>
+          <t>Rapid Bucuresti</t>
         </is>
       </c>
       <c r="E655" t="n">
-        <v>9</v>
+        <v>9.470000000000001</v>
       </c>
       <c r="F655" t="n">
-        <v>1.86</v>
+        <v>-0.18</v>
       </c>
     </row>
     <row r="656">
@@ -17462,258 +17462,440 @@
       </c>
       <c r="B656" t="inlineStr">
         <is>
-          <t>Spain - Segunda</t>
+          <t>Romania - Liga 1</t>
         </is>
       </c>
       <c r="C656" t="inlineStr">
         <is>
-          <t>Real Oviedo</t>
+          <t>Petrolul Ploiesti</t>
         </is>
       </c>
       <c r="D656" t="inlineStr">
         <is>
-          <t>Burgos</t>
+          <t>Corvinul Hunedoara</t>
         </is>
       </c>
       <c r="E656" t="n">
-        <v>9.09</v>
+        <v>8.33</v>
       </c>
       <c r="F656" t="n">
-        <v>1.6</v>
+        <v>0.36</v>
       </c>
     </row>
     <row r="657">
       <c r="A657" s="1" t="n">
-        <v>46272</v>
+        <v>46271</v>
       </c>
       <c r="B657" t="inlineStr">
         <is>
-          <t>Finland - Ykkosliiga</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="C657" t="inlineStr">
         <is>
-          <t>HJK Klubi 04</t>
+          <t>Almeria</t>
         </is>
       </c>
       <c r="D657" t="inlineStr">
         <is>
-          <t>KaPa</t>
+          <t>Cadiz</t>
         </is>
       </c>
       <c r="E657" t="n">
-        <v>10.53</v>
+        <v>9.710000000000001</v>
       </c>
       <c r="F657" t="n">
-        <v>0.9399999999999999</v>
+        <v>2.23</v>
       </c>
     </row>
     <row r="658">
       <c r="A658" s="1" t="n">
-        <v>46272</v>
+        <v>46271</v>
       </c>
       <c r="B658" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="C658" t="inlineStr">
         <is>
-          <t>Pogon Szczecin</t>
+          <t>Castellon</t>
         </is>
       </c>
       <c r="D658" t="inlineStr">
         <is>
-          <t>Wisla Plock</t>
+          <t>Albacete</t>
         </is>
       </c>
       <c r="E658" t="n">
-        <v>10.45</v>
+        <v>10.32</v>
       </c>
       <c r="F658" t="n">
-        <v>0.9399999999999999</v>
+        <v>2.53</v>
       </c>
     </row>
     <row r="659">
       <c r="A659" s="1" t="n">
-        <v>46272</v>
+        <v>46271</v>
       </c>
       <c r="B659" t="inlineStr">
         <is>
-          <t>Romania - Liga 1</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="C659" t="inlineStr">
         <is>
-          <t>Universitatea Craiova</t>
+          <t>Eibar</t>
         </is>
       </c>
       <c r="D659" t="inlineStr">
         <is>
-          <t>Universitatea Cluj</t>
+          <t>Granada</t>
         </is>
       </c>
       <c r="E659" t="n">
-        <v>9.34</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="F659" t="n">
-        <v>2.67</v>
+        <v>1.85</v>
       </c>
     </row>
     <row r="660">
       <c r="A660" s="1" t="n">
-        <v>46272</v>
+        <v>46271</v>
       </c>
       <c r="B660" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="C660" t="inlineStr">
         <is>
-          <t>Orebro SK</t>
+          <t>Real Oviedo</t>
         </is>
       </c>
       <c r="D660" t="inlineStr">
         <is>
-          <t>Ostersunds FK</t>
+          <t>Burgos</t>
         </is>
       </c>
       <c r="E660" t="n">
-        <v>10.13</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="F660" t="n">
-        <v>-0.02</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="661">
       <c r="A661" s="1" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B661" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Finland - Ykkosliiga</t>
         </is>
       </c>
       <c r="C661" t="inlineStr">
         <is>
-          <t>Cuiaba</t>
+          <t>HJK Klubi 04</t>
         </is>
       </c>
       <c r="D661" t="inlineStr">
         <is>
-          <t>Athletic Club</t>
+          <t>KaPa</t>
         </is>
       </c>
       <c r="E661" t="n">
-        <v>10.14</v>
+        <v>10.53</v>
       </c>
       <c r="F661" t="n">
-        <v>2.16</v>
+        <v>0.9399999999999999</v>
       </c>
     </row>
     <row r="662">
       <c r="A662" s="1" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B662" t="inlineStr">
         <is>
-          <t>Finland - Veikkausliiga</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C662" t="inlineStr">
         <is>
-          <t>FC Lahti</t>
+          <t>Pogon Szczecin</t>
         </is>
       </c>
       <c r="D662" t="inlineStr">
         <is>
-          <t>IFK Mariehamn</t>
+          <t>Wisla Plock</t>
         </is>
       </c>
       <c r="E662" t="n">
-        <v>10.53</v>
+        <v>10.45</v>
       </c>
       <c r="F662" t="n">
-        <v>2.96</v>
+        <v>0.9399999999999999</v>
       </c>
     </row>
     <row r="663">
       <c r="A663" s="1" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B663" t="inlineStr">
         <is>
-          <t>Finland - Veikkausliiga</t>
+          <t>Romania - Liga 1</t>
         </is>
       </c>
       <c r="C663" t="inlineStr">
         <is>
-          <t>Gnistan</t>
+          <t>Universitatea Craiova</t>
         </is>
       </c>
       <c r="D663" t="inlineStr">
         <is>
-          <t>KuPS</t>
+          <t>Universitatea Cluj</t>
         </is>
       </c>
       <c r="E663" t="n">
-        <v>10.3</v>
+        <v>9.34</v>
       </c>
       <c r="F663" t="n">
-        <v>-0.57</v>
+        <v>2.67</v>
       </c>
     </row>
     <row r="664">
       <c r="A664" s="1" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B664" t="inlineStr">
         <is>
-          <t>Finland - Veikkausliiga</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="C664" t="inlineStr">
         <is>
-          <t>Ilves</t>
+          <t>Sabadell</t>
         </is>
       </c>
       <c r="D664" t="inlineStr">
         <is>
-          <t>Jaro</t>
+          <t>Cordoba</t>
         </is>
       </c>
       <c r="E664" t="n">
-        <v>10.22</v>
+        <v>9.279999999999999</v>
       </c>
       <c r="F664" t="n">
-        <v>2.2</v>
+        <v>0.96</v>
       </c>
     </row>
     <row r="665">
       <c r="A665" s="1" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B665" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C665" t="inlineStr">
+        <is>
+          <t>Orebro SK</t>
+        </is>
+      </c>
+      <c r="D665" t="inlineStr">
+        <is>
+          <t>Ostersunds FK</t>
+        </is>
+      </c>
+      <c r="E665" t="n">
+        <v>10.13</v>
+      </c>
+      <c r="F665" t="n">
+        <v>-0.02</v>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" s="1" t="n">
         <v>46273</v>
       </c>
-      <c r="B665" t="inlineStr">
+      <c r="B666" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C666" t="inlineStr">
+        <is>
+          <t>Cuiaba</t>
+        </is>
+      </c>
+      <c r="D666" t="inlineStr">
+        <is>
+          <t>Athletic Club</t>
+        </is>
+      </c>
+      <c r="E666" t="n">
+        <v>10.14</v>
+      </c>
+      <c r="F666" t="n">
+        <v>2.16</v>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" s="1" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B667" t="inlineStr">
         <is>
           <t>Finland - Veikkausliiga</t>
         </is>
       </c>
-      <c r="C665" t="inlineStr">
+      <c r="C667" t="inlineStr">
+        <is>
+          <t>FC Lahti</t>
+        </is>
+      </c>
+      <c r="D667" t="inlineStr">
+        <is>
+          <t>IFK Mariehamn</t>
+        </is>
+      </c>
+      <c r="E667" t="n">
+        <v>10.51</v>
+      </c>
+      <c r="F667" t="n">
+        <v>2.96</v>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" s="1" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B668" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C668" t="inlineStr">
+        <is>
+          <t>Gnistan</t>
+        </is>
+      </c>
+      <c r="D668" t="inlineStr">
+        <is>
+          <t>KuPS</t>
+        </is>
+      </c>
+      <c r="E668" t="n">
+        <v>10.11</v>
+      </c>
+      <c r="F668" t="n">
+        <v>-0.13</v>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" s="1" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B669" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C669" t="inlineStr">
+        <is>
+          <t>Ilves</t>
+        </is>
+      </c>
+      <c r="D669" t="inlineStr">
+        <is>
+          <t>Jaro</t>
+        </is>
+      </c>
+      <c r="E669" t="n">
+        <v>10.05</v>
+      </c>
+      <c r="F669" t="n">
+        <v>2.2</v>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" s="1" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B670" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C670" t="inlineStr">
+        <is>
+          <t>TPS</t>
+        </is>
+      </c>
+      <c r="D670" t="inlineStr">
+        <is>
+          <t>SJK</t>
+        </is>
+      </c>
+      <c r="E670" t="n">
+        <v>10.69</v>
+      </c>
+      <c r="F670" t="n">
+        <v>-0.46</v>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" s="1" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B671" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C671" t="inlineStr">
         <is>
           <t>VPS</t>
         </is>
       </c>
-      <c r="D665" t="inlineStr">
+      <c r="D671" t="inlineStr">
         <is>
           <t>AC Oulu</t>
         </is>
       </c>
-      <c r="E665" t="n">
-        <v>9.74</v>
-      </c>
-      <c r="F665" t="n">
-        <v>1</v>
+      <c r="E671" t="n">
+        <v>9.65</v>
+      </c>
+      <c r="F671" t="n">
+        <v>1.02</v>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" s="1" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B672" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C672" t="inlineStr">
+        <is>
+          <t>Criciuma</t>
+        </is>
+      </c>
+      <c r="D672" t="inlineStr">
+        <is>
+          <t>Juventude</t>
+        </is>
+      </c>
+      <c r="E672" t="n">
+        <v>10.49</v>
+      </c>
+      <c r="F672" t="n">
+        <v>1.98</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily scrape output - 2026-09-07
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F672"/>
+  <dimension ref="A1:F674"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17632,10 +17632,10 @@
         </is>
       </c>
       <c r="E662" t="n">
-        <v>10.45</v>
+        <v>10.51</v>
       </c>
       <c r="F662" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.61</v>
       </c>
     </row>
     <row r="663">
@@ -17644,24 +17644,24 @@
       </c>
       <c r="B663" t="inlineStr">
         <is>
-          <t>Romania - Liga 1</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C663" t="inlineStr">
         <is>
-          <t>Universitatea Craiova</t>
+          <t>Wieczysta Krakow</t>
         </is>
       </c>
       <c r="D663" t="inlineStr">
         <is>
-          <t>Universitatea Cluj</t>
+          <t>Zaglebie Lubin</t>
         </is>
       </c>
       <c r="E663" t="n">
-        <v>9.34</v>
+        <v>10.81</v>
       </c>
       <c r="F663" t="n">
-        <v>2.67</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="664">
@@ -17670,24 +17670,24 @@
       </c>
       <c r="B664" t="inlineStr">
         <is>
-          <t>Spain - Segunda</t>
+          <t>Romania - Liga 1</t>
         </is>
       </c>
       <c r="C664" t="inlineStr">
         <is>
-          <t>Sabadell</t>
+          <t>Universitatea Craiova</t>
         </is>
       </c>
       <c r="D664" t="inlineStr">
         <is>
-          <t>Cordoba</t>
+          <t>Universitatea Cluj</t>
         </is>
       </c>
       <c r="E664" t="n">
-        <v>9.279999999999999</v>
+        <v>9.34</v>
       </c>
       <c r="F664" t="n">
-        <v>0.96</v>
+        <v>2.67</v>
       </c>
     </row>
     <row r="665">
@@ -17696,76 +17696,76 @@
       </c>
       <c r="B665" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Romania - Liga 1</t>
         </is>
       </c>
       <c r="C665" t="inlineStr">
         <is>
-          <t>Orebro SK</t>
+          <t>Voluntari</t>
         </is>
       </c>
       <c r="D665" t="inlineStr">
         <is>
-          <t>Ostersunds FK</t>
+          <t>Arges Pitesti</t>
         </is>
       </c>
       <c r="E665" t="n">
-        <v>10.13</v>
+        <v>8</v>
       </c>
       <c r="F665" t="n">
-        <v>-0.02</v>
+        <v>-0.04</v>
       </c>
     </row>
     <row r="666">
       <c r="A666" s="1" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B666" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="C666" t="inlineStr">
         <is>
-          <t>Cuiaba</t>
+          <t>Sabadell</t>
         </is>
       </c>
       <c r="D666" t="inlineStr">
         <is>
-          <t>Athletic Club</t>
+          <t>Cordoba</t>
         </is>
       </c>
       <c r="E666" t="n">
-        <v>10.14</v>
+        <v>9.279999999999999</v>
       </c>
       <c r="F666" t="n">
-        <v>2.16</v>
+        <v>0.96</v>
       </c>
     </row>
     <row r="667">
       <c r="A667" s="1" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B667" t="inlineStr">
         <is>
-          <t>Finland - Veikkausliiga</t>
+          <t>Sweden - Superettan</t>
         </is>
       </c>
       <c r="C667" t="inlineStr">
         <is>
-          <t>FC Lahti</t>
+          <t>Orebro SK</t>
         </is>
       </c>
       <c r="D667" t="inlineStr">
         <is>
-          <t>IFK Mariehamn</t>
+          <t>Ostersunds FK</t>
         </is>
       </c>
       <c r="E667" t="n">
-        <v>10.51</v>
+        <v>10.13</v>
       </c>
       <c r="F667" t="n">
-        <v>2.96</v>
+        <v>-0.02</v>
       </c>
     </row>
     <row r="668">
@@ -17774,24 +17774,24 @@
       </c>
       <c r="B668" t="inlineStr">
         <is>
-          <t>Finland - Veikkausliiga</t>
+          <t>Brazil - Serie B</t>
         </is>
       </c>
       <c r="C668" t="inlineStr">
         <is>
-          <t>Gnistan</t>
+          <t>Cuiaba</t>
         </is>
       </c>
       <c r="D668" t="inlineStr">
         <is>
-          <t>KuPS</t>
+          <t>Athletic Club</t>
         </is>
       </c>
       <c r="E668" t="n">
-        <v>10.11</v>
+        <v>10.09</v>
       </c>
       <c r="F668" t="n">
-        <v>-0.13</v>
+        <v>2.84</v>
       </c>
     </row>
     <row r="669">
@@ -17805,19 +17805,19 @@
       </c>
       <c r="C669" t="inlineStr">
         <is>
-          <t>Ilves</t>
+          <t>FC Lahti</t>
         </is>
       </c>
       <c r="D669" t="inlineStr">
         <is>
-          <t>Jaro</t>
+          <t>IFK Mariehamn</t>
         </is>
       </c>
       <c r="E669" t="n">
-        <v>10.05</v>
+        <v>10.5</v>
       </c>
       <c r="F669" t="n">
-        <v>2.2</v>
+        <v>2.72</v>
       </c>
     </row>
     <row r="670">
@@ -17831,19 +17831,19 @@
       </c>
       <c r="C670" t="inlineStr">
         <is>
-          <t>TPS</t>
+          <t>Gnistan</t>
         </is>
       </c>
       <c r="D670" t="inlineStr">
         <is>
-          <t>SJK</t>
+          <t>KuPS</t>
         </is>
       </c>
       <c r="E670" t="n">
-        <v>10.69</v>
+        <v>10.11</v>
       </c>
       <c r="F670" t="n">
-        <v>-0.46</v>
+        <v>-0.14</v>
       </c>
     </row>
     <row r="671">
@@ -17857,45 +17857,97 @@
       </c>
       <c r="C671" t="inlineStr">
         <is>
-          <t>VPS</t>
+          <t>Ilves</t>
         </is>
       </c>
       <c r="D671" t="inlineStr">
         <is>
-          <t>AC Oulu</t>
+          <t>Jaro</t>
         </is>
       </c>
       <c r="E671" t="n">
-        <v>9.65</v>
+        <v>10.05</v>
       </c>
       <c r="F671" t="n">
-        <v>1.02</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="672">
       <c r="A672" s="1" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B672" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C672" t="inlineStr">
+        <is>
+          <t>TPS</t>
+        </is>
+      </c>
+      <c r="D672" t="inlineStr">
+        <is>
+          <t>SJK</t>
+        </is>
+      </c>
+      <c r="E672" t="n">
+        <v>10.69</v>
+      </c>
+      <c r="F672" t="n">
+        <v>-0.49</v>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" s="1" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B673" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C673" t="inlineStr">
+        <is>
+          <t>VPS</t>
+        </is>
+      </c>
+      <c r="D673" t="inlineStr">
+        <is>
+          <t>AC Oulu</t>
+        </is>
+      </c>
+      <c r="E673" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="F673" t="n">
+        <v>1.02</v>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" s="1" t="n">
         <v>46274</v>
       </c>
-      <c r="B672" t="inlineStr">
+      <c r="B674" t="inlineStr">
         <is>
           <t>Brazil - Serie B</t>
         </is>
       </c>
-      <c r="C672" t="inlineStr">
+      <c r="C674" t="inlineStr">
         <is>
           <t>Criciuma</t>
         </is>
       </c>
-      <c r="D672" t="inlineStr">
+      <c r="D674" t="inlineStr">
         <is>
           <t>Juventude</t>
         </is>
       </c>
-      <c r="E672" t="n">
-        <v>10.49</v>
-      </c>
-      <c r="F672" t="n">
-        <v>1.98</v>
+      <c r="E674" t="n">
+        <v>10.89</v>
+      </c>
+      <c r="F674" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily scrape output - 2026-09-08
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -17788,10 +17788,10 @@
         </is>
       </c>
       <c r="E668" t="n">
-        <v>10.09</v>
+        <v>9.69</v>
       </c>
       <c r="F668" t="n">
-        <v>2.84</v>
+        <v>2.15</v>
       </c>
     </row>
     <row r="669">
@@ -17814,7 +17814,7 @@
         </is>
       </c>
       <c r="E669" t="n">
-        <v>10.5</v>
+        <v>10.37</v>
       </c>
       <c r="F669" t="n">
         <v>2.72</v>
@@ -17840,10 +17840,10 @@
         </is>
       </c>
       <c r="E670" t="n">
-        <v>10.11</v>
+        <v>10.15</v>
       </c>
       <c r="F670" t="n">
-        <v>-0.14</v>
+        <v>-0.51</v>
       </c>
     </row>
     <row r="671">
@@ -17869,7 +17869,7 @@
         <v>10.05</v>
       </c>
       <c r="F671" t="n">
-        <v>2.2</v>
+        <v>1.99</v>
       </c>
     </row>
     <row r="672">
@@ -17918,10 +17918,10 @@
         </is>
       </c>
       <c r="E673" t="n">
-        <v>9.6</v>
+        <v>9.44</v>
       </c>
       <c r="F673" t="n">
-        <v>1.02</v>
+        <v>1.15</v>
       </c>
     </row>
     <row r="674">
@@ -17944,10 +17944,10 @@
         </is>
       </c>
       <c r="E674" t="n">
-        <v>10.89</v>
+        <v>10.48</v>
       </c>
       <c r="F674" t="n">
-        <v>2</v>
+        <v>1.69</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily scrape output - 2026-09-09
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F674"/>
+  <dimension ref="A1:F686"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17935,19 +17935,331 @@
       </c>
       <c r="C674" t="inlineStr">
         <is>
+          <t>America Mineiro</t>
+        </is>
+      </c>
+      <c r="D674" t="inlineStr">
+        <is>
+          <t>Nautico</t>
+        </is>
+      </c>
+      <c r="E674" t="n">
+        <v>10.85</v>
+      </c>
+      <c r="F674" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" s="1" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B675" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C675" t="inlineStr">
+        <is>
+          <t>Botafogo SP</t>
+        </is>
+      </c>
+      <c r="D675" t="inlineStr">
+        <is>
+          <t>Gremio Novorizontino</t>
+        </is>
+      </c>
+      <c r="E675" t="n">
+        <v>11.16</v>
+      </c>
+      <c r="F675" t="n">
+        <v>0.42</v>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" s="1" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B676" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C676" t="inlineStr">
+        <is>
           <t>Criciuma</t>
         </is>
       </c>
-      <c r="D674" t="inlineStr">
+      <c r="D676" t="inlineStr">
         <is>
           <t>Juventude</t>
         </is>
       </c>
-      <c r="E674" t="n">
+      <c r="E676" t="n">
         <v>10.48</v>
       </c>
-      <c r="F674" t="n">
+      <c r="F676" t="n">
         <v>1.69</v>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" s="1" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B677" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C677" t="inlineStr">
+        <is>
+          <t>Fortaleza</t>
+        </is>
+      </c>
+      <c r="D677" t="inlineStr">
+        <is>
+          <t>Avai</t>
+        </is>
+      </c>
+      <c r="E677" t="n">
+        <v>10.36</v>
+      </c>
+      <c r="F677" t="n">
+        <v>2.89</v>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" s="1" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B678" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C678" t="inlineStr">
+        <is>
+          <t>Operario Ferroviario</t>
+        </is>
+      </c>
+      <c r="D678" t="inlineStr">
+        <is>
+          <t>CRB</t>
+        </is>
+      </c>
+      <c r="E678" t="n">
+        <v>10.58</v>
+      </c>
+      <c r="F678" t="n">
+        <v>0.93</v>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" s="1" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B679" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C679" t="inlineStr">
+        <is>
+          <t>HJK Helsinki</t>
+        </is>
+      </c>
+      <c r="D679" t="inlineStr">
+        <is>
+          <t>Inter Turku</t>
+        </is>
+      </c>
+      <c r="E679" t="n">
+        <v>10.05</v>
+      </c>
+      <c r="F679" t="n">
+        <v>-0.04</v>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" s="1" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B680" t="inlineStr">
+        <is>
+          <t>Iceland - 1. Deild</t>
+        </is>
+      </c>
+      <c r="C680" t="inlineStr">
+        <is>
+          <t>HK Kopavogur</t>
+        </is>
+      </c>
+      <c r="D680" t="inlineStr">
+        <is>
+          <t>Fylkir</t>
+        </is>
+      </c>
+      <c r="E680" t="n">
+        <v>11.69</v>
+      </c>
+      <c r="F680" t="n">
+        <v>-0.34</v>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" s="1" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B681" t="inlineStr">
+        <is>
+          <t>Iceland - 1. Deild</t>
+        </is>
+      </c>
+      <c r="C681" t="inlineStr">
+        <is>
+          <t>UMF Njardvik</t>
+        </is>
+      </c>
+      <c r="D681" t="inlineStr">
+        <is>
+          <t>Throttur Reykjavik</t>
+        </is>
+      </c>
+      <c r="E681" t="n">
+        <v>11.02</v>
+      </c>
+      <c r="F681" t="n">
+        <v>0.43</v>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" s="1" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B682" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C682" t="inlineStr">
+        <is>
+          <t>Landskrona</t>
+        </is>
+      </c>
+      <c r="D682" t="inlineStr">
+        <is>
+          <t>Helsingborgs</t>
+        </is>
+      </c>
+      <c r="E682" t="n">
+        <v>10.16</v>
+      </c>
+      <c r="F682" t="n">
+        <v>1.54</v>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" s="1" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B683" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C683" t="inlineStr">
+        <is>
+          <t>Ljungskile</t>
+        </is>
+      </c>
+      <c r="D683" t="inlineStr">
+        <is>
+          <t>Norrby</t>
+        </is>
+      </c>
+      <c r="E683" t="n">
+        <v>10.54</v>
+      </c>
+      <c r="F683" t="n">
+        <v>1.33</v>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" s="1" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B684" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C684" t="inlineStr">
+        <is>
+          <t>Nordic United</t>
+        </is>
+      </c>
+      <c r="D684" t="inlineStr">
+        <is>
+          <t>Varnamo</t>
+        </is>
+      </c>
+      <c r="E684" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="F684" t="n">
+        <v>1.48</v>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" s="1" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B685" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C685" t="inlineStr">
+        <is>
+          <t>Sandvikens IF</t>
+        </is>
+      </c>
+      <c r="D685" t="inlineStr">
+        <is>
+          <t>Oddevold</t>
+        </is>
+      </c>
+      <c r="E685" t="n">
+        <v>9.949999999999999</v>
+      </c>
+      <c r="F685" t="n">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" s="1" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B686" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C686" t="inlineStr">
+        <is>
+          <t>Atletico Goianiense</t>
+        </is>
+      </c>
+      <c r="D686" t="inlineStr">
+        <is>
+          <t>Ceara</t>
+        </is>
+      </c>
+      <c r="E686" t="n">
+        <v>10.04</v>
+      </c>
+      <c r="F686" t="n">
+        <v>1.06</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily scrape output - 2026-09-10
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F686"/>
+  <dimension ref="A1:F692"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18262,6 +18262,162 @@
         <v>1.06</v>
       </c>
     </row>
+    <row r="687">
+      <c r="A687" s="1" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B687" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C687" t="inlineStr">
+        <is>
+          <t>Sao Bernardo</t>
+        </is>
+      </c>
+      <c r="D687" t="inlineStr">
+        <is>
+          <t>Londrina</t>
+        </is>
+      </c>
+      <c r="E687" t="n">
+        <v>10.63</v>
+      </c>
+      <c r="F687" t="n">
+        <v>1.98</v>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" s="1" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B688" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C688" t="inlineStr">
+        <is>
+          <t>Vila Nova</t>
+        </is>
+      </c>
+      <c r="D688" t="inlineStr">
+        <is>
+          <t>Goias</t>
+        </is>
+      </c>
+      <c r="E688" t="n">
+        <v>10.11</v>
+      </c>
+      <c r="F688" t="n">
+        <v>1.18</v>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" s="1" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B689" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C689" t="inlineStr">
+        <is>
+          <t>Falkenbergs</t>
+        </is>
+      </c>
+      <c r="D689" t="inlineStr">
+        <is>
+          <t>Osters</t>
+        </is>
+      </c>
+      <c r="E689" t="n">
+        <v>9.83</v>
+      </c>
+      <c r="F689" t="n">
+        <v>1.42</v>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" s="1" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B690" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C690" t="inlineStr">
+        <is>
+          <t>Sundsvall</t>
+        </is>
+      </c>
+      <c r="D690" t="inlineStr">
+        <is>
+          <t>Orebro SK</t>
+        </is>
+      </c>
+      <c r="E690" t="n">
+        <v>10.28</v>
+      </c>
+      <c r="F690" t="n">
+        <v>-0.52</v>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" s="1" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B691" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C691" t="inlineStr">
+        <is>
+          <t>Varbergs BoIS</t>
+        </is>
+      </c>
+      <c r="D691" t="inlineStr">
+        <is>
+          <t>Norrkoping</t>
+        </is>
+      </c>
+      <c r="E691" t="n">
+        <v>10.38</v>
+      </c>
+      <c r="F691" t="n">
+        <v>-0.37</v>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" s="1" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B692" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C692" t="inlineStr">
+        <is>
+          <t>Sport Recife</t>
+        </is>
+      </c>
+      <c r="D692" t="inlineStr">
+        <is>
+          <t>Ponte Preta</t>
+        </is>
+      </c>
+      <c r="E692" t="n">
+        <v>11.16</v>
+      </c>
+      <c r="F692" t="n">
+        <v>3.56</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily scrape output - 2026-09-11
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F692"/>
+  <dimension ref="A1:F740"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18418,6 +18418,1254 @@
         <v>3.56</v>
       </c>
     </row>
+    <row r="693">
+      <c r="A693" s="1" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B693" t="inlineStr">
+        <is>
+          <t>Finland - Ykkosliiga</t>
+        </is>
+      </c>
+      <c r="C693" t="inlineStr">
+        <is>
+          <t>KTP</t>
+        </is>
+      </c>
+      <c r="D693" t="inlineStr">
+        <is>
+          <t>JaPS</t>
+        </is>
+      </c>
+      <c r="E693" t="n">
+        <v>10.68</v>
+      </c>
+      <c r="F693" t="n">
+        <v>2.51</v>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" s="1" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B694" t="inlineStr">
+        <is>
+          <t>Finland - Ykkosliiga</t>
+        </is>
+      </c>
+      <c r="C694" t="inlineStr">
+        <is>
+          <t>KaPa</t>
+        </is>
+      </c>
+      <c r="D694" t="inlineStr">
+        <is>
+          <t>PK-35</t>
+        </is>
+      </c>
+      <c r="E694" t="n">
+        <v>10.49</v>
+      </c>
+      <c r="F694" t="n">
+        <v>-1.11</v>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" s="1" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B695" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C695" t="inlineStr">
+        <is>
+          <t>Polonia Warsaw</t>
+        </is>
+      </c>
+      <c r="D695" t="inlineStr">
+        <is>
+          <t>Polonia Bytom</t>
+        </is>
+      </c>
+      <c r="E695" t="n">
+        <v>10.96</v>
+      </c>
+      <c r="F695" t="n">
+        <v>1.15</v>
+      </c>
+    </row>
+    <row r="696">
+      <c r="A696" s="1" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B696" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C696" t="inlineStr">
+        <is>
+          <t>Puszcza Niepolomice</t>
+        </is>
+      </c>
+      <c r="D696" t="inlineStr">
+        <is>
+          <t>LKS Lodz</t>
+        </is>
+      </c>
+      <c r="E696" t="n">
+        <v>10.33</v>
+      </c>
+      <c r="F696" t="n">
+        <v>-0.61</v>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" s="1" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B697" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C697" t="inlineStr">
+        <is>
+          <t>Rakow Czestochowa</t>
+        </is>
+      </c>
+      <c r="D697" t="inlineStr">
+        <is>
+          <t>Motor Lublin</t>
+        </is>
+      </c>
+      <c r="E697" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="F697" t="n">
+        <v>1.42</v>
+      </c>
+    </row>
+    <row r="698">
+      <c r="A698" s="1" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B698" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C698" t="inlineStr">
+        <is>
+          <t>Wisla Krakow</t>
+        </is>
+      </c>
+      <c r="D698" t="inlineStr">
+        <is>
+          <t>Jagiellonia Bialystok</t>
+        </is>
+      </c>
+      <c r="E698" t="n">
+        <v>10.05</v>
+      </c>
+      <c r="F698" t="n">
+        <v>0.33</v>
+      </c>
+    </row>
+    <row r="699">
+      <c r="A699" s="1" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B699" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C699" t="inlineStr">
+        <is>
+          <t>Csikszereda</t>
+        </is>
+      </c>
+      <c r="D699" t="inlineStr">
+        <is>
+          <t>Dinamo Bucuresti</t>
+        </is>
+      </c>
+      <c r="E699" t="n">
+        <v>9.27</v>
+      </c>
+      <c r="F699" t="n">
+        <v>-2.59</v>
+      </c>
+    </row>
+    <row r="700">
+      <c r="A700" s="1" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B700" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C700" t="inlineStr">
+        <is>
+          <t>Farul Constanta</t>
+        </is>
+      </c>
+      <c r="D700" t="inlineStr">
+        <is>
+          <t>UTA Arad</t>
+        </is>
+      </c>
+      <c r="E700" t="n">
+        <v>9.720000000000001</v>
+      </c>
+      <c r="F700" t="n">
+        <v>0.65</v>
+      </c>
+    </row>
+    <row r="701">
+      <c r="A701" s="1" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B701" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C701" t="inlineStr">
+        <is>
+          <t>Burgos</t>
+        </is>
+      </c>
+      <c r="D701" t="inlineStr">
+        <is>
+          <t>Ceuta</t>
+        </is>
+      </c>
+      <c r="E701" t="n">
+        <v>8.550000000000001</v>
+      </c>
+      <c r="F701" t="n">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="702">
+      <c r="A702" s="1" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B702" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C702" t="inlineStr">
+        <is>
+          <t>AC Oulu</t>
+        </is>
+      </c>
+      <c r="D702" t="inlineStr">
+        <is>
+          <t>Gnistan</t>
+        </is>
+      </c>
+      <c r="E702" t="n">
+        <v>9.119999999999999</v>
+      </c>
+      <c r="F702" t="n">
+        <v>0.57</v>
+      </c>
+    </row>
+    <row r="703">
+      <c r="A703" s="1" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B703" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C703" t="inlineStr">
+        <is>
+          <t>IFK Mariehamn</t>
+        </is>
+      </c>
+      <c r="D703" t="inlineStr">
+        <is>
+          <t>TPS</t>
+        </is>
+      </c>
+      <c r="E703" t="n">
+        <v>10.29</v>
+      </c>
+      <c r="F703" t="n">
+        <v>-0.02</v>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" s="1" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B704" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C704" t="inlineStr">
+        <is>
+          <t>Ilves</t>
+        </is>
+      </c>
+      <c r="D704" t="inlineStr">
+        <is>
+          <t>FC Lahti</t>
+        </is>
+      </c>
+      <c r="E704" t="n">
+        <v>10.28</v>
+      </c>
+      <c r="F704" t="n">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" s="1" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B705" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C705" t="inlineStr">
+        <is>
+          <t>Jaro</t>
+        </is>
+      </c>
+      <c r="D705" t="inlineStr">
+        <is>
+          <t>SJK</t>
+        </is>
+      </c>
+      <c r="E705" t="n">
+        <v>9.609999999999999</v>
+      </c>
+      <c r="F705" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="706">
+      <c r="A706" s="1" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B706" t="inlineStr">
+        <is>
+          <t>Finland - Ykkosliiga</t>
+        </is>
+      </c>
+      <c r="C706" t="inlineStr">
+        <is>
+          <t>EIF</t>
+        </is>
+      </c>
+      <c r="D706" t="inlineStr">
+        <is>
+          <t>FC Haka</t>
+        </is>
+      </c>
+      <c r="E706" t="n">
+        <v>10.53</v>
+      </c>
+      <c r="F706" t="n">
+        <v>-0.91</v>
+      </c>
+    </row>
+    <row r="707">
+      <c r="A707" s="1" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B707" t="inlineStr">
+        <is>
+          <t>Finland - Ykkosliiga</t>
+        </is>
+      </c>
+      <c r="C707" t="inlineStr">
+        <is>
+          <t>JIPPO</t>
+        </is>
+      </c>
+      <c r="D707" t="inlineStr">
+        <is>
+          <t>HJK Klubi 04</t>
+        </is>
+      </c>
+      <c r="E707" t="n">
+        <v>10.13</v>
+      </c>
+      <c r="F707" t="n">
+        <v>2.47</v>
+      </c>
+    </row>
+    <row r="708">
+      <c r="A708" s="1" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B708" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C708" t="inlineStr">
+        <is>
+          <t>Bryne</t>
+        </is>
+      </c>
+      <c r="D708" t="inlineStr">
+        <is>
+          <t>Stabaek</t>
+        </is>
+      </c>
+      <c r="E708" t="n">
+        <v>10.66</v>
+      </c>
+      <c r="F708" t="n">
+        <v>-0.64</v>
+      </c>
+    </row>
+    <row r="709">
+      <c r="A709" s="1" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B709" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C709" t="inlineStr">
+        <is>
+          <t>Chrobry Glogow</t>
+        </is>
+      </c>
+      <c r="D709" t="inlineStr">
+        <is>
+          <t>Pogon Siedlce</t>
+        </is>
+      </c>
+      <c r="E709" t="n">
+        <v>10.73</v>
+      </c>
+      <c r="F709" t="n">
+        <v>1.57</v>
+      </c>
+    </row>
+    <row r="710">
+      <c r="A710" s="1" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B710" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C710" t="inlineStr">
+        <is>
+          <t>Zaglebie Lubin</t>
+        </is>
+      </c>
+      <c r="D710" t="inlineStr">
+        <is>
+          <t>GKS Katowice</t>
+        </is>
+      </c>
+      <c r="E710" t="n">
+        <v>10.01</v>
+      </c>
+      <c r="F710" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+    </row>
+    <row r="711">
+      <c r="A711" s="1" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B711" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C711" t="inlineStr">
+        <is>
+          <t>Cadiz</t>
+        </is>
+      </c>
+      <c r="D711" t="inlineStr">
+        <is>
+          <t>Las Palmas</t>
+        </is>
+      </c>
+      <c r="E711" t="n">
+        <v>9.09</v>
+      </c>
+      <c r="F711" t="n">
+        <v>-0.15</v>
+      </c>
+    </row>
+    <row r="712">
+      <c r="A712" s="1" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B712" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C712" t="inlineStr">
+        <is>
+          <t>Cordoba</t>
+        </is>
+      </c>
+      <c r="D712" t="inlineStr">
+        <is>
+          <t>Almeria</t>
+        </is>
+      </c>
+      <c r="E712" t="n">
+        <v>9.880000000000001</v>
+      </c>
+      <c r="F712" t="n">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="713">
+      <c r="A713" s="1" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B713" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C713" t="inlineStr">
+        <is>
+          <t>FC Andorra</t>
+        </is>
+      </c>
+      <c r="D713" t="inlineStr">
+        <is>
+          <t>Real Sociedad II</t>
+        </is>
+      </c>
+      <c r="E713" t="n">
+        <v>9.51</v>
+      </c>
+      <c r="F713" t="n">
+        <v>2.59</v>
+      </c>
+    </row>
+    <row r="714">
+      <c r="A714" s="1" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B714" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C714" t="inlineStr">
+        <is>
+          <t>Granada</t>
+        </is>
+      </c>
+      <c r="D714" t="inlineStr">
+        <is>
+          <t>Albacete</t>
+        </is>
+      </c>
+      <c r="E714" t="n">
+        <v>9.550000000000001</v>
+      </c>
+      <c r="F714" t="n">
+        <v>1.72</v>
+      </c>
+    </row>
+    <row r="715">
+      <c r="A715" s="1" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B715" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C715" t="inlineStr">
+        <is>
+          <t>Atletico Goianiense</t>
+        </is>
+      </c>
+      <c r="D715" t="inlineStr">
+        <is>
+          <t>Criciuma</t>
+        </is>
+      </c>
+      <c r="E715" t="n">
+        <v>10.47</v>
+      </c>
+      <c r="F715" t="n">
+        <v>0.54</v>
+      </c>
+    </row>
+    <row r="716">
+      <c r="A716" s="1" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B716" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C716" t="inlineStr">
+        <is>
+          <t>Fortaleza</t>
+        </is>
+      </c>
+      <c r="D716" t="inlineStr">
+        <is>
+          <t>Ceara</t>
+        </is>
+      </c>
+      <c r="E716" t="n">
+        <v>10.54</v>
+      </c>
+      <c r="F716" t="n">
+        <v>1.46</v>
+      </c>
+    </row>
+    <row r="717">
+      <c r="A717" s="1" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B717" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C717" t="inlineStr">
+        <is>
+          <t>Gremio Novorizontino</t>
+        </is>
+      </c>
+      <c r="D717" t="inlineStr">
+        <is>
+          <t>Cuiaba</t>
+        </is>
+      </c>
+      <c r="E717" t="n">
+        <v>10.45</v>
+      </c>
+      <c r="F717" t="n">
+        <v>1.65</v>
+      </c>
+    </row>
+    <row r="718">
+      <c r="A718" s="1" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B718" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C718" t="inlineStr">
+        <is>
+          <t>Juventude</t>
+        </is>
+      </c>
+      <c r="D718" t="inlineStr">
+        <is>
+          <t>Athletic Club</t>
+        </is>
+      </c>
+      <c r="E718" t="n">
+        <v>10.04</v>
+      </c>
+      <c r="F718" t="n">
+        <v>1.85</v>
+      </c>
+    </row>
+    <row r="719">
+      <c r="A719" s="1" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B719" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C719" t="inlineStr">
+        <is>
+          <t>KuPS</t>
+        </is>
+      </c>
+      <c r="D719" t="inlineStr">
+        <is>
+          <t>HJK Helsinki</t>
+        </is>
+      </c>
+      <c r="E719" t="n">
+        <v>10.09</v>
+      </c>
+      <c r="F719" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="720">
+      <c r="A720" s="1" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B720" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C720" t="inlineStr">
+        <is>
+          <t>Egersunds</t>
+        </is>
+      </c>
+      <c r="D720" t="inlineStr">
+        <is>
+          <t>Kongsvinger</t>
+        </is>
+      </c>
+      <c r="E720" t="n">
+        <v>10.66</v>
+      </c>
+      <c r="F720" t="n">
+        <v>-0.47</v>
+      </c>
+    </row>
+    <row r="721">
+      <c r="A721" s="1" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B721" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C721" t="inlineStr">
+        <is>
+          <t>Moss</t>
+        </is>
+      </c>
+      <c r="D721" t="inlineStr">
+        <is>
+          <t>Haugesund</t>
+        </is>
+      </c>
+      <c r="E721" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="F721" t="n">
+        <v>-1.33</v>
+      </c>
+    </row>
+    <row r="722">
+      <c r="A722" s="1" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B722" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C722" t="inlineStr">
+        <is>
+          <t>Raufoss</t>
+        </is>
+      </c>
+      <c r="D722" t="inlineStr">
+        <is>
+          <t>Odd BK</t>
+        </is>
+      </c>
+      <c r="E722" t="n">
+        <v>11.02</v>
+      </c>
+      <c r="F722" t="n">
+        <v>-2.09</v>
+      </c>
+    </row>
+    <row r="723">
+      <c r="A723" s="1" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B723" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C723" t="inlineStr">
+        <is>
+          <t>Sogndal</t>
+        </is>
+      </c>
+      <c r="D723" t="inlineStr">
+        <is>
+          <t>Strommen</t>
+        </is>
+      </c>
+      <c r="E723" t="n">
+        <v>11.09</v>
+      </c>
+      <c r="F723" t="n">
+        <v>1.07</v>
+      </c>
+    </row>
+    <row r="724">
+      <c r="A724" s="1" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B724" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C724" t="inlineStr">
+        <is>
+          <t>Stromsgodset</t>
+        </is>
+      </c>
+      <c r="D724" t="inlineStr">
+        <is>
+          <t>Sandnes Ulf</t>
+        </is>
+      </c>
+      <c r="E724" t="n">
+        <v>11.48</v>
+      </c>
+      <c r="F724" t="n">
+        <v>3.4</v>
+      </c>
+    </row>
+    <row r="725">
+      <c r="A725" s="1" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B725" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C725" t="inlineStr">
+        <is>
+          <t>Odra Opole</t>
+        </is>
+      </c>
+      <c r="D725" t="inlineStr">
+        <is>
+          <t>Stal Rzeszow</t>
+        </is>
+      </c>
+      <c r="E725" t="n">
+        <v>10.65</v>
+      </c>
+      <c r="F725" t="n">
+        <v>1.21</v>
+      </c>
+    </row>
+    <row r="726">
+      <c r="A726" s="1" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B726" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C726" t="inlineStr">
+        <is>
+          <t>Legia Warsaw</t>
+        </is>
+      </c>
+      <c r="D726" t="inlineStr">
+        <is>
+          <t>Widzew Lodz</t>
+        </is>
+      </c>
+      <c r="E726" t="n">
+        <v>9.789999999999999</v>
+      </c>
+      <c r="F726" t="n">
+        <v>1.65</v>
+      </c>
+    </row>
+    <row r="727">
+      <c r="A727" s="1" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B727" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C727" t="inlineStr">
+        <is>
+          <t>Wisla Plock</t>
+        </is>
+      </c>
+      <c r="D727" t="inlineStr">
+        <is>
+          <t>Cracovia Krakow</t>
+        </is>
+      </c>
+      <c r="E727" t="n">
+        <v>10.72</v>
+      </c>
+      <c r="F727" t="n">
+        <v>0.38</v>
+      </c>
+    </row>
+    <row r="728">
+      <c r="A728" s="1" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B728" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C728" t="inlineStr">
+        <is>
+          <t>Arges Pitesti</t>
+        </is>
+      </c>
+      <c r="D728" t="inlineStr">
+        <is>
+          <t>Botosani</t>
+        </is>
+      </c>
+      <c r="E728" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="F728" t="n">
+        <v>1.06</v>
+      </c>
+    </row>
+    <row r="729">
+      <c r="A729" s="1" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B729" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C729" t="inlineStr">
+        <is>
+          <t>Ljungskile</t>
+        </is>
+      </c>
+      <c r="D729" t="inlineStr">
+        <is>
+          <t>Falkenbergs</t>
+        </is>
+      </c>
+      <c r="E729" t="n">
+        <v>10.29</v>
+      </c>
+      <c r="F729" t="n">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="730">
+      <c r="A730" s="1" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B730" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C730" t="inlineStr">
+        <is>
+          <t>Norrkoping</t>
+        </is>
+      </c>
+      <c r="D730" t="inlineStr">
+        <is>
+          <t>Oddevold</t>
+        </is>
+      </c>
+      <c r="E730" t="n">
+        <v>10.16</v>
+      </c>
+      <c r="F730" t="n">
+        <v>1.97</v>
+      </c>
+    </row>
+    <row r="731">
+      <c r="A731" s="1" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B731" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C731" t="inlineStr">
+        <is>
+          <t>America Mineiro</t>
+        </is>
+      </c>
+      <c r="D731" t="inlineStr">
+        <is>
+          <t>Sao Bernardo</t>
+        </is>
+      </c>
+      <c r="E731" t="n">
+        <v>10.63</v>
+      </c>
+      <c r="F731" t="n">
+        <v>1.01</v>
+      </c>
+    </row>
+    <row r="732">
+      <c r="A732" s="1" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B732" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C732" t="inlineStr">
+        <is>
+          <t>Botafogo SP</t>
+        </is>
+      </c>
+      <c r="D732" t="inlineStr">
+        <is>
+          <t>Goias</t>
+        </is>
+      </c>
+      <c r="E732" t="n">
+        <v>10.65</v>
+      </c>
+      <c r="F732" t="n">
+        <v>1.34</v>
+      </c>
+    </row>
+    <row r="733">
+      <c r="A733" s="1" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B733" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C733" t="inlineStr">
+        <is>
+          <t>Inter Turku</t>
+        </is>
+      </c>
+      <c r="D733" t="inlineStr">
+        <is>
+          <t>VPS</t>
+        </is>
+      </c>
+      <c r="E733" t="n">
+        <v>9.84</v>
+      </c>
+      <c r="F733" t="n">
+        <v>1.88</v>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734" s="1" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B734" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C734" t="inlineStr">
+        <is>
+          <t>Radomiak Radom</t>
+        </is>
+      </c>
+      <c r="D734" t="inlineStr">
+        <is>
+          <t>Piast Gliwice</t>
+        </is>
+      </c>
+      <c r="E734" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="F734" t="n">
+        <v>0.34</v>
+      </c>
+    </row>
+    <row r="735">
+      <c r="A735" s="1" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B735" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C735" t="inlineStr">
+        <is>
+          <t>FCSB</t>
+        </is>
+      </c>
+      <c r="D735" t="inlineStr">
+        <is>
+          <t>Petrolul Ploiesti</t>
+        </is>
+      </c>
+      <c r="E735" t="n">
+        <v>10.11</v>
+      </c>
+      <c r="F735" t="n">
+        <v>3.25</v>
+      </c>
+    </row>
+    <row r="736">
+      <c r="A736" s="1" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B736" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C736" t="inlineStr">
+        <is>
+          <t>Universitatea Cluj</t>
+        </is>
+      </c>
+      <c r="D736" t="inlineStr">
+        <is>
+          <t>Otelul Galati</t>
+        </is>
+      </c>
+      <c r="E736" t="n">
+        <v>9.66</v>
+      </c>
+      <c r="F736" t="n">
+        <v>1.54</v>
+      </c>
+    </row>
+    <row r="737">
+      <c r="A737" s="1" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B737" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C737" t="inlineStr">
+        <is>
+          <t>Norrby</t>
+        </is>
+      </c>
+      <c r="D737" t="inlineStr">
+        <is>
+          <t>Varbergs BoIS</t>
+        </is>
+      </c>
+      <c r="E737" t="n">
+        <v>10.55</v>
+      </c>
+      <c r="F737" t="n">
+        <v>-0.5600000000000001</v>
+      </c>
+    </row>
+    <row r="738">
+      <c r="A738" s="1" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B738" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C738" t="inlineStr">
+        <is>
+          <t>Orebro SK</t>
+        </is>
+      </c>
+      <c r="D738" t="inlineStr">
+        <is>
+          <t>Nordic United</t>
+        </is>
+      </c>
+      <c r="E738" t="n">
+        <v>10.17</v>
+      </c>
+      <c r="F738" t="n">
+        <v>0.71</v>
+      </c>
+    </row>
+    <row r="739">
+      <c r="A739" s="1" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B739" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C739" t="inlineStr">
+        <is>
+          <t>Ostersunds FK</t>
+        </is>
+      </c>
+      <c r="D739" t="inlineStr">
+        <is>
+          <t>Helsingborgs</t>
+        </is>
+      </c>
+      <c r="E739" t="n">
+        <v>9.98</v>
+      </c>
+      <c r="F739" t="n">
+        <v>1.46</v>
+      </c>
+    </row>
+    <row r="740">
+      <c r="A740" s="1" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B740" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C740" t="inlineStr">
+        <is>
+          <t>Avai</t>
+        </is>
+      </c>
+      <c r="D740" t="inlineStr">
+        <is>
+          <t>Vila Nova</t>
+        </is>
+      </c>
+      <c r="E740" t="n">
+        <v>10.28</v>
+      </c>
+      <c r="F740" t="n">
+        <v>0.13</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily scrape output - 2026-09-12
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F740"/>
+  <dimension ref="A1:F757"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18672,10 +18672,10 @@
         </is>
       </c>
       <c r="E702" t="n">
-        <v>9.119999999999999</v>
+        <v>9.48</v>
       </c>
       <c r="F702" t="n">
-        <v>0.57</v>
+        <v>0.65</v>
       </c>
     </row>
     <row r="703">
@@ -18698,10 +18698,10 @@
         </is>
       </c>
       <c r="E703" t="n">
-        <v>10.29</v>
+        <v>10.69</v>
       </c>
       <c r="F703" t="n">
-        <v>-0.02</v>
+        <v>-0.05</v>
       </c>
     </row>
     <row r="704">
@@ -18724,10 +18724,10 @@
         </is>
       </c>
       <c r="E704" t="n">
-        <v>10.28</v>
+        <v>10.24</v>
       </c>
       <c r="F704" t="n">
-        <v>0.04</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="705">
@@ -18814,24 +18814,24 @@
       </c>
       <c r="B708" t="inlineStr">
         <is>
-          <t>Norway - 1st Division</t>
+          <t>Finland - Ykkosliiga</t>
         </is>
       </c>
       <c r="C708" t="inlineStr">
         <is>
-          <t>Bryne</t>
+          <t>Mikkelin Palloilijat</t>
         </is>
       </c>
       <c r="D708" t="inlineStr">
         <is>
-          <t>Stabaek</t>
+          <t>SJK Akatemia</t>
         </is>
       </c>
       <c r="E708" t="n">
-        <v>10.66</v>
+        <v>10.34</v>
       </c>
       <c r="F708" t="n">
-        <v>-0.64</v>
+        <v>1.05</v>
       </c>
     </row>
     <row r="709">
@@ -18840,24 +18840,24 @@
       </c>
       <c r="B709" t="inlineStr">
         <is>
-          <t>Poland - 1st Liga</t>
+          <t>Norway - 1st Division</t>
         </is>
       </c>
       <c r="C709" t="inlineStr">
         <is>
-          <t>Chrobry Glogow</t>
+          <t>Bryne</t>
         </is>
       </c>
       <c r="D709" t="inlineStr">
         <is>
-          <t>Pogon Siedlce</t>
+          <t>Stabaek</t>
         </is>
       </c>
       <c r="E709" t="n">
-        <v>10.73</v>
+        <v>10.66</v>
       </c>
       <c r="F709" t="n">
-        <v>1.57</v>
+        <v>-0.64</v>
       </c>
     </row>
     <row r="710">
@@ -18866,24 +18866,24 @@
       </c>
       <c r="B710" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="C710" t="inlineStr">
         <is>
-          <t>Zaglebie Lubin</t>
+          <t>Chrobry Glogow</t>
         </is>
       </c>
       <c r="D710" t="inlineStr">
         <is>
-          <t>GKS Katowice</t>
+          <t>Pogon Siedlce</t>
         </is>
       </c>
       <c r="E710" t="n">
-        <v>10.01</v>
+        <v>10.61</v>
       </c>
       <c r="F710" t="n">
-        <v>-0.07000000000000001</v>
+        <v>1.57</v>
       </c>
     </row>
     <row r="711">
@@ -18892,24 +18892,24 @@
       </c>
       <c r="B711" t="inlineStr">
         <is>
-          <t>Spain - Segunda</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="C711" t="inlineStr">
         <is>
-          <t>Cadiz</t>
+          <t>Ruch Chorzow</t>
         </is>
       </c>
       <c r="D711" t="inlineStr">
         <is>
-          <t>Las Palmas</t>
+          <t>Podbeskidzie Bielsko-Biala</t>
         </is>
       </c>
       <c r="E711" t="n">
-        <v>9.09</v>
+        <v>10.11</v>
       </c>
       <c r="F711" t="n">
-        <v>-0.15</v>
+        <v>0.61</v>
       </c>
     </row>
     <row r="712">
@@ -18918,24 +18918,24 @@
       </c>
       <c r="B712" t="inlineStr">
         <is>
-          <t>Spain - Segunda</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C712" t="inlineStr">
         <is>
-          <t>Cordoba</t>
+          <t>Gornik Zabrze</t>
         </is>
       </c>
       <c r="D712" t="inlineStr">
         <is>
-          <t>Almeria</t>
+          <t>Lech Poznan</t>
         </is>
       </c>
       <c r="E712" t="n">
-        <v>9.880000000000001</v>
+        <v>10.43</v>
       </c>
       <c r="F712" t="n">
-        <v>1.4</v>
+        <v>0.44</v>
       </c>
     </row>
     <row r="713">
@@ -18944,24 +18944,24 @@
       </c>
       <c r="B713" t="inlineStr">
         <is>
-          <t>Spain - Segunda</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C713" t="inlineStr">
         <is>
-          <t>FC Andorra</t>
+          <t>Slask Wroclaw</t>
         </is>
       </c>
       <c r="D713" t="inlineStr">
         <is>
-          <t>Real Sociedad II</t>
+          <t>Korona Kielce</t>
         </is>
       </c>
       <c r="E713" t="n">
-        <v>9.51</v>
+        <v>9.69</v>
       </c>
       <c r="F713" t="n">
-        <v>2.59</v>
+        <v>0.34</v>
       </c>
     </row>
     <row r="714">
@@ -18970,206 +18970,206 @@
       </c>
       <c r="B714" t="inlineStr">
         <is>
-          <t>Spain - Segunda</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C714" t="inlineStr">
         <is>
-          <t>Granada</t>
+          <t>Zaglebie Lubin</t>
         </is>
       </c>
       <c r="D714" t="inlineStr">
         <is>
-          <t>Albacete</t>
+          <t>GKS Katowice</t>
         </is>
       </c>
       <c r="E714" t="n">
-        <v>9.550000000000001</v>
+        <v>9.779999999999999</v>
       </c>
       <c r="F714" t="n">
-        <v>1.72</v>
+        <v>-0.05</v>
       </c>
     </row>
     <row r="715">
       <c r="A715" s="1" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B715" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Romania - Liga 1</t>
         </is>
       </c>
       <c r="C715" t="inlineStr">
         <is>
-          <t>Atletico Goianiense</t>
+          <t>Rapid Bucuresti</t>
         </is>
       </c>
       <c r="D715" t="inlineStr">
         <is>
-          <t>Criciuma</t>
+          <t>Voluntari</t>
         </is>
       </c>
       <c r="E715" t="n">
-        <v>10.47</v>
+        <v>9.640000000000001</v>
       </c>
       <c r="F715" t="n">
-        <v>0.54</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="716">
       <c r="A716" s="1" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B716" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Romania - Liga 1</t>
         </is>
       </c>
       <c r="C716" t="inlineStr">
         <is>
-          <t>Fortaleza</t>
+          <t>Sepsi</t>
         </is>
       </c>
       <c r="D716" t="inlineStr">
         <is>
-          <t>Ceara</t>
+          <t>CFR Cluj</t>
         </is>
       </c>
       <c r="E716" t="n">
-        <v>10.54</v>
+        <v>9.57</v>
       </c>
       <c r="F716" t="n">
-        <v>1.46</v>
+        <v>-0.12</v>
       </c>
     </row>
     <row r="717">
       <c r="A717" s="1" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B717" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="C717" t="inlineStr">
         <is>
-          <t>Gremio Novorizontino</t>
+          <t>Cadiz</t>
         </is>
       </c>
       <c r="D717" t="inlineStr">
         <is>
-          <t>Cuiaba</t>
+          <t>Las Palmas</t>
         </is>
       </c>
       <c r="E717" t="n">
-        <v>10.45</v>
+        <v>8.859999999999999</v>
       </c>
       <c r="F717" t="n">
-        <v>1.65</v>
+        <v>0.35</v>
       </c>
     </row>
     <row r="718">
       <c r="A718" s="1" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B718" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="C718" t="inlineStr">
         <is>
-          <t>Juventude</t>
+          <t>Cordoba</t>
         </is>
       </c>
       <c r="D718" t="inlineStr">
         <is>
-          <t>Athletic Club</t>
+          <t>Almeria</t>
         </is>
       </c>
       <c r="E718" t="n">
-        <v>10.04</v>
+        <v>10.2</v>
       </c>
       <c r="F718" t="n">
-        <v>1.85</v>
+        <v>1.38</v>
       </c>
     </row>
     <row r="719">
       <c r="A719" s="1" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B719" t="inlineStr">
         <is>
-          <t>Finland - Veikkausliiga</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="C719" t="inlineStr">
         <is>
-          <t>KuPS</t>
+          <t>FC Andorra</t>
         </is>
       </c>
       <c r="D719" t="inlineStr">
         <is>
-          <t>HJK Helsinki</t>
+          <t>Real Sociedad II</t>
         </is>
       </c>
       <c r="E719" t="n">
-        <v>10.09</v>
+        <v>9.33</v>
       </c>
       <c r="F719" t="n">
-        <v>0.4</v>
+        <v>2.43</v>
       </c>
     </row>
     <row r="720">
       <c r="A720" s="1" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B720" t="inlineStr">
         <is>
-          <t>Norway - 1st Division</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="C720" t="inlineStr">
         <is>
-          <t>Egersunds</t>
+          <t>Girona</t>
         </is>
       </c>
       <c r="D720" t="inlineStr">
         <is>
-          <t>Kongsvinger</t>
+          <t>Castellon</t>
         </is>
       </c>
       <c r="E720" t="n">
-        <v>10.66</v>
+        <v>9.16</v>
       </c>
       <c r="F720" t="n">
-        <v>-0.47</v>
+        <v>0.82</v>
       </c>
     </row>
     <row r="721">
       <c r="A721" s="1" t="n">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="B721" t="inlineStr">
         <is>
-          <t>Norway - 1st Division</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="C721" t="inlineStr">
         <is>
-          <t>Moss</t>
+          <t>Granada</t>
         </is>
       </c>
       <c r="D721" t="inlineStr">
         <is>
-          <t>Haugesund</t>
+          <t>Albacete</t>
         </is>
       </c>
       <c r="E721" t="n">
-        <v>11.2</v>
+        <v>9.609999999999999</v>
       </c>
       <c r="F721" t="n">
-        <v>-1.33</v>
+        <v>1.72</v>
       </c>
     </row>
     <row r="722">
@@ -19178,24 +19178,24 @@
       </c>
       <c r="B722" t="inlineStr">
         <is>
-          <t>Norway - 1st Division</t>
+          <t>Brazil - Serie B</t>
         </is>
       </c>
       <c r="C722" t="inlineStr">
         <is>
-          <t>Raufoss</t>
+          <t>Atletico Goianiense</t>
         </is>
       </c>
       <c r="D722" t="inlineStr">
         <is>
-          <t>Odd BK</t>
+          <t>Criciuma</t>
         </is>
       </c>
       <c r="E722" t="n">
-        <v>11.02</v>
+        <v>10.32</v>
       </c>
       <c r="F722" t="n">
-        <v>-2.09</v>
+        <v>0.55</v>
       </c>
     </row>
     <row r="723">
@@ -19204,24 +19204,24 @@
       </c>
       <c r="B723" t="inlineStr">
         <is>
-          <t>Norway - 1st Division</t>
+          <t>Brazil - Serie B</t>
         </is>
       </c>
       <c r="C723" t="inlineStr">
         <is>
-          <t>Sogndal</t>
+          <t>Fortaleza</t>
         </is>
       </c>
       <c r="D723" t="inlineStr">
         <is>
-          <t>Strommen</t>
+          <t>Ceara</t>
         </is>
       </c>
       <c r="E723" t="n">
-        <v>11.09</v>
+        <v>10.54</v>
       </c>
       <c r="F723" t="n">
-        <v>1.07</v>
+        <v>1.46</v>
       </c>
     </row>
     <row r="724">
@@ -19230,24 +19230,24 @@
       </c>
       <c r="B724" t="inlineStr">
         <is>
-          <t>Norway - 1st Division</t>
+          <t>Brazil - Serie B</t>
         </is>
       </c>
       <c r="C724" t="inlineStr">
         <is>
-          <t>Stromsgodset</t>
+          <t>Gremio Novorizontino</t>
         </is>
       </c>
       <c r="D724" t="inlineStr">
         <is>
-          <t>Sandnes Ulf</t>
+          <t>Cuiaba</t>
         </is>
       </c>
       <c r="E724" t="n">
-        <v>11.48</v>
+        <v>10.45</v>
       </c>
       <c r="F724" t="n">
-        <v>3.4</v>
+        <v>1.65</v>
       </c>
     </row>
     <row r="725">
@@ -19256,24 +19256,24 @@
       </c>
       <c r="B725" t="inlineStr">
         <is>
-          <t>Poland - 1st Liga</t>
+          <t>Brazil - Serie B</t>
         </is>
       </c>
       <c r="C725" t="inlineStr">
         <is>
-          <t>Odra Opole</t>
+          <t>Juventude</t>
         </is>
       </c>
       <c r="D725" t="inlineStr">
         <is>
-          <t>Stal Rzeszow</t>
+          <t>Athletic Club</t>
         </is>
       </c>
       <c r="E725" t="n">
-        <v>10.65</v>
+        <v>10.04</v>
       </c>
       <c r="F725" t="n">
-        <v>1.21</v>
+        <v>1.85</v>
       </c>
     </row>
     <row r="726">
@@ -19282,24 +19282,24 @@
       </c>
       <c r="B726" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Finland - Veikkausliiga</t>
         </is>
       </c>
       <c r="C726" t="inlineStr">
         <is>
-          <t>Legia Warsaw</t>
+          <t>KuPS</t>
         </is>
       </c>
       <c r="D726" t="inlineStr">
         <is>
-          <t>Widzew Lodz</t>
+          <t>HJK Helsinki</t>
         </is>
       </c>
       <c r="E726" t="n">
-        <v>9.789999999999999</v>
+        <v>10.05</v>
       </c>
       <c r="F726" t="n">
-        <v>1.65</v>
+        <v>0.66</v>
       </c>
     </row>
     <row r="727">
@@ -19308,24 +19308,24 @@
       </c>
       <c r="B727" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Iceland - 1. Deild</t>
         </is>
       </c>
       <c r="C727" t="inlineStr">
         <is>
-          <t>Wisla Plock</t>
+          <t>Throttur Reykjavik</t>
         </is>
       </c>
       <c r="D727" t="inlineStr">
         <is>
-          <t>Cracovia Krakow</t>
+          <t>UMF Njardvik</t>
         </is>
       </c>
       <c r="E727" t="n">
-        <v>10.72</v>
+        <v>11.55</v>
       </c>
       <c r="F727" t="n">
-        <v>0.38</v>
+        <v>1.03</v>
       </c>
     </row>
     <row r="728">
@@ -19334,24 +19334,24 @@
       </c>
       <c r="B728" t="inlineStr">
         <is>
-          <t>Romania - Liga 1</t>
+          <t>Norway - 1st Division</t>
         </is>
       </c>
       <c r="C728" t="inlineStr">
         <is>
-          <t>Arges Pitesti</t>
+          <t>Egersunds</t>
         </is>
       </c>
       <c r="D728" t="inlineStr">
         <is>
-          <t>Botosani</t>
+          <t>Kongsvinger</t>
         </is>
       </c>
       <c r="E728" t="n">
-        <v>9.6</v>
+        <v>10.66</v>
       </c>
       <c r="F728" t="n">
-        <v>1.06</v>
+        <v>-0.47</v>
       </c>
     </row>
     <row r="729">
@@ -19360,24 +19360,24 @@
       </c>
       <c r="B729" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Norway - 1st Division</t>
         </is>
       </c>
       <c r="C729" t="inlineStr">
         <is>
-          <t>Ljungskile</t>
+          <t>Hodd</t>
         </is>
       </c>
       <c r="D729" t="inlineStr">
         <is>
-          <t>Falkenbergs</t>
+          <t>Lyn</t>
         </is>
       </c>
       <c r="E729" t="n">
-        <v>10.29</v>
+        <v>10.7</v>
       </c>
       <c r="F729" t="n">
-        <v>0.9</v>
+        <v>-1.19</v>
       </c>
     </row>
     <row r="730">
@@ -19386,284 +19386,726 @@
       </c>
       <c r="B730" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Norway - 1st Division</t>
         </is>
       </c>
       <c r="C730" t="inlineStr">
         <is>
-          <t>Norrkoping</t>
+          <t>Moss</t>
         </is>
       </c>
       <c r="D730" t="inlineStr">
         <is>
-          <t>Oddevold</t>
+          <t>Haugesund</t>
         </is>
       </c>
       <c r="E730" t="n">
-        <v>10.16</v>
+        <v>11.2</v>
       </c>
       <c r="F730" t="n">
-        <v>1.97</v>
+        <v>-1.33</v>
       </c>
     </row>
     <row r="731">
       <c r="A731" s="1" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B731" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Norway - 1st Division</t>
         </is>
       </c>
       <c r="C731" t="inlineStr">
         <is>
-          <t>America Mineiro</t>
+          <t>Raufoss</t>
         </is>
       </c>
       <c r="D731" t="inlineStr">
         <is>
-          <t>Sao Bernardo</t>
+          <t>Odd BK</t>
         </is>
       </c>
       <c r="E731" t="n">
-        <v>10.63</v>
+        <v>11.02</v>
       </c>
       <c r="F731" t="n">
-        <v>1.01</v>
+        <v>-2.09</v>
       </c>
     </row>
     <row r="732">
       <c r="A732" s="1" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B732" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Norway - 1st Division</t>
         </is>
       </c>
       <c r="C732" t="inlineStr">
         <is>
-          <t>Botafogo SP</t>
+          <t>Sogndal</t>
         </is>
       </c>
       <c r="D732" t="inlineStr">
         <is>
-          <t>Goias</t>
+          <t>Strommen</t>
         </is>
       </c>
       <c r="E732" t="n">
-        <v>10.65</v>
+        <v>11.09</v>
       </c>
       <c r="F732" t="n">
-        <v>1.34</v>
+        <v>1.07</v>
       </c>
     </row>
     <row r="733">
       <c r="A733" s="1" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B733" t="inlineStr">
         <is>
-          <t>Finland - Veikkausliiga</t>
+          <t>Norway - 1st Division</t>
         </is>
       </c>
       <c r="C733" t="inlineStr">
         <is>
-          <t>Inter Turku</t>
+          <t>Stromsgodset</t>
         </is>
       </c>
       <c r="D733" t="inlineStr">
         <is>
-          <t>VPS</t>
+          <t>Sandnes Ulf</t>
         </is>
       </c>
       <c r="E733" t="n">
-        <v>9.84</v>
+        <v>11.48</v>
       </c>
       <c r="F733" t="n">
-        <v>1.88</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="734">
       <c r="A734" s="1" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B734" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="C734" t="inlineStr">
         <is>
-          <t>Radomiak Radom</t>
+          <t>Odra Opole</t>
         </is>
       </c>
       <c r="D734" t="inlineStr">
         <is>
-          <t>Piast Gliwice</t>
+          <t>Stal Rzeszow</t>
         </is>
       </c>
       <c r="E734" t="n">
-        <v>10.5</v>
+        <v>10.67</v>
       </c>
       <c r="F734" t="n">
-        <v>0.34</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="735">
       <c r="A735" s="1" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B735" t="inlineStr">
         <is>
-          <t>Romania - Liga 1</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C735" t="inlineStr">
         <is>
-          <t>FCSB</t>
+          <t>Legia Warsaw</t>
         </is>
       </c>
       <c r="D735" t="inlineStr">
         <is>
-          <t>Petrolul Ploiesti</t>
+          <t>Widzew Lodz</t>
         </is>
       </c>
       <c r="E735" t="n">
-        <v>10.11</v>
+        <v>9.789999999999999</v>
       </c>
       <c r="F735" t="n">
-        <v>3.25</v>
+        <v>1.65</v>
       </c>
     </row>
     <row r="736">
       <c r="A736" s="1" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B736" t="inlineStr">
         <is>
-          <t>Romania - Liga 1</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C736" t="inlineStr">
         <is>
-          <t>Universitatea Cluj</t>
+          <t>Wisla Plock</t>
         </is>
       </c>
       <c r="D736" t="inlineStr">
         <is>
-          <t>Otelul Galati</t>
+          <t>Cracovia Krakow</t>
         </is>
       </c>
       <c r="E736" t="n">
-        <v>9.66</v>
+        <v>10.72</v>
       </c>
       <c r="F736" t="n">
-        <v>1.54</v>
+        <v>0.38</v>
       </c>
     </row>
     <row r="737">
       <c r="A737" s="1" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B737" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Romania - Liga 1</t>
         </is>
       </c>
       <c r="C737" t="inlineStr">
         <is>
-          <t>Norrby</t>
+          <t>Arges Pitesti</t>
         </is>
       </c>
       <c r="D737" t="inlineStr">
         <is>
-          <t>Varbergs BoIS</t>
+          <t>Botosani</t>
         </is>
       </c>
       <c r="E737" t="n">
-        <v>10.55</v>
+        <v>9.6</v>
       </c>
       <c r="F737" t="n">
-        <v>-0.5600000000000001</v>
+        <v>1.06</v>
       </c>
     </row>
     <row r="738">
       <c r="A738" s="1" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B738" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="C738" t="inlineStr">
         <is>
-          <t>Orebro SK</t>
+          <t>Mallorca</t>
         </is>
       </c>
       <c r="D738" t="inlineStr">
         <is>
-          <t>Nordic United</t>
+          <t>Sabadell</t>
         </is>
       </c>
       <c r="E738" t="n">
-        <v>10.17</v>
+        <v>8.609999999999999</v>
       </c>
       <c r="F738" t="n">
-        <v>0.71</v>
+        <v>1.04</v>
       </c>
     </row>
     <row r="739">
       <c r="A739" s="1" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B739" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="C739" t="inlineStr">
         <is>
-          <t>Ostersunds FK</t>
+          <t>Real Valladolid</t>
         </is>
       </c>
       <c r="D739" t="inlineStr">
         <is>
-          <t>Helsingborgs</t>
+          <t>Real Oviedo</t>
         </is>
       </c>
       <c r="E739" t="n">
-        <v>9.98</v>
+        <v>8.609999999999999</v>
       </c>
       <c r="F739" t="n">
-        <v>1.46</v>
+        <v>0.72</v>
       </c>
     </row>
     <row r="740">
       <c r="A740" s="1" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B740" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C740" t="inlineStr">
+        <is>
+          <t>Sporting Gijon</t>
+        </is>
+      </c>
+      <c r="D740" t="inlineStr">
+        <is>
+          <t>Eldense</t>
+        </is>
+      </c>
+      <c r="E740" t="n">
+        <v>9.59</v>
+      </c>
+      <c r="F740" t="n">
+        <v>1.43</v>
+      </c>
+    </row>
+    <row r="741">
+      <c r="A741" s="1" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B741" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C741" t="inlineStr">
+        <is>
+          <t>Tenerife</t>
+        </is>
+      </c>
+      <c r="D741" t="inlineStr">
+        <is>
+          <t>Leganes</t>
+        </is>
+      </c>
+      <c r="E741" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="F741" t="n">
+        <v>1.38</v>
+      </c>
+    </row>
+    <row r="742">
+      <c r="A742" s="1" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B742" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C742" t="inlineStr">
+        <is>
+          <t>Ljungskile</t>
+        </is>
+      </c>
+      <c r="D742" t="inlineStr">
+        <is>
+          <t>Falkenbergs</t>
+        </is>
+      </c>
+      <c r="E742" t="n">
+        <v>10.29</v>
+      </c>
+      <c r="F742" t="n">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="743">
+      <c r="A743" s="1" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B743" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C743" t="inlineStr">
+        <is>
+          <t>Norrkoping</t>
+        </is>
+      </c>
+      <c r="D743" t="inlineStr">
+        <is>
+          <t>Oddevold</t>
+        </is>
+      </c>
+      <c r="E743" t="n">
+        <v>10.16</v>
+      </c>
+      <c r="F743" t="n">
+        <v>1.97</v>
+      </c>
+    </row>
+    <row r="744">
+      <c r="A744" s="1" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B744" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C744" t="inlineStr">
+        <is>
+          <t>America Mineiro</t>
+        </is>
+      </c>
+      <c r="D744" t="inlineStr">
+        <is>
+          <t>Sao Bernardo</t>
+        </is>
+      </c>
+      <c r="E744" t="n">
+        <v>10.63</v>
+      </c>
+      <c r="F744" t="n">
+        <v>1.01</v>
+      </c>
+    </row>
+    <row r="745">
+      <c r="A745" s="1" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B745" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C745" t="inlineStr">
+        <is>
+          <t>Botafogo SP</t>
+        </is>
+      </c>
+      <c r="D745" t="inlineStr">
+        <is>
+          <t>Goias</t>
+        </is>
+      </c>
+      <c r="E745" t="n">
+        <v>10.65</v>
+      </c>
+      <c r="F745" t="n">
+        <v>1.34</v>
+      </c>
+    </row>
+    <row r="746">
+      <c r="A746" s="1" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B746" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C746" t="inlineStr">
+        <is>
+          <t>Inter Turku</t>
+        </is>
+      </c>
+      <c r="D746" t="inlineStr">
+        <is>
+          <t>VPS</t>
+        </is>
+      </c>
+      <c r="E746" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="F746" t="n">
+        <v>1.88</v>
+      </c>
+    </row>
+    <row r="747">
+      <c r="A747" s="1" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B747" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C747" t="inlineStr">
+        <is>
+          <t>Radomiak Radom</t>
+        </is>
+      </c>
+      <c r="D747" t="inlineStr">
+        <is>
+          <t>Piast Gliwice</t>
+        </is>
+      </c>
+      <c r="E747" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="F747" t="n">
+        <v>0.34</v>
+      </c>
+    </row>
+    <row r="748">
+      <c r="A748" s="1" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B748" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C748" t="inlineStr">
+        <is>
+          <t>FCSB</t>
+        </is>
+      </c>
+      <c r="D748" t="inlineStr">
+        <is>
+          <t>Petrolul Ploiesti</t>
+        </is>
+      </c>
+      <c r="E748" t="n">
+        <v>10.11</v>
+      </c>
+      <c r="F748" t="n">
+        <v>3.25</v>
+      </c>
+    </row>
+    <row r="749">
+      <c r="A749" s="1" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B749" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C749" t="inlineStr">
+        <is>
+          <t>Universitatea Cluj</t>
+        </is>
+      </c>
+      <c r="D749" t="inlineStr">
+        <is>
+          <t>Otelul Galati</t>
+        </is>
+      </c>
+      <c r="E749" t="n">
+        <v>9.66</v>
+      </c>
+      <c r="F749" t="n">
+        <v>1.54</v>
+      </c>
+    </row>
+    <row r="750">
+      <c r="A750" s="1" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B750" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C750" t="inlineStr">
+        <is>
+          <t>Norrby</t>
+        </is>
+      </c>
+      <c r="D750" t="inlineStr">
+        <is>
+          <t>Varbergs BoIS</t>
+        </is>
+      </c>
+      <c r="E750" t="n">
+        <v>10.55</v>
+      </c>
+      <c r="F750" t="n">
+        <v>-0.5600000000000001</v>
+      </c>
+    </row>
+    <row r="751">
+      <c r="A751" s="1" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B751" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C751" t="inlineStr">
+        <is>
+          <t>Orebro SK</t>
+        </is>
+      </c>
+      <c r="D751" t="inlineStr">
+        <is>
+          <t>Nordic United</t>
+        </is>
+      </c>
+      <c r="E751" t="n">
+        <v>10.17</v>
+      </c>
+      <c r="F751" t="n">
+        <v>0.71</v>
+      </c>
+    </row>
+    <row r="752">
+      <c r="A752" s="1" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B752" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C752" t="inlineStr">
+        <is>
+          <t>Ostersunds FK</t>
+        </is>
+      </c>
+      <c r="D752" t="inlineStr">
+        <is>
+          <t>Helsingborgs</t>
+        </is>
+      </c>
+      <c r="E752" t="n">
+        <v>9.98</v>
+      </c>
+      <c r="F752" t="n">
+        <v>1.46</v>
+      </c>
+    </row>
+    <row r="753">
+      <c r="A753" s="1" t="n">
         <v>46280</v>
       </c>
-      <c r="B740" t="inlineStr">
+      <c r="B753" t="inlineStr">
         <is>
           <t>Brazil - Serie B</t>
         </is>
       </c>
-      <c r="C740" t="inlineStr">
+      <c r="C753" t="inlineStr">
         <is>
           <t>Avai</t>
         </is>
       </c>
-      <c r="D740" t="inlineStr">
+      <c r="D753" t="inlineStr">
         <is>
           <t>Vila Nova</t>
         </is>
       </c>
-      <c r="E740" t="n">
-        <v>10.28</v>
-      </c>
-      <c r="F740" t="n">
-        <v>0.13</v>
+      <c r="E753" t="n">
+        <v>9.82</v>
+      </c>
+      <c r="F753" t="n">
+        <v>0.17</v>
+      </c>
+    </row>
+    <row r="754">
+      <c r="A754" s="1" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B754" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C754" t="inlineStr">
+        <is>
+          <t>Nautico</t>
+        </is>
+      </c>
+      <c r="D754" t="inlineStr">
+        <is>
+          <t>Operario Ferroviario</t>
+        </is>
+      </c>
+      <c r="E754" t="n">
+        <v>10.69</v>
+      </c>
+      <c r="F754" t="n">
+        <v>2.09</v>
+      </c>
+    </row>
+    <row r="755">
+      <c r="A755" s="1" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B755" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C755" t="inlineStr">
+        <is>
+          <t>Brage</t>
+        </is>
+      </c>
+      <c r="D755" t="inlineStr">
+        <is>
+          <t>Sandvikens IF</t>
+        </is>
+      </c>
+      <c r="E755" t="n">
+        <v>10.55</v>
+      </c>
+      <c r="F755" t="n">
+        <v>-0.17</v>
+      </c>
+    </row>
+    <row r="756">
+      <c r="A756" s="1" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B756" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C756" t="inlineStr">
+        <is>
+          <t>Landskrona</t>
+        </is>
+      </c>
+      <c r="D756" t="inlineStr">
+        <is>
+          <t>Sundsvall</t>
+        </is>
+      </c>
+      <c r="E756" t="n">
+        <v>10.39</v>
+      </c>
+      <c r="F756" t="n">
+        <v>2.43</v>
+      </c>
+    </row>
+    <row r="757">
+      <c r="A757" s="1" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B757" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C757" t="inlineStr">
+        <is>
+          <t>Varnamo</t>
+        </is>
+      </c>
+      <c r="D757" t="inlineStr">
+        <is>
+          <t>Osters</t>
+        </is>
+      </c>
+      <c r="E757" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="F757" t="n">
+        <v>1.35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>